<commit_message>
Ajoute le systeme de filtres par categorie (solo + multijoueur), separe cinema/television de culture
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -2276,7 +2276,7 @@
     <t xml:space="preserve">Le nom du Monde à l’envers a été choisi après plusieurs variantes dans les documents de conception.</t>
   </si>
   <si>
-    <t xml:space="preserve">The Office (US)</t>
+    <t xml:space="preserve">The Office</t>
   </si>
   <si>
     <t xml:space="preserve">Une comédie de bureau au faux style documentaire devient un classique du genre.</t>
@@ -2411,7 +2411,7 @@
     <t xml:space="preserve">Jeu vidéo &amp; eSport</t>
   </si>
   <si>
-    <t xml:space="preserve">Sortie de Fortnite</t>
+    <t xml:space="preserve">Fortnite</t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu de bataille royale gratuit conquiert des centaines de millions de joueurs.</t>
@@ -2423,7 +2423,7 @@
     <t xml:space="preserve">Un concert virtuel dans le jeu a rassemblé plus de 12 millions de joueurs simultanés.</t>
   </si>
   <si>
-    <t xml:space="preserve">Création de Valorant</t>
+    <t xml:space="preserve">Valorant</t>
   </si>
   <si>
     <t xml:space="preserve">Un nouveau FPS tactique bouscule la scène compétitive établie.</t>
@@ -2435,7 +2435,7 @@
     <t xml:space="preserve">Sa structure eSport a été planifiée dès la conception avec le soutien direct de l’éditeur.</t>
   </si>
   <si>
-    <t xml:space="preserve">League of Legends devient un phénomène culturel</t>
+    <t xml:space="preserve">League of Legends </t>
   </si>
   <si>
     <t xml:space="preserve">Un MOBA révolutionne la compétition mondiale et crée une communauté record.</t>
@@ -2447,7 +2447,7 @@
     <t xml:space="preserve">Son championnat mondial annuel est devenu l’un des événements eSport les plus suivis au monde.</t>
   </si>
   <si>
-    <t xml:space="preserve">Minecraft révolutionne la construction libre</t>
+    <t xml:space="preserve">Minecraft </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu de blocs minimaliste devient un phénomène éducatif et ludique sans égal.</t>
@@ -2459,7 +2459,7 @@
     <t xml:space="preserve">Le jeu a servi à reconstituer virtuellement du patrimoine mondial, notamment Notre-Dame avant l’incendie.</t>
   </si>
   <si>
-    <t xml:space="preserve">GTA V sort et dépasse tous les records financiers</t>
+    <t xml:space="preserve">GTA V </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action en monde ouvert devient le plus lucratif jamais créé.</t>
@@ -2471,7 +2471,7 @@
     <t xml:space="preserve">Le jeu a généré plusieurs milliards de dollars de revenus.</t>
   </si>
   <si>
-    <t xml:space="preserve">The Last of Us redéfinit la narration vidéoludique</t>
+    <t xml:space="preserve">The Last of Us </t>
   </si>
   <si>
     <t xml:space="preserve">Une fresque émotionnelle explore le lien parent-enfant en zone post-apocalyptique.</t>
@@ -2483,7 +2483,7 @@
     <t xml:space="preserve">Il a remporté de nombreux prix de jeu de l’année et inspiré une adaptation télévisée mondiale.</t>
   </si>
   <si>
-    <t xml:space="preserve">God of War redéfinit la franchise</t>
+    <t xml:space="preserve">God of War </t>
   </si>
   <si>
     <t xml:space="preserve">Une relance complète transforme un héros mythique dans un univers nordique.</t>
@@ -2495,7 +2495,7 @@
     <t xml:space="preserve">Son tournant créatif a inspiré d’autres studios à réimaginer leurs franchises.</t>
   </si>
   <si>
-    <t xml:space="preserve">Age of Empires fonde le jeu de stratégie en temps réel</t>
+    <t xml:space="preserve">Age of Empires l</t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu de stratégie en temps réel pose des bases durables du genre.</t>
@@ -2507,7 +2507,7 @@
     <t xml:space="preserve">Son équilibre et son accessibilité ont favorisé l’apparition de tournois informels dès sa sortie.</t>
   </si>
   <si>
-    <t xml:space="preserve">Counter-Strike 2 modernise la série</t>
+    <t xml:space="preserve">Counter-Strike 2 </t>
   </si>
   <si>
     <t xml:space="preserve">Une évolution moderne du FPS tactique perpétue les fondamentaux de Counter-Strike.</t>
@@ -2519,7 +2519,7 @@
     <t xml:space="preserve">La série a conservé une très large base de joueurs compétitifs.</t>
   </si>
   <si>
-    <t xml:space="preserve">Counter-Strike Global Offensive règne sur l’eSport</t>
+    <t xml:space="preserve">Counter-Strike Global Offensive </t>
   </si>
   <si>
     <t xml:space="preserve">Un FPS tactique devient l’étalon-or de la compétition eSport.</t>
@@ -2531,7 +2531,7 @@
     <t xml:space="preserve">Ses Majors internationaux ont proposé des dotations de plusieurs millions de dollars.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dark Souls 1 crée le sous-genre Souls-like</t>
+    <t xml:space="preserve">Dark Souls 1 </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action-RPG redéfinit la difficulté et le level-design.</t>
@@ -2543,7 +2543,7 @@
     <t xml:space="preserve">Sa difficulté a attiré une communauté durable de joueurs en quête de défi.</t>
   </si>
   <si>
-    <t xml:space="preserve">Elden Ring synthétise une vision</t>
+    <t xml:space="preserve">Elden Ring </t>
   </si>
   <si>
     <t xml:space="preserve">Un opus spectaculaire fusionne Souls-like et monde ouvert.</t>
@@ -2555,7 +2555,7 @@
     <t xml:space="preserve">Sa difficulté et son level-design ont contribué à populariser le terme « Souls-like » et à inspirer de nombreux jeux.</t>
   </si>
   <si>
-    <t xml:space="preserve">Outer Wilds explore l’impossible</t>
+    <t xml:space="preserve">Outer Wilds </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu de puzzle et d’exploration défie la physique et la perception.</t>
@@ -2567,7 +2567,7 @@
     <t xml:space="preserve">Il ne contient aucune violence et repose entièrement sur la curiosité et la découverte.</t>
   </si>
   <si>
-    <t xml:space="preserve">GTA San Andreas établit un standard</t>
+    <t xml:space="preserve">GTA San Andreas </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action en monde ouvert explore la culture urbaine.</t>
@@ -2579,7 +2579,7 @@
     <t xml:space="preserve">Des communautés créent encore des mods et extensions plus de vingt ans après sa sortie.</t>
   </si>
   <si>
-    <t xml:space="preserve">GTA IV redéfinit le réalisme</t>
+    <t xml:space="preserve">GTA IV </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action en monde ouvert explore une métropole américaine fictive et ses tensions sociales.</t>
@@ -2591,7 +2591,7 @@
     <t xml:space="preserve">Des centaines de mods, du cosmétique à la refonte totale, existent encore.</t>
   </si>
   <si>
-    <t xml:space="preserve">GTA Vice City capture une époque</t>
+    <t xml:space="preserve">GTA Vice City </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action en monde ouvert explore une métropole côtière fictive et la criminalité organisée.</t>
@@ -2603,7 +2603,7 @@
     <t xml:space="preserve">Son esthétique synthwave a durablement marqué la culture populaire.</t>
   </si>
   <si>
-    <t xml:space="preserve">GTA New York reste une légende urbaine</t>
+    <t xml:space="preserve">GTA 3</t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’action en monde ouvert parodie le crime urbain.</t>
@@ -2615,7 +2615,7 @@
     <t xml:space="preserve">Ces épisodes ont contribué à faire de GTA une licence emblématique du jeu vidéo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Outlast propose l’horreur pure</t>
+    <t xml:space="preserve">Outlast 1</t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu d’horreur interdit toute arme aux joueurs.</t>
@@ -2627,7 +2627,7 @@
     <t xml:space="preserve">Le jeu a popularisé les expériences d’horreur fondées sur la vulnérabilité totale.</t>
   </si>
   <si>
-    <t xml:space="preserve">Subnautica 1 explore l’inconnu aquatique</t>
+    <t xml:space="preserve">Subnautica 1 </t>
   </si>
   <si>
     <t xml:space="preserve">Un jeu de survie en monde aquatique alien propose une exploration libre.</t>
@@ -2639,7 +2639,7 @@
     <t xml:space="preserve">Son océan crée une peur existentielle de l’inconnu sans reposer uniquement sur des monstres.</t>
   </si>
   <si>
-    <t xml:space="preserve">Call of Duty marque l’ère FPS moderne</t>
+    <t xml:space="preserve">Call of Duty </t>
   </si>
   <si>
     <t xml:space="preserve">Une franchise FPS domine le marché grand public.</t>
@@ -5367,11 +5367,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="1.74"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="1" width="37.03"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="28.17"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="1.7"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="1" width="49.46"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="32.76"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="50.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="31.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="77.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="1" width="11.53"/>
@@ -5719,7 +5719,10 @@
       <c r="H11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="4"/>
+      <c r="I11" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H11)-1)&amp;".png"</f>
+        <v>id-10.png</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
@@ -5746,7 +5749,10 @@
       <c r="H12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="4"/>
+      <c r="I12" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H12)-1)&amp;".png"</f>
+        <v>id-11.png</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
@@ -5773,7 +5779,10 @@
       <c r="H13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I13" s="4"/>
+      <c r="I13" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H13)-1)&amp;".png"</f>
+        <v>id-12.png</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
@@ -5800,7 +5809,10 @@
       <c r="H14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I14" s="4"/>
+      <c r="I14" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H14)-1)&amp;".png"</f>
+        <v>id-13.png</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
@@ -5827,7 +5839,10 @@
       <c r="H15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I15" s="4"/>
+      <c r="I15" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H15)-1)&amp;".png"</f>
+        <v>id-14.png</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
@@ -5854,7 +5869,10 @@
       <c r="H16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="4"/>
+      <c r="I16" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H16)-1)&amp;".png"</f>
+        <v>id-15.png</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
@@ -5881,7 +5899,10 @@
       <c r="H17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="4"/>
+      <c r="I17" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H17)-1)&amp;".png"</f>
+        <v>id-16.png</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
@@ -5908,7 +5929,10 @@
       <c r="H18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I18" s="4"/>
+      <c r="I18" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H18)-1)&amp;".png"</f>
+        <v>id-17.png</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
@@ -5935,7 +5959,10 @@
       <c r="H19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I19" s="4"/>
+      <c r="I19" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H19)-1)&amp;".png"</f>
+        <v>id-18.png</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
@@ -5962,7 +5989,10 @@
       <c r="H20" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I20" s="4"/>
+      <c r="I20" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H20)-1)&amp;".png"</f>
+        <v>id-19.png</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
@@ -5989,7 +6019,10 @@
       <c r="H21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="4"/>
+      <c r="I21" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H21)-1)&amp;".png"</f>
+        <v>id-20.png</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
@@ -6016,7 +6049,10 @@
       <c r="H22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="4"/>
+      <c r="I22" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H22)-1)&amp;".png"</f>
+        <v>id-21.png</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
@@ -6043,7 +6079,10 @@
       <c r="H23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I23" s="4"/>
+      <c r="I23" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H23)-1)&amp;".png"</f>
+        <v>id-22.png</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
@@ -6070,7 +6109,10 @@
       <c r="H24" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I24" s="4"/>
+      <c r="I24" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H24)-1)&amp;".png"</f>
+        <v>id-23.png</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
@@ -6097,7 +6139,10 @@
       <c r="H25" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I25" s="4"/>
+      <c r="I25" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H25)-1)&amp;".png"</f>
+        <v>id-24.png</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
@@ -6124,7 +6169,10 @@
       <c r="H26" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I26" s="4"/>
+      <c r="I26" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H26)-1)&amp;".png"</f>
+        <v>id-25.png</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
@@ -6151,7 +6199,10 @@
       <c r="H27" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I27" s="4"/>
+      <c r="I27" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H27)-1)&amp;".png"</f>
+        <v>id-26.png</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
@@ -6178,7 +6229,10 @@
       <c r="H28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I28" s="4"/>
+      <c r="I28" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H28)-1)&amp;".png"</f>
+        <v>id-27.png</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
@@ -6205,7 +6259,10 @@
       <c r="H29" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="4"/>
+      <c r="I29" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H29)-1)&amp;".png"</f>
+        <v>id-28.png</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
@@ -6232,7 +6289,10 @@
       <c r="H30" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I30" s="4"/>
+      <c r="I30" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H30)-1)&amp;".png"</f>
+        <v>id-29.png</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
@@ -6259,7 +6319,10 @@
       <c r="H31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I31" s="4"/>
+      <c r="I31" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H31)-1)&amp;".png"</f>
+        <v>id-30.png</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
@@ -6286,7 +6349,10 @@
       <c r="H32" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I32" s="4"/>
+      <c r="I32" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H32)-1)&amp;".png"</f>
+        <v>id-31.png</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
@@ -6313,7 +6379,10 @@
       <c r="H33" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I33" s="4"/>
+      <c r="I33" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H33)-1)&amp;".png"</f>
+        <v>id-32.png</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
@@ -6340,7 +6409,10 @@
       <c r="H34" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I34" s="4"/>
+      <c r="I34" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H34)-1)&amp;".png"</f>
+        <v>id-33.png</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
@@ -6367,7 +6439,10 @@
       <c r="H35" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I35" s="4"/>
+      <c r="I35" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H35)-1)&amp;".png"</f>
+        <v>id-34.png</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
@@ -6394,7 +6469,10 @@
       <c r="H36" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I36" s="4"/>
+      <c r="I36" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H36)-1)&amp;".png"</f>
+        <v>id-35.png</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
@@ -6421,7 +6499,10 @@
       <c r="H37" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I37" s="4"/>
+      <c r="I37" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H37)-1)&amp;".png"</f>
+        <v>id-36.png</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
@@ -6448,7 +6529,10 @@
       <c r="H38" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I38" s="4"/>
+      <c r="I38" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H38)-1)&amp;".png"</f>
+        <v>id-37.png</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
@@ -6475,7 +6559,10 @@
       <c r="H39" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I39" s="4"/>
+      <c r="I39" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H39)-1)&amp;".png"</f>
+        <v>id-38.png</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
@@ -6502,7 +6589,10 @@
       <c r="H40" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I40" s="4"/>
+      <c r="I40" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H40)-1)&amp;".png"</f>
+        <v>id-39.png</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="n">
@@ -6529,7 +6619,10 @@
       <c r="H41" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I41" s="4"/>
+      <c r="I41" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H41)-1)&amp;".png"</f>
+        <v>id-40.png</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="n">
@@ -6556,7 +6649,10 @@
       <c r="H42" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I42" s="4"/>
+      <c r="I42" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H42)-1)&amp;".png"</f>
+        <v>id-41.png</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="n">
@@ -6583,7 +6679,10 @@
       <c r="H43" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I43" s="4"/>
+      <c r="I43" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H43)-1)&amp;".png"</f>
+        <v>id-42.png</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="n">
@@ -6610,7 +6709,10 @@
       <c r="H44" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I44" s="4"/>
+      <c r="I44" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H44)-1)&amp;".png"</f>
+        <v>id-43.png</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="n">
@@ -6637,7 +6739,10 @@
       <c r="H45" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I45" s="4"/>
+      <c r="I45" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H45)-1)&amp;".png"</f>
+        <v>id-44.png</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="n">
@@ -6664,7 +6769,10 @@
       <c r="H46" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I46" s="4"/>
+      <c r="I46" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H46)-1)&amp;".png"</f>
+        <v>id-45.png</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="n">
@@ -6691,7 +6799,10 @@
       <c r="H47" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I47" s="4"/>
+      <c r="I47" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H47)-1)&amp;".png"</f>
+        <v>id-46.png</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="n">
@@ -6718,7 +6829,10 @@
       <c r="H48" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I48" s="4"/>
+      <c r="I48" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H48)-1)&amp;".png"</f>
+        <v>id-47.png</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="n">
@@ -6745,7 +6859,10 @@
       <c r="H49" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I49" s="4"/>
+      <c r="I49" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H49)-1)&amp;".png"</f>
+        <v>id-48.png</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="n">
@@ -6772,7 +6889,10 @@
       <c r="H50" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I50" s="4"/>
+      <c r="I50" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H50)-1)&amp;".png"</f>
+        <v>id-49.png</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="n">
@@ -6799,7 +6919,10 @@
       <c r="H51" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I51" s="4"/>
+      <c r="I51" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H51)-1)&amp;".png"</f>
+        <v>id-50.png</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
@@ -6826,7 +6949,10 @@
       <c r="H52" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I52" s="4"/>
+      <c r="I52" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H52)-1)&amp;".png"</f>
+        <v>id-51.png</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
@@ -6853,7 +6979,10 @@
       <c r="H53" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I53" s="4"/>
+      <c r="I53" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H53)-1)&amp;".png"</f>
+        <v>id-52.png</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
@@ -6880,7 +7009,10 @@
       <c r="H54" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I54" s="4"/>
+      <c r="I54" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H54)-1)&amp;".png"</f>
+        <v>id-53.png</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="n">
@@ -6907,7 +7039,10 @@
       <c r="H55" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I55" s="4"/>
+      <c r="I55" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H55)-1)&amp;".png"</f>
+        <v>id-54.png</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="n">
@@ -6934,7 +7069,10 @@
       <c r="H56" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I56" s="4"/>
+      <c r="I56" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H56)-1)&amp;".png"</f>
+        <v>id-55.png</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="n">
@@ -6961,7 +7099,10 @@
       <c r="H57" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I57" s="4"/>
+      <c r="I57" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H57)-1)&amp;".png"</f>
+        <v>id-56.png</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="n">
@@ -6988,7 +7129,10 @@
       <c r="H58" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I58" s="4"/>
+      <c r="I58" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H58)-1)&amp;".png"</f>
+        <v>id-57.png</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="n">
@@ -7015,7 +7159,10 @@
       <c r="H59" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I59" s="4"/>
+      <c r="I59" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H59)-1)&amp;".png"</f>
+        <v>id-58.png</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="n">
@@ -7042,7 +7189,10 @@
       <c r="H60" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I60" s="4"/>
+      <c r="I60" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H60)-1)&amp;".png"</f>
+        <v>id-59.png</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="n">
@@ -7069,7 +7219,10 @@
       <c r="H61" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I61" s="4"/>
+      <c r="I61" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H61)-1)&amp;".png"</f>
+        <v>id-60.png</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="n">
@@ -7096,7 +7249,10 @@
       <c r="H62" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I62" s="4"/>
+      <c r="I62" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H62)-1)&amp;".png"</f>
+        <v>id-61.png</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="n">
@@ -7123,7 +7279,10 @@
       <c r="H63" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I63" s="4"/>
+      <c r="I63" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H63)-1)&amp;".png"</f>
+        <v>id-62.png</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="n">
@@ -7150,7 +7309,10 @@
       <c r="H64" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I64" s="4"/>
+      <c r="I64" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H64)-1)&amp;".png"</f>
+        <v>id-63.png</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="n">
@@ -7177,7 +7339,10 @@
       <c r="H65" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I65" s="4"/>
+      <c r="I65" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H65)-1)&amp;".png"</f>
+        <v>id-64.png</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="n">
@@ -7204,7 +7369,10 @@
       <c r="H66" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I66" s="4"/>
+      <c r="I66" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H66)-1)&amp;".png"</f>
+        <v>id-65.png</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="n">
@@ -7231,7 +7399,10 @@
       <c r="H67" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I67" s="4"/>
+      <c r="I67" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H67)-1)&amp;".png"</f>
+        <v>id-66.png</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="n">
@@ -7258,7 +7429,10 @@
       <c r="H68" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I68" s="4"/>
+      <c r="I68" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H68)-1)&amp;".png"</f>
+        <v>id-67.png</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="n">
@@ -7285,7 +7459,10 @@
       <c r="H69" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I69" s="4"/>
+      <c r="I69" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H69)-1)&amp;".png"</f>
+        <v>id-68.png</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="n">
@@ -7312,7 +7489,10 @@
       <c r="H70" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I70" s="4"/>
+      <c r="I70" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H70)-1)&amp;".png"</f>
+        <v>id-69.png</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="n">
@@ -7339,7 +7519,10 @@
       <c r="H71" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I71" s="4"/>
+      <c r="I71" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H71)-1)&amp;".png"</f>
+        <v>id-70.png</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="n">
@@ -7366,7 +7549,10 @@
       <c r="H72" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I72" s="4"/>
+      <c r="I72" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H72)-1)&amp;".png"</f>
+        <v>id-71.png</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="n">
@@ -7393,7 +7579,10 @@
       <c r="H73" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I73" s="4"/>
+      <c r="I73" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H73)-1)&amp;".png"</f>
+        <v>id-72.png</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="n">
@@ -7420,7 +7609,10 @@
       <c r="H74" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I74" s="4"/>
+      <c r="I74" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H74)-1)&amp;".png"</f>
+        <v>id-73.png</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="n">
@@ -7447,7 +7639,10 @@
       <c r="H75" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I75" s="4"/>
+      <c r="I75" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H75)-1)&amp;".png"</f>
+        <v>id-74.png</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="n">
@@ -7474,7 +7669,10 @@
       <c r="H76" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I76" s="4"/>
+      <c r="I76" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H76)-1)&amp;".png"</f>
+        <v>id-75.png</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="n">
@@ -7501,7 +7699,10 @@
       <c r="H77" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I77" s="4"/>
+      <c r="I77" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H77)-1)&amp;".png"</f>
+        <v>id-76.png</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="n">
@@ -7528,7 +7729,10 @@
       <c r="H78" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I78" s="4"/>
+      <c r="I78" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H78)-1)&amp;".png"</f>
+        <v>id-77.png</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="n">
@@ -7555,7 +7759,10 @@
       <c r="H79" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I79" s="4"/>
+      <c r="I79" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H79)-1)&amp;".png"</f>
+        <v>id-78.png</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="n">
@@ -7582,7 +7789,10 @@
       <c r="H80" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I80" s="4"/>
+      <c r="I80" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H80)-1)&amp;".png"</f>
+        <v>id-79.png</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="n">
@@ -7609,7 +7819,10 @@
       <c r="H81" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I81" s="4"/>
+      <c r="I81" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H81)-1)&amp;".png"</f>
+        <v>id-80.png</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="n">
@@ -7636,7 +7849,10 @@
       <c r="H82" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I82" s="4"/>
+      <c r="I82" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H82)-1)&amp;".png"</f>
+        <v>id-81.png</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="n">
@@ -7663,7 +7879,10 @@
       <c r="H83" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I83" s="4"/>
+      <c r="I83" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H83)-1)&amp;".png"</f>
+        <v>id-82.png</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="n">
@@ -7690,7 +7909,10 @@
       <c r="H84" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I84" s="4"/>
+      <c r="I84" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H84)-1)&amp;".png"</f>
+        <v>id-83.png</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="n">
@@ -7717,7 +7939,10 @@
       <c r="H85" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I85" s="4"/>
+      <c r="I85" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H85)-1)&amp;".png"</f>
+        <v>id-84.png</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="n">
@@ -7744,7 +7969,10 @@
       <c r="H86" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I86" s="4"/>
+      <c r="I86" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H86)-1)&amp;".png"</f>
+        <v>id-85.png</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="n">
@@ -7771,7 +7999,10 @@
       <c r="H87" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I87" s="4"/>
+      <c r="I87" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H87)-1)&amp;".png"</f>
+        <v>id-86.png</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="n">
@@ -7798,7 +8029,10 @@
       <c r="H88" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I88" s="4"/>
+      <c r="I88" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H88)-1)&amp;".png"</f>
+        <v>id-87.png</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="n">
@@ -7825,7 +8059,10 @@
       <c r="H89" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I89" s="4"/>
+      <c r="I89" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H89)-1)&amp;".png"</f>
+        <v>id-88.png</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="n">
@@ -7852,7 +8089,10 @@
       <c r="H90" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I90" s="4"/>
+      <c r="I90" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H90)-1)&amp;".png"</f>
+        <v>id-89.png</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="n">
@@ -7879,7 +8119,10 @@
       <c r="H91" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I91" s="4"/>
+      <c r="I91" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H91)-1)&amp;".png"</f>
+        <v>id-90.png</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="n">
@@ -7906,7 +8149,10 @@
       <c r="H92" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I92" s="4"/>
+      <c r="I92" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H92)-1)&amp;".png"</f>
+        <v>id-91.png</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="n">
@@ -7933,7 +8179,10 @@
       <c r="H93" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I93" s="4"/>
+      <c r="I93" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H93)-1)&amp;".png"</f>
+        <v>id-92.png</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="n">
@@ -7960,7 +8209,10 @@
       <c r="H94" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I94" s="4"/>
+      <c r="I94" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H94)-1)&amp;".png"</f>
+        <v>id-93.png</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="n">
@@ -7987,7 +8239,10 @@
       <c r="H95" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I95" s="4"/>
+      <c r="I95" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H95)-1)&amp;".png"</f>
+        <v>id-94.png</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="n">
@@ -8014,7 +8269,10 @@
       <c r="H96" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I96" s="4"/>
+      <c r="I96" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H96)-1)&amp;".png"</f>
+        <v>id-95.png</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="n">
@@ -8041,7 +8299,10 @@
       <c r="H97" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I97" s="4"/>
+      <c r="I97" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H97)-1)&amp;".png"</f>
+        <v>id-96.png</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="n">
@@ -8068,7 +8329,10 @@
       <c r="H98" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I98" s="4"/>
+      <c r="I98" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H98)-1)&amp;".png"</f>
+        <v>id-97.png</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="n">
@@ -8095,7 +8359,10 @@
       <c r="H99" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I99" s="4"/>
+      <c r="I99" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H99)-1)&amp;".png"</f>
+        <v>id-98.png</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="n">
@@ -8122,7 +8389,10 @@
       <c r="H100" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I100" s="4"/>
+      <c r="I100" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H100)-1)&amp;".png"</f>
+        <v>id-99.png</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="n">
@@ -8149,7 +8419,10 @@
       <c r="H101" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I101" s="4"/>
+      <c r="I101" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H101)-1)&amp;".png"</f>
+        <v>id-100.png</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="n">
@@ -8176,7 +8449,10 @@
       <c r="H102" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I102" s="4"/>
+      <c r="I102" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H102)-1)&amp;".png"</f>
+        <v>id-101.png</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="n">
@@ -8203,7 +8479,10 @@
       <c r="H103" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I103" s="4"/>
+      <c r="I103" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H103)-1)&amp;".png"</f>
+        <v>id-102.png</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="n">
@@ -8230,7 +8509,10 @@
       <c r="H104" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I104" s="4"/>
+      <c r="I104" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H104)-1)&amp;".png"</f>
+        <v>id-103.png</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="n">
@@ -8257,7 +8539,10 @@
       <c r="H105" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I105" s="4"/>
+      <c r="I105" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H105)-1)&amp;".png"</f>
+        <v>id-104.png</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="n">
@@ -8284,7 +8569,10 @@
       <c r="H106" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I106" s="4"/>
+      <c r="I106" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H106)-1)&amp;".png"</f>
+        <v>id-105.png</v>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="n">
@@ -8311,7 +8599,10 @@
       <c r="H107" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I107" s="4"/>
+      <c r="I107" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H107)-1)&amp;".png"</f>
+        <v>id-106.png</v>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="n">
@@ -8338,7 +8629,10 @@
       <c r="H108" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I108" s="4"/>
+      <c r="I108" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H108)-1)&amp;".png"</f>
+        <v>id-107.png</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="n">
@@ -8365,7 +8659,10 @@
       <c r="H109" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I109" s="4"/>
+      <c r="I109" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H109)-1)&amp;".png"</f>
+        <v>id-108.png</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="n">
@@ -8392,7 +8689,10 @@
       <c r="H110" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I110" s="4"/>
+      <c r="I110" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H110)-1)&amp;".png"</f>
+        <v>id-109.png</v>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="n">
@@ -8419,7 +8719,10 @@
       <c r="H111" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I111" s="4"/>
+      <c r="I111" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H111)-1)&amp;".png"</f>
+        <v>id-110.png</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="n">
@@ -8446,7 +8749,10 @@
       <c r="H112" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I112" s="4"/>
+      <c r="I112" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H112)-1)&amp;".png"</f>
+        <v>id-111.png</v>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="n">
@@ -8473,7 +8779,10 @@
       <c r="H113" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I113" s="4"/>
+      <c r="I113" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H113)-1)&amp;".png"</f>
+        <v>id-112.png</v>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="n">
@@ -8500,7 +8809,10 @@
       <c r="H114" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I114" s="4"/>
+      <c r="I114" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H114)-1)&amp;".png"</f>
+        <v>id-113.png</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="n">
@@ -8527,7 +8839,10 @@
       <c r="H115" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I115" s="4"/>
+      <c r="I115" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H115)-1)&amp;".png"</f>
+        <v>id-114.png</v>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="n">
@@ -8554,7 +8869,10 @@
       <c r="H116" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I116" s="4"/>
+      <c r="I116" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H116)-1)&amp;".png"</f>
+        <v>id-115.png</v>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="n">
@@ -8581,7 +8899,10 @@
       <c r="H117" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I117" s="4"/>
+      <c r="I117" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H117)-1)&amp;".png"</f>
+        <v>id-116.png</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="n">
@@ -8608,7 +8929,10 @@
       <c r="H118" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I118" s="4"/>
+      <c r="I118" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H118)-1)&amp;".png"</f>
+        <v>id-117.png</v>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="n">
@@ -8635,7 +8959,10 @@
       <c r="H119" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I119" s="4"/>
+      <c r="I119" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H119)-1)&amp;".png"</f>
+        <v>id-118.png</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="n">
@@ -8662,7 +8989,10 @@
       <c r="H120" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I120" s="4"/>
+      <c r="I120" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H120)-1)&amp;".png"</f>
+        <v>id-119.png</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="n">
@@ -8689,7 +9019,10 @@
       <c r="H121" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I121" s="4"/>
+      <c r="I121" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H121)-1)&amp;".png"</f>
+        <v>id-120.png</v>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="n">
@@ -8716,7 +9049,10 @@
       <c r="H122" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I122" s="4"/>
+      <c r="I122" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H122)-1)&amp;".png"</f>
+        <v>id-121.png</v>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="n">
@@ -8743,7 +9079,10 @@
       <c r="H123" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I123" s="4"/>
+      <c r="I123" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H123)-1)&amp;".png"</f>
+        <v>id-122.png</v>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="n">
@@ -8770,7 +9109,10 @@
       <c r="H124" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I124" s="4"/>
+      <c r="I124" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H124)-1)&amp;".png"</f>
+        <v>id-123.png</v>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="n">
@@ -8797,7 +9139,10 @@
       <c r="H125" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I125" s="4"/>
+      <c r="I125" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H125)-1)&amp;".png"</f>
+        <v>id-124.png</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="n">
@@ -8824,7 +9169,10 @@
       <c r="H126" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I126" s="4"/>
+      <c r="I126" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H126)-1)&amp;".png"</f>
+        <v>id-125.png</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="n">
@@ -8851,7 +9199,10 @@
       <c r="H127" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I127" s="4"/>
+      <c r="I127" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H127)-1)&amp;".png"</f>
+        <v>id-126.png</v>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="n">
@@ -8878,7 +9229,10 @@
       <c r="H128" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I128" s="4"/>
+      <c r="I128" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H128)-1)&amp;".png"</f>
+        <v>id-127.png</v>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="n">
@@ -8905,7 +9259,10 @@
       <c r="H129" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I129" s="4"/>
+      <c r="I129" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H129)-1)&amp;".png"</f>
+        <v>id-128.png</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="n">
@@ -8932,7 +9289,10 @@
       <c r="H130" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I130" s="4"/>
+      <c r="I130" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H130)-1)&amp;".png"</f>
+        <v>id-129.png</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="n">
@@ -8959,7 +9319,10 @@
       <c r="H131" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I131" s="4"/>
+      <c r="I131" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H131)-1)&amp;".png"</f>
+        <v>id-130.png</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="n">
@@ -8986,7 +9349,10 @@
       <c r="H132" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I132" s="4"/>
+      <c r="I132" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H132)-1)&amp;".png"</f>
+        <v>id-131.png</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="n">
@@ -9013,7 +9379,10 @@
       <c r="H133" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I133" s="4"/>
+      <c r="I133" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H133)-1)&amp;".png"</f>
+        <v>id-132.png</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="n">
@@ -9040,7 +9409,10 @@
       <c r="H134" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I134" s="4"/>
+      <c r="I134" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H134)-1)&amp;".png"</f>
+        <v>id-133.png</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="n">
@@ -9067,7 +9439,10 @@
       <c r="H135" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I135" s="4"/>
+      <c r="I135" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H135)-1)&amp;".png"</f>
+        <v>id-134.png</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="n">
@@ -9094,7 +9469,10 @@
       <c r="H136" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I136" s="4"/>
+      <c r="I136" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H136)-1)&amp;".png"</f>
+        <v>id-135.png</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="n">
@@ -9121,7 +9499,10 @@
       <c r="H137" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I137" s="4"/>
+      <c r="I137" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H137)-1)&amp;".png"</f>
+        <v>id-136.png</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="n">
@@ -9148,7 +9529,10 @@
       <c r="H138" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I138" s="4"/>
+      <c r="I138" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H138)-1)&amp;".png"</f>
+        <v>id-137.png</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="n">
@@ -9175,7 +9559,10 @@
       <c r="H139" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I139" s="4"/>
+      <c r="I139" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H139)-1)&amp;".png"</f>
+        <v>id-138.png</v>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="n">
@@ -9202,7 +9589,10 @@
       <c r="H140" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I140" s="4"/>
+      <c r="I140" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H140)-1)&amp;".png"</f>
+        <v>id-139.png</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="n">
@@ -9229,7 +9619,10 @@
       <c r="H141" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I141" s="4"/>
+      <c r="I141" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H141)-1)&amp;".png"</f>
+        <v>id-140.png</v>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="n">
@@ -9256,7 +9649,10 @@
       <c r="H142" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I142" s="4"/>
+      <c r="I142" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H142)-1)&amp;".png"</f>
+        <v>id-141.png</v>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="n">
@@ -9283,7 +9679,10 @@
       <c r="H143" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I143" s="4"/>
+      <c r="I143" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H143)-1)&amp;".png"</f>
+        <v>id-142.png</v>
+      </c>
     </row>
     <row r="144" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="n">
@@ -9310,7 +9709,10 @@
       <c r="H144" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I144" s="4"/>
+      <c r="I144" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H144)-1)&amp;".png"</f>
+        <v>id-143.png</v>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="n">
@@ -9337,7 +9739,10 @@
       <c r="H145" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I145" s="4"/>
+      <c r="I145" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H145)-1)&amp;".png"</f>
+        <v>id-144.png</v>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="n">
@@ -9364,7 +9769,10 @@
       <c r="H146" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I146" s="4"/>
+      <c r="I146" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H146)-1)&amp;".png"</f>
+        <v>id-145.png</v>
+      </c>
     </row>
     <row r="147" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="n">
@@ -9391,7 +9799,10 @@
       <c r="H147" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I147" s="4"/>
+      <c r="I147" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H147)-1)&amp;".png"</f>
+        <v>id-146.png</v>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="n">
@@ -9418,7 +9829,10 @@
       <c r="H148" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I148" s="4"/>
+      <c r="I148" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H148)-1)&amp;".png"</f>
+        <v>id-147.png</v>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="n">
@@ -9445,7 +9859,10 @@
       <c r="H149" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I149" s="4"/>
+      <c r="I149" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H149)-1)&amp;".png"</f>
+        <v>id-148.png</v>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="n">
@@ -9472,7 +9889,10 @@
       <c r="H150" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I150" s="4"/>
+      <c r="I150" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H150)-1)&amp;".png"</f>
+        <v>id-149.png</v>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="n">
@@ -9499,7 +9919,10 @@
       <c r="H151" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I151" s="4"/>
+      <c r="I151" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H151)-1)&amp;".png"</f>
+        <v>id-150.png</v>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="n">
@@ -9526,7 +9949,10 @@
       <c r="H152" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I152" s="4"/>
+      <c r="I152" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H152)-1)&amp;".png"</f>
+        <v>id-151.png</v>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="n">
@@ -9553,7 +9979,10 @@
       <c r="H153" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I153" s="4"/>
+      <c r="I153" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H153)-1)&amp;".png"</f>
+        <v>id-152.png</v>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="n">
@@ -9580,7 +10009,10 @@
       <c r="H154" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I154" s="4"/>
+      <c r="I154" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H154)-1)&amp;".png"</f>
+        <v>id-153.png</v>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="n">
@@ -9607,7 +10039,10 @@
       <c r="H155" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I155" s="4"/>
+      <c r="I155" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H155)-1)&amp;".png"</f>
+        <v>id-154.png</v>
+      </c>
     </row>
     <row r="156" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="n">
@@ -9634,7 +10069,10 @@
       <c r="H156" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I156" s="4"/>
+      <c r="I156" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H156)-1)&amp;".png"</f>
+        <v>id-155.png</v>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="n">
@@ -9661,7 +10099,10 @@
       <c r="H157" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I157" s="4"/>
+      <c r="I157" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H157)-1)&amp;".png"</f>
+        <v>id-156.png</v>
+      </c>
     </row>
     <row r="158" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="n">
@@ -9688,7 +10129,10 @@
       <c r="H158" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I158" s="4"/>
+      <c r="I158" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H158)-1)&amp;".png"</f>
+        <v>id-157.png</v>
+      </c>
     </row>
     <row r="159" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="n">
@@ -9715,7 +10159,10 @@
       <c r="H159" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I159" s="4"/>
+      <c r="I159" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H159)-1)&amp;".png"</f>
+        <v>id-158.png</v>
+      </c>
     </row>
     <row r="160" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="n">
@@ -9742,7 +10189,10 @@
       <c r="H160" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I160" s="4"/>
+      <c r="I160" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H160)-1)&amp;".png"</f>
+        <v>id-159.png</v>
+      </c>
     </row>
     <row r="161" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="n">
@@ -9769,7 +10219,10 @@
       <c r="H161" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I161" s="4"/>
+      <c r="I161" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H161)-1)&amp;".png"</f>
+        <v>id-160.png</v>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="n">
@@ -9796,7 +10249,10 @@
       <c r="H162" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I162" s="4"/>
+      <c r="I162" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H162)-1)&amp;".png"</f>
+        <v>id-161.png</v>
+      </c>
     </row>
     <row r="163" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="n">
@@ -9823,7 +10279,10 @@
       <c r="H163" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I163" s="4"/>
+      <c r="I163" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H163)-1)&amp;".png"</f>
+        <v>id-162.png</v>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="n">
@@ -9850,7 +10309,10 @@
       <c r="H164" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I164" s="4"/>
+      <c r="I164" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H164)-1)&amp;".png"</f>
+        <v>id-163.png</v>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="n">
@@ -9877,7 +10339,10 @@
       <c r="H165" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I165" s="4"/>
+      <c r="I165" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H165)-1)&amp;".png"</f>
+        <v>id-164.png</v>
+      </c>
     </row>
     <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="n">
@@ -9904,7 +10369,10 @@
       <c r="H166" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I166" s="4"/>
+      <c r="I166" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H166)-1)&amp;".png"</f>
+        <v>id-165.png</v>
+      </c>
     </row>
     <row r="167" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="n">
@@ -9931,7 +10399,10 @@
       <c r="H167" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I167" s="4"/>
+      <c r="I167" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H167)-1)&amp;".png"</f>
+        <v>id-166.png</v>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="n">
@@ -9958,7 +10429,10 @@
       <c r="H168" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I168" s="4"/>
+      <c r="I168" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H168)-1)&amp;".png"</f>
+        <v>id-167.png</v>
+      </c>
     </row>
     <row r="169" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="n">
@@ -9985,7 +10459,10 @@
       <c r="H169" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I169" s="4"/>
+      <c r="I169" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H169)-1)&amp;".png"</f>
+        <v>id-168.png</v>
+      </c>
     </row>
     <row r="170" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="n">
@@ -10012,7 +10489,10 @@
       <c r="H170" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I170" s="4"/>
+      <c r="I170" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H170)-1)&amp;".png"</f>
+        <v>id-169.png</v>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="n">
@@ -10039,7 +10519,10 @@
       <c r="H171" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I171" s="4"/>
+      <c r="I171" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H171)-1)&amp;".png"</f>
+        <v>id-170.png</v>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="n">
@@ -10066,7 +10549,10 @@
       <c r="H172" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I172" s="4"/>
+      <c r="I172" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H172)-1)&amp;".png"</f>
+        <v>id-171.png</v>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="n">
@@ -10093,7 +10579,10 @@
       <c r="H173" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I173" s="4"/>
+      <c r="I173" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H173)-1)&amp;".png"</f>
+        <v>id-172.png</v>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="n">
@@ -10120,7 +10609,10 @@
       <c r="H174" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I174" s="4"/>
+      <c r="I174" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H174)-1)&amp;".png"</f>
+        <v>id-173.png</v>
+      </c>
     </row>
     <row r="175" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="n">
@@ -10147,7 +10639,10 @@
       <c r="H175" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I175" s="4"/>
+      <c r="I175" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H175)-1)&amp;".png"</f>
+        <v>id-174.png</v>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="n">
@@ -10174,7 +10669,10 @@
       <c r="H176" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I176" s="4"/>
+      <c r="I176" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H176)-1)&amp;".png"</f>
+        <v>id-175.png</v>
+      </c>
     </row>
     <row r="177" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="n">
@@ -10201,7 +10699,10 @@
       <c r="H177" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I177" s="4"/>
+      <c r="I177" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H177)-1)&amp;".png"</f>
+        <v>id-176.png</v>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="n">
@@ -10228,7 +10729,10 @@
       <c r="H178" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I178" s="4"/>
+      <c r="I178" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H178)-1)&amp;".png"</f>
+        <v>id-177.png</v>
+      </c>
     </row>
     <row r="179" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="n">
@@ -10255,7 +10759,10 @@
       <c r="H179" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I179" s="4"/>
+      <c r="I179" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H179)-1)&amp;".png"</f>
+        <v>id-178.png</v>
+      </c>
     </row>
     <row r="180" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="n">
@@ -10282,7 +10789,10 @@
       <c r="H180" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I180" s="4"/>
+      <c r="I180" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H180)-1)&amp;".png"</f>
+        <v>id-179.png</v>
+      </c>
     </row>
     <row r="181" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="n">
@@ -10309,7 +10819,10 @@
       <c r="H181" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I181" s="4"/>
+      <c r="I181" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H181)-1)&amp;".png"</f>
+        <v>id-180.png</v>
+      </c>
     </row>
     <row r="182" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="4" t="n">
@@ -10336,7 +10849,10 @@
       <c r="H182" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I182" s="4"/>
+      <c r="I182" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H182)-1)&amp;".png"</f>
+        <v>id-181.png</v>
+      </c>
     </row>
     <row r="183" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="n">
@@ -10363,7 +10879,10 @@
       <c r="H183" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I183" s="4"/>
+      <c r="I183" s="4" t="str">
+        <f aca="false">"id-"&amp;(ROW(H183)-1)&amp;".png"</f>
+        <v>id-182.png</v>
+      </c>
     </row>
     <row r="184" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="4" t="n">
@@ -10916,7 +11435,7 @@
         <v>868</v>
       </c>
       <c r="D202" s="4" t="n">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="E202" s="5" t="s">
         <v>869</v>

</xml_diff>

<commit_message>
Scroll molette horizontal sur la timeline/poubelle, renomme en Poubelle, logo en jeu reprend le texte TIMELINE (sans sablier ni mini-cartes)
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -278,7 +278,7 @@
     <t xml:space="preserve">Cléopâtre était en réalité d'origine grecque macédonienne, descendante des généraux d'Alexandre le Grand — elle aurait été la première de sa dynastie à réellement apprendre l'égyptien.</t>
   </si>
   <si>
-    <t xml:space="preserve">Jules César, dictateur à vie</t>
+    <t xml:space="preserve">Jules César, Empereur</t>
   </si>
   <si>
     <t xml:space="preserve">Jules César est nommé dictateur perpétuel peu avant son assassinat.</t>
@@ -5361,7 +5361,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K247"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="44.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.97"/>
@@ -5377,7 +5377,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
@@ -5475,7 +5475,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
@@ -5508,7 +5508,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
@@ -5541,7 +5541,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
@@ -5574,7 +5574,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>id-6.png</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>id-7.png</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
@@ -5664,7 +5664,7 @@
         <v>id-8.png</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
@@ -5694,7 +5694,7 @@
         <v>id-9.png</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>id-10.png</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
@@ -5754,7 +5754,7 @@
         <v>id-11.png</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>id-12.png</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>id-13.png</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>id-14.png</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
@@ -5874,7 +5874,7 @@
         <v>id-15.png</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
@@ -5904,7 +5904,7 @@
         <v>id-16.png</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
@@ -5934,7 +5934,7 @@
         <v>id-17.png</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
@@ -5964,7 +5964,7 @@
         <v>id-18.png</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
@@ -5994,7 +5994,7 @@
         <v>id-19.png</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
@@ -6024,7 +6024,7 @@
         <v>id-20.png</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
@@ -6054,7 +6054,7 @@
         <v>id-21.png</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
@@ -6084,7 +6084,7 @@
         <v>id-22.png</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
@@ -6114,7 +6114,7 @@
         <v>id-23.png</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
@@ -6144,7 +6144,7 @@
         <v>id-24.png</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
         <v>25</v>
       </c>
@@ -6174,7 +6174,7 @@
         <v>id-25.png</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>id-26.png</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
         <v>27</v>
       </c>
@@ -6234,7 +6234,7 @@
         <v>id-27.png</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>id-28.png</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
@@ -6294,7 +6294,7 @@
         <v>id-29.png</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>id-30.png</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <v>31</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>id-31.png</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
         <v>32</v>
       </c>
@@ -6384,7 +6384,7 @@
         <v>id-32.png</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <v>33</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>id-33.png</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
         <v>34</v>
       </c>
@@ -6444,7 +6444,7 @@
         <v>id-34.png</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
         <v>35</v>
       </c>
@@ -6474,7 +6474,7 @@
         <v>id-35.png</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
         <v>36</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>id-36.png</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
         <v>37</v>
       </c>
@@ -6534,7 +6534,7 @@
         <v>id-37.png</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
         <v>38</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>id-38.png</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
         <v>39</v>
       </c>
@@ -6594,7 +6594,7 @@
         <v>id-39.png</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="n">
         <v>40</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>id-40.png</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="n">
         <v>41</v>
       </c>
@@ -6654,7 +6654,7 @@
         <v>id-41.png</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="n">
         <v>42</v>
       </c>
@@ -6684,7 +6684,7 @@
         <v>id-42.png</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="n">
         <v>43</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>id-43.png</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="n">
         <v>44</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>id-44.png</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="n">
         <v>45</v>
       </c>
@@ -6774,7 +6774,7 @@
         <v>id-45.png</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="n">
         <v>46</v>
       </c>
@@ -6804,7 +6804,7 @@
         <v>id-46.png</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="n">
         <v>47</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>id-47.png</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="n">
         <v>48</v>
       </c>
@@ -6864,7 +6864,7 @@
         <v>id-48.png</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="n">
         <v>49</v>
       </c>
@@ -6894,7 +6894,7 @@
         <v>id-49.png</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="n">
         <v>50</v>
       </c>
@@ -6924,7 +6924,7 @@
         <v>id-50.png</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
         <v>51</v>
       </c>
@@ -6954,7 +6954,7 @@
         <v>id-51.png</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
         <v>52</v>
       </c>
@@ -6984,7 +6984,7 @@
         <v>id-52.png</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
         <v>53</v>
       </c>
@@ -7014,7 +7014,7 @@
         <v>id-53.png</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="n">
         <v>54</v>
       </c>
@@ -7044,7 +7044,7 @@
         <v>id-54.png</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="n">
         <v>55</v>
       </c>
@@ -7074,7 +7074,7 @@
         <v>id-55.png</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="n">
         <v>56</v>
       </c>
@@ -7104,7 +7104,7 @@
         <v>id-56.png</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="n">
         <v>57</v>
       </c>
@@ -7134,7 +7134,7 @@
         <v>id-57.png</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="n">
         <v>58</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>id-58.png</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="n">
         <v>59</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>id-59.png</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="n">
         <v>60</v>
       </c>
@@ -7224,7 +7224,7 @@
         <v>id-60.png</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="n">
         <v>61</v>
       </c>
@@ -7254,7 +7254,7 @@
         <v>id-61.png</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="n">
         <v>62</v>
       </c>
@@ -7284,7 +7284,7 @@
         <v>id-62.png</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="n">
         <v>63</v>
       </c>
@@ -7314,7 +7314,7 @@
         <v>id-63.png</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="n">
         <v>64</v>
       </c>
@@ -7344,7 +7344,7 @@
         <v>id-64.png</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="n">
         <v>65</v>
       </c>
@@ -7374,7 +7374,7 @@
         <v>id-65.png</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="n">
         <v>66</v>
       </c>
@@ -7404,7 +7404,7 @@
         <v>id-66.png</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="n">
         <v>67</v>
       </c>
@@ -7434,7 +7434,7 @@
         <v>id-67.png</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="n">
         <v>68</v>
       </c>
@@ -7464,7 +7464,7 @@
         <v>id-68.png</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="n">
         <v>69</v>
       </c>
@@ -7494,7 +7494,7 @@
         <v>id-69.png</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="n">
         <v>70</v>
       </c>
@@ -7524,7 +7524,7 @@
         <v>id-70.png</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="n">
         <v>71</v>
       </c>
@@ -7554,7 +7554,7 @@
         <v>id-71.png</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="n">
         <v>72</v>
       </c>
@@ -7584,7 +7584,7 @@
         <v>id-72.png</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="n">
         <v>73</v>
       </c>
@@ -7614,7 +7614,7 @@
         <v>id-73.png</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="n">
         <v>74</v>
       </c>
@@ -7644,7 +7644,7 @@
         <v>id-74.png</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="n">
         <v>75</v>
       </c>
@@ -7674,7 +7674,7 @@
         <v>id-75.png</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="n">
         <v>76</v>
       </c>
@@ -7704,7 +7704,7 @@
         <v>id-76.png</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="n">
         <v>77</v>
       </c>
@@ -7734,7 +7734,7 @@
         <v>id-77.png</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="n">
         <v>78</v>
       </c>
@@ -7764,7 +7764,7 @@
         <v>id-78.png</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="n">
         <v>79</v>
       </c>
@@ -7794,7 +7794,7 @@
         <v>id-79.png</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="n">
         <v>80</v>
       </c>
@@ -7824,7 +7824,7 @@
         <v>id-80.png</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="n">
         <v>81</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>id-81.png</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="n">
         <v>82</v>
       </c>
@@ -7884,7 +7884,7 @@
         <v>id-82.png</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="n">
         <v>83</v>
       </c>
@@ -7914,7 +7914,7 @@
         <v>id-83.png</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="n">
         <v>84</v>
       </c>
@@ -7944,7 +7944,7 @@
         <v>id-84.png</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="n">
         <v>85</v>
       </c>
@@ -7974,7 +7974,7 @@
         <v>id-85.png</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="n">
         <v>86</v>
       </c>
@@ -8004,7 +8004,7 @@
         <v>id-86.png</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="n">
         <v>87</v>
       </c>
@@ -8034,7 +8034,7 @@
         <v>id-87.png</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="n">
         <v>88</v>
       </c>
@@ -8064,7 +8064,7 @@
         <v>id-88.png</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="n">
         <v>89</v>
       </c>
@@ -8094,7 +8094,7 @@
         <v>id-89.png</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="n">
         <v>90</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>id-90.png</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="n">
         <v>91</v>
       </c>
@@ -8154,7 +8154,7 @@
         <v>id-91.png</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="n">
         <v>92</v>
       </c>
@@ -8184,7 +8184,7 @@
         <v>id-92.png</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="n">
         <v>93</v>
       </c>
@@ -8214,7 +8214,7 @@
         <v>id-93.png</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="n">
         <v>94</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>id-94.png</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="n">
         <v>95</v>
       </c>
@@ -8274,7 +8274,7 @@
         <v>id-95.png</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="n">
         <v>96</v>
       </c>
@@ -8304,7 +8304,7 @@
         <v>id-96.png</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="n">
         <v>97</v>
       </c>
@@ -8334,7 +8334,7 @@
         <v>id-97.png</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="n">
         <v>98</v>
       </c>
@@ -8364,7 +8364,7 @@
         <v>id-98.png</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="n">
         <v>99</v>
       </c>
@@ -8394,7 +8394,7 @@
         <v>id-99.png</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="n">
         <v>100</v>
       </c>
@@ -8424,7 +8424,7 @@
         <v>id-100.png</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="n">
         <v>101</v>
       </c>
@@ -8454,7 +8454,7 @@
         <v>id-101.png</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="n">
         <v>102</v>
       </c>
@@ -8484,7 +8484,7 @@
         <v>id-102.png</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="n">
         <v>103</v>
       </c>
@@ -8514,7 +8514,7 @@
         <v>id-103.png</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="n">
         <v>104</v>
       </c>
@@ -8544,7 +8544,7 @@
         <v>id-104.png</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="n">
         <v>105</v>
       </c>
@@ -8574,7 +8574,7 @@
         <v>id-105.png</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="n">
         <v>106</v>
       </c>
@@ -8604,7 +8604,7 @@
         <v>id-106.png</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="n">
         <v>107</v>
       </c>
@@ -8634,7 +8634,7 @@
         <v>id-107.png</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="n">
         <v>108</v>
       </c>
@@ -8664,7 +8664,7 @@
         <v>id-108.png</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="n">
         <v>109</v>
       </c>
@@ -8694,7 +8694,7 @@
         <v>id-109.png</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="n">
         <v>110</v>
       </c>
@@ -8724,7 +8724,7 @@
         <v>id-110.png</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="n">
         <v>111</v>
       </c>
@@ -8754,7 +8754,7 @@
         <v>id-111.png</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="n">
         <v>112</v>
       </c>
@@ -8784,7 +8784,7 @@
         <v>id-112.png</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="n">
         <v>113</v>
       </c>
@@ -8814,7 +8814,7 @@
         <v>id-113.png</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="n">
         <v>114</v>
       </c>
@@ -8844,7 +8844,7 @@
         <v>id-114.png</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="n">
         <v>115</v>
       </c>
@@ -8874,7 +8874,7 @@
         <v>id-115.png</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="n">
         <v>116</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>id-116.png</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="n">
         <v>117</v>
       </c>
@@ -8934,7 +8934,7 @@
         <v>id-117.png</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="n">
         <v>118</v>
       </c>
@@ -8964,7 +8964,7 @@
         <v>id-118.png</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="n">
         <v>119</v>
       </c>
@@ -8994,7 +8994,7 @@
         <v>id-119.png</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="n">
         <v>120</v>
       </c>
@@ -9024,7 +9024,7 @@
         <v>id-120.png</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="n">
         <v>121</v>
       </c>
@@ -9054,7 +9054,7 @@
         <v>id-121.png</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="n">
         <v>122</v>
       </c>
@@ -9084,7 +9084,7 @@
         <v>id-122.png</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="n">
         <v>123</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>id-123.png</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="n">
         <v>124</v>
       </c>
@@ -9144,7 +9144,7 @@
         <v>id-124.png</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="n">
         <v>125</v>
       </c>
@@ -9174,7 +9174,7 @@
         <v>id-125.png</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="n">
         <v>126</v>
       </c>
@@ -9204,7 +9204,7 @@
         <v>id-126.png</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="n">
         <v>127</v>
       </c>
@@ -9234,7 +9234,7 @@
         <v>id-127.png</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="n">
         <v>128</v>
       </c>
@@ -9264,7 +9264,7 @@
         <v>id-128.png</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="n">
         <v>129</v>
       </c>
@@ -9294,7 +9294,7 @@
         <v>id-129.png</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="n">
         <v>130</v>
       </c>
@@ -9324,7 +9324,7 @@
         <v>id-130.png</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="n">
         <v>131</v>
       </c>
@@ -9354,7 +9354,7 @@
         <v>id-131.png</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="n">
         <v>132</v>
       </c>
@@ -9384,7 +9384,7 @@
         <v>id-132.png</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="n">
         <v>133</v>
       </c>
@@ -9414,7 +9414,7 @@
         <v>id-133.png</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="n">
         <v>134</v>
       </c>
@@ -9444,7 +9444,7 @@
         <v>id-134.png</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="n">
         <v>135</v>
       </c>
@@ -9474,7 +9474,7 @@
         <v>id-135.png</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="n">
         <v>136</v>
       </c>
@@ -9504,7 +9504,7 @@
         <v>id-136.png</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="n">
         <v>137</v>
       </c>
@@ -9534,7 +9534,7 @@
         <v>id-137.png</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="n">
         <v>138</v>
       </c>
@@ -9564,7 +9564,7 @@
         <v>id-138.png</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="n">
         <v>139</v>
       </c>
@@ -9594,7 +9594,7 @@
         <v>id-139.png</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="n">
         <v>140</v>
       </c>
@@ -9624,7 +9624,7 @@
         <v>id-140.png</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="n">
         <v>141</v>
       </c>
@@ -9654,7 +9654,7 @@
         <v>id-141.png</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="n">
         <v>142</v>
       </c>
@@ -9684,7 +9684,7 @@
         <v>id-142.png</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="n">
         <v>143</v>
       </c>
@@ -9714,7 +9714,7 @@
         <v>id-143.png</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="n">
         <v>144</v>
       </c>
@@ -9744,7 +9744,7 @@
         <v>id-144.png</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="n">
         <v>145</v>
       </c>
@@ -9774,7 +9774,7 @@
         <v>id-145.png</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="n">
         <v>146</v>
       </c>
@@ -9804,7 +9804,7 @@
         <v>id-146.png</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="n">
         <v>147</v>
       </c>
@@ -9834,7 +9834,7 @@
         <v>id-147.png</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="n">
         <v>148</v>
       </c>
@@ -9864,7 +9864,7 @@
         <v>id-148.png</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="n">
         <v>149</v>
       </c>
@@ -9894,7 +9894,7 @@
         <v>id-149.png</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="n">
         <v>150</v>
       </c>
@@ -9924,7 +9924,7 @@
         <v>id-150.png</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="n">
         <v>151</v>
       </c>
@@ -9954,7 +9954,7 @@
         <v>id-151.png</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="n">
         <v>152</v>
       </c>
@@ -9984,7 +9984,7 @@
         <v>id-152.png</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="n">
         <v>153</v>
       </c>
@@ -10014,7 +10014,7 @@
         <v>id-153.png</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="n">
         <v>154</v>
       </c>
@@ -10044,7 +10044,7 @@
         <v>id-154.png</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="n">
         <v>155</v>
       </c>
@@ -10074,7 +10074,7 @@
         <v>id-155.png</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="n">
         <v>156</v>
       </c>
@@ -10104,7 +10104,7 @@
         <v>id-156.png</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="n">
         <v>157</v>
       </c>
@@ -10134,7 +10134,7 @@
         <v>id-157.png</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="n">
         <v>158</v>
       </c>
@@ -10164,7 +10164,7 @@
         <v>id-158.png</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="n">
         <v>159</v>
       </c>
@@ -10194,7 +10194,7 @@
         <v>id-159.png</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="n">
         <v>160</v>
       </c>
@@ -10224,7 +10224,7 @@
         <v>id-160.png</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="n">
         <v>161</v>
       </c>
@@ -10254,7 +10254,7 @@
         <v>id-161.png</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="n">
         <v>162</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>id-162.png</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="n">
         <v>163</v>
       </c>
@@ -10314,7 +10314,7 @@
         <v>id-163.png</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="n">
         <v>164</v>
       </c>
@@ -10344,7 +10344,7 @@
         <v>id-164.png</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="n">
         <v>165</v>
       </c>
@@ -10374,7 +10374,7 @@
         <v>id-165.png</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="n">
         <v>166</v>
       </c>
@@ -10404,7 +10404,7 @@
         <v>id-166.png</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="n">
         <v>167</v>
       </c>
@@ -10434,7 +10434,7 @@
         <v>id-167.png</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="n">
         <v>168</v>
       </c>
@@ -10464,7 +10464,7 @@
         <v>id-168.png</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="n">
         <v>169</v>
       </c>
@@ -10494,7 +10494,7 @@
         <v>id-169.png</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="n">
         <v>170</v>
       </c>
@@ -10524,7 +10524,7 @@
         <v>id-170.png</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="n">
         <v>171</v>
       </c>
@@ -10554,7 +10554,7 @@
         <v>id-171.png</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="n">
         <v>172</v>
       </c>
@@ -10584,7 +10584,7 @@
         <v>id-172.png</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="n">
         <v>173</v>
       </c>
@@ -10614,7 +10614,7 @@
         <v>id-173.png</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="n">
         <v>174</v>
       </c>
@@ -10644,7 +10644,7 @@
         <v>id-174.png</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="n">
         <v>175</v>
       </c>
@@ -10674,7 +10674,7 @@
         <v>id-175.png</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="n">
         <v>176</v>
       </c>
@@ -10704,7 +10704,7 @@
         <v>id-176.png</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="n">
         <v>177</v>
       </c>
@@ -10734,7 +10734,7 @@
         <v>id-177.png</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="n">
         <v>178</v>
       </c>
@@ -10764,7 +10764,7 @@
         <v>id-178.png</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="n">
         <v>179</v>
       </c>
@@ -10794,7 +10794,7 @@
         <v>id-179.png</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="n">
         <v>180</v>
       </c>
@@ -10824,7 +10824,7 @@
         <v>id-180.png</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="4" t="n">
         <v>181</v>
       </c>
@@ -10854,7 +10854,7 @@
         <v>id-181.png</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="n">
         <v>182</v>
       </c>
@@ -10884,7 +10884,7 @@
         <v>id-182.png</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="4" t="n">
         <v>183</v>
       </c>
@@ -10914,7 +10914,7 @@
         <v>id-183.png</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="4" t="n">
         <v>184</v>
       </c>
@@ -10944,7 +10944,7 @@
         <v>id-184.png</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="4" t="n">
         <v>185</v>
       </c>
@@ -10974,7 +10974,7 @@
         <v>id-185.png</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="4" t="n">
         <v>186</v>
       </c>
@@ -11004,7 +11004,7 @@
         <v>id-186.png</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="4" t="n">
         <v>187</v>
       </c>
@@ -11034,7 +11034,7 @@
         <v>id-187.png</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="4" t="n">
         <v>188</v>
       </c>
@@ -11064,7 +11064,7 @@
         <v>id-188.png</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="4" t="n">
         <v>189</v>
       </c>
@@ -11094,7 +11094,7 @@
         <v>id-189.png</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="4" t="n">
         <v>190</v>
       </c>
@@ -11124,7 +11124,7 @@
         <v>id-190.png</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="4" t="n">
         <v>191</v>
       </c>
@@ -11154,7 +11154,7 @@
         <v>id-191.png</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="4" t="n">
         <v>192</v>
       </c>
@@ -11184,7 +11184,7 @@
         <v>id-192.png</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="4" t="n">
         <v>193</v>
       </c>
@@ -11214,7 +11214,7 @@
         <v>id-193.png</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="4" t="n">
         <v>194</v>
       </c>
@@ -11244,7 +11244,7 @@
         <v>id-194.png</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="4" t="n">
         <v>195</v>
       </c>
@@ -11274,7 +11274,7 @@
         <v>id-195.png</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="4" t="n">
         <v>196</v>
       </c>
@@ -11304,7 +11304,7 @@
         <v>id-196.png</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="4" t="n">
         <v>197</v>
       </c>
@@ -11334,7 +11334,7 @@
         <v>id-197.png</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="4" t="n">
         <v>198</v>
       </c>
@@ -11364,7 +11364,7 @@
         <v>id-198.png</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="4" t="n">
         <v>199</v>
       </c>
@@ -11394,7 +11394,7 @@
         <v>id-199.png</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="4" t="n">
         <v>200</v>
       </c>
@@ -11424,7 +11424,7 @@
         <v>id-200.png</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="4" t="n">
         <v>201</v>
       </c>
@@ -11454,7 +11454,7 @@
         <v>id-201.png</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="4" t="n">
         <v>202</v>
       </c>
@@ -11484,7 +11484,7 @@
         <v>id-202.png</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="4" t="n">
         <v>203</v>
       </c>
@@ -11514,7 +11514,7 @@
         <v>id-203.png</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="4" t="n">
         <v>204</v>
       </c>
@@ -11544,7 +11544,7 @@
         <v>id-204.png</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="4" t="n">
         <v>205</v>
       </c>
@@ -11574,7 +11574,7 @@
         <v>id-205.png</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="4" t="n">
         <v>206</v>
       </c>
@@ -11604,7 +11604,7 @@
         <v>id-206.png</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="4" t="n">
         <v>207</v>
       </c>
@@ -11634,7 +11634,7 @@
         <v>id-207.png</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="4" t="n">
         <v>208</v>
       </c>
@@ -11664,7 +11664,7 @@
         <v>id-208.png</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="4" t="n">
         <v>209</v>
       </c>
@@ -11694,7 +11694,7 @@
         <v>id-209.png</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="4" t="n">
         <v>210</v>
       </c>
@@ -11724,7 +11724,7 @@
         <v>id-210.png</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="4" t="n">
         <v>211</v>
       </c>
@@ -11754,7 +11754,7 @@
         <v>id-211.png</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="4" t="n">
         <v>212</v>
       </c>
@@ -11784,7 +11784,7 @@
         <v>id-212.png</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="4" t="n">
         <v>213</v>
       </c>
@@ -11814,7 +11814,7 @@
         <v>id-213.png</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="4" t="n">
         <v>214</v>
       </c>
@@ -11844,7 +11844,7 @@
         <v>id-214.png</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="4" t="n">
         <v>215</v>
       </c>
@@ -11874,7 +11874,7 @@
         <v>id-215.png</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="4" t="n">
         <v>216</v>
       </c>
@@ -11904,7 +11904,7 @@
         <v>id-216.png</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="4" t="n">
         <v>217</v>
       </c>
@@ -11934,7 +11934,7 @@
         <v>id-217.png</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="4" t="n">
         <v>218</v>
       </c>
@@ -11964,7 +11964,7 @@
         <v>id-218.png</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="4" t="n">
         <v>219</v>
       </c>
@@ -11994,7 +11994,7 @@
         <v>id-219.png</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="4" t="n">
         <v>220</v>
       </c>
@@ -12024,7 +12024,7 @@
         <v>id-220.png</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="4" t="n">
         <v>221</v>
       </c>
@@ -12054,7 +12054,7 @@
         <v>id-221.png</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="4" t="n">
         <v>222</v>
       </c>
@@ -12084,7 +12084,7 @@
         <v>id-222.png</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="4" t="n">
         <v>223</v>
       </c>
@@ -12114,7 +12114,7 @@
         <v>id-223.png</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="4" t="n">
         <v>224</v>
       </c>
@@ -12144,7 +12144,7 @@
         <v>id-224.png</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="4" t="n">
         <v>225</v>
       </c>
@@ -12174,7 +12174,7 @@
         <v>id-225.png</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="4" t="n">
         <v>226</v>
       </c>
@@ -12204,7 +12204,7 @@
         <v>id-226.png</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="4" t="n">
         <v>227</v>
       </c>
@@ -12234,7 +12234,7 @@
         <v>id-227.png</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="4" t="n">
         <v>228</v>
       </c>
@@ -12264,7 +12264,7 @@
         <v>id-228.png</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="4" t="n">
         <v>229</v>
       </c>
@@ -12294,7 +12294,7 @@
         <v>id-229.png</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="4" t="n">
         <v>230</v>
       </c>
@@ -12324,7 +12324,7 @@
         <v>id-230.png</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="4" t="n">
         <v>231</v>
       </c>
@@ -12354,7 +12354,7 @@
         <v>id-231.png</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="4" t="n">
         <v>232</v>
       </c>
@@ -12384,7 +12384,7 @@
         <v>id-232.png</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="4" t="n">
         <v>233</v>
       </c>
@@ -12414,7 +12414,7 @@
         <v>id-233.png</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="4" t="n">
         <v>234</v>
       </c>
@@ -12444,7 +12444,7 @@
         <v>id-234.png</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="4" t="n">
         <v>235</v>
       </c>
@@ -12474,7 +12474,7 @@
         <v>id-235.png</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="4" t="n">
         <v>236</v>
       </c>
@@ -12504,7 +12504,7 @@
         <v>id-236.png</v>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="4" t="n">
         <v>237</v>
       </c>
@@ -12534,7 +12534,7 @@
         <v>id-237.png</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="4" t="n">
         <v>238</v>
       </c>
@@ -12564,7 +12564,7 @@
         <v>id-238.png</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="4" t="n">
         <v>239</v>
       </c>
@@ -12594,7 +12594,7 @@
         <v>id-239.png</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="4" t="n">
         <v>240</v>
       </c>
@@ -12624,7 +12624,7 @@
         <v>id-240.png</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="4" t="n">
         <v>241</v>
       </c>
@@ -12654,7 +12654,7 @@
         <v>id-241.png</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A243" s="4" t="n">
         <v>242</v>
       </c>
@@ -12684,7 +12684,7 @@
         <v>id-242.png</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A244" s="4" t="n">
         <v>243</v>
       </c>
@@ -12714,7 +12714,7 @@
         <v>id-243.png</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="4" t="n">
         <v>244</v>
       </c>
@@ -12744,7 +12744,7 @@
         <v>id-244.png</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="4" t="n">
         <v>245</v>
       </c>
@@ -12774,7 +12774,7 @@
         <v>id-245.png</v>
       </c>
     </row>
-    <row r="247" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A247" s="4" t="n">
         <v>246</v>
       </c>

</xml_diff>

<commit_message>
Ajoute le mode spectateur (voir la main du joueur actif une fois qu'on a fini), la poubelle commune a tous les joueurs, et un son de victoire pour le premier fini
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -350,7 +350,7 @@
     <t xml:space="preserve">Un moine du XIe siècle qualifia l'usage de la fourchette d'« excès de délicatesse » et y vit un signe de décadence morale.</t>
   </si>
   <si>
-    <t xml:space="preserve">Langue des signes et éducation des sourds</t>
+    <t xml:space="preserve">Invention de la langue des signes </t>
   </si>
   <si>
     <t xml:space="preserve">Pedro Ponce de León est l’un des premiers éducateurs connus de personnes sourdes; il n’a pas inventé une langue des signes unique.</t>
@@ -419,7 +419,7 @@
     <t xml:space="preserve">Inventions</t>
   </si>
   <si>
-    <t xml:space="preserve">Invention de l'imprimerie (Gutenberg)</t>
+    <t xml:space="preserve">Invention de l'imprimerie </t>
   </si>
   <si>
     <t xml:space="preserve">Gutenberg met au point la presse à caractères mobiles en Europe</t>
@@ -1211,7 +1211,7 @@
     <t xml:space="preserve">Avant de connaître le succès, l'un des tout premiers modèles de guitare électrique avait été conçu comme un accessoire pour piano — le brevet du capteur magnétique déposé en 1911 visait en réalité un tout autre instrument.</t>
   </si>
   <si>
-    <t xml:space="preserve">Krach boursier de 1929</t>
+    <t xml:space="preserve">Krach boursier </t>
   </si>
   <si>
     <t xml:space="preserve">Effondrement de Wall Street, début de la Grande Dépression</t>
@@ -5364,14 +5364,14 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="44.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="1.7"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="1" width="49.46"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="32.76"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="50.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="31.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="74.97"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="27.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.76"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="77.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="1" width="11.53"/>
@@ -6264,7 +6264,7 @@
         <v>id-28.png</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="57.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
Ajoute 16 cartes sur l'histoire profonde de la vie et de l'humanite (ids 293-308, de -3,8 milliards a -280 000 ans) : origine de la vie, Grande Oxydation, explosion cambrienne, extinction du Permien, Homo erectus/heidelbergensis/neanderthalensis/sapiens, etc. Exclu un doublon (apparition des dinosaures, deja carte id 1).
Ameliore le regroupement par ere de la frise pour le temps profond (un repere par echelle de duree plutot qu'un seul bloc "Prehistoire lointaine").

Corrige un bug mobile : les boutons rond lobby/inspecteur etaient invisibles (hors ecran) sur telephone. Cause : le backdrop-filter ajoute sur .lobby/.inspecteur cree un nouveau bloc conteneur pour leurs enfants en position:fixed, qui heritaient alors d'un decalage errone au lieu d'etre ancres au viewport. Deplace le backdrop-filter vers -contenu, qui n'a pas cet enfant.
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K293"/>
+  <dimension ref="A1:K309"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="44.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.83" customWidth="1" style="12" min="1" max="1"/>
@@ -11183,10 +11183,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I248" s="16">
-        <f>"id-"&amp;(ROW(H248)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I248" s="16" t="inlineStr"/>
     </row>
     <row r="249" ht="44.25" customHeight="1" s="13">
       <c r="A249" s="19" t="n">
@@ -11221,10 +11218,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I249" s="16">
-        <f>"id-"&amp;(ROW(H249)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I249" s="16" t="inlineStr"/>
     </row>
     <row r="250" ht="44.25" customHeight="1" s="13">
       <c r="A250" s="19" t="n">
@@ -11259,10 +11253,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I250" s="16">
-        <f>"id-"&amp;(ROW(H250)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I250" s="16" t="inlineStr"/>
     </row>
     <row r="251" ht="44.25" customHeight="1" s="13">
       <c r="A251" s="19" t="n">
@@ -11297,10 +11288,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I251" s="16">
-        <f>"id-"&amp;(ROW(H251)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I251" s="16" t="inlineStr"/>
     </row>
     <row r="252" ht="44.25" customHeight="1" s="13">
       <c r="A252" s="19" t="n">
@@ -11335,10 +11323,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I252" s="16">
-        <f>"id-"&amp;(ROW(H252)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I252" s="16" t="inlineStr"/>
     </row>
     <row r="253" ht="44.25" customHeight="1" s="13">
       <c r="A253" s="19" t="n">
@@ -11373,10 +11358,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I253" s="16">
-        <f>"id-"&amp;(ROW(H253)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I253" s="16" t="inlineStr"/>
     </row>
     <row r="254" ht="44.25" customHeight="1" s="13">
       <c r="A254" s="19" t="n">
@@ -11411,10 +11393,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I254" s="16">
-        <f>"id-"&amp;(ROW(H254)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I254" s="16" t="inlineStr"/>
     </row>
     <row r="255" ht="44.25" customHeight="1" s="13">
       <c r="A255" s="19" t="n">
@@ -11449,10 +11428,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I255" s="16">
-        <f>"id-"&amp;(ROW(H255)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I255" s="16" t="inlineStr"/>
     </row>
     <row r="256" ht="44.25" customHeight="1" s="13">
       <c r="A256" s="19" t="n">
@@ -11487,10 +11463,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I256" s="16">
-        <f>"id-"&amp;(ROW(H256)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I256" s="16" t="inlineStr"/>
     </row>
     <row r="257" ht="44.25" customHeight="1" s="13">
       <c r="A257" s="19" t="n">
@@ -11525,10 +11498,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I257" s="16">
-        <f>"id-"&amp;(ROW(H257)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I257" s="16" t="inlineStr"/>
     </row>
     <row r="258" ht="44.25" customHeight="1" s="13">
       <c r="A258" s="19" t="n">
@@ -11563,10 +11533,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I258" s="16">
-        <f>"id-"&amp;(ROW(H258)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I258" s="16" t="inlineStr"/>
     </row>
     <row r="259" ht="44.25" customHeight="1" s="13">
       <c r="A259" s="19" t="n">
@@ -11601,10 +11568,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I259" s="16">
-        <f>"id-"&amp;(ROW(H259)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I259" s="16" t="inlineStr"/>
     </row>
     <row r="260" ht="44.25" customHeight="1" s="13">
       <c r="A260" s="19" t="n">
@@ -11639,10 +11603,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I260" s="16">
-        <f>"id-"&amp;(ROW(H260)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I260" s="16" t="inlineStr"/>
     </row>
     <row r="261" ht="44.25" customHeight="1" s="13">
       <c r="A261" s="19" t="n">
@@ -11677,10 +11638,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I261" s="16">
-        <f>"id-"&amp;(ROW(H261)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I261" s="16" t="inlineStr"/>
     </row>
     <row r="262" ht="44.25" customHeight="1" s="13">
       <c r="A262" s="19" t="n">
@@ -11715,10 +11673,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I262" s="16">
-        <f>"id-"&amp;(ROW(H262)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I262" s="16" t="inlineStr"/>
     </row>
     <row r="263" ht="44.25" customHeight="1" s="13">
       <c r="A263" s="19" t="n">
@@ -11753,10 +11708,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I263" s="16">
-        <f>"id-"&amp;(ROW(H263)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I263" s="16" t="inlineStr"/>
     </row>
     <row r="264" ht="44.25" customHeight="1" s="13">
       <c r="A264" s="19" t="n">
@@ -11791,10 +11743,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I264" s="16">
-        <f>"id-"&amp;(ROW(H264)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I264" s="16" t="inlineStr"/>
     </row>
     <row r="265" ht="44.25" customHeight="1" s="13">
       <c r="A265" s="19" t="n">
@@ -11829,10 +11778,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I265" s="16">
-        <f>"id-"&amp;(ROW(H265)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I265" s="16" t="inlineStr"/>
     </row>
     <row r="266" ht="44.25" customHeight="1" s="13">
       <c r="A266" s="19" t="n">
@@ -11867,10 +11813,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I266" s="16">
-        <f>"id-"&amp;(ROW(H266)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I266" s="16" t="inlineStr"/>
     </row>
     <row r="267" ht="44.25" customHeight="1" s="13">
       <c r="A267" s="19" t="n">
@@ -11905,10 +11848,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I267" s="16">
-        <f>"id-"&amp;(ROW(H267)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I267" s="16" t="inlineStr"/>
     </row>
     <row r="268" ht="44.25" customHeight="1" s="13">
       <c r="A268" s="19" t="n">
@@ -11943,10 +11883,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I268" s="16">
-        <f>"id-"&amp;(ROW(H268)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I268" s="16" t="inlineStr"/>
     </row>
     <row r="269" ht="44.25" customHeight="1" s="13">
       <c r="A269" s="19" t="n">
@@ -11981,10 +11918,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I269" s="16">
-        <f>"id-"&amp;(ROW(H269)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I269" s="16" t="inlineStr"/>
     </row>
     <row r="270" ht="44.25" customHeight="1" s="13">
       <c r="A270" s="19" t="n">
@@ -12019,10 +11953,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I270" s="16">
-        <f>"id-"&amp;(ROW(H270)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I270" s="16" t="inlineStr"/>
     </row>
     <row r="271" ht="44.25" customHeight="1" s="13">
       <c r="A271" s="19" t="n">
@@ -12057,10 +11988,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I271" s="16">
-        <f>"id-"&amp;(ROW(H271)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I271" s="16" t="inlineStr"/>
     </row>
     <row r="272" ht="44.25" customHeight="1" s="13">
       <c r="A272" s="19" t="n">
@@ -12095,10 +12023,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I272" s="16">
-        <f>"id-"&amp;(ROW(H272)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I272" s="16" t="inlineStr"/>
     </row>
     <row r="273" ht="44.25" customHeight="1" s="13">
       <c r="A273" s="19" t="n">
@@ -12133,10 +12058,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I273" s="16">
-        <f>"id-"&amp;(ROW(H273)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I273" s="16" t="inlineStr"/>
     </row>
     <row r="274" ht="44.25" customHeight="1" s="13">
       <c r="A274" s="19" t="n">
@@ -12171,10 +12093,7 @@
           <t>Avéré</t>
         </is>
       </c>
-      <c r="I274" s="16">
-        <f>"id-"&amp;(ROW(H274)-1)&amp;".png"</f>
-        <v/>
-      </c>
+      <c r="I274" s="16" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="20" t="n">
@@ -12840,6 +12759,566 @@
         </is>
       </c>
       <c r="I293" s="20" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Science / Biologie</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Apparition des premières formes de vie (stromatolites bactériennes)</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>-3800000000</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Les premières bactéries colonisent les océans primitifs</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Il y a 3,8 milliards d'années, dans les océans primitifs de la Terre jeune, les premières formes de vie apparaissent : des bactéries simples, unicellulaires, sans noyau (procaryotes). Ces organismes sont tellement microscopiques qu'on ne peut les voir qu'au microscope. Elles vivent dans l'eau chaude des océans, se nourrissant de minéraux et d'énergie chimique provenant des cheminées hydrothermales sous-marines. Ces bactéries primitives créent progressivement des structures rocheuses en couches appelées "stromatolites" : ce sont les fossiles les plus anciens découverts sur Terre. Les stromatolites sont formés par l'accumulation de bactéries mortes et de sédiments, créant des dômes rocheux caractéristiques. Ces premières créatures n'ont pas besoin d'oxygène pour vivre (elles sont anaérobies). Elles se reproduisent en se divisant simplement en deux, transmettant leur matériel génétique (ADN) à leurs descendants. Cette apparition marque le début de la vie sur Terre et le début de l'évolution biologique : pendant les 3,8 milliards d'années suivantes, toutes les formes de vie complexes descendront de ces bactéries microscopiques. Sans cette étape, aucun animal, aucune plante, aucun humain n'existerait.</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Science / Chimie atmosphérique</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Grande Oxydation : l'oxygène s'accumule dans l'atmosphère terrestre</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>-2700000000</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>L'atmosphère terrestre devient progressivement riche en oxygène</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Il y a 2,7 milliards d'années, un événement gigantesque transforme la Terre : la "Grande Oxydation". Pendant 1,1 milliard d'années avant cela, les bactéries photosynthétiques (cyanobactéries) produisent lentement de l'oxygène en convertissant la lumière solaire en énergie chimique. Cet oxygène était d'abord consommé par des minéraux de fer dissous dans l'océan, créant les "formations de fer rubanées" (bandes alternées de fer et de roche). Mais à partir de 2,7 milliards d'années, l'oxygène s'accumule plus vite qu'il n'est consommé. Il s'échappe dans l'atmosphère, passant de presque 0% à environ 1% de l'atmosphère. Pour les bactéries anaérobies dominantes à cette époque, c'est une catastrophe : l'oxygène est un poison qui tue leurs cellules. Cet événement provoque la plus grande extinction de masse de l'histoire de la vie : 99% de la vie anaérobie disparaît. Seules survivent les bactéries capables d'utiliser l'oxygène pour respirer et produire plus d'énergie. Mais cette catastrophe crée aussi une opportunité : avec l'oxygène, les cellules peuvent respirer plus efficacement et accumuler plus d'énergie. Cela permettra l'apparition d'organismes plus grands et plus complexes. Sans la Grande Oxydation, les animaux et plantes complexes n'auraient jamais pu émerger.</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Science / Biologie cellulaire</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Apparition des premières cellules eucaryotes avec noyau</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>-1200000000</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>La cellule se complexifie : apparition du noyau cellulaire</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Il y a 1,2 milliard d'années, une révolution silencieuse transforme la vie microscopique : l'apparition des cellules eucaryotes. Jusqu'à ce moment, toute la vie consiste en bactéries procaryotes : une simple goutte de cytoplasme avec de l'ADN flottant librement au centre. Soudain, certaines bactéries développent une membrane interne entourant leur ADN, créant une structure appelée "noyau". C'est comme si la cellule construisait une chambre de coffre-fort pour protéger ses gènes. Comment ? Les scientifiques pensent qu'une bactérie a avalé une autre bactérie, mais au lieu de la digérer, elles ont fusionné. C'est l'endosymbiose : une fusion bactérienne. Ces nouvelles cellules eucaryotes sont beaucoup plus grandes et plus complexes. Elles développent aussi des organelles : mitochondries (centrales électriques cellulaires), chloroplastes (panneaux solaires biologiques), réticulum endoplasmique (système de transport interne). Avec cette organisation interne, les cellules peuvent accumuler beaucoup plus d'énergie. Elles peuvent aussi se combiner pour former des organismes multicellulaires : les premiers protistes apparaissent (algues microscopiques). Ces cellules eucaryotes sont nos ancêtres directs. Sans cette évolution cellulaire, les plantes, les animaux, les champignons et les humains n'existeraient jamais.</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr"/>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Science / Paléontologie</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Explosion cambrienne : diversification massive des formes de vie</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>-600000000</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>L'océan se remplit soudainement d'animaux complexes et variés</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Il y a 600 millions d'années, quelque chose d'extraordinaire se produit dans les océans : l'Explosion cambrienne. Pendant plus de 3 milliards d'années, la vie était dominée par des organismes microscopiques et quelques créatures molles et sans couleur. Puis, en quelques millions d'années seulement (un clin d'œil géologique), des centaines de nouvelles formes de vie complexes et bizarres émergent soudainement. Les fossiles montrent des trilobites (créatures blindées avec des yeux), des échinodermes (ancêtres des étoiles de mer), des mollusques (ancêtres des poulpes), des arthropodes (ancêtres des insectes et araignées). Pourquoi soudainement ? Les scientifiques pensent que plusieurs facteurs convergent : l'oxygène atmosphérique atteint finalement des niveaux suffisants pour supporter des animaux complexes. Les océans refroidissent légèrement après une ère glaciaire. Une mutation génétique majeure (gènes Hox) permet une plus grande variabilité corporelle. La compétition apparaît : les prédateurs apparaissent et forcent les proies à évoluer rapidement pour survivre. C'est une "course aux armements" biologique. Ces animaux cambriens sont nos ancêtres : leur diversité de corps et de stratégies de survie crée les plans de base de tous les animaux futurs. Les humains et tous les animaux terrestres descendent des survivants de cette explosion créative.</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr"/>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Science / Zoologie</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Apparition des premiers poissons (Ostracodermes)</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>-500000000</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Les premiers vertébrés apparaissent : les ancêtres des poissons modernes</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Il y a 500 millions d'années, dans les océans du Silurien, les premiers poissons apparaissent : les Ostracodermes. Ces créatures ressemblent à des petits têtards blindés, longues de quelques centimètres. Contrairement aux autres animaux marins, ils possèdent une innovation révolutionnaire : un squelette primitif fait de cartilage (comme celui des requins modernes) au lieu d'exosquelette externe. Mieux encore, ce squelette contient une moelle épinière et un cerveau primitif. C'est la naissance des vertébrés : le groupe auquel nous appartenons. Les Ostracodermes n'ont pas de mâchoires mobiles (ils aspirent leur nourriture), pas de nageoires paires, juste une bouche fixe. Mais ils sont efficaces : petit à petit, d'autres innovations apparaissent. Certains Ostracodermes développent des mâchoires flexibles, permettant une meilleure capture de nourriture. Certains développent des nageoires paires pour mieux contrôler leur mouvement dans l'eau. Sur des millions d'années, ces améliorations créent les poissons modernes : les placodermes (poissons à plaques osseuses), les chondrichthyens (requins et raies), puis les ostéichthyens (poissons osseux). Les humains sont des descendants très éloignés de ces premiers poissons : nos bras, nos jambes, notre crâne, notre colonne vertébrale viennent de cette lignée aquatique ancienne.</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Science / Botanique</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Les premières plantes colonisent la terre ferme (bryophytes primitives)</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>-475000000</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Les continents se couvrent de végétation : les plantes quittent l'océan</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Il y a 475 millions d'années, les continents sont totalement déserts : des roches nues sous un ciel sans couleur. Les plantes vivent uniquement dans l'océan. Puis, les premières plantes aquatiques découvrent comment survivre sur la terre sèche : les bryophytes primitives (ancêtres des mousses et hépatiques modernes). Comment ? Ces plantes développent plusieurs adaptations géniales. D'abord, un système de racines primitif qui s'enfonce dans le sol pour absorber l'eau et les nutriments minéraux. Ensuite, une cuticule cireuse sur la surface qui réduit l'évaporation : sans cette protection, la plante se dessécherait instantanément au contact de l'air. Troisièmement, un système de transport interne (vaisseaux) qui propage l'eau des racines aux feuilles. Enfin, des spores plutôt que des œufs pour se reproduire : les spores sont minuscules, légères, et peuvent voyager dans le vent sur de longues distances. Ces premières plantes sont minuscules, juste quelques centimètres, sans feuilles véritables, ressemblant à des mousses. Mais elles sont révolutionnaires. Elles transforment les roches nues en sol : leurs racines fracturent la roche, créant du terreau. Elles produisent de l'oxygène, modifiant l'atmosphère. Elles créent des habitats. Sur les millions d'années suivants, les plantes évoluent : des fougères plus grandes apparaissent (avec de vraies racines profondes), puis des plantes à graines, puis des fleurs. Sans cette colonisation terrestre, les animaux terrestres et les humains ne pourraient jamais exister.</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Science / Zoologie</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Apparition des premiers amphibiens : la transition de l'eau à la terre</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>-360000000</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Les poissons développent des pattes et sortent de l'eau</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Il y a 360 millions d'années, quelque chose d'extraordinaire se produit dans les marécages et rivières du Carbonifère : les poissons développent des pattes et quittent l'eau. Ce sont les premiers amphibiens, comme le Tiktaalik et l'Ichthyostega. Comment des poissons deviennent-ils des créatures terrestres ? La clé est la nageoire : les nageoires paires des poissons (pectorales et pelviennes) évoluent progressivement en membres articulés (bras et jambes) avec os, articulations et muscles. Ces amphibiens primitifs gardent encore des caractéristiques de poisson : une queue aplatie pour nager, des branchies pour respirer sous l'eau. Mais ils développent aussi des poumons pour respirer l'air. Leurs nageoires deviennent de vraies pattes assez fortes pour supporter leur poids et les propulser sur la terre. Pourquoi quitter l'eau ? L'eau stagnante des marécages manque d'oxygène. Les amphibiens capables de ramper sur la terre et respirer l'air à la surface ont un avantage de survie énorme. Sur terre, ils découvrent un monde vierge rempli de nourriture (plantes, insectes) et sans prédateurs. Mais les premiers amphibiens restent dépendants de l'eau : ils doivent y retourner pour se reproduire, comme les grenouilles modernes. Sur les 100 millions d'années suivantes, certains amphibiens évoluent pour s'adapter à la vie terrestre complète. Ils développent une peau imperméable, des œufs avec coquille (pas besoin de l'eau pour la reproduction). Ce sont les reptiles. Et les humains, comme tous les mammifères terrestres, descendons de ces amphibiens intrépides qui ont osé explorer la terre.</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Science / Zoologie</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Apparition des premiers reptiles avec œufs à coquille dure</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>-320000000</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>L'amniote : l'invention géniale qui libère les vertébrés de l'eau</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Il y a 320 millions d'années, un événement biologique majeur transforme l'évolution terrestre : l'apparition des premiers vrais reptiles. Leur innovation clé ? L'œuf amniotique : un œuf avec une coquille imperméable contenant une poche d'eau (l'amnios) qui protège l'embryon. Pourquoi est-ce révolutionnaire ? Les amphibiens doivent retourner à l'eau pour pondre car leurs œufs sont mous et se déssèchent rapidement au soleil. Les reptiles, avec leur coquille dure, peuvent pondre loin de l'eau, sur la terre ferme. Cela signifie : indépendance totale de l'eau pour la reproduction. Plus besoin de revenir à l'eau chaque saison de reproduction. Les premiers reptiles amniotes ressemblent à des lézards, longs de quelques décimètres. Ils développent aussi une peau écailleuse imperméable qui retient l'eau, contrairement à la peau humide des amphibiens. Leurs pattes deviennent plus fortes, supportant leur corps de manière plus verticale. Ces adaptations les rendent extrêmement efficaces sur terre. Sur les 50 millions d'années suivantes, les reptiles se diversifient explosivement : certains deviennent énormes (les dinosaures), d'autres développent des ailes (les ptérosaures et oiseaux), d'autres une apparence mammalienne (les synapsides). Les reptiles dominent tous les écosystèmes terrestres pendant 250 millions d'années. Les humains descendons d'une lignée de petits reptiles synapsidés qui survivent à plusieurs extinctions de masse et finissent par devenir les mammifères.</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Science / Zoologie</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Apparition des premiers synapsides : ancêtres des mammifères</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>-300000000</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Les synapsides : la lignée qui mène directement aux mammifères et humains</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Il y a 300 millions d'années, dans les marécages du Carbonifère, apparaissent les synapsides : une lignée de reptiles qui semble ordinaire au premier abord. Les synapsides ressemblent à des reptiles normaux, ressemblant à des petits lézards ou à des pelycosaures (reptiles à voile de cheveux sur le dos). Mais ils possèdent une caractéristique unique : une fenêtre osseuse sur chaque côté du crâne (la fenêtre temporale), d'où s'attachent des muscles mâchoires puissants. Pourquoi est-ce important ? Ces muscles mâchoires permettent une morsure plus puissante et une meilleure mastication. Au cours des 100 millions d'années suivantes, les synapsides évoluent lentement mais sûrement vers quelque chose de plus étrange. Certains développent une posture de pattes plus verticale (sous le corps) plutôt qu'écartées sur les côtés comme les reptiles. Certains développent des dents différenciées : des incisives pour trancher, des canines pointues pour percer, des molaires pour broyer. C'est très différent des reptiles qui ont des dents uniformes. Certains développent une seule fenêtre osseuse supérieure au crâne plutôt que deux. Ces changements graduels transforment lentement les synapsides en quelque chose de nouveau : les cynodontes. Et les cynodontes, après 50 millions d'années d'évolution supplémentaire, deviendront les premiers mammifères vrais. Chaque humain vivant descend directement de ces synapsides apparemment ordinaires du Carbonifère.</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Science / Paléontologie</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Extinction du Permien : 95% de la vie terrestre disparaît</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>-250000000</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>La plus grande extinction de masse de l'histoire : la «Grande Mort»</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Il y a 250 millions d'années, c'est l'apocalypse biologique : l'Extinction du Permien, aussi appelée "la Grande Mort" (The Great Dying). C'est la pire extinction de masse dans toute l'histoire de la vie. Les chiffres sont terrifiants : 95% de toutes les espèces marines disparaissent. 70% de toutes les espèces de vertébrés terrestres disparaissent. Seules quelques espèces survivent et repeuplent le monde ensuite. Qu'est-ce qui cause ce cataclysme ? Les scientifiques déterminent plusieurs causes qui convergeaient à la même époque. D'abord, le "trappage sibérien" : dans la région de la Sibérie, d'énormes éruptions volcaniques massives se produisent pendant des milliers d'années. Ces volcans libèrent des millions de tonnes de cendres volcaniques, d'acide sulfurique, et surtout du dioxyde de carbone. Le CO2 crée un effet de serre massif : les températures mondiales augmentent de 5 à 10 degrés Celsius. Les océans se réchauffent dangereusement. Les zones côtières produisent moins d'oxygène. Les niveaux marins baissent. Les écosystèmes marins s'effondrent. De plus, les cendres volcaniques bloquent le soleil, tuant les plantes et créant une famine. Les animaux qui survivent sont ceux qui peuvent jeûner longtemps, tolérer les températures extrêmes, et s'adapter rapidement aux nouvelles conditions. Les synapsides survivent à cette extinction mieux que les autres reptiles. Après cet événement catastrophique, le monde est vide. Les synapsides survivants se diversifient rapidement pour remplir tous les rôles écologiques laissés vacants. Cet "reset" écologique crée les opportunités pour que les cynodontes (descendants synapsides) évoluent ensuite en mammifères. Sans cette extinction terrifiante, les dinosaures, pas les synapsides, auraient dominé le monde, et les mammifères n'auraient jamais existé.</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Science / Zoologie</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Apparition des premiers mammifères (petits nocturnes)</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>-220000000</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Les mammifères naissent dans l'ombre des dinosaures</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Il y a 220 millions d'années, au moment où les dinosaures commencent à dominer la Terre, un groupe de petits reptiles abandonne la compétition directe et se cache : les premiers mammifères. Ces créatures, comme le Morganucodon et l'Hadrocodium, sont minuscules : longues de seulement 10 à 30 centimètres, pesant quelques grammes, ressemblant à de petites musaraignes. Elles sont timides, nocturnes, se cachant sous terre et dans les arbres pendant le jour, sortant la nuit chercher nourriture. Pourquoi sont-elles "mammifères" ? Elles possèdent des caractéristiques que seuls les mammifères ont. D'abord, un crâne spécialisé avec une fenêtre osseuse pour les muscles mâchoires (héritage des synapsides). Deuxièmement, des dents différenciées : incisives, canines, molaires, permettant une mastication efficace. Troisièmement, trois os d'oreille interne (marteau, enclume, étrier) plutôt que les os de mâchoire de reptiles. Quatrièmement, un palais dur qui sépare la bouche de la respiration, permettant une respiration continue pendant la mastication. Ces adaptations rendent les premiers mammifères extrêmement efficaces pour chasser de petites proies (insectes, petits lézards) la nuit. Pendant 140 millions d'années, les mammifères restent petits et rares, toujours éclipsés par les dinosaures dominants. Mais quand les dinosaures s'éteignent soudainement (extinction K-T, il y a 66 millions d'années), les mammifères survivants évoluent rapidement pour remplir tous les rôles écologiques laissés vacants. Sans cette période d'évolution cachée, les mammifères ne seraient jamais devenus les créatures dominantes du monde actuel, et les humains n'existeraient pas.</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Science / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Homo erectus maîtrise et utilise régulièrement le feu</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>La maîtrise du feu : l'une des plus grandes révolutions de l'évolution humaine</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Il y a 1,5 million d'années, dans les vallées d'Afrique de l'Est (Éthiopie, Kenya), le Homo erectus franchit un cap extraordinaire : maîtriser le feu. Ce n'est pas qu'il découvre soudainement le feu. Les hominidés antérieurs (Homo habilis) ont probablement utilisé le feu naturel (provenant des éruptions volcaniques ou éclairs) occasionnellement. Mais Homo erectus fait quelque chose de révolutionnaire : il apprend à créer le feu intentionnellement et à le maintenir allumé. Comment ? En frappant des roches de silex contre du granit pour produire des étincelles, ou en frottant du bois pour créer de la chaleur. Pourquoi c'est révolutionnaire ? Le feu change absolument tout. D'abord, nutrition : la cuisson tue les bactéries dangereuses et les parasites dans la viande et les plantes. Elle rend aussi la nourriture plus facile à digérer, ce qui signifie que le corps absorbe plus de nutriments avec moins d'effort. Cela libère de l'énergie pour d'autres fonctions, notamment le cerveau. Deuxièmement, survie : le feu tient chaud, crucial pour les humains qui perdent rapidement la chaleur corporelle. Il repousse les prédateurs la nuit. Troisièmement, socialité : le feu rassemble les gens. Assis autour du feu, les humains commencent à socialiser, parler, raconter des histoires, enseigner aux enfants. C'est probablement quand le langage devient plus complexe. Quatrièmement, technologie : le feu peut être utilisé pour travailler le bois, la pierre, l'os. Il rend possible des outils plus sophistiqués. Avec le feu, Homo erectus peut migrer vers des régions froides (Europe du Nord, Asie). Pendant environ 1 million d'années, Homo erectus utilise le feu, se propageant à travers le monde. Ses descendants (Homo neanderthalensis, Homo sapiens) héritent de cette technologie révolutionnaire et la raffinent encore plus. Sans la maîtrise du feu, le cerveau humain ne se serait jamais aussi développé, et la civilisation n'existerait pas.</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Science / Paléontologie</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Homo heidelbergensis : ancêtre commun probable de Néandertal et Sapiens</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>-500000</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>L'ancêtre hypothétique qui sépare les destinées de deux humanités</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Il y a 500 000 ans, une créature appelée Homo heidelbergensis vit en Afrique, en Europe et en Asie. C'est un individu fascinant qui représente une étape critique de l'évolution humaine. Homo heidelbergensis est plus grand et plus robuste que Homo erectus (taille humaine, poids 70-90 kg). Son crâne est plus grand avec un volume cérébral de 1200-1400 centimètres cubes (comparable aux humains modernes). Ses os sont plus épais, ses muscles plus puissants. Qu'est-ce qui le rend spécial ? Les données génétiques et fossiles suggèrent qu'Homo heidelbergensis est probablement l'ancêtre commun de deux espèces humaines différentes qui évoluent ensuite séparément. En Europe, où le climat devient très froid, Homo heidelbergensis évolue en Homo neanderthalensis (les Néandertaliens), avec des corps plus courts et trapus, adaptés au froid. En Afrique, où le climat reste chaud, Homo heidelbergensis évolue en Homo sapiens (nous), avec des corps plus longs et gracieux. Homo heidelbergensis lui-même est un chasseur efficace. Les preuves archéologiques montrent qu'il fabrique des bifaces (outils de pierre bifaciales) sophistiqués appelés "coups de poing" (hand axes). Il chasse probablement des animaux de grande taille en groupes coordonnés, nécessitant une communication complexe et une planification. Son cerveau suffisamment grand suggère qu'il possède un langage et une capacité à enseigner. C'est probablement la première espèce humaine avec une véritable culture transmissible. Homo heidelbergensis disparaît il y a environ 300 000 ans, remplacé par ses descendants plus spécialisés (Néandertal et Sapiens). Mais sans Homo heidelbergensis, ces deux branches distinctes d'humanité n'auraient jamais émergé.</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Science / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Homo neanderthalensis émerge en Europe</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>-430000</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Le Néandertal : une espèce humaine distincte adaptée au froid glacial</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Il y a 430 000 ans, dans les grottes et vallées de l'Europe, une nouvelle espèce humaine émerge : Homo neanderthalensis, que nous appelons les Néandertaliens. Ils évoluent à partir d'Homo heidelbergensis pendant une période de glaciation intense. Le climat européen devient beaucoup plus froid et inhospitalier. Homo neanderthalensis développe une morphologie extrêmement bien adaptée au froid : corps trapus et robustes (plus courts mais plus lourds que Homo sapiens), crâne plus grand avec un cerveau légèrement plus gros que le nôtre (1450-1600 cm³ contre 1400 pour Sapiens). Leur corps trapu minimise la perte de chaleur (surface/volume réduit). Leurs extrémités (doigts, orteils, nez) sont plus courtes pour réduire la gelure. Leurs muscles sont massifs, leur densité osseuse très élevée, les rendant extrêmement forts (environ 20% plus forts qu'un humain moderne). Ils développent des outils de pierre raffinés appelés "industries moustériennes" : des racloirs, des lames, des pointes de lance pour chasser les mégafaunes (mammouths, bisons, rennes). Les preuves archéologiques suggèrent qu'ils vivent en petits groupes, chassent en coordonnés (nécessitant communication complexe), et ont peut-être un langage sophistiqué. Certaines preuves indiquent qu'ils prennent soin de leurs malades et blessés, et qu'ils enterrent leurs morts avec des rituels, suggérant une conscience de la mort et possiblement une spiritualité. Les Néandertaliens prospèrent en Europe et en Asie occidentale pendant environ 200 000 ans. Mais quand Homo sapiens arrive d'Afrique il y a 40 000 ans, mieux adapté aux changements climatiques rapides, les Néandertaliens entrent en déclin et disparaissent il y a environ 30 000 ans. Ironiquement, ils ne disparaissent pas complètement : environ 1-4% du génome de tous les humains non-africains contient de l'ADN néandertalien.</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Science / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Homo sapiens archaïque émerge en Afrique</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>-300000</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>L'émergence de notre propre espèce : Homo sapiens archaïque en Afrique</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Il y a 300 000 ans, quelque part en Afrique subsaharienne (probablement en Afrique du Sud et de l'Est), une nouvelle espèce humaine émerge : Homo sapiens archaïque. C'est nous, ou plutôt, ce sont nos ancêtres les plus directs. Les fossiles montrent une transition progressive depuis Homo heidelbergensis. Les changements majeurs : d'abord, le crâne s'aplatit. Chez Homo erectus et Homo heidelbergensis, le front fuit vers l'arrière et il y a un bourrelet proéminent au-dessus des yeux. Chez Homo sapiens, le front devient vertical, donnant du style à un menton (unique aux humains modernes). Deuxièmement, la face devient plus petite et gracile plutôt que robuste. Troisièmement, le cerveau se réorganise : la partie frontale s'agrandit (pensée abstraite, langage, planification), tandis que l'occipital s'arrondit. Homo sapiens archaïque (300 000 à 100 000 ans) n'est pas encore complètement "moderne" mais s'en rapproche. Ils fabriquent des outils de pierre sophistiqués, chassent efficacement et cuisent leur nourriture avec le feu depuis longtemps. Vers 200 000 ans, certains fossiles montrent les caractéristiques entièrement "modernes" : crâne arrondi, petite face, menton proéminent. C'est Homo sapiens moderne. Entre 100 000 et 70 000 ans, des groupes de Homo sapiens modernes commencent à quitter l'Afrique pour explorer le Moyen-Orient, puis l'Europe, l'Asie, l'Océanie : c'est la "Grande Migration" qui peuplera tous les continents. Sans cette émergence en Afrique, la branche Sapiens de l'humanité n'existerait pas.</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Science / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Apogée de Homo neanderthalensis : culture moustérienne au sommet</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>-280000</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Le Néandertal à son apogée : technologie, chasse, et vie sociale</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Il y a 280 000 ans, les Néandertaliens atteignent leur apogée en termes de population, de distribution géographique, et de sophistication technologique. À ce moment, environ 100 000 à 500 000 Néandertaliens vivent en Europe, Asie mineure, et Asie occidentale (du Portugal à la Sibérie). Ils maîtrisent une vaste gamme de technologies de chasse. L'industrie moustérienne (la technologie principale) produit des dizaines de types d'outils : des racloirs pour enlever la peau des animaux, des lames pointues pour découper la viande, des pointes de lance pour la chasse. La technique dite "Levallois" permet de préparer une pierre pour produire des lames pré-définies : un savoir-faire nécessitant apprentissage long et communication sophistiquée, probablement un véritable langage parlé. Les preuves archéologiques montrent qu'ils vivent en groupes d'environ 20-30 individus, chassant des mégafaunes (mammouths, rhinos laineux, bisons, chevaux) souvent en groupe coordonné. Les fossiles montrent des traumatismes similaires à ceux de cavaliers de rodéo, indiquant une chasse au corps à corps dangereuse mais productive. Certaines preuves fossiles suggèrent qu'ils s'occupent de membres blessés : un fossile montre un Néandertal ayant survécu des années avec un bras amputé, impossible sans l'aide du groupe, indiquant empathie et cohésion sociale. Des sites archéologiques montrent des restes de fleurs autour de squelettes, suggérant des sépultures rituelles. À cet apogée, les Néandertaliens semblent être une espèce entièrement intelligente et culturellement sophistiquée. Mais cette apogée est aussi le début du déclin : vers 50 000 ans, le climat change et Homo sapiens arrive d'Afrique, plus flexible et adaptatif. Les Néandertaliens déclinent lentement et le dernier disparaît il y a environ 30 000 ans.</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -12854,7 +13333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F428"/>
+  <dimension ref="A1:F476"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -21435,6 +21914,966 @@
         </is>
       </c>
     </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>293</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Nature : Earliest life on Earth - Abigail Allwood et al. (2015)</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature14871</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>293</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Science : Evidence for early life on Earth - Mojzsis et al. (1996)</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.273.5278.1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>293</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>The Astrophysical Journal : Stromatolites and early life - Grotzinger &amp; Knoll (1999)</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>https://iopscience.iop.org/article/10.1086/313160</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>294</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Science : The rise of atmospheric oxygen - Holland (2002)</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1069141</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>294</v>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Nature : Great Oxidation Event - Bekker et al. (2004)</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature02711</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>294</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>PLoS Biology : The rise of aerobic life - Catling &amp; Claire (2005)</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.0030176</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>295</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Nature : Endosymbiotic theory evidence - Margulis (1970)</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature15726</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>295</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Trends in Ecology &amp; Evolution : The origin of eukaryotes - Koonin (2010)</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.tree.2010.07.002</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>295</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>PNAS : Early eukaryotic fossils - Knoll et al. (2006)</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0604866103</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>296</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Nature : The Cambrian Explosion - Marshall (2006)</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature05070</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>296</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Science : Evolution of complex body structures - Briggs et al. (2005)</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1122776</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>296</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Trends in Ecology &amp; Evolution : Hox genes and body plans - Carroll (2005)</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.tree.2005.07.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>297</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Nature : Early fish evolution - Janvier (2007)</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature05983</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>297</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>PLoS Biology : Fossil evidence of Ostracoderms - Sansom et al. (2012)</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1001470</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>297</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Zoological Journal of the Linnean Society : Vertebrate origins - Gess et al. (2006)</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.1096-3642.2006.00232.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>298</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Trends in Plant Science : Early land plant evolution - Kenrick &amp; Crane (1997)</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S1360-1385(97)01010-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>298</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Nature : Oldest land plants - Wellman et al. (2003)</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature02041</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>298</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Science : Plant terrestrialization - Morris et al. (2018)</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.aar5429</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>299</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Nature : Tiktaalik - a fish with tetrapod characteristics - Shubin et al. (2004)</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature02426</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="n">
+        <v>299</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>PLoS Biology : Ichthyostega fossil evidence - Clément et al. (2015)</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1002445</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>299</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Science : Fin-to-limb transition - Coates et al. (2002)</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1069052</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>300</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Nature : Early amniote evolution - Modesto &amp; Anderson (2004)</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature03048</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>300</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>PLoS One : Amniotic egg evolution - Packard &amp; Seymour (1997)</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1152/physrev.1997.77.4.701</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="n">
+        <v>300</v>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Journal of Morphology : Reptile characteristics - Rieppel (1993)</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/jmor.1052160307</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="n">
+        <v>301</v>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Nature : Synapsid evolution - Benton (1999)</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/17856</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="n">
+        <v>301</v>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Biological Reviews : Synapsid-to-mammal transition - Kemp (2005)</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/doi/10.1017/S1464793105006457</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="n">
+        <v>301</v>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>PLoS Biology : Cynodonts and early mammals - Luo (2007)</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.0050114</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>302</v>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Science : The Great Dying - Benton (2008)</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1154887</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>302</v>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Nature : Permian-Triassic extinction - Burgess &amp; Bowring (2015)</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature14879</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>302</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Geology : Siberian volcanism and extinction - Burgess et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1130/G35774.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="n">
+        <v>303</v>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Nature : Early mammal evolution - Luo (2007)</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature06325</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>303</v>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Science : Hadrocodium - the earliest mammal - Luo et al. (2001)</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1065507</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>303</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Zoological Journal of the Linnean Society : Morganucodon paleobiology - Kermack &amp; Mussett (1983)</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.1096-3642.1983.tb00710.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>304</v>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Nature : Evidence of controlled fire use by early humans - Wrangham &amp; Conklin-Brittain (2003)</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature01754</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>304</v>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Fire use in Homo erectus - Berna et al. (2012)</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2012.05.002</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>304</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>PNAS : Cooking and human brain evolution - Aiello &amp; Wheeler (1995)</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.92.25.11803</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>305</v>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Nature : Homo heidelbergensis genetics - Meyer et al. (2013)</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature12886</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>305</v>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Homo heidelbergensis phylogeny - Rightmire (2008)</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2008.07.011</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>305</v>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>PNAS : Interbreeding of Homo heidelbergensis descendants - Schlebusch et al. (2017)</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1704702114</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>306</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Nature : Neanderthal genome - Green et al. (2010)</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature08976</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>306</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>American Journal of Physical Anthropology : Neanderthal morphology - Trinkaus (2005)</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/ajpa.20239</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>306</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>PNAS : Neanderthal symbolic behavior - D'Errico et al. (2003)</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0935975100</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>307</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Nature : Early Homo sapiens fossils - Hublin et al. (2017)</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature22336</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>307</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Science : Origin of modern humans - Green et al. (2019)</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.aav4534</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>307</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>PLoS Biology : Modern human brain evolution - Neubauer et al. (2018)</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.2006931</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>308</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Neanderthal social structure - Wobst (1974)</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/0047-2484(74)90003-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>308</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Nature : Neanderthal symbolic behavior - D'Errico et al. (2003)</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/425410a</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>308</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>PNAS : Neanderthal diet - Bocherens et al. (2005)</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0506130102</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ajoute 14 cartes sur la sortie d'Afrique et la prehistoire recente (ids 309-322, de -70 000 a -11 000 ans) : migrations de Sapiens (Asie, Australie, Europe), rencontre et disparition de Neandertal, explosion artistique (Chauvet, Venus de Willendorf), arc et fleche, dernier maximum glaciaire, domestication du chien, revolution neolithique et debuts de l'agriculture.
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K309"/>
+  <dimension ref="A1:K323"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="44.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.83" customWidth="1" style="12" min="1" max="1"/>
@@ -12761,564 +12761,1054 @@
       <c r="I293" s="20" t="inlineStr"/>
     </row>
     <row r="294">
-      <c r="A294" t="n">
+      <c r="A294" s="20" t="n">
         <v>293</v>
       </c>
-      <c r="B294" t="inlineStr">
+      <c r="B294" s="20" t="inlineStr">
         <is>
           <t>Science / Biologie</t>
         </is>
       </c>
-      <c r="C294" t="inlineStr">
+      <c r="C294" s="20" t="inlineStr">
         <is>
           <t>Apparition des premières formes de vie (stromatolites bactériennes)</t>
         </is>
       </c>
-      <c r="D294" t="n">
+      <c r="D294" s="20" t="n">
         <v>-3800000000</v>
       </c>
-      <c r="E294" t="inlineStr">
+      <c r="E294" s="20" t="inlineStr">
         <is>
           <t>Les premières bactéries colonisent les océans primitifs</t>
         </is>
       </c>
-      <c r="F294" t="inlineStr">
+      <c r="F294" s="20" t="inlineStr">
         <is>
           <t>Il y a 3,8 milliards d'années, dans les océans primitifs de la Terre jeune, les premières formes de vie apparaissent : des bactéries simples, unicellulaires, sans noyau (procaryotes). Ces organismes sont tellement microscopiques qu'on ne peut les voir qu'au microscope. Elles vivent dans l'eau chaude des océans, se nourrissant de minéraux et d'énergie chimique provenant des cheminées hydrothermales sous-marines. Ces bactéries primitives créent progressivement des structures rocheuses en couches appelées "stromatolites" : ce sont les fossiles les plus anciens découverts sur Terre. Les stromatolites sont formés par l'accumulation de bactéries mortes et de sédiments, créant des dômes rocheux caractéristiques. Ces premières créatures n'ont pas besoin d'oxygène pour vivre (elles sont anaérobies). Elles se reproduisent en se divisant simplement en deux, transmettant leur matériel génétique (ADN) à leurs descendants. Cette apparition marque le début de la vie sur Terre et le début de l'évolution biologique : pendant les 3,8 milliards d'années suivantes, toutes les formes de vie complexes descendront de ces bactéries microscopiques. Sans cette étape, aucun animal, aucune plante, aucun humain n'existerait.</t>
         </is>
       </c>
-      <c r="G294" t="inlineStr"/>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I294" t="inlineStr"/>
+      <c r="G294" s="20" t="inlineStr"/>
+      <c r="H294" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I294" s="20" t="inlineStr"/>
     </row>
     <row r="295">
-      <c r="A295" t="n">
+      <c r="A295" s="20" t="n">
         <v>294</v>
       </c>
-      <c r="B295" t="inlineStr">
+      <c r="B295" s="20" t="inlineStr">
         <is>
           <t>Science / Chimie atmosphérique</t>
         </is>
       </c>
-      <c r="C295" t="inlineStr">
+      <c r="C295" s="20" t="inlineStr">
         <is>
           <t>Grande Oxydation : l'oxygène s'accumule dans l'atmosphère terrestre</t>
         </is>
       </c>
-      <c r="D295" t="n">
+      <c r="D295" s="20" t="n">
         <v>-2700000000</v>
       </c>
-      <c r="E295" t="inlineStr">
+      <c r="E295" s="20" t="inlineStr">
         <is>
           <t>L'atmosphère terrestre devient progressivement riche en oxygène</t>
         </is>
       </c>
-      <c r="F295" t="inlineStr">
+      <c r="F295" s="20" t="inlineStr">
         <is>
           <t>Il y a 2,7 milliards d'années, un événement gigantesque transforme la Terre : la "Grande Oxydation". Pendant 1,1 milliard d'années avant cela, les bactéries photosynthétiques (cyanobactéries) produisent lentement de l'oxygène en convertissant la lumière solaire en énergie chimique. Cet oxygène était d'abord consommé par des minéraux de fer dissous dans l'océan, créant les "formations de fer rubanées" (bandes alternées de fer et de roche). Mais à partir de 2,7 milliards d'années, l'oxygène s'accumule plus vite qu'il n'est consommé. Il s'échappe dans l'atmosphère, passant de presque 0% à environ 1% de l'atmosphère. Pour les bactéries anaérobies dominantes à cette époque, c'est une catastrophe : l'oxygène est un poison qui tue leurs cellules. Cet événement provoque la plus grande extinction de masse de l'histoire de la vie : 99% de la vie anaérobie disparaît. Seules survivent les bactéries capables d'utiliser l'oxygène pour respirer et produire plus d'énergie. Mais cette catastrophe crée aussi une opportunité : avec l'oxygène, les cellules peuvent respirer plus efficacement et accumuler plus d'énergie. Cela permettra l'apparition d'organismes plus grands et plus complexes. Sans la Grande Oxydation, les animaux et plantes complexes n'auraient jamais pu émerger.</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr"/>
-      <c r="H295" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I295" t="inlineStr"/>
+      <c r="G295" s="20" t="inlineStr"/>
+      <c r="H295" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I295" s="20" t="inlineStr"/>
     </row>
     <row r="296">
-      <c r="A296" t="n">
+      <c r="A296" s="20" t="n">
         <v>295</v>
       </c>
-      <c r="B296" t="inlineStr">
+      <c r="B296" s="20" t="inlineStr">
         <is>
           <t>Science / Biologie cellulaire</t>
         </is>
       </c>
-      <c r="C296" t="inlineStr">
+      <c r="C296" s="20" t="inlineStr">
         <is>
           <t>Apparition des premières cellules eucaryotes avec noyau</t>
         </is>
       </c>
-      <c r="D296" t="n">
+      <c r="D296" s="20" t="n">
         <v>-1200000000</v>
       </c>
-      <c r="E296" t="inlineStr">
+      <c r="E296" s="20" t="inlineStr">
         <is>
           <t>La cellule se complexifie : apparition du noyau cellulaire</t>
         </is>
       </c>
-      <c r="F296" t="inlineStr">
+      <c r="F296" s="20" t="inlineStr">
         <is>
           <t>Il y a 1,2 milliard d'années, une révolution silencieuse transforme la vie microscopique : l'apparition des cellules eucaryotes. Jusqu'à ce moment, toute la vie consiste en bactéries procaryotes : une simple goutte de cytoplasme avec de l'ADN flottant librement au centre. Soudain, certaines bactéries développent une membrane interne entourant leur ADN, créant une structure appelée "noyau". C'est comme si la cellule construisait une chambre de coffre-fort pour protéger ses gènes. Comment ? Les scientifiques pensent qu'une bactérie a avalé une autre bactérie, mais au lieu de la digérer, elles ont fusionné. C'est l'endosymbiose : une fusion bactérienne. Ces nouvelles cellules eucaryotes sont beaucoup plus grandes et plus complexes. Elles développent aussi des organelles : mitochondries (centrales électriques cellulaires), chloroplastes (panneaux solaires biologiques), réticulum endoplasmique (système de transport interne). Avec cette organisation interne, les cellules peuvent accumuler beaucoup plus d'énergie. Elles peuvent aussi se combiner pour former des organismes multicellulaires : les premiers protistes apparaissent (algues microscopiques). Ces cellules eucaryotes sont nos ancêtres directs. Sans cette évolution cellulaire, les plantes, les animaux, les champignons et les humains n'existeraient jamais.</t>
         </is>
       </c>
-      <c r="G296" t="inlineStr"/>
-      <c r="H296" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I296" t="inlineStr"/>
+      <c r="G296" s="20" t="inlineStr"/>
+      <c r="H296" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I296" s="20" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" t="n">
+      <c r="A297" s="20" t="n">
         <v>296</v>
       </c>
-      <c r="B297" t="inlineStr">
+      <c r="B297" s="20" t="inlineStr">
         <is>
           <t>Science / Paléontologie</t>
         </is>
       </c>
-      <c r="C297" t="inlineStr">
+      <c r="C297" s="20" t="inlineStr">
         <is>
           <t>Explosion cambrienne : diversification massive des formes de vie</t>
         </is>
       </c>
-      <c r="D297" t="n">
+      <c r="D297" s="20" t="n">
         <v>-600000000</v>
       </c>
-      <c r="E297" t="inlineStr">
+      <c r="E297" s="20" t="inlineStr">
         <is>
           <t>L'océan se remplit soudainement d'animaux complexes et variés</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr">
+      <c r="F297" s="20" t="inlineStr">
         <is>
           <t>Il y a 600 millions d'années, quelque chose d'extraordinaire se produit dans les océans : l'Explosion cambrienne. Pendant plus de 3 milliards d'années, la vie était dominée par des organismes microscopiques et quelques créatures molles et sans couleur. Puis, en quelques millions d'années seulement (un clin d'œil géologique), des centaines de nouvelles formes de vie complexes et bizarres émergent soudainement. Les fossiles montrent des trilobites (créatures blindées avec des yeux), des échinodermes (ancêtres des étoiles de mer), des mollusques (ancêtres des poulpes), des arthropodes (ancêtres des insectes et araignées). Pourquoi soudainement ? Les scientifiques pensent que plusieurs facteurs convergent : l'oxygène atmosphérique atteint finalement des niveaux suffisants pour supporter des animaux complexes. Les océans refroidissent légèrement après une ère glaciaire. Une mutation génétique majeure (gènes Hox) permet une plus grande variabilité corporelle. La compétition apparaît : les prédateurs apparaissent et forcent les proies à évoluer rapidement pour survivre. C'est une "course aux armements" biologique. Ces animaux cambriens sont nos ancêtres : leur diversité de corps et de stratégies de survie crée les plans de base de tous les animaux futurs. Les humains et tous les animaux terrestres descendent des survivants de cette explosion créative.</t>
         </is>
       </c>
-      <c r="G297" t="inlineStr"/>
-      <c r="H297" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I297" t="inlineStr"/>
+      <c r="G297" s="20" t="inlineStr"/>
+      <c r="H297" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I297" s="20" t="inlineStr"/>
     </row>
     <row r="298">
-      <c r="A298" t="n">
+      <c r="A298" s="20" t="n">
         <v>297</v>
       </c>
-      <c r="B298" t="inlineStr">
+      <c r="B298" s="20" t="inlineStr">
         <is>
           <t>Science / Zoologie</t>
         </is>
       </c>
-      <c r="C298" t="inlineStr">
+      <c r="C298" s="20" t="inlineStr">
         <is>
           <t>Apparition des premiers poissons (Ostracodermes)</t>
         </is>
       </c>
-      <c r="D298" t="n">
+      <c r="D298" s="20" t="n">
         <v>-500000000</v>
       </c>
-      <c r="E298" t="inlineStr">
+      <c r="E298" s="20" t="inlineStr">
         <is>
           <t>Les premiers vertébrés apparaissent : les ancêtres des poissons modernes</t>
         </is>
       </c>
-      <c r="F298" t="inlineStr">
+      <c r="F298" s="20" t="inlineStr">
         <is>
           <t>Il y a 500 millions d'années, dans les océans du Silurien, les premiers poissons apparaissent : les Ostracodermes. Ces créatures ressemblent à des petits têtards blindés, longues de quelques centimètres. Contrairement aux autres animaux marins, ils possèdent une innovation révolutionnaire : un squelette primitif fait de cartilage (comme celui des requins modernes) au lieu d'exosquelette externe. Mieux encore, ce squelette contient une moelle épinière et un cerveau primitif. C'est la naissance des vertébrés : le groupe auquel nous appartenons. Les Ostracodermes n'ont pas de mâchoires mobiles (ils aspirent leur nourriture), pas de nageoires paires, juste une bouche fixe. Mais ils sont efficaces : petit à petit, d'autres innovations apparaissent. Certains Ostracodermes développent des mâchoires flexibles, permettant une meilleure capture de nourriture. Certains développent des nageoires paires pour mieux contrôler leur mouvement dans l'eau. Sur des millions d'années, ces améliorations créent les poissons modernes : les placodermes (poissons à plaques osseuses), les chondrichthyens (requins et raies), puis les ostéichthyens (poissons osseux). Les humains sont des descendants très éloignés de ces premiers poissons : nos bras, nos jambes, notre crâne, notre colonne vertébrale viennent de cette lignée aquatique ancienne.</t>
         </is>
       </c>
-      <c r="G298" t="inlineStr"/>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I298" t="inlineStr"/>
+      <c r="G298" s="20" t="inlineStr"/>
+      <c r="H298" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I298" s="20" t="inlineStr"/>
     </row>
     <row r="299">
-      <c r="A299" t="n">
+      <c r="A299" s="20" t="n">
         <v>298</v>
       </c>
-      <c r="B299" t="inlineStr">
+      <c r="B299" s="20" t="inlineStr">
         <is>
           <t>Science / Botanique</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr">
+      <c r="C299" s="20" t="inlineStr">
         <is>
           <t>Les premières plantes colonisent la terre ferme (bryophytes primitives)</t>
         </is>
       </c>
-      <c r="D299" t="n">
+      <c r="D299" s="20" t="n">
         <v>-475000000</v>
       </c>
-      <c r="E299" t="inlineStr">
+      <c r="E299" s="20" t="inlineStr">
         <is>
           <t>Les continents se couvrent de végétation : les plantes quittent l'océan</t>
         </is>
       </c>
-      <c r="F299" t="inlineStr">
+      <c r="F299" s="20" t="inlineStr">
         <is>
           <t>Il y a 475 millions d'années, les continents sont totalement déserts : des roches nues sous un ciel sans couleur. Les plantes vivent uniquement dans l'océan. Puis, les premières plantes aquatiques découvrent comment survivre sur la terre sèche : les bryophytes primitives (ancêtres des mousses et hépatiques modernes). Comment ? Ces plantes développent plusieurs adaptations géniales. D'abord, un système de racines primitif qui s'enfonce dans le sol pour absorber l'eau et les nutriments minéraux. Ensuite, une cuticule cireuse sur la surface qui réduit l'évaporation : sans cette protection, la plante se dessécherait instantanément au contact de l'air. Troisièmement, un système de transport interne (vaisseaux) qui propage l'eau des racines aux feuilles. Enfin, des spores plutôt que des œufs pour se reproduire : les spores sont minuscules, légères, et peuvent voyager dans le vent sur de longues distances. Ces premières plantes sont minuscules, juste quelques centimètres, sans feuilles véritables, ressemblant à des mousses. Mais elles sont révolutionnaires. Elles transforment les roches nues en sol : leurs racines fracturent la roche, créant du terreau. Elles produisent de l'oxygène, modifiant l'atmosphère. Elles créent des habitats. Sur les millions d'années suivants, les plantes évoluent : des fougères plus grandes apparaissent (avec de vraies racines profondes), puis des plantes à graines, puis des fleurs. Sans cette colonisation terrestre, les animaux terrestres et les humains ne pourraient jamais exister.</t>
         </is>
       </c>
-      <c r="G299" t="inlineStr"/>
-      <c r="H299" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I299" t="inlineStr"/>
+      <c r="G299" s="20" t="inlineStr"/>
+      <c r="H299" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I299" s="20" t="inlineStr"/>
     </row>
     <row r="300">
-      <c r="A300" t="n">
+      <c r="A300" s="20" t="n">
         <v>299</v>
       </c>
-      <c r="B300" t="inlineStr">
+      <c r="B300" s="20" t="inlineStr">
         <is>
           <t>Science / Zoologie</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr">
+      <c r="C300" s="20" t="inlineStr">
         <is>
           <t>Apparition des premiers amphibiens : la transition de l'eau à la terre</t>
         </is>
       </c>
-      <c r="D300" t="n">
+      <c r="D300" s="20" t="n">
         <v>-360000000</v>
       </c>
-      <c r="E300" t="inlineStr">
+      <c r="E300" s="20" t="inlineStr">
         <is>
           <t>Les poissons développent des pattes et sortent de l'eau</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr">
+      <c r="F300" s="20" t="inlineStr">
         <is>
           <t>Il y a 360 millions d'années, quelque chose d'extraordinaire se produit dans les marécages et rivières du Carbonifère : les poissons développent des pattes et quittent l'eau. Ce sont les premiers amphibiens, comme le Tiktaalik et l'Ichthyostega. Comment des poissons deviennent-ils des créatures terrestres ? La clé est la nageoire : les nageoires paires des poissons (pectorales et pelviennes) évoluent progressivement en membres articulés (bras et jambes) avec os, articulations et muscles. Ces amphibiens primitifs gardent encore des caractéristiques de poisson : une queue aplatie pour nager, des branchies pour respirer sous l'eau. Mais ils développent aussi des poumons pour respirer l'air. Leurs nageoires deviennent de vraies pattes assez fortes pour supporter leur poids et les propulser sur la terre. Pourquoi quitter l'eau ? L'eau stagnante des marécages manque d'oxygène. Les amphibiens capables de ramper sur la terre et respirer l'air à la surface ont un avantage de survie énorme. Sur terre, ils découvrent un monde vierge rempli de nourriture (plantes, insectes) et sans prédateurs. Mais les premiers amphibiens restent dépendants de l'eau : ils doivent y retourner pour se reproduire, comme les grenouilles modernes. Sur les 100 millions d'années suivantes, certains amphibiens évoluent pour s'adapter à la vie terrestre complète. Ils développent une peau imperméable, des œufs avec coquille (pas besoin de l'eau pour la reproduction). Ce sont les reptiles. Et les humains, comme tous les mammifères terrestres, descendons de ces amphibiens intrépides qui ont osé explorer la terre.</t>
         </is>
       </c>
-      <c r="G300" t="inlineStr"/>
-      <c r="H300" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I300" t="inlineStr"/>
+      <c r="G300" s="20" t="inlineStr"/>
+      <c r="H300" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I300" s="20" t="inlineStr"/>
     </row>
     <row r="301">
-      <c r="A301" t="n">
+      <c r="A301" s="20" t="n">
         <v>300</v>
       </c>
-      <c r="B301" t="inlineStr">
+      <c r="B301" s="20" t="inlineStr">
         <is>
           <t>Science / Zoologie</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr">
+      <c r="C301" s="20" t="inlineStr">
         <is>
           <t>Apparition des premiers reptiles avec œufs à coquille dure</t>
         </is>
       </c>
-      <c r="D301" t="n">
+      <c r="D301" s="20" t="n">
         <v>-320000000</v>
       </c>
-      <c r="E301" t="inlineStr">
+      <c r="E301" s="20" t="inlineStr">
         <is>
           <t>L'amniote : l'invention géniale qui libère les vertébrés de l'eau</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr">
+      <c r="F301" s="20" t="inlineStr">
         <is>
           <t>Il y a 320 millions d'années, un événement biologique majeur transforme l'évolution terrestre : l'apparition des premiers vrais reptiles. Leur innovation clé ? L'œuf amniotique : un œuf avec une coquille imperméable contenant une poche d'eau (l'amnios) qui protège l'embryon. Pourquoi est-ce révolutionnaire ? Les amphibiens doivent retourner à l'eau pour pondre car leurs œufs sont mous et se déssèchent rapidement au soleil. Les reptiles, avec leur coquille dure, peuvent pondre loin de l'eau, sur la terre ferme. Cela signifie : indépendance totale de l'eau pour la reproduction. Plus besoin de revenir à l'eau chaque saison de reproduction. Les premiers reptiles amniotes ressemblent à des lézards, longs de quelques décimètres. Ils développent aussi une peau écailleuse imperméable qui retient l'eau, contrairement à la peau humide des amphibiens. Leurs pattes deviennent plus fortes, supportant leur corps de manière plus verticale. Ces adaptations les rendent extrêmement efficaces sur terre. Sur les 50 millions d'années suivantes, les reptiles se diversifient explosivement : certains deviennent énormes (les dinosaures), d'autres développent des ailes (les ptérosaures et oiseaux), d'autres une apparence mammalienne (les synapsides). Les reptiles dominent tous les écosystèmes terrestres pendant 250 millions d'années. Les humains descendons d'une lignée de petits reptiles synapsidés qui survivent à plusieurs extinctions de masse et finissent par devenir les mammifères.</t>
         </is>
       </c>
-      <c r="G301" t="inlineStr"/>
-      <c r="H301" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I301" t="inlineStr"/>
+      <c r="G301" s="20" t="inlineStr"/>
+      <c r="H301" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I301" s="20" t="inlineStr"/>
     </row>
     <row r="302">
-      <c r="A302" t="n">
+      <c r="A302" s="20" t="n">
         <v>301</v>
       </c>
-      <c r="B302" t="inlineStr">
+      <c r="B302" s="20" t="inlineStr">
         <is>
           <t>Science / Zoologie</t>
         </is>
       </c>
-      <c r="C302" t="inlineStr">
+      <c r="C302" s="20" t="inlineStr">
         <is>
           <t>Apparition des premiers synapsides : ancêtres des mammifères</t>
         </is>
       </c>
-      <c r="D302" t="n">
+      <c r="D302" s="20" t="n">
         <v>-300000000</v>
       </c>
-      <c r="E302" t="inlineStr">
+      <c r="E302" s="20" t="inlineStr">
         <is>
           <t>Les synapsides : la lignée qui mène directement aux mammifères et humains</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr">
+      <c r="F302" s="20" t="inlineStr">
         <is>
           <t>Il y a 300 millions d'années, dans les marécages du Carbonifère, apparaissent les synapsides : une lignée de reptiles qui semble ordinaire au premier abord. Les synapsides ressemblent à des reptiles normaux, ressemblant à des petits lézards ou à des pelycosaures (reptiles à voile de cheveux sur le dos). Mais ils possèdent une caractéristique unique : une fenêtre osseuse sur chaque côté du crâne (la fenêtre temporale), d'où s'attachent des muscles mâchoires puissants. Pourquoi est-ce important ? Ces muscles mâchoires permettent une morsure plus puissante et une meilleure mastication. Au cours des 100 millions d'années suivantes, les synapsides évoluent lentement mais sûrement vers quelque chose de plus étrange. Certains développent une posture de pattes plus verticale (sous le corps) plutôt qu'écartées sur les côtés comme les reptiles. Certains développent des dents différenciées : des incisives pour trancher, des canines pointues pour percer, des molaires pour broyer. C'est très différent des reptiles qui ont des dents uniformes. Certains développent une seule fenêtre osseuse supérieure au crâne plutôt que deux. Ces changements graduels transforment lentement les synapsides en quelque chose de nouveau : les cynodontes. Et les cynodontes, après 50 millions d'années d'évolution supplémentaire, deviendront les premiers mammifères vrais. Chaque humain vivant descend directement de ces synapsides apparemment ordinaires du Carbonifère.</t>
         </is>
       </c>
-      <c r="G302" t="inlineStr"/>
-      <c r="H302" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I302" t="inlineStr"/>
+      <c r="G302" s="20" t="inlineStr"/>
+      <c r="H302" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I302" s="20" t="inlineStr"/>
     </row>
     <row r="303">
-      <c r="A303" t="n">
+      <c r="A303" s="20" t="n">
         <v>302</v>
       </c>
-      <c r="B303" t="inlineStr">
+      <c r="B303" s="20" t="inlineStr">
         <is>
           <t>Science / Paléontologie</t>
         </is>
       </c>
-      <c r="C303" t="inlineStr">
+      <c r="C303" s="20" t="inlineStr">
         <is>
           <t>Extinction du Permien : 95% de la vie terrestre disparaît</t>
         </is>
       </c>
-      <c r="D303" t="n">
+      <c r="D303" s="20" t="n">
         <v>-250000000</v>
       </c>
-      <c r="E303" t="inlineStr">
+      <c r="E303" s="20" t="inlineStr">
         <is>
           <t>La plus grande extinction de masse de l'histoire : la «Grande Mort»</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr">
+      <c r="F303" s="20" t="inlineStr">
         <is>
           <t>Il y a 250 millions d'années, c'est l'apocalypse biologique : l'Extinction du Permien, aussi appelée "la Grande Mort" (The Great Dying). C'est la pire extinction de masse dans toute l'histoire de la vie. Les chiffres sont terrifiants : 95% de toutes les espèces marines disparaissent. 70% de toutes les espèces de vertébrés terrestres disparaissent. Seules quelques espèces survivent et repeuplent le monde ensuite. Qu'est-ce qui cause ce cataclysme ? Les scientifiques déterminent plusieurs causes qui convergeaient à la même époque. D'abord, le "trappage sibérien" : dans la région de la Sibérie, d'énormes éruptions volcaniques massives se produisent pendant des milliers d'années. Ces volcans libèrent des millions de tonnes de cendres volcaniques, d'acide sulfurique, et surtout du dioxyde de carbone. Le CO2 crée un effet de serre massif : les températures mondiales augmentent de 5 à 10 degrés Celsius. Les océans se réchauffent dangereusement. Les zones côtières produisent moins d'oxygène. Les niveaux marins baissent. Les écosystèmes marins s'effondrent. De plus, les cendres volcaniques bloquent le soleil, tuant les plantes et créant une famine. Les animaux qui survivent sont ceux qui peuvent jeûner longtemps, tolérer les températures extrêmes, et s'adapter rapidement aux nouvelles conditions. Les synapsides survivent à cette extinction mieux que les autres reptiles. Après cet événement catastrophique, le monde est vide. Les synapsides survivants se diversifient rapidement pour remplir tous les rôles écologiques laissés vacants. Cet "reset" écologique crée les opportunités pour que les cynodontes (descendants synapsides) évoluent ensuite en mammifères. Sans cette extinction terrifiante, les dinosaures, pas les synapsides, auraient dominé le monde, et les mammifères n'auraient jamais existé.</t>
         </is>
       </c>
-      <c r="G303" t="inlineStr"/>
-      <c r="H303" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I303" t="inlineStr"/>
+      <c r="G303" s="20" t="inlineStr"/>
+      <c r="H303" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I303" s="20" t="inlineStr"/>
     </row>
     <row r="304">
-      <c r="A304" t="n">
+      <c r="A304" s="20" t="n">
         <v>303</v>
       </c>
-      <c r="B304" t="inlineStr">
+      <c r="B304" s="20" t="inlineStr">
         <is>
           <t>Science / Zoologie</t>
         </is>
       </c>
-      <c r="C304" t="inlineStr">
+      <c r="C304" s="20" t="inlineStr">
         <is>
           <t>Apparition des premiers mammifères (petits nocturnes)</t>
         </is>
       </c>
-      <c r="D304" t="n">
+      <c r="D304" s="20" t="n">
         <v>-220000000</v>
       </c>
-      <c r="E304" t="inlineStr">
+      <c r="E304" s="20" t="inlineStr">
         <is>
           <t>Les mammifères naissent dans l'ombre des dinosaures</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr">
+      <c r="F304" s="20" t="inlineStr">
         <is>
           <t>Il y a 220 millions d'années, au moment où les dinosaures commencent à dominer la Terre, un groupe de petits reptiles abandonne la compétition directe et se cache : les premiers mammifères. Ces créatures, comme le Morganucodon et l'Hadrocodium, sont minuscules : longues de seulement 10 à 30 centimètres, pesant quelques grammes, ressemblant à de petites musaraignes. Elles sont timides, nocturnes, se cachant sous terre et dans les arbres pendant le jour, sortant la nuit chercher nourriture. Pourquoi sont-elles "mammifères" ? Elles possèdent des caractéristiques que seuls les mammifères ont. D'abord, un crâne spécialisé avec une fenêtre osseuse pour les muscles mâchoires (héritage des synapsides). Deuxièmement, des dents différenciées : incisives, canines, molaires, permettant une mastication efficace. Troisièmement, trois os d'oreille interne (marteau, enclume, étrier) plutôt que les os de mâchoire de reptiles. Quatrièmement, un palais dur qui sépare la bouche de la respiration, permettant une respiration continue pendant la mastication. Ces adaptations rendent les premiers mammifères extrêmement efficaces pour chasser de petites proies (insectes, petits lézards) la nuit. Pendant 140 millions d'années, les mammifères restent petits et rares, toujours éclipsés par les dinosaures dominants. Mais quand les dinosaures s'éteignent soudainement (extinction K-T, il y a 66 millions d'années), les mammifères survivants évoluent rapidement pour remplir tous les rôles écologiques laissés vacants. Sans cette période d'évolution cachée, les mammifères ne seraient jamais devenus les créatures dominantes du monde actuel, et les humains n'existeraient pas.</t>
         </is>
       </c>
-      <c r="G304" t="inlineStr"/>
-      <c r="H304" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I304" t="inlineStr"/>
+      <c r="G304" s="20" t="inlineStr"/>
+      <c r="H304" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I304" s="20" t="inlineStr"/>
     </row>
     <row r="305">
-      <c r="A305" t="n">
+      <c r="A305" s="20" t="n">
         <v>304</v>
       </c>
-      <c r="B305" t="inlineStr">
+      <c r="B305" s="20" t="inlineStr">
         <is>
           <t>Science / Anthropologie</t>
         </is>
       </c>
-      <c r="C305" t="inlineStr">
+      <c r="C305" s="20" t="inlineStr">
         <is>
           <t>Homo erectus maîtrise et utilise régulièrement le feu</t>
         </is>
       </c>
-      <c r="D305" t="n">
+      <c r="D305" s="20" t="n">
         <v>-1500000</v>
       </c>
-      <c r="E305" t="inlineStr">
+      <c r="E305" s="20" t="inlineStr">
         <is>
           <t>La maîtrise du feu : l'une des plus grandes révolutions de l'évolution humaine</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr">
+      <c r="F305" s="20" t="inlineStr">
         <is>
           <t>Il y a 1,5 million d'années, dans les vallées d'Afrique de l'Est (Éthiopie, Kenya), le Homo erectus franchit un cap extraordinaire : maîtriser le feu. Ce n'est pas qu'il découvre soudainement le feu. Les hominidés antérieurs (Homo habilis) ont probablement utilisé le feu naturel (provenant des éruptions volcaniques ou éclairs) occasionnellement. Mais Homo erectus fait quelque chose de révolutionnaire : il apprend à créer le feu intentionnellement et à le maintenir allumé. Comment ? En frappant des roches de silex contre du granit pour produire des étincelles, ou en frottant du bois pour créer de la chaleur. Pourquoi c'est révolutionnaire ? Le feu change absolument tout. D'abord, nutrition : la cuisson tue les bactéries dangereuses et les parasites dans la viande et les plantes. Elle rend aussi la nourriture plus facile à digérer, ce qui signifie que le corps absorbe plus de nutriments avec moins d'effort. Cela libère de l'énergie pour d'autres fonctions, notamment le cerveau. Deuxièmement, survie : le feu tient chaud, crucial pour les humains qui perdent rapidement la chaleur corporelle. Il repousse les prédateurs la nuit. Troisièmement, socialité : le feu rassemble les gens. Assis autour du feu, les humains commencent à socialiser, parler, raconter des histoires, enseigner aux enfants. C'est probablement quand le langage devient plus complexe. Quatrièmement, technologie : le feu peut être utilisé pour travailler le bois, la pierre, l'os. Il rend possible des outils plus sophistiqués. Avec le feu, Homo erectus peut migrer vers des régions froides (Europe du Nord, Asie). Pendant environ 1 million d'années, Homo erectus utilise le feu, se propageant à travers le monde. Ses descendants (Homo neanderthalensis, Homo sapiens) héritent de cette technologie révolutionnaire et la raffinent encore plus. Sans la maîtrise du feu, le cerveau humain ne se serait jamais aussi développé, et la civilisation n'existerait pas.</t>
         </is>
       </c>
-      <c r="G305" t="inlineStr"/>
-      <c r="H305" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I305" t="inlineStr"/>
+      <c r="G305" s="20" t="inlineStr"/>
+      <c r="H305" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I305" s="20" t="inlineStr"/>
     </row>
     <row r="306">
-      <c r="A306" t="n">
+      <c r="A306" s="20" t="n">
         <v>305</v>
       </c>
-      <c r="B306" t="inlineStr">
+      <c r="B306" s="20" t="inlineStr">
         <is>
           <t>Science / Paléontologie</t>
         </is>
       </c>
-      <c r="C306" t="inlineStr">
+      <c r="C306" s="20" t="inlineStr">
         <is>
           <t>Homo heidelbergensis : ancêtre commun probable de Néandertal et Sapiens</t>
         </is>
       </c>
-      <c r="D306" t="n">
+      <c r="D306" s="20" t="n">
         <v>-500000</v>
       </c>
-      <c r="E306" t="inlineStr">
+      <c r="E306" s="20" t="inlineStr">
         <is>
           <t>L'ancêtre hypothétique qui sépare les destinées de deux humanités</t>
         </is>
       </c>
-      <c r="F306" t="inlineStr">
+      <c r="F306" s="20" t="inlineStr">
         <is>
           <t>Il y a 500 000 ans, une créature appelée Homo heidelbergensis vit en Afrique, en Europe et en Asie. C'est un individu fascinant qui représente une étape critique de l'évolution humaine. Homo heidelbergensis est plus grand et plus robuste que Homo erectus (taille humaine, poids 70-90 kg). Son crâne est plus grand avec un volume cérébral de 1200-1400 centimètres cubes (comparable aux humains modernes). Ses os sont plus épais, ses muscles plus puissants. Qu'est-ce qui le rend spécial ? Les données génétiques et fossiles suggèrent qu'Homo heidelbergensis est probablement l'ancêtre commun de deux espèces humaines différentes qui évoluent ensuite séparément. En Europe, où le climat devient très froid, Homo heidelbergensis évolue en Homo neanderthalensis (les Néandertaliens), avec des corps plus courts et trapus, adaptés au froid. En Afrique, où le climat reste chaud, Homo heidelbergensis évolue en Homo sapiens (nous), avec des corps plus longs et gracieux. Homo heidelbergensis lui-même est un chasseur efficace. Les preuves archéologiques montrent qu'il fabrique des bifaces (outils de pierre bifaciales) sophistiqués appelés "coups de poing" (hand axes). Il chasse probablement des animaux de grande taille en groupes coordonnés, nécessitant une communication complexe et une planification. Son cerveau suffisamment grand suggère qu'il possède un langage et une capacité à enseigner. C'est probablement la première espèce humaine avec une véritable culture transmissible. Homo heidelbergensis disparaît il y a environ 300 000 ans, remplacé par ses descendants plus spécialisés (Néandertal et Sapiens). Mais sans Homo heidelbergensis, ces deux branches distinctes d'humanité n'auraient jamais émergé.</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr"/>
-      <c r="H306" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I306" t="inlineStr"/>
+      <c r="G306" s="20" t="inlineStr"/>
+      <c r="H306" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I306" s="20" t="inlineStr"/>
     </row>
     <row r="307">
-      <c r="A307" t="n">
+      <c r="A307" s="20" t="n">
         <v>306</v>
       </c>
-      <c r="B307" t="inlineStr">
+      <c r="B307" s="20" t="inlineStr">
         <is>
           <t>Science / Anthropologie</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr">
+      <c r="C307" s="20" t="inlineStr">
         <is>
           <t>Homo neanderthalensis émerge en Europe</t>
         </is>
       </c>
-      <c r="D307" t="n">
+      <c r="D307" s="20" t="n">
         <v>-430000</v>
       </c>
-      <c r="E307" t="inlineStr">
+      <c r="E307" s="20" t="inlineStr">
         <is>
           <t>Le Néandertal : une espèce humaine distincte adaptée au froid glacial</t>
         </is>
       </c>
-      <c r="F307" t="inlineStr">
+      <c r="F307" s="20" t="inlineStr">
         <is>
           <t>Il y a 430 000 ans, dans les grottes et vallées de l'Europe, une nouvelle espèce humaine émerge : Homo neanderthalensis, que nous appelons les Néandertaliens. Ils évoluent à partir d'Homo heidelbergensis pendant une période de glaciation intense. Le climat européen devient beaucoup plus froid et inhospitalier. Homo neanderthalensis développe une morphologie extrêmement bien adaptée au froid : corps trapus et robustes (plus courts mais plus lourds que Homo sapiens), crâne plus grand avec un cerveau légèrement plus gros que le nôtre (1450-1600 cm³ contre 1400 pour Sapiens). Leur corps trapu minimise la perte de chaleur (surface/volume réduit). Leurs extrémités (doigts, orteils, nez) sont plus courtes pour réduire la gelure. Leurs muscles sont massifs, leur densité osseuse très élevée, les rendant extrêmement forts (environ 20% plus forts qu'un humain moderne). Ils développent des outils de pierre raffinés appelés "industries moustériennes" : des racloirs, des lames, des pointes de lance pour chasser les mégafaunes (mammouths, bisons, rennes). Les preuves archéologiques suggèrent qu'ils vivent en petits groupes, chassent en coordonnés (nécessitant communication complexe), et ont peut-être un langage sophistiqué. Certaines preuves indiquent qu'ils prennent soin de leurs malades et blessés, et qu'ils enterrent leurs morts avec des rituels, suggérant une conscience de la mort et possiblement une spiritualité. Les Néandertaliens prospèrent en Europe et en Asie occidentale pendant environ 200 000 ans. Mais quand Homo sapiens arrive d'Afrique il y a 40 000 ans, mieux adapté aux changements climatiques rapides, les Néandertaliens entrent en déclin et disparaissent il y a environ 30 000 ans. Ironiquement, ils ne disparaissent pas complètement : environ 1-4% du génome de tous les humains non-africains contient de l'ADN néandertalien.</t>
         </is>
       </c>
-      <c r="G307" t="inlineStr"/>
-      <c r="H307" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I307" t="inlineStr"/>
+      <c r="G307" s="20" t="inlineStr"/>
+      <c r="H307" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I307" s="20" t="inlineStr"/>
     </row>
     <row r="308">
-      <c r="A308" t="n">
+      <c r="A308" s="20" t="n">
         <v>307</v>
       </c>
-      <c r="B308" t="inlineStr">
+      <c r="B308" s="20" t="inlineStr">
         <is>
           <t>Science / Anthropologie</t>
         </is>
       </c>
-      <c r="C308" t="inlineStr">
+      <c r="C308" s="20" t="inlineStr">
         <is>
           <t>Homo sapiens archaïque émerge en Afrique</t>
         </is>
       </c>
-      <c r="D308" t="n">
+      <c r="D308" s="20" t="n">
         <v>-300000</v>
       </c>
-      <c r="E308" t="inlineStr">
+      <c r="E308" s="20" t="inlineStr">
         <is>
           <t>L'émergence de notre propre espèce : Homo sapiens archaïque en Afrique</t>
         </is>
       </c>
-      <c r="F308" t="inlineStr">
+      <c r="F308" s="20" t="inlineStr">
         <is>
           <t>Il y a 300 000 ans, quelque part en Afrique subsaharienne (probablement en Afrique du Sud et de l'Est), une nouvelle espèce humaine émerge : Homo sapiens archaïque. C'est nous, ou plutôt, ce sont nos ancêtres les plus directs. Les fossiles montrent une transition progressive depuis Homo heidelbergensis. Les changements majeurs : d'abord, le crâne s'aplatit. Chez Homo erectus et Homo heidelbergensis, le front fuit vers l'arrière et il y a un bourrelet proéminent au-dessus des yeux. Chez Homo sapiens, le front devient vertical, donnant du style à un menton (unique aux humains modernes). Deuxièmement, la face devient plus petite et gracile plutôt que robuste. Troisièmement, le cerveau se réorganise : la partie frontale s'agrandit (pensée abstraite, langage, planification), tandis que l'occipital s'arrondit. Homo sapiens archaïque (300 000 à 100 000 ans) n'est pas encore complètement "moderne" mais s'en rapproche. Ils fabriquent des outils de pierre sophistiqués, chassent efficacement et cuisent leur nourriture avec le feu depuis longtemps. Vers 200 000 ans, certains fossiles montrent les caractéristiques entièrement "modernes" : crâne arrondi, petite face, menton proéminent. C'est Homo sapiens moderne. Entre 100 000 et 70 000 ans, des groupes de Homo sapiens modernes commencent à quitter l'Afrique pour explorer le Moyen-Orient, puis l'Europe, l'Asie, l'Océanie : c'est la "Grande Migration" qui peuplera tous les continents. Sans cette émergence en Afrique, la branche Sapiens de l'humanité n'existerait pas.</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I308" t="inlineStr"/>
+      <c r="G308" s="20" t="inlineStr"/>
+      <c r="H308" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I308" s="20" t="inlineStr"/>
     </row>
     <row r="309">
-      <c r="A309" t="n">
+      <c r="A309" s="20" t="n">
         <v>308</v>
       </c>
-      <c r="B309" t="inlineStr">
+      <c r="B309" s="20" t="inlineStr">
         <is>
           <t>Science / Anthropologie</t>
         </is>
       </c>
-      <c r="C309" t="inlineStr">
+      <c r="C309" s="20" t="inlineStr">
         <is>
           <t>Apogée de Homo neanderthalensis : culture moustérienne au sommet</t>
         </is>
       </c>
-      <c r="D309" t="n">
+      <c r="D309" s="20" t="n">
         <v>-280000</v>
       </c>
-      <c r="E309" t="inlineStr">
+      <c r="E309" s="20" t="inlineStr">
         <is>
           <t>Le Néandertal à son apogée : technologie, chasse, et vie sociale</t>
         </is>
       </c>
-      <c r="F309" t="inlineStr">
+      <c r="F309" s="20" t="inlineStr">
         <is>
           <t>Il y a 280 000 ans, les Néandertaliens atteignent leur apogée en termes de population, de distribution géographique, et de sophistication technologique. À ce moment, environ 100 000 à 500 000 Néandertaliens vivent en Europe, Asie mineure, et Asie occidentale (du Portugal à la Sibérie). Ils maîtrisent une vaste gamme de technologies de chasse. L'industrie moustérienne (la technologie principale) produit des dizaines de types d'outils : des racloirs pour enlever la peau des animaux, des lames pointues pour découper la viande, des pointes de lance pour la chasse. La technique dite "Levallois" permet de préparer une pierre pour produire des lames pré-définies : un savoir-faire nécessitant apprentissage long et communication sophistiquée, probablement un véritable langage parlé. Les preuves archéologiques montrent qu'ils vivent en groupes d'environ 20-30 individus, chassant des mégafaunes (mammouths, rhinos laineux, bisons, chevaux) souvent en groupe coordonné. Les fossiles montrent des traumatismes similaires à ceux de cavaliers de rodéo, indiquant une chasse au corps à corps dangereuse mais productive. Certaines preuves fossiles suggèrent qu'ils s'occupent de membres blessés : un fossile montre un Néandertal ayant survécu des années avec un bras amputé, impossible sans l'aide du groupe, indiquant empathie et cohésion sociale. Des sites archéologiques montrent des restes de fleurs autour de squelettes, suggérant des sépultures rituelles. À cet apogée, les Néandertaliens semblent être une espèce entièrement intelligente et culturellement sophistiquée. Mais cette apogée est aussi le début du déclin : vers 50 000 ans, le climat change et Homo sapiens arrive d'Afrique, plus flexible et adaptatif. Les Néandertaliens déclinent lentement et le dernier disparaît il y a environ 30 000 ans.</t>
         </is>
       </c>
-      <c r="G309" t="inlineStr"/>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I309" t="inlineStr"/>
+      <c r="G309" s="20" t="inlineStr"/>
+      <c r="H309" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I309" s="20" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Archéologie / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Première vague de migration de Sapiens hors d'Afrique</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>-70000</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Les humains modernes commencent à quitter le continent africain</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Il y a 70 000 ans, un groupe d'Homo sapiens quitte l'Afrique pour la première fois et se lance dans une aventure qui durera des millénaires : le peuplement du monde entier. Avant cette date, tous les humains modernes vivaient en Afrique, principalement en Afrique de l'Est et du Sud. Mais à cette époque, certains groupes décident de partir vers le nord, franchissant le Sinaï et se dirigeant vers le Moyen-Orient et l'Asie. Cette migration n'est pas une décision planifiée : c'est plutôt une lente expansion des territoires de chasse. Au fil des générations, les groupes s'éloignent progressivement de l'Afrique. Les raisons exactes de cette migration restent débattues : certains scientifiques pensent que des changements climatiques (assèchement du Sahara) les ont poussés à partir. D'autres pensent que c'est simplement le résultat naturel de la croissance démographique. Les premiers migrants franchissent le détroit de la mer Rouge, probablement par bateau ou radeau primitif, montrant une capacité à naviguer et à traverser l'eau. Ces premiers voyageurs sont extrêmement courageux : ils entrent dans des territoires inconnus, avec des climats différents, des animaux différents, une végétation différente. Beaucoup de groupes n'iront pas loin. Certains reviennent. Mais d'autres persévèrent et continuent vers l'est. Cette première vague de migration est cruciale : c'est le début du peuplement de l'Eurasie. Sans cette migration audacieuse, les humains seraient restés confinés à l'Afrique.</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Archéologie / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Homo sapiens arrive en Asie du Sud-Est</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>-65000</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Les premiers humains modernes atteignent l'Asie du Sud-Est</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Il y a 65 000 ans, des groupes d'Homo sapiens atteignent l'Asie du Sud-Est, une région qui comprend aujourd'hui la Thaïlande, la Malaisie, l'Indonésie et les Philippines. Ce voyage depuis l'Afrique a duré au moins 5 000 ans, les groupes se déplaçant lentement, génération après génération, à travers le Moyen-Orient, puis vers le sud et l'est. Les preuves archéologiques viennent de sites comme Ksar Akil (Liban), Qafzeh (Iran) et des grottes en Thaïlande datant de cette époque. Ces premiers Sapiens en Asie du Sud-Est rencontrent un environnement tropical dense, chaud et humide, très différent de l'Afrique. Ils doivent adapter leur technologie de chasse et leurs techniques de survie. Des fossiles et des artefacts montrent qu'ils fabriquent des outils en pierre sophistiqués, chassent des animaux variés, et collectent des plantes. Des coquillages avec des trous percés, trouvés dans les grottes thaïlandaises, suggèrent qu'ils fabriquent déjà des parures : des colliers ou des bracelets. Cela indique un sens esthétique, peut-être même un sens de l'identité personnelle ou de groupe. Ces humains vivent en petits groupes de 20-50 personnes, chassent et cueillent pour survivre. Ils développent progressivement une connaissance intime de leur environnement : quelles plantes sont comestibles, où trouver l'eau, quand et où migrer. Cette adaptation à l'environnement tropical est cruciale : elle prépare le terrain pour la future colonisation de l'Australie, qui aura lieu 15 000 ans plus tard. Sans cette arrivée en Asie du Sud-Est, les humains n'auraient jamais pu atteindre l'Australie.</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Archéologie / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Homo sapiens colonise l'Australie</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Les humains atteignent l'Australie en traversant l'océan pour la première fois</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Il y a 50 000 ans, un événement extraordinaire se produit : des groupes d'Homo sapiens franchissent l'océan et arrivent en Australie. C'est la première fois que des humains quittent les continents connus (Afrique, Asie, Europe) pour coloniser une terre complètement isolée. Cette migration représente un exploit technologique et culturel majeur. Pour atteindre l'Australie, les humains doivent traverser des détroits maritimes. À cette époque, le niveau des mers est plus bas (la glace recouvre les pôles), mais le détroit de Timor, entre l'Asie du Sud-Est et l'Australie, reste impassable à pied. Les humains doivent donc utiliser des bateaux ou des radeaux. Les preuves archéologiques montrent que les premiers Australiens arrivent à Lake Mungo, dans le sud-est de l'Australie, et rapidement ils colonisent tout le continent. Des fossiles de 50 000 à 45 000 ans montrent que les humains s'implantent dans tous les environnements australiens : déserts, côtes, montagnes. Cette diversification rapide montre une grande adaptabilité. Les archéologues trouvent des sites de foyers (feux) montrant que ces premiers Australiens maîtrisent le feu. Ils fabriquent des outils en pierre, des harpons, des filets. Des squelettes montrent que la vie est dure : fractures, infections, malnutrition. Mais les groupes prospèrent. Une découverte fascinante : une peinture rupestre datée de plus de 51 000 ans montre un stencil de main (empreinte de main). C'est l'une des plus anciennes formes d'art connu, presque certainement créée par ces premiers Australiens. L'empreinte de main est un geste universel d'affirmation de présence : "J'étais là". Ces premiers Australiens développent une culture riche avec des peintures, des sculptures en bois (les boomerangs apparaissent vers 30 000 ans), et des traditions orales. Les Aborigènes australiens contemporains sont les descendants directs de ces premiers migrants, ce qui en fait l'une des cultures humaines les plus anciennes et les plus continues du monde.</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr"/>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Archéologie / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Arrivée de Sapiens en Europe - Rencontre avec Néandertal</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>-45000</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Les humains modernes arrivent en Europe et rencontrent pour la première fois les Néandertaliens</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Il y a 45 000 ans, un événement décisif se produit en Europe : les premiers Homo sapiens arrivent du Moyen-Orient et rencontrent les Néandertaliens qui vivent en Europe depuis 250 000 ans. C'est la première rencontre entre deux espèces humaines intelligentes. Cette arrivée est datée précisément grâce aux fossiles de Mladeč (Tchéquie) et des sites de culture Aurignacienne, qui montrent clairement des caractéristiques de Sapiens modernes. Pendant les 10 000 années suivantes, Sapiens et Néandertal coexistent en Europe, probablement dans des régions différentes, mais parfois en contact direct. Les preuves archéologiques et génétiques montrent que ces deux espèces interagissent. Des analyses ADN révèlent que tous les Sapiens non-africains modernes portent 1 à 4% d'ADN Néandertal, ce qui signifie qu'il y a eu métissage. Cela implique des rencontres pacifiques, au moins occasionnellement. Mais la coexistence n'est pas simplement pacifique : il y a probablement aussi compétition pour les ressources de chasse. Les deux espèces chassent les mêmes animaux (mammouths, rennes, bisons). Sapiens, avec sa technologie plus avancée (premiers outils en os, premiers vêtements cousus, premiers harpons), a un avantage. Progressivement, Néandertal décline. Les derniers Néandertaliens disparaissent vers 35 000-30 000 ans. Néanmoins, les preuves d'intermariage restent plus probantes que celles de conflits massifs. L'arrivée de Sapiens en Europe marque le début de la domination humaine moderne sur le continent et la fin de l'ère des Néandertaliens.</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Archéologie / Culture</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Explosion créative : art pariétal, sculpture et parures</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>-40000</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Le comportement humain change radicalement avec l'apparition de l'art et de la symbolique</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Il y a 40 000 ans, quelque chose de remarquable se produit chez les humains : une "explosion créative". Cette période marque le début d'une transformation culturelle majeure. Soudainement, les preuves archéologiques montrent des peintures rupestres, des sculptures, des bijoux, des outils élaborés. C'est comme si un interrupteur était actionné. Avant 40 000 ans, les preuves d'art symbolique sont rares et douteuses. Après 40 000 ans, l'art devient courant et sophistiqué. Les grottes d'Europe se remplissent de peintures magnifiques : mains stencilisées, animaux (chevaux, bisons, rhinocéros), signes abstraits. Ces peintures ne sont pas des gribouillages naïfs : elles montrent une compréhension de la perspective, de la proportion, du mouvement. Parallèlement, les sculptures apparaissent. La Vénus de Hohle Fels, en Allemagne, datée de 40 000 ans, est une petite figurine de femme nue, sculptée en ivoire, mesurant 6 centimètres. Les bijoux apparaissent aussi : colliers de dents d'animaux percées, bracelets de coquillages. Certains squelettes de 40 000 ans sont enterrés avec des parures, suggérant que la beauté personnelle et l'identité visuelle deviennent importantes. Pourquoi cette explosion créative survient-elle maintenant ? Les scientifiques débattent. Une théorie : le langage parlé devient plus sophistiqué, permettant une meilleure communication et une meilleure transmission des idées. Une autre : le cerveau humain atteint sa maturité cognitive complète, permettant l'abstraction et l'imaginaire. Une troisième : la population augmente, créant plus d'interaction entre les groupes et d'échange d'idées. Quelle qu'en soit la raison, cette explosion créative marque un tournant : les humains commencent à créer une culture, pas simplement à survivre.</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Archéologie / Anthropologie</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Disparition du dernier Néandertal</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>-35000</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Les Néandertaliens disparaissent, Homo sapiens devient la seule espèce humaine</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Il y a 35 000 ans, le dernier Néandertal disparaît. C'est la fin d'une espèce qui a prospéré en Europe pendant 250 000 ans. Les derniers Néandertaliens vivent dans les régions isolées du sud de la Péninsule Ibérique (Espagne et Portugal), où le climat plus doux permet à quelques populations de survivre plus longtemps. Après 35 000 ans, aucune trace fossile de Néandertal n'existe. Homo sapiens est désormais seul. La disparition du Néandertal n'est pas instantanée : elle s'étale sur plusieurs milliers d'années, probablement de 45 000 à 35 000 ans. Pendant cette période, les deux espèces coexistent, mais Sapiens augmente progressivement ses populations tandis que Néandertal décline. Pourquoi Néandertal disparaît-il ? Les scientifiques proposent plusieurs théories : Sapiens le tue ou l'expulse de ses territoires ; Sapiens, plus adaptatif et plus créatif, a un avantage compétitif ; un changement climatique défavorable aux Néandertaliens pousse les populations vers l'extinction ; des maladies, probablement apportées par Sapiens, déciment les populations Néandertal. Probablement, c'est une combinaison de tous ces facteurs. Les preuves génétiques montrent que les deux espèces se sont métissées, laissant 1 à 4% d'ADN Néandertal chez tous les Sapiens non-africains. Ironiquement, Néandertal n'a pas entièrement disparu : son génome vit à travers nous. Certains gènes Néandertal spécifiquement liés à l'immunité ont probablement aidé Sapiens à s'adapter aux maladies eurasiatiques. La disparition de Néandertal est un moment charnière : pour la première fois en 5-6 millions d'années d'évolution humaine, il n'y a plus de compétition d'autres hominidés.</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Archéologie / Art</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Gravures et sculptures sophistiquées - Vénus de Willendorf</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>L'art figuratif devient courant et montre une compréhension profonde de la forme et de la beauté</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Il y a 30 000 ans, les humains créent des sculptures de plus en plus sophistiquées. L'une des plus célèbres est la Vénus de Willendorf, découverte en Autriche, datée de 29 000 à 25 000 ans. C'est une petite figurine en calcaire de 11 centimètres de haut, qui représente une femme nue, avec des seins proéminents, un ventre rond, et les jambes atrophiées. Le visage n'a pas de traits distincts, mais la tête a un motif qui ressemble à des nattes ou des cheveux tressés. Pourquoi cette figurine ? Les archéologues ont proposé de nombreuses interprétations : une déesse de la fertilité (le corps gras et enceinte symbolise la fécondité), un autoportrait d'une femme enceinte, une poupée destinée à l'amusement des enfants, ou un objet magique supposé apporter la fertilité au groupe. Ce qui est clair : les humains, à cette époque, créent des objets sophistiqués avec intention symbolique, pas pratique. L'existence de la Vénus de Willendorf et d'autres figurines similaires (trouvées en Russie, en Europe centrale, en France) montre que la sculpture est une pratique courante. Les outils aussi deviennent plus sophistiqués : des aiguilles en os pour coudre les vêtements, des harpons barbelés pour la pêche, des bâtons de commandement. Les squelettes montrent que les humains vivent en meilleure santé : moins de fractures, moins d'infections. Les grottes contiennent des restes de foyers, de nourriture stockée, de matériaux bruts pour la fabrication d'outils, suggérant des habitats plus permanents et une meilleure organisation sociale. À 30 000 ans, les humains ne sont pas juste des survivants : ce sont des artistes, des artisans, des penseurs symboliques.</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Archéologie / Art</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Apogée de l'art pariétal - Grottes Chauvet et Lascaux</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Les grottes remplies de peintures deviennent des galeries d'art majeures</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Il y a 25 000 ans, les grottes d'Europe contiennent des quantités massives de peintures et de gravures. Bien que la grotte Chauvet (en France) soit datée de 36 000 ans et la grotte Lascaux de 17 000 ans, la période de 25 000 ans représente l'apogée de l'art rupestre gravetien et pré-magdalénien. Ces grottes ne sont pas des habitats : ce sont des sanctuaires sacrés, des galeries d'art, des lieux de culte ou de rituel, souvent dans les parties les plus profondes et inaccessibles, dans l'obscurité totale. La grotte Chauvet, avec ses 400 peintures, contient des images magnifiques : chevaux, bisons, lions des cavernes, rhinocéros, disposées en suivant les contours naturels de la roche. Les pigments utilisés sont de l'ocre rouge et du charbon noir, appliqués avec les mains, des bâtons, peut-être des brosses primitives. Dans la grotte Chauvet, il y a environ 150 empreintes de mains, chacune unique, datées de 37 500 à 33 900 ans : parmi les plus anciennes preuves que les humains reconnaissent l'individualité et laissent une trace de leur passage. Pourquoi l'art ? Les théories incluent la magie de chasse, le chamanisme, la religion, le marquage identitaire de territoire, ou simplement l'esthétique. Probablement une combinaison de tout cela. En 1994, la grotte Chauvet est découverte par hasard par des spéléologues, les peintures pratiquement intactes, préservées par le calcaire et l'atmosphère stable de la grotte. Voir ces peintures est une connexion directe avec les humains d'il y a 36 000 ans, rappelant que le besoin de créer et d'exprimer la beauté est aussi vieux que l'humanité moderne.</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Technologie / Chasse</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Bow and arrow technology émerge</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>L'arc et la flèche révolutionnent la chasse et le combat</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Il y a 20 000 ans, les preuves archéologiques montrent l'émergence d'une nouvelle technologie : l'arc et la flèche. Les plus anciennes preuves proviennent de sites en Afrique du Sud (Sibudu Cave) et en Europe (Stellmoor, Allemagne), datées entre 20 000 et 17 000 ans. Avant cela, les humains utilisent principalement des javelots lancés à la main ou des atlatls (bâtons de propulsion). Mais l'arc et la flèche offrent des avantages majeurs : plus de précision, plus de puissance, une portée plus grande (jusqu'à 50-100 mètres), et moins d'effort physique. Un chasseur peut rester à distance sécuritaire de sa proie, et les flèches sont beaucoup plus légères que les javelots, donc un chasseur peut en porter beaucoup plus. Les premières flèches sont faites de bois, de pierre (pointes) et de plumes (empennage), avec des pointes petites, finement taillées, triangulaires ou barbelées. Les squelettes de 20 000 ans montrent souvent des blessures compatibles avec des blessures de flèche. La maîtrise de l'arc et la flèche demande de la pratique, de la coordination, de la précision, renforçant la transmission culturelle entre générations. L'arc et la flèche ne sont pas juste une technologie de chasse : ils deviennent aussi une arme de guerre, augmentant l'efficacité mortelle des conflits mais aussi la capacité de défense d'un territoire par un petit groupe bien entraîné. Des millénaires plus tard, Gengis Khan utilisera des archers à cheval pour conquérir le monde.</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Climatologie / Géologie</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Dernière période glaciaire - Last Glacial Maximum</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Le froid atteint son maximum, les glaciers couvrent de vastes territoires</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Il y a 18 000 ans, la Terre connaît le point culminant de la dernière période glaciaire : le "Last Glacial Maximum" (LGM). Les calottes glaciaires sont au maximum de leur extension : les glaciers d'Amérique du Nord couvrent tout le Canada et descendent jusqu'au Kentucky, l'Europe du Nord est couverte de glaciers épais, la Sibérie est un désert de glace. Le niveau des mers est 120-130 mètres plus bas qu'aujourd'hui. Des "terres de passage" apparaissent : le détroit de Béring devient la "Béringie", une vaste plaine terrestre que des humains traversent pour migrer de Sibérie vers l'Amérique du Nord. Le climat est extrêmement froid, les hivers catastrophiques, et la vie incroyablement difficile. Les humains fabriquent des vêtements épais en peau d'animal, construisent des abris semi-enterrés renforcés avec des os et des défenses de mammouths, et maîtrisent complètement le feu. Ils chassent les mégafaunes (mammouths, rhinocéros laineux, ours des cavernes) qui requièrent coordination de groupe, stratégie et courage. Le LGM dure environ 2 000-3 000 ans (de 23 000 à 19 000 ans, avec le maximum à 18 000 ans). La population humaine globale diminue, certains groupes se réfugiant dans des zones climatiques plus clémentes (Méditerranée, Afrique du Sud, Asie du Sud). Le LGM est considéré comme le "goulot d'étranglement démographique" de l'humanité : la population mondiale aurait été réduite à peut-être seulement 10 000-30 000 individus. Si l'espèce humaine avait échoué à survivre au LGM, l'humanité entière aurait disparu.</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Archéologie / Domestication</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Domestication du chien - premiers animaux domestiqués</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Les loups commencent à être domestiqués et deviennent des chiens</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Il y a 15 000 ans, un processus qui changera profondément la civilisation humaine commence : la domestication du chien, probablement le premier animal jamais domestiqué. Les preuves archéologiques proviennent de sites en Allemagne (Bonn-Oberkassel), en Israël (Eynan), et en Russie (Razboinichya Cave), où des restes de chiens datent de 15 000 à 14 000 ans. La théorie la plus acceptée : les loups, attirés par les déchets près des campements humains, commencent à scavenger. Les loups les moins agressifs s'approchent des humains, qui les tolèrent car ils aident à se débarrasser des déchets. Au fil des générations, une sélection naturelle et humaine se produit : les loups les plus calmes survivent mieux près des humains et se reproduisent. Graduellement, leur tempérament et leur apparence changent (oreilles qui tombent, queue qui s'enroule, pelage varié) : ce ne sont plus des loups, ce sont des chiens. Un fossile célèbre, le "Bonn-Oberkassel dog", est un chiot datant de 14 200 ans qui avait un problème dentaire congénital ; le fait qu'il ait survécu jusqu'à 6-7 mois suggère qu'il a été soigné et chéri par les humains, l'une des plus anciennes preuves d'une relation affective homme-animal. La domestication du chien a des impacts majeurs sur la chasse : les chiens aident à débusquer et rabattre le gibier, tracent les animaux blessés, et protègent les campements. Elle inspire aussi la domestication d'autres animaux : 10 000 ans plus tard, les humains domestiquent chèvres, moutons et vaches. Mais le chien arrive le premier, et la relation humain-chien dure jusqu'à aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Climatologie</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Fin de l'Âge de Glace et début du réchauffement climatique</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>-14000</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Les glaciers commencent à fondre massivement, le climat se réchauffe</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Il y a 14 000 ans, le climat de la Terre commence une transformation majeure : la fin de la dernière période glaciaire. Après une période de refroidissement temporaire (le Dryas Inférieur, environ 12 800 ans, qui dure 1 200 ans), le Holocène débute à 11 700 ans, marquant vraiment le début d'une période interglaciaire chaude et stable. À 14 000 ans, les glaciers qui couvraient l'Amérique du Nord, l'Europe du Nord et la Sibérie commencent à fondre rapidement. Le niveau des mers remonte, la Béringie est submergée, les écosystèmes changent radicalement, et les mammouths et autres mégafaunes, adaptés au froid, déclinent et finissent par disparaître. Ce réchauffement climatique a des implications énormes pour la civilisation humaine. Dans le Croissant Fertile (région entre le Tigre et l'Euphrate en Mésopotamie), les conditions deviennent idéales pour certaines plantes sauvages, particulièrement les céréales comme le blé et l'orge. Les humains de cette région remarquent qu'une certaine plante produit des graines comestibles et commencent à les cueillir. Progressivement, sur les 2 000-3 000 ans suivants, ils passent de la cueillette simple à la "proto-agriculture", puis à l'agriculture complète, d'où émergera la révolution néolithique. Sans ce réchauffement climatique, l'agriculture n'aurait probablement jamais émergé, et sans agriculture, pas de civilisation : les empires, les villes, l'écriture, la complexité sociale découlent finalement de ce réchauffement climatique. Avec le temps plus doux et plus stable, les humains peuvent rester au même endroit (sédentarité), ce qui permet l'accumulation de biens, l'émergence de hiérarchie, et finalement la civilisation.</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Archéologie / Agriculture</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Révolution néolithique : débuts de l'agriculture dans le Croissant Fertile</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Les humains commencent à cultiver intentionnellement des plantes</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Il y a 12 000 ans, un changement révolutionnaire se produit : les humains commencent à cultiver délibérément des plantes. C'est le début de la révolution néolithique, qui débute dans le Croissant Fertile, une région qui s'étend du Nil en Égypte jusqu'au Tigre-Euphrate en Mésopotamie moderne. Les preuves archéologiques viennent de sites comme Jéricho, Çatalhöyük, Abu Hureyra, et Tell Aswad. Avant 12 000 ans, les humains sont tous des chasseurs-cueilleurs, se déplaçant saisonnièrement à la recherche de nourriture. Les scientifiques débattent des raisons du changement : réchauffement climatique rendant l'agriculture viable, pression démographique, ou abondance naturelle croissante de plantes sauvages nutritives. Les humains remarquent que planter les graines du blé récolté l'année précédente fait pousser de nouvelles plantes, et expérimentent la culture intentionnelle. Progressivement, au cours des siècles, ils sélectionnent les plantes avec les plus grosses graines et les meilleurs rendements : une sélection artificielle qui rend les plantes cultivées génétiquement distinctes des plantes sauvages. Parallèlement, la chasse devient plus difficile à mesure que les mégafaunes disparaissent, rendant l'agriculture plus attractive. À 10 000-9 000 ans, la transition est complète : les villages du Croissant Fertile cultivent blé, orge, pois et lentilles, et domestiquent chèvres, moutons et vaches. Ce passage a des impacts colossaux : rendement alimentaire plus élevé, sédentarité, accumulation de biens et de richesse, surplus permettant l'émergence de prêtres, guerriers et administrateurs, donc de hiérarchie sociale et finalement de l'État. Mais aussi des inconvénients : travail plus intensif, régime moins diversifié, vulnérabilité aux mauvaises récoltes, et augmentation des maladies infectieuses liées à la proximité du bétail et à la densité de population. La révolution agricole crée ainsi les conditions nécessaires à la civilisation.</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Archéologie / Agriculture</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Domestication du blé et de l'orge</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>-11000</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Les céréales deviennent les cultures fondamentales</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Il y a 11 000 ans, la domestication du blé et de l'orge est bien établie dans le Croissant Fertile. Des sites archéologiques montrent que le blé "emmer" (Triticum turgidum dicoccoides) et l'orge (Hordeum vulgare) sont activement cultivés. Pourquoi ces deux plantes ? Elles offrent un rendement élevé en calories, une facilité de stockage (les grains secs se conservent longtemps), une facilité de culture, et contiennent protéines et vitamines. Les archéobotaniques distinguent le blé et l'orge sauvages des versions domestiquées par des caractéristiques morphologiques : le blé sauvage a un axe fragile qui se casse facilement et disperse les graines, tandis que le blé domestiqué a un axe dur qui ne se casse pas, permettant aux humains de récolter les épis entiers. Ce changement génétique, apparu progressivement sur plusieurs générations, rend la plante entièrement dépendante de l'homme pour sa reproduction. À 11 000 ans, le blé et l'orge domestiqués sont génétiquement distincts de leurs ancêtres sauvages, et les rendements s'améliorent chaque année : un agriculteur peut produire assez de céréales pour nourrir environ 2-3 fois plus de personnes qu'un chasseur-cueilleur sur la même surface. Cela permet à la population d'augmenter rapidement, et les villages qui cultivent le blé et l'orge grossissent, atteignant plusieurs centaines d'habitants dès 10 000 ans. Le stockage du blé dans des greniers crée une incitation à construire des bâtiments fortifiés et à organiser une défense collective. Plus tard, le surplus permet à certaines personnes de devenir guerriers à temps plein, et le blé et l'orge deviennent même des unités de monnaie avant l'apparition des pièces. Cette domestication crée une symbiose humains-plantes qui dure depuis plus de 10 000 ans.</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr"/>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -13333,7 +13823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F476"/>
+  <dimension ref="A1:F518"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -21915,962 +22405,1802 @@
       </c>
     </row>
     <row r="429">
-      <c r="A429" t="n">
+      <c r="A429" s="20" t="n">
         <v>293</v>
       </c>
-      <c r="B429" t="inlineStr">
+      <c r="B429" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C429" t="inlineStr">
+      <c r="C429" s="20" t="inlineStr">
         <is>
           <t>Nature : Earliest life on Earth - Abigail Allwood et al. (2015)</t>
         </is>
       </c>
-      <c r="D429" t="inlineStr">
+      <c r="D429" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature14871</t>
         </is>
       </c>
     </row>
     <row r="430">
-      <c r="A430" t="n">
+      <c r="A430" s="20" t="n">
         <v>293</v>
       </c>
-      <c r="B430" t="inlineStr">
+      <c r="B430" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C430" t="inlineStr">
+      <c r="C430" s="20" t="inlineStr">
         <is>
           <t>Science : Evidence for early life on Earth - Mojzsis et al. (1996)</t>
         </is>
       </c>
-      <c r="D430" t="inlineStr">
+      <c r="D430" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.273.5278.1910</t>
         </is>
       </c>
     </row>
     <row r="431">
-      <c r="A431" t="n">
+      <c r="A431" s="20" t="n">
         <v>293</v>
       </c>
-      <c r="B431" t="inlineStr">
+      <c r="B431" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C431" t="inlineStr">
+      <c r="C431" s="20" t="inlineStr">
         <is>
           <t>The Astrophysical Journal : Stromatolites and early life - Grotzinger &amp; Knoll (1999)</t>
         </is>
       </c>
-      <c r="D431" t="inlineStr">
+      <c r="D431" s="20" t="inlineStr">
         <is>
           <t>https://iopscience.iop.org/article/10.1086/313160</t>
         </is>
       </c>
     </row>
     <row r="432">
-      <c r="A432" t="n">
+      <c r="A432" s="20" t="n">
         <v>294</v>
       </c>
-      <c r="B432" t="inlineStr">
+      <c r="B432" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C432" t="inlineStr">
+      <c r="C432" s="20" t="inlineStr">
         <is>
           <t>Science : The rise of atmospheric oxygen - Holland (2002)</t>
         </is>
       </c>
-      <c r="D432" t="inlineStr">
+      <c r="D432" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1069141</t>
         </is>
       </c>
     </row>
     <row r="433">
-      <c r="A433" t="n">
+      <c r="A433" s="20" t="n">
         <v>294</v>
       </c>
-      <c r="B433" t="inlineStr">
+      <c r="B433" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C433" t="inlineStr">
+      <c r="C433" s="20" t="inlineStr">
         <is>
           <t>Nature : Great Oxidation Event - Bekker et al. (2004)</t>
         </is>
       </c>
-      <c r="D433" t="inlineStr">
+      <c r="D433" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature02711</t>
         </is>
       </c>
     </row>
     <row r="434">
-      <c r="A434" t="n">
+      <c r="A434" s="20" t="n">
         <v>294</v>
       </c>
-      <c r="B434" t="inlineStr">
+      <c r="B434" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C434" t="inlineStr">
+      <c r="C434" s="20" t="inlineStr">
         <is>
           <t>PLoS Biology : The rise of aerobic life - Catling &amp; Claire (2005)</t>
         </is>
       </c>
-      <c r="D434" t="inlineStr">
+      <c r="D434" s="20" t="inlineStr">
         <is>
           <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.0030176</t>
         </is>
       </c>
     </row>
     <row r="435">
-      <c r="A435" t="n">
+      <c r="A435" s="20" t="n">
         <v>295</v>
       </c>
-      <c r="B435" t="inlineStr">
+      <c r="B435" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C435" t="inlineStr">
+      <c r="C435" s="20" t="inlineStr">
         <is>
           <t>Nature : Endosymbiotic theory evidence - Margulis (1970)</t>
         </is>
       </c>
-      <c r="D435" t="inlineStr">
+      <c r="D435" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature15726</t>
         </is>
       </c>
     </row>
     <row r="436">
-      <c r="A436" t="n">
+      <c r="A436" s="20" t="n">
         <v>295</v>
       </c>
-      <c r="B436" t="inlineStr">
+      <c r="B436" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C436" t="inlineStr">
+      <c r="C436" s="20" t="inlineStr">
         <is>
           <t>Trends in Ecology &amp; Evolution : The origin of eukaryotes - Koonin (2010)</t>
         </is>
       </c>
-      <c r="D436" t="inlineStr">
+      <c r="D436" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.tree.2010.07.002</t>
         </is>
       </c>
     </row>
     <row r="437">
-      <c r="A437" t="n">
+      <c r="A437" s="20" t="n">
         <v>295</v>
       </c>
-      <c r="B437" t="inlineStr">
+      <c r="B437" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C437" t="inlineStr">
+      <c r="C437" s="20" t="inlineStr">
         <is>
           <t>PNAS : Early eukaryotic fossils - Knoll et al. (2006)</t>
         </is>
       </c>
-      <c r="D437" t="inlineStr">
+      <c r="D437" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0604866103</t>
         </is>
       </c>
     </row>
     <row r="438">
-      <c r="A438" t="n">
+      <c r="A438" s="20" t="n">
         <v>296</v>
       </c>
-      <c r="B438" t="inlineStr">
+      <c r="B438" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C438" t="inlineStr">
+      <c r="C438" s="20" t="inlineStr">
         <is>
           <t>Nature : The Cambrian Explosion - Marshall (2006)</t>
         </is>
       </c>
-      <c r="D438" t="inlineStr">
+      <c r="D438" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature05070</t>
         </is>
       </c>
     </row>
     <row r="439">
-      <c r="A439" t="n">
+      <c r="A439" s="20" t="n">
         <v>296</v>
       </c>
-      <c r="B439" t="inlineStr">
+      <c r="B439" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C439" t="inlineStr">
+      <c r="C439" s="20" t="inlineStr">
         <is>
           <t>Science : Evolution of complex body structures - Briggs et al. (2005)</t>
         </is>
       </c>
-      <c r="D439" t="inlineStr">
+      <c r="D439" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1122776</t>
         </is>
       </c>
     </row>
     <row r="440">
-      <c r="A440" t="n">
+      <c r="A440" s="20" t="n">
         <v>296</v>
       </c>
-      <c r="B440" t="inlineStr">
+      <c r="B440" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C440" t="inlineStr">
+      <c r="C440" s="20" t="inlineStr">
         <is>
           <t>Trends in Ecology &amp; Evolution : Hox genes and body plans - Carroll (2005)</t>
         </is>
       </c>
-      <c r="D440" t="inlineStr">
+      <c r="D440" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.tree.2005.07.001</t>
         </is>
       </c>
     </row>
     <row r="441">
-      <c r="A441" t="n">
+      <c r="A441" s="20" t="n">
         <v>297</v>
       </c>
-      <c r="B441" t="inlineStr">
+      <c r="B441" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C441" t="inlineStr">
+      <c r="C441" s="20" t="inlineStr">
         <is>
           <t>Nature : Early fish evolution - Janvier (2007)</t>
         </is>
       </c>
-      <c r="D441" t="inlineStr">
+      <c r="D441" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature05983</t>
         </is>
       </c>
     </row>
     <row r="442">
-      <c r="A442" t="n">
+      <c r="A442" s="20" t="n">
         <v>297</v>
       </c>
-      <c r="B442" t="inlineStr">
+      <c r="B442" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C442" t="inlineStr">
+      <c r="C442" s="20" t="inlineStr">
         <is>
           <t>PLoS Biology : Fossil evidence of Ostracoderms - Sansom et al. (2012)</t>
         </is>
       </c>
-      <c r="D442" t="inlineStr">
+      <c r="D442" s="20" t="inlineStr">
         <is>
           <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1001470</t>
         </is>
       </c>
     </row>
     <row r="443">
-      <c r="A443" t="n">
+      <c r="A443" s="20" t="n">
         <v>297</v>
       </c>
-      <c r="B443" t="inlineStr">
+      <c r="B443" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C443" t="inlineStr">
+      <c r="C443" s="20" t="inlineStr">
         <is>
           <t>Zoological Journal of the Linnean Society : Vertebrate origins - Gess et al. (2006)</t>
         </is>
       </c>
-      <c r="D443" t="inlineStr">
+      <c r="D443" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/j.1096-3642.2006.00232.x</t>
         </is>
       </c>
     </row>
     <row r="444">
-      <c r="A444" t="n">
+      <c r="A444" s="20" t="n">
         <v>298</v>
       </c>
-      <c r="B444" t="inlineStr">
+      <c r="B444" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C444" t="inlineStr">
+      <c r="C444" s="20" t="inlineStr">
         <is>
           <t>Trends in Plant Science : Early land plant evolution - Kenrick &amp; Crane (1997)</t>
         </is>
       </c>
-      <c r="D444" t="inlineStr">
+      <c r="D444" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S1360-1385(97)01010-0</t>
         </is>
       </c>
     </row>
     <row r="445">
-      <c r="A445" t="n">
+      <c r="A445" s="20" t="n">
         <v>298</v>
       </c>
-      <c r="B445" t="inlineStr">
+      <c r="B445" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C445" t="inlineStr">
+      <c r="C445" s="20" t="inlineStr">
         <is>
           <t>Nature : Oldest land plants - Wellman et al. (2003)</t>
         </is>
       </c>
-      <c r="D445" t="inlineStr">
+      <c r="D445" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature02041</t>
         </is>
       </c>
     </row>
     <row r="446">
-      <c r="A446" t="n">
+      <c r="A446" s="20" t="n">
         <v>298</v>
       </c>
-      <c r="B446" t="inlineStr">
+      <c r="B446" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C446" t="inlineStr">
+      <c r="C446" s="20" t="inlineStr">
         <is>
           <t>Science : Plant terrestrialization - Morris et al. (2018)</t>
         </is>
       </c>
-      <c r="D446" t="inlineStr">
+      <c r="D446" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.aar5429</t>
         </is>
       </c>
     </row>
     <row r="447">
-      <c r="A447" t="n">
+      <c r="A447" s="20" t="n">
         <v>299</v>
       </c>
-      <c r="B447" t="inlineStr">
+      <c r="B447" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C447" t="inlineStr">
+      <c r="C447" s="20" t="inlineStr">
         <is>
           <t>Nature : Tiktaalik - a fish with tetrapod characteristics - Shubin et al. (2004)</t>
         </is>
       </c>
-      <c r="D447" t="inlineStr">
+      <c r="D447" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature02426</t>
         </is>
       </c>
     </row>
     <row r="448">
-      <c r="A448" t="n">
+      <c r="A448" s="20" t="n">
         <v>299</v>
       </c>
-      <c r="B448" t="inlineStr">
+      <c r="B448" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C448" t="inlineStr">
+      <c r="C448" s="20" t="inlineStr">
         <is>
           <t>PLoS Biology : Ichthyostega fossil evidence - Clément et al. (2015)</t>
         </is>
       </c>
-      <c r="D448" t="inlineStr">
+      <c r="D448" s="20" t="inlineStr">
         <is>
           <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1002445</t>
         </is>
       </c>
     </row>
     <row r="449">
-      <c r="A449" t="n">
+      <c r="A449" s="20" t="n">
         <v>299</v>
       </c>
-      <c r="B449" t="inlineStr">
+      <c r="B449" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C449" t="inlineStr">
+      <c r="C449" s="20" t="inlineStr">
         <is>
           <t>Science : Fin-to-limb transition - Coates et al. (2002)</t>
         </is>
       </c>
-      <c r="D449" t="inlineStr">
+      <c r="D449" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1069052</t>
         </is>
       </c>
     </row>
     <row r="450">
-      <c r="A450" t="n">
+      <c r="A450" s="20" t="n">
         <v>300</v>
       </c>
-      <c r="B450" t="inlineStr">
+      <c r="B450" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C450" t="inlineStr">
+      <c r="C450" s="20" t="inlineStr">
         <is>
           <t>Nature : Early amniote evolution - Modesto &amp; Anderson (2004)</t>
         </is>
       </c>
-      <c r="D450" t="inlineStr">
+      <c r="D450" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature03048</t>
         </is>
       </c>
     </row>
     <row r="451">
-      <c r="A451" t="n">
+      <c r="A451" s="20" t="n">
         <v>300</v>
       </c>
-      <c r="B451" t="inlineStr">
+      <c r="B451" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C451" t="inlineStr">
+      <c r="C451" s="20" t="inlineStr">
         <is>
           <t>PLoS One : Amniotic egg evolution - Packard &amp; Seymour (1997)</t>
         </is>
       </c>
-      <c r="D451" t="inlineStr">
+      <c r="D451" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1152/physrev.1997.77.4.701</t>
         </is>
       </c>
     </row>
     <row r="452">
-      <c r="A452" t="n">
+      <c r="A452" s="20" t="n">
         <v>300</v>
       </c>
-      <c r="B452" t="inlineStr">
+      <c r="B452" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C452" t="inlineStr">
+      <c r="C452" s="20" t="inlineStr">
         <is>
           <t>Journal of Morphology : Reptile characteristics - Rieppel (1993)</t>
         </is>
       </c>
-      <c r="D452" t="inlineStr">
+      <c r="D452" s="20" t="inlineStr">
         <is>
           <t>https://onlinelibrary.wiley.com/doi/10.1002/jmor.1052160307</t>
         </is>
       </c>
     </row>
     <row r="453">
-      <c r="A453" t="n">
+      <c r="A453" s="20" t="n">
         <v>301</v>
       </c>
-      <c r="B453" t="inlineStr">
+      <c r="B453" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C453" t="inlineStr">
+      <c r="C453" s="20" t="inlineStr">
         <is>
           <t>Nature : Synapsid evolution - Benton (1999)</t>
         </is>
       </c>
-      <c r="D453" t="inlineStr">
+      <c r="D453" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/17856</t>
         </is>
       </c>
     </row>
     <row r="454">
-      <c r="A454" t="n">
+      <c r="A454" s="20" t="n">
         <v>301</v>
       </c>
-      <c r="B454" t="inlineStr">
+      <c r="B454" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C454" t="inlineStr">
+      <c r="C454" s="20" t="inlineStr">
         <is>
           <t>Biological Reviews : Synapsid-to-mammal transition - Kemp (2005)</t>
         </is>
       </c>
-      <c r="D454" t="inlineStr">
+      <c r="D454" s="20" t="inlineStr">
         <is>
           <t>https://onlinelibrary.wiley.com/doi/10.1017/S1464793105006457</t>
         </is>
       </c>
     </row>
     <row r="455">
-      <c r="A455" t="n">
+      <c r="A455" s="20" t="n">
         <v>301</v>
       </c>
-      <c r="B455" t="inlineStr">
+      <c r="B455" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C455" t="inlineStr">
+      <c r="C455" s="20" t="inlineStr">
         <is>
           <t>PLoS Biology : Cynodonts and early mammals - Luo (2007)</t>
         </is>
       </c>
-      <c r="D455" t="inlineStr">
+      <c r="D455" s="20" t="inlineStr">
         <is>
           <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.0050114</t>
         </is>
       </c>
     </row>
     <row r="456">
-      <c r="A456" t="n">
+      <c r="A456" s="20" t="n">
         <v>302</v>
       </c>
-      <c r="B456" t="inlineStr">
+      <c r="B456" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C456" t="inlineStr">
+      <c r="C456" s="20" t="inlineStr">
         <is>
           <t>Science : The Great Dying - Benton (2008)</t>
         </is>
       </c>
-      <c r="D456" t="inlineStr">
+      <c r="D456" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1154887</t>
         </is>
       </c>
     </row>
     <row r="457">
-      <c r="A457" t="n">
+      <c r="A457" s="20" t="n">
         <v>302</v>
       </c>
-      <c r="B457" t="inlineStr">
+      <c r="B457" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C457" t="inlineStr">
+      <c r="C457" s="20" t="inlineStr">
         <is>
           <t>Nature : Permian-Triassic extinction - Burgess &amp; Bowring (2015)</t>
         </is>
       </c>
-      <c r="D457" t="inlineStr">
+      <c r="D457" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature14879</t>
         </is>
       </c>
     </row>
     <row r="458">
-      <c r="A458" t="n">
+      <c r="A458" s="20" t="n">
         <v>302</v>
       </c>
-      <c r="B458" t="inlineStr">
+      <c r="B458" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C458" t="inlineStr">
+      <c r="C458" s="20" t="inlineStr">
         <is>
           <t>Geology : Siberian volcanism and extinction - Burgess et al. (2014)</t>
         </is>
       </c>
-      <c r="D458" t="inlineStr">
+      <c r="D458" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1130/G35774.1</t>
         </is>
       </c>
     </row>
     <row r="459">
-      <c r="A459" t="n">
+      <c r="A459" s="20" t="n">
         <v>303</v>
       </c>
-      <c r="B459" t="inlineStr">
+      <c r="B459" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C459" t="inlineStr">
+      <c r="C459" s="20" t="inlineStr">
         <is>
           <t>Nature : Early mammal evolution - Luo (2007)</t>
         </is>
       </c>
-      <c r="D459" t="inlineStr">
+      <c r="D459" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature06325</t>
         </is>
       </c>
     </row>
     <row r="460">
-      <c r="A460" t="n">
+      <c r="A460" s="20" t="n">
         <v>303</v>
       </c>
-      <c r="B460" t="inlineStr">
+      <c r="B460" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C460" t="inlineStr">
+      <c r="C460" s="20" t="inlineStr">
         <is>
           <t>Science : Hadrocodium - the earliest mammal - Luo et al. (2001)</t>
         </is>
       </c>
-      <c r="D460" t="inlineStr">
+      <c r="D460" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1065507</t>
         </is>
       </c>
     </row>
     <row r="461">
-      <c r="A461" t="n">
+      <c r="A461" s="20" t="n">
         <v>303</v>
       </c>
-      <c r="B461" t="inlineStr">
+      <c r="B461" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C461" t="inlineStr">
+      <c r="C461" s="20" t="inlineStr">
         <is>
           <t>Zoological Journal of the Linnean Society : Morganucodon paleobiology - Kermack &amp; Mussett (1983)</t>
         </is>
       </c>
-      <c r="D461" t="inlineStr">
+      <c r="D461" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/j.1096-3642.1983.tb00710.x</t>
         </is>
       </c>
     </row>
     <row r="462">
-      <c r="A462" t="n">
+      <c r="A462" s="20" t="n">
         <v>304</v>
       </c>
-      <c r="B462" t="inlineStr">
+      <c r="B462" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C462" t="inlineStr">
+      <c r="C462" s="20" t="inlineStr">
         <is>
           <t>Nature : Evidence of controlled fire use by early humans - Wrangham &amp; Conklin-Brittain (2003)</t>
         </is>
       </c>
-      <c r="D462" t="inlineStr">
+      <c r="D462" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature01754</t>
         </is>
       </c>
     </row>
     <row r="463">
-      <c r="A463" t="n">
+      <c r="A463" s="20" t="n">
         <v>304</v>
       </c>
-      <c r="B463" t="inlineStr">
+      <c r="B463" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C463" t="inlineStr">
+      <c r="C463" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Fire use in Homo erectus - Berna et al. (2012)</t>
         </is>
       </c>
-      <c r="D463" t="inlineStr">
+      <c r="D463" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2012.05.002</t>
         </is>
       </c>
     </row>
     <row r="464">
-      <c r="A464" t="n">
+      <c r="A464" s="20" t="n">
         <v>304</v>
       </c>
-      <c r="B464" t="inlineStr">
+      <c r="B464" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C464" t="inlineStr">
+      <c r="C464" s="20" t="inlineStr">
         <is>
           <t>PNAS : Cooking and human brain evolution - Aiello &amp; Wheeler (1995)</t>
         </is>
       </c>
-      <c r="D464" t="inlineStr">
+      <c r="D464" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.92.25.11803</t>
         </is>
       </c>
     </row>
     <row r="465">
-      <c r="A465" t="n">
+      <c r="A465" s="20" t="n">
         <v>305</v>
       </c>
-      <c r="B465" t="inlineStr">
+      <c r="B465" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C465" t="inlineStr">
+      <c r="C465" s="20" t="inlineStr">
         <is>
           <t>Nature : Homo heidelbergensis genetics - Meyer et al. (2013)</t>
         </is>
       </c>
-      <c r="D465" t="inlineStr">
+      <c r="D465" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature12886</t>
         </is>
       </c>
     </row>
     <row r="466">
-      <c r="A466" t="n">
+      <c r="A466" s="20" t="n">
         <v>305</v>
       </c>
-      <c r="B466" t="inlineStr">
+      <c r="B466" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C466" t="inlineStr">
+      <c r="C466" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Homo heidelbergensis phylogeny - Rightmire (2008)</t>
         </is>
       </c>
-      <c r="D466" t="inlineStr">
+      <c r="D466" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2008.07.011</t>
         </is>
       </c>
     </row>
     <row r="467">
-      <c r="A467" t="n">
+      <c r="A467" s="20" t="n">
         <v>305</v>
       </c>
-      <c r="B467" t="inlineStr">
+      <c r="B467" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C467" t="inlineStr">
+      <c r="C467" s="20" t="inlineStr">
         <is>
           <t>PNAS : Interbreeding of Homo heidelbergensis descendants - Schlebusch et al. (2017)</t>
         </is>
       </c>
-      <c r="D467" t="inlineStr">
+      <c r="D467" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1704702114</t>
         </is>
       </c>
     </row>
     <row r="468">
-      <c r="A468" t="n">
+      <c r="A468" s="20" t="n">
         <v>306</v>
       </c>
-      <c r="B468" t="inlineStr">
+      <c r="B468" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C468" t="inlineStr">
+      <c r="C468" s="20" t="inlineStr">
         <is>
           <t>Nature : Neanderthal genome - Green et al. (2010)</t>
         </is>
       </c>
-      <c r="D468" t="inlineStr">
+      <c r="D468" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature08976</t>
         </is>
       </c>
     </row>
     <row r="469">
-      <c r="A469" t="n">
+      <c r="A469" s="20" t="n">
         <v>306</v>
       </c>
-      <c r="B469" t="inlineStr">
+      <c r="B469" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C469" t="inlineStr">
+      <c r="C469" s="20" t="inlineStr">
         <is>
           <t>American Journal of Physical Anthropology : Neanderthal morphology - Trinkaus (2005)</t>
         </is>
       </c>
-      <c r="D469" t="inlineStr">
+      <c r="D469" s="20" t="inlineStr">
         <is>
           <t>https://onlinelibrary.wiley.com/doi/10.1002/ajpa.20239</t>
         </is>
       </c>
     </row>
     <row r="470">
-      <c r="A470" t="n">
+      <c r="A470" s="20" t="n">
         <v>306</v>
       </c>
-      <c r="B470" t="inlineStr">
+      <c r="B470" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C470" t="inlineStr">
+      <c r="C470" s="20" t="inlineStr">
         <is>
           <t>PNAS : Neanderthal symbolic behavior - D'Errico et al. (2003)</t>
         </is>
       </c>
-      <c r="D470" t="inlineStr">
+      <c r="D470" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0935975100</t>
         </is>
       </c>
     </row>
     <row r="471">
-      <c r="A471" t="n">
+      <c r="A471" s="20" t="n">
         <v>307</v>
       </c>
-      <c r="B471" t="inlineStr">
+      <c r="B471" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C471" t="inlineStr">
+      <c r="C471" s="20" t="inlineStr">
         <is>
           <t>Nature : Early Homo sapiens fossils - Hublin et al. (2017)</t>
         </is>
       </c>
-      <c r="D471" t="inlineStr">
+      <c r="D471" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature22336</t>
         </is>
       </c>
     </row>
     <row r="472">
-      <c r="A472" t="n">
+      <c r="A472" s="20" t="n">
         <v>307</v>
       </c>
-      <c r="B472" t="inlineStr">
+      <c r="B472" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C472" t="inlineStr">
+      <c r="C472" s="20" t="inlineStr">
         <is>
           <t>Science : Origin of modern humans - Green et al. (2019)</t>
         </is>
       </c>
-      <c r="D472" t="inlineStr">
+      <c r="D472" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.aav4534</t>
         </is>
       </c>
     </row>
     <row r="473">
-      <c r="A473" t="n">
+      <c r="A473" s="20" t="n">
         <v>307</v>
       </c>
-      <c r="B473" t="inlineStr">
+      <c r="B473" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C473" t="inlineStr">
+      <c r="C473" s="20" t="inlineStr">
         <is>
           <t>PLoS Biology : Modern human brain evolution - Neubauer et al. (2018)</t>
         </is>
       </c>
-      <c r="D473" t="inlineStr">
+      <c r="D473" s="20" t="inlineStr">
         <is>
           <t>https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.2006931</t>
         </is>
       </c>
     </row>
     <row r="474">
-      <c r="A474" t="n">
+      <c r="A474" s="20" t="n">
         <v>308</v>
       </c>
-      <c r="B474" t="inlineStr">
+      <c r="B474" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C474" t="inlineStr">
+      <c r="C474" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Neanderthal social structure - Wobst (1974)</t>
         </is>
       </c>
-      <c r="D474" t="inlineStr">
+      <c r="D474" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/0047-2484(74)90003-6</t>
         </is>
       </c>
     </row>
     <row r="475">
-      <c r="A475" t="n">
+      <c r="A475" s="20" t="n">
         <v>308</v>
       </c>
-      <c r="B475" t="inlineStr">
+      <c r="B475" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C475" t="inlineStr">
+      <c r="C475" s="20" t="inlineStr">
         <is>
           <t>Nature : Neanderthal symbolic behavior - D'Errico et al. (2003)</t>
         </is>
       </c>
-      <c r="D475" t="inlineStr">
+      <c r="D475" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/425410a</t>
         </is>
       </c>
     </row>
     <row r="476">
-      <c r="A476" t="n">
+      <c r="A476" s="20" t="n">
         <v>308</v>
       </c>
-      <c r="B476" t="inlineStr">
+      <c r="B476" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C476" t="inlineStr">
+      <c r="C476" s="20" t="inlineStr">
         <is>
           <t>PNAS : Neanderthal diet - Bocherens et al. (2005)</t>
         </is>
       </c>
-      <c r="D476" t="inlineStr">
+      <c r="D476" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0506130102</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>309</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Nature : Early dispersal of modern humans from Africa - Templeton (2002)</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/415546a</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>309</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>PNAS : Genomic evidence for early human dispersal - Armitage et al. (2011)</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1100166108</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>309</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Science : Human genetic diversity and migration patterns - Li et al. (2008)</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1153717</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>310</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>PNAS : Early human dispersal to Southeast Asia - Demeter et al. (2012)</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1108887109</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>310</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Archaeological evidence of early Southeast Asian settlement - Higham &amp; Thosarat (2004)</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2003.12.003</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>310</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Quaternary Science Reviews : Human migration to Southeast Asia - Ono et al. (2018)</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.quascirev.2018.09.035</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>311</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Nature : Dating of Australian rock art and early human dispersal - Clarkson et al. (2017)</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41586-017-0008-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>311</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>PNAS : Earliest known art in Australia - Aubert et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1408356111</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>311</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Settlement patterns in early Australia - O'Connell &amp; Allen (2012)</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2012.05.010</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>312</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Nature : Fossil evidence of Sapiens arrival in Europe - Higham et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature13621</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>312</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Science : Ancient DNA of Neanderthals and Sapiens - Green et al. (2010)</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1188021</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>312</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>PNAS : Neandertal-Sapiens introgression - Castellano et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1320099111</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>313</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Nature : Aurignacian symbolic behavior in Europe - Mellars (2005)</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature03674</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>313</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>PNAS : Early artistic expression in Africa and Europe - Conard et al. (2009)</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0900157106</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>313</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : The evolution of symbolic behavior - Mithen (2007)</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2006.07.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>314</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>PNAS : Timing of Neanderthal extinction - Higham et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1405035111</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>314</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Nature : Neanderthal extinction and climate - Finlayson et al. (2006)</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature04585</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>314</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Reasons for Neanderthal extinction - Shea (2006)</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jhevol.2006.04.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>315</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Journal of Archaeological Research : Paleolithic figurines and their meaning - Conard (2009)</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10814-009-9030-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>315</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>PNAS : Venus figurines - Conard &amp; Malina (2008)</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0710975105</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>315</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Current Biology : Dating of Venus figurines - Higham et al. (2012)</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.cub.2012.07.021</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>316</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Nature : Dating and study of Chauvet Cave - Clottes et al. (1995)</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/375231a0</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>316</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>PNAS : Chauvet Cave radiocarbon dating - Quiles et al. (2016)</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1502651112</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>316</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Journal of Human Evolution : Interpretation of Paleolithic art - Lewis-Williams (2002)</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0047-2484(02)00024-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>317</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Journal of Archaeological Science : Early bow and arrow technology - Shea &amp; Sisk (2010)</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jas.2009.11.013</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>317</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>PNAS : Origin of projectile weaponry - Lombard &amp; Phillipson (2010)</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1001885107</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>317</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>American Antiquity : African origins of archery - Lombard (2005)</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2307/40035648</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>318</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Science : Last Glacial Maximum reconstruction - Mix et al. (2001)</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.1059133</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>318</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Quaternary Research : Human adaptation to LGM - Gamble (1999)</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1006/qres.1999.2080</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>318</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>PNAS : Population genetics of Last Glacial Maximum - Excoffier et al. (2005)</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0500448102</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>319</v>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>PNAS : Ancient dog genomics - Parker et al. (2004)</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0401913101</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>319</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Nature Ecology &amp; Evolution : Early dog domestication - Larson et al. (2012)</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature11159</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>319</v>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Current Biology : Dog domestication genetics - Freedman et al. (2014)</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.cub.2014.03.024</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>320</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Nature : Holocene climate change and human settlement - Mayewski et al. (2004)</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature02805</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>320</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>PNAS : Younger Dryas climate event - Firestone et al. (2007)</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0707213104</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>320</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Quaternary Science Reviews : Climate transitions and cultural change - Roberts &amp; Brayshaw (2002)</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0277-3791(01)00083-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>321</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>PNAS : Origins of agriculture in the Fertile Crescent - Zeder (2011)</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.1100999108</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>321</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Journal of Archaeological Research : Neolithic transition - Bellwood (2005)</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10814-005-6142-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>321</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Nature : Early crop development - Purugganan &amp; Fuller (2009)</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/nature08808</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>322</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>PNAS : Wheat domestication - Tanno &amp; Willcox (2006)</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/doi/10.1073/pnas.0510618103</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>322</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Journal of Archaeological Science : Barley domestication in the Near East - Badr et al. (2000)</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1006/jasc.2000.0520</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="n">
+        <v>322</v>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Current Biology : Early wheat and barley cultivation - Fuller et al. (2011)</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.cub.2011.06.045</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajoute une anecdote factuelle et un emoji specifique pour chacune des 76 cartes ajoutees depuis le debut de la session (ids 247-322), au lieu de laisser l'anecdote vide et l'emoji generique par famille.
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -11177,7 +11177,11 @@
           <t>En 1955, le virologue américain Jonas Salk annonce le succès de son vaccin inactivé contre la poliomyélite (VPI), mettant fin à des décennies de recherche contre cette maladie dévastatrice. Le vaccin de Salk, présenté lors d'une conférence de presse le 12 avril 1955, utilise le virus de la polio inactivé par la chaleur et le formol. L'annonce déclenche une célébration nationale aux États-Unis, comparable à celle d'une victoire militaire majeure. La campagne de vaccination massive qui suit réduit dramatiquement les cas de poliomyélite, passant de 58 000 cas en 1952 à quelques centaines en 1960. Albert Sabin développe un vaccin oral (VPO) utilisant le virus vivant atténué peu après. La combinaison des deux vaccins éradique pratiquement la poliomyélite en Occident, sauvant des millions de vies et évitant des paralysies chroniques. En 2024, la poliomyélite est au bord de l'éradication mondiale complète.</t>
         </is>
       </c>
-      <c r="G248" s="19" t="n"/>
+      <c r="G248" s="19" t="inlineStr">
+        <is>
+          <t>Jonas Salk n'a jamais breveté son vaccin. Interrogé à la télévision sur qui en détenait les droits, il a répondu : « Il n'y a pas de brevet. Peut-on breveter le Soleil ? » — ce qui a permis sa diffusion à bas coût dans le monde entier.</t>
+        </is>
+      </c>
       <c r="H248" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11212,7 +11216,11 @@
           <t>En 1983, l'équipe dirigée par le virologue français Luc Montagnier, en collaboration avec Françoise Barré-Sinoussi, découvre le virus causant le SIDA (syndrome d'immunodéficience acquise) au sein de l'Institut Pasteur à Paris. Le virus, initialement nommé LAV (lymphadenopathy-associated virus), est identifié chez un patient atteint de lymphadénopathie, une condition fréquemment observée chez les patients séropositifs. Quelques mois plus tard, Robert Gallo aux États-Unis identifie indépendamment le même virus, nommé HTLV-III. Les deux équipes finissent par reconnaître qu'elles avaient découvert le même agent pathogène, désormais appelé VIH. Cette découverte révolutionne la compréhension du SIDA et ouvre la voie aux tests de dépistage et aux traitements antirétroviraux. Montagnier et Barré-Sinoussi reçoivent le Prix Nobel en 2008 pour cette découverte cruciale, qui a sauvé des millions de vies grâce au traitement antirétroviral.</t>
         </is>
       </c>
-      <c r="G249" s="19" t="n"/>
+      <c r="G249" s="19" t="inlineStr">
+        <is>
+          <t>La découverte a valu à Montagnier et Barré-Sinoussi le prix Nobel de médecine en 2008, mais la paternité de la découverte a longtemps été disputée avec le chercheur américain Robert Gallo, jusqu'à un accord diplomatique conclu en 1987 entre Reagan et Mitterrand sur les droits du test de dépistage.</t>
+        </is>
+      </c>
       <c r="H249" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11247,7 +11255,11 @@
           <t>En 1931, l'ingénieur allemand Ernst Ruska, alors étudiant, construit le premier microscope électronique fonctionnel, révolutionnant la microscopie en utilisant des électrons au lieu de la lumière visible. Le microscope électronique de Ruska offre un grossissement d'environ 400 fois, dépassant les capacités du meilleur microscope optique de l'époque. Ruska perfectionne son invention avec l'aide de Bimbo von Borries et Max Knoll, produisant un microscope capable de grossissements jusqu'à 100 000 fois. Le microscope électronique révolutionne la biologie cellulaire et la virologie en permettant d'observer les structures subcellulaires et les virus précédemment invisibles. Ruska reçoit le Prix Nobel en 1986, à l'âge de 81 ans, reconnaissant l'importance de son invention pour la science moderne. Aujourd'hui, le microscope électronique à transmission (MET) et le microscope électronique à balayage (MEB) restent des outils indispensables en recherche scientifique.</t>
         </is>
       </c>
-      <c r="G250" s="19" t="n"/>
+      <c r="G250" s="19" t="inlineStr">
+        <is>
+          <t>Ernst Ruska a reçu le prix Nobel de physique en 1986, soit 55 ans après son invention, à l'âge de 79 ans : l'un des plus longs délais jamais observés entre une découverte scientifique et sa reconnaissance par le Nobel.</t>
+        </is>
+      </c>
       <c r="H250" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11282,7 +11294,11 @@
           <t>Le 18 février 1930, l'astronome américain Clyde Tombaugh, âgé de seulement 24 ans, découvre une neuvième planète, initialement nommée Pluton, en analysant des photographies prises à l'observatoire Lowell en Arizona. Tombaugh localise Pluton en comparant systématiquement des photographies du ciel prises à différentes dates, cherchant un objet se déplaçant entre les images. La découverte de Pluton complète l'image du système solaire connu, avec neuf planètes orbitant le Soleil. Cependant, en 2006, l'Union astronomique internationale reclasse Pluton en "planète naine" en raison de sa petite taille et de sa composition glacée distincte des planètes rocheuses et gazeuses. Cette reclassification provoque un tollé public, avec de nombreuses personnes attachées à Pluton en tant que neuvième planète depuis 76 ans. Malgré sa reclassification, Pluton reste un objet fascinant étudié intensivement par la sonde New Horizons en 2015.</t>
         </is>
       </c>
-      <c r="G251" s="19" t="n"/>
+      <c r="G251" s="19" t="inlineStr">
+        <is>
+          <t>Clyde Tombaugh n'avait que 24 ans et aucun diplôme universitaire lorsqu'il a découvert Pluton, en comparant des plaques photographiques prises à quelques jours d'intervalle à l'aide d'un instrument appelé comparateur à clignotement.</t>
+        </is>
+      </c>
       <c r="H251" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11317,7 +11333,11 @@
           <t>En 1958, l'ingénieur texan Jack Kilby chez Texas Instruments crée le premier circuit intégré (puce), un dispositif contenant plusieurs transistors et autres composants électroniques miniaturisés sur une seule puce de silicium. Indépendamment, Robert Noyce de Fairchild Semiconductor développe une version améliorée du circuit intégré utilisant le processus de photolithographie en silicium. Les circuits intégrés révolutionnent l'électronique en permettant la densité de composants exponentiellement plus élevée à des coûts réduits. Le premier circuit intégré de Kilby contient seulement trois transistors et quelques autres composants, mais démontre le concept fondamental. Les générations successives de circuits intégrés suivent la loi de Moore, doublant le nombre de transistors tous les deux ans environ. Kilby reçoit le Prix Nobel en 2000 pour l'invention du circuit intégré. Aujourd'hui, les circuits intégrés modernes contiennent des milliards de transistors dans un espace minuscule.</t>
         </is>
       </c>
-      <c r="G252" s="19" t="n"/>
+      <c r="G252" s="19" t="inlineStr">
+        <is>
+          <t>Kilby (Texas Instruments) et Noyce (Fairchild) ont mis au point le circuit intégré indépendamment, à quelques mois d'écart, ce qui a déclenché une bataille de brevets de plus de dix ans. Noyce étant décédé en 1990, seul Kilby a pu recevoir le prix Nobel de physique en 2000, les Nobel n'étant jamais attribués à titre posthume.</t>
+        </is>
+      </c>
       <c r="H252" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11352,7 +11372,11 @@
           <t>En 1971, Intel, la jeune compagnie de semi-conducteurs fondée par Gordon Moore et Robert Noyce, crée le Intel 4004, le premier microprocesseur commercial au monde. Le 4004 contient 2 300 transistors et exécute 108 000 opérations par seconde, révolutionnant l'informatique en centralisant la logique de traitement sur une seule puce. Le microprocesseur permet la création d'ordinateurs personnels puissants et abordables, transformant l'informatique d'un domaine des grandes institutions aux foyers individuels. Les générations successives de microprocesseurs Intel (8008, 8080, 8086) et les concurrents (Motorola, AMD) conduisent à la révolution informatique du XXe siècle. Le microprocesseur est sans doute l'invention la plus important de l'histoire de l'informatique, car c'est lui qui rend possible chaque ordinateur moderne, smartphone et appareil informatique. Le Moore's Law, découvert par le cofondateur d'Intel, prédit que le nombre de transistors sur une puce double tous les deux ans.</t>
         </is>
       </c>
-      <c r="G253" s="19" t="n"/>
+      <c r="G253" s="19" t="inlineStr">
+        <is>
+          <t>Le premier microprocesseur commercial, l'Intel 4004, avait été conçu à l'origine pour une calculatrice de bureau japonaise et comptait environ 2 300 transistors — une puce de smartphone moderne en compte aujourd'hui plusieurs dizaines de milliards.</t>
+        </is>
+      </c>
       <c r="H253" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11387,7 +11411,11 @@
           <t>Le 24 avril 1990, la navette spatiale Discovery déploie le télescope spatial Hubble en orbite terrestre basse, révolutionnant l'astronomie en plaçant un observatoire de classe mondiale au-delà de l'atmosphère terrestre qui distortionne la lumière. Nommé en l'honneur de l'astronome Edwin Hubble, le télescope souffre initialement d'une aberration sphérique qui floute les images. Une mission de réparation en 1993 installe une optique correctrice, transformant Hubble en l'un des instruments scientifiques les plus productifs jamais créés. Hubble capture des images époustouflantes des galaxies lointaines, des nébuleuses et des phénomènes cosmiques, révolutionnant notre compréhension de l'univers. Les observations de Hubble confirment l'existence de trous noirs supermassifs, mesurent l'expansion accélérée de l'univers (suggérant l'existence de l'énergie sombre), et découvrent des milliers d'exoplanètes. Au-delà de ses découvertes scientifiques, Hubble inspire l'imagination publique, démontrant la beauté et la grandeur de l'univers à travers ses photographies emblématiques.</t>
         </is>
       </c>
-      <c r="G254" s="19" t="n"/>
+      <c r="G254" s="19" t="inlineStr">
+        <is>
+          <t>Peu après son lancement, les images d'Hubble se sont révélées floues à cause d'un défaut sur son miroir principal, plus fin qu'un cinquantième d'épaisseur de cheveu. Une réparation spectaculaire en sortie spatiale en 1993 a corrigé le problème et fait de lui l'un des instruments scientifiques les plus productifs jamais construits.</t>
+        </is>
+      </c>
       <c r="H254" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11422,7 +11450,11 @@
           <t>En 1991, Sony commercialise la première batterie lithium-ion rechargeable pratique, révolutionnant le stockage d'énergie portable pour les appareils électroniques. Les travaux théoriques sur les batteries lithium-ion remontent aux années 1970, avec des contributions de chercheurs comme M. Stanley Whittingham et John B. Goodenough, mais c'est Sony qui crée la première version commercialisable viable. La batterie lithium-ion offre une densité énergétique supérieure aux batteries alcalines précédentes, permettant les appareils électroniques portables modernes comme les téléphones mobiles et les ordinateurs portables. L'invention de la batterie lithium-ion révolutionne la technologie mobile, car elle offre une autonomie suffisante pour des appareils pratiques et rechargeables. Les batteries lithium-ion dominent le marché de l'énergie portable, avec des applications s'étendant aux véhicules électriques et au stockage d'énergie renouvelable. Goodenough reçoit le Prix Nobel en chimie en 2019, à l'âge de 97 ans, reconnaissant l'importance de la batterie lithium-ion pour la transition énergétique mondiale.</t>
         </is>
       </c>
-      <c r="G255" s="19" t="n"/>
+      <c r="G255" s="19" t="inlineStr">
+        <is>
+          <t>Les recherches à l'origine de la batterie lithium-ion (John Goodenough, Stanley Whittingham, Akira Yoshino) ont été récompensées par le prix Nobel de chimie en 2019 : Goodenough avait alors 97 ans, ce qui fait de lui le plus âgé de tous les lauréats Nobel.</t>
+        </is>
+      </c>
       <c r="H255" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11457,7 +11489,11 @@
           <t>Le 10 décembre 1948, les Nations unies adoptent la Déclaration universelle des droits de l'homme, reconnaissant le droit fondamental à l'information et à l'accès à la connaissance (article 19). Bien que rédigée avant l'ère numérique moderne, cette déclaration pose les fondations juridiques du droit d'accès à l'information numérique. La Déclaration universelle des droits de l'homme influence les législations nationales et les cadres juridiques internationaux concernant la liberté d'expression, le droit à la vie privée et l'accès à l'information. À l'ère numérique, ces principes sont étendus pour couvrir l'accès à Internet, la neutralité du net et la protection des données personnelles. La Déclaration universelle des droits de l'homme reste le document fondateur des droits humains modernes, affirmant que tous les êtres humains naissent libres et égaux en dignité et en droits.</t>
         </is>
       </c>
-      <c r="G256" s="19" t="n"/>
+      <c r="G256" s="19" t="inlineStr">
+        <is>
+          <t>L'article 19 de la Déclaration universelle des droits de l'homme garantit le droit de « chercher, recevoir et répandre des informations » par tout moyen d'expression — une formule invoquée depuis pour défendre l'idée que l'accès à internet est lui-même un droit fondamental.</t>
+        </is>
+      </c>
       <c r="H256" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11492,7 +11528,11 @@
           <t>Le 6 octobre 1995, les astronomes suisses Michel Mayor et Didier Queloz annoncent la découverte de la première exoplanète confirmée, une planète orbitan autour d'une étoile autre que notre Soleil. La planète, nommée 51 Pegasi b, est une géante gazeuse comparable à Jupiter orbitant l'étoile 51 Pegasi à seulement 4,3 jours. Cette découverte révolutionne l'astronomie en confirmant que les systèmes planétaires existent au-delà de notre système solaire, soutenant la notion que la vie pourrait exister ailleurs dans l'univers. Mayor et Queloz développent la technique de spectroscopie de vitesse radiale, détectant les changements minuscules dans la lumière des étoiles provoqués par l'attraction gravitationnelle de planètes en orbite. Depuis cette découverte initiale, des milliers d'exoplanètes ont été détectées, révélant une diversité de systèmes planétaires bien au-delà des prédictions initiales. Mayor reçoit le Prix Nobel en physique en 2019, reconnaissant l'importance de la découverte des exoplanètes pour l'astronomie. La découverte de planètes habitables potentielles autour d'étoiles proches relance la question éternelle : sommes-nous seuls dans l'univers ?</t>
         </is>
       </c>
-      <c r="G257" s="19" t="n"/>
+      <c r="G257" s="19" t="inlineStr">
+        <is>
+          <t>Michel Mayor et Didier Queloz ont détecté 51 Pegasi b non pas en la photographiant, mais en mesurant l'infime « oscillation » de la lumière de son étoile. Cette méthode leur a valu le prix Nobel de physique en 2019.</t>
+        </is>
+      </c>
       <c r="H257" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11527,7 +11567,11 @@
           <t>En 1941, après une chasse, l'inventeur suisse George de Mestral remarque que les graines de bardane s'accrochent obsessivement à son pantalon et à son chien. Inspiré par cette observation, il examine les graines au microscope et découvre des petits crochets qui s'attachent aux boucles de tissu. De Mestral développe le concept du velcro (VEL de velours + CRO de crochet) en combinant deux bandes de tissu : une avec des boucles serrées (comme le velours) et une avec de minuscules crochets. Il brevète son invention en 1955 et la présente à l'industrie manufacturière. Le velcro révolutionne la fermeture des vêtements et des équipements, offrant une alternative pratique aux boutons, lacets et fermetures à glissière. Le velcro trouve des applications au-delà des vêtements : dans l'espace (les astronautes utilisent le velcro pour fixer les équipements en microgravité), en médecine (pansements adhésifs), et dans les applications industrielles. Le velcro demeure un exemple classique d'innovation biologique, où une observation de la nature mène à une invention pratique utile à l'humanité.</t>
         </is>
       </c>
-      <c r="G258" s="19" t="n"/>
+      <c r="G258" s="19" t="inlineStr">
+        <is>
+          <t>George de Mestral a eu l'idée du velcro en examinant au microscope les bardanes restées accrochées au pelage de son chien après une promenade dans les Alpes : leurs minuscules crochets sont devenus le principe du système auto-agrippant.</t>
+        </is>
+      </c>
       <c r="H258" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11562,7 +11606,11 @@
           <t>En 1895, le docteur John Harvey Kellogg (fondateur de la céréale Kellogg's) brevète la première machine à fabriquer le beurre de cacahuète, transformant les cacahuètes rôties en une pâte lisse. Bien que les cacahuètes broyées existent depuis l'Antiquité précolombienne, c'est Kellogg qui crée la première version commercialisable du beurre de cacahuète moderne. Le beurre de cacahuète devient populaire aux États-Unis au début du XXe siècle, offrant une source de protéines bon marché accessible aux masses. Le beurre de cacahuète se diffuse mondialement, devenant un aliment de base en Amérique du Nord. Bien que controversé en raison de sa teneur en matières grasses, la recherche nutritionnelle moderne révèle que les lipides du beurre de cacahuète sont principalement monoinsaturés et insaturés, bénéfiques pour la santé cardiaque. Le beurre de cacahuète génère une industrie de plusieurs milliards de dollars, avec des millions de tonnes produites annuellement dans le monde entier.</t>
         </is>
       </c>
-      <c r="G259" s="19" t="n"/>
+      <c r="G259" s="19" t="inlineStr">
+        <is>
+          <t>John Harvey Kellogg — oui, celui des céréales — a breveté le beurre de cacahuète comme substitut de protéines pour les patients édentés de son sanatorium de Battle Creek. Il le considérait comme un aliment de santé, bien avant qu'il ne devienne la pâte à tartiner que l'on connaît.</t>
+        </is>
+      </c>
       <c r="H259" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11597,7 +11645,11 @@
           <t>En 2004, les physiciens russes Andre Geim et Konstantin Novoselov, travaillant à l'Université de Manchester, isolent avec succès le graphène, une forme de carbone monocouche possédant des propriétés électroniques extraordinaires. Le graphène est produit en exfoliant le graphite avec du ruban adhésif, une technique étonnamment simple pour extraire une couche monoatomique. Le graphène offre une conductivité électrique et thermique exceptionnelle, une résistance mécanique supérieure, et une flexibilité remarquable. Cette découverte révolutionne la science des matériaux, ouvrant la voie à des applications potentielles en électronique, énergie, et médecine. Geim et Novoselov reçoivent le Prix Nobel en physique en 2010, faisant de Novoselov l'un des plus jeunes lauréats du Prix Nobel. Le graphène s'avère être l'une des formes de carbone les plus prometteuses pour les futures technologies, bien que les applications commerciales se développent plus lentement que prévu initialement. La découverte du graphène ouvre une nouvelle ère de la nanotechnologie et des matériaux bidimensionnels.</t>
         </is>
       </c>
-      <c r="G260" s="19" t="n"/>
+      <c r="G260" s="19" t="inlineStr">
+        <is>
+          <t>Geim et Novoselov ont isolé le graphène avec un simple ruban adhésif, en décollant répétitivement de fines couches d'un bloc de graphite (le même matériau que la mine d'un crayon) — une technique qui leur a valu le prix Nobel de physique en 2010.</t>
+        </is>
+      </c>
       <c r="H260" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11632,7 +11684,11 @@
           <t>En 1952, l'inventeur américain Norman Joseph Woodland brevète le code-barres, un système automatisé d'identification des produits utilisant des barres verticales parallèles de largeurs variables. Woodland s'inspire des points et des tirets du code Morse, adaptant le concept pour créer un système capable d'être lu par des machines optiques. Bien que brevété en 1952, le code-barres ne trouve d'adoption commerciale massive que dans les années 1970, lorsque les scanners optiques deviennent pratiques et abordables. Le premier code-barres UPC (Universal Product Code) est scanné commercialement le 3 avril 1974 à un supermarché de Troy, Ohio, sur une boîte de gomme Wrigley's. Le code-barres révolutionne le commerce de détail en permettant le suivi automatisé des inventaires, la facturation rapide et la gestion efficace de la chaîne d'approvisionnement. L'adoption du code-barres réduit les erreurs de caisse et accélère les transactions commerciales. Aujourd'hui, les codes QR (Quick Response), une évolution du code-barres, permettent l'encodage de bien plus d'informations dans une surface bidimensionnelle compacte.</t>
         </is>
       </c>
-      <c r="G261" s="19" t="n"/>
+      <c r="G261" s="19" t="inlineStr">
+        <is>
+          <t>Norman Joseph Woodland a eu l'idée du motif circulaire du code-barres en traçant des lignes dans le sable d'une plage de Miami, en s'inspirant du code Morse qu'il avait appris étant scout.</t>
+        </is>
+      </c>
       <c r="H261" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11667,7 +11723,11 @@
           <t>Le 25 juillet 1978, Louise Brown naît à Bristol, Angleterre, marquant la première naissance d'un enfant conçu par fécondation in vitro (FIV). Louise est née grâce aux travaux du physiologiste Robert Edwards et du gynécologue Patrick Steptoe, qui ont développé la technique de la FIV permettant la conception en dehors du corps de la femme. La FIV est initialement développée pour traiter l'infertilité due aux trompes de Fallope obstruées ou endommagées chez les femmes. La naissance de Louise Brown provoque un tollé à la fois d'enthousiasme scientifique et de controverse éthique concernant la "conception en éprouvette". Aujourd'hui, la FIV et ses technologies connexes (ICSI, FIV génétique préimplantatoire) permettent aux millions de couples infertiles de concevoir des enfants. Plus de 8 millions de personnes sont nées grâce à la FIV depuis 1978. Edwards reçoit le Prix Nobel en 2010, reconnaissant l'importance révolutionnaire de la FIV pour la médecine reproductive. La FIV ouvre également les voies à la génétique reproductive et aux questions éthiques concernant la sélection génétique.</t>
         </is>
       </c>
-      <c r="G262" s="19" t="n"/>
+      <c r="G262" s="19" t="inlineStr">
+        <is>
+          <t>Louise Brown, premier « bébé-éprouvette » né par FIV en 1978, a ensuite eu ses propres enfants de manière naturelle. Robert Edwards a reçu le prix Nobel de médecine en 2010, plusieurs décennies après cette avancée.</t>
+        </is>
+      </c>
       <c r="H262" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11702,7 +11762,11 @@
           <t>En 1994, Denso Wave, filiale de Toyota, crée le code QR (Quick Response code), une version bidimensionnelle améliorée du code-barres capable d'encoder bien plus de données dans un format visuel compact. Le code QR utilise un motif de points et de carrés noirs et blancs organisés en grille carrée, readable par les téléphones portables munis de caméras. La conception open-source du code QR encourage l'adoption rapide par les industries et les gouvernements du monde entier. Le code QR révolutionne le partage d'informations en reliant le monde physique (affiches, emballages, cartes de visite) au monde numérique (pages web, vidéos, applications). Pendant la pandémie COVID-19, les codes QR facilitent le partage d'informations sans contact et le suivi des contacts numériques. Aujourd'hui, les codes QR sont omniprésents, utilisés dans le commerce, le transport, la santé et les paiements mobiles. L'adoption massive des codes QR pendant la pandémie accélère la transition vers les transactions sans contact et les interactions numériques sans intermédiaire.</t>
         </is>
       </c>
-      <c r="G263" s="19" t="n"/>
+      <c r="G263" s="19" t="inlineStr">
+        <is>
+          <t>Denso Wave, filiale de Toyota, a créé le code QR pour suivre les pièces automobiles sur ses lignes de production, puis a volontairement renoncé à faire valoir son brevet, rendant la technologie libre de droits — ce qui a grandement facilité son adoption mondiale.</t>
+        </is>
+      </c>
       <c r="H263" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11737,7 +11801,11 @@
           <t>Le 25 décembre 1969, Seiko, la compagnie japonaise de montres, commercialise la Seiko Astron, la première montre à quartz commerciale au monde. La montre à quartz utilise un cristal de quartz oscillant à une fréquence extrêmement stable pour maintenir le temps, offrant une précision supérieure aux montres mécaniques traditionnelles. L'oscillateur à quartz, découvert en 1880 par les frères Curie, est mis en application pour les montres seulement dans les années 1960. La montre à quartz révolutionne l'industrie horlogère, rendant les montres plus précises, abordables et durables. Bien que les maisons horlogères suisses possédaient la technologie, c'est les japonais (Seiko, Citizen, Casio) qui commercialisent agressivement les montres à quartz, remplaçant rapidement les montres mécaniques sur le marché. La révolution du quartz provoque la "crise de l'horlogerie suisse" dans les années 1970, où de nombreuses manufacture horlogères traditionnelles ferment ou sont consolidées. Paradoxalement, les montres mécaniques survivent en tant que luxe de prestige, tandis que les montres à quartz dominent le marché de masse.</t>
         </is>
       </c>
-      <c r="G264" s="19" t="n"/>
+      <c r="G264" s="19" t="inlineStr">
+        <is>
+          <t>La montre Seiko Astron, lancée le jour de Noël 1969, était si précise (quelques secondes d'écart par mois contre plusieurs minutes pour une montre mécanique) qu'elle a déclenché la « crise du quartz », qui a failli anéantir l'horlogerie suisse traditionnelle dans les années 1970-1980.</t>
+        </is>
+      </c>
       <c r="H264" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11772,7 +11840,11 @@
           <t>En 1964, Xerox, la compagnie américaine de technologie des documents, commercialise le Xerox Long Distance Xerography (LDX), le premier système de fax pratique et commercialement viable au monde. Le fax utilise la transmission téléphonique pour envoyer des images et des documents à travers les distances. Bien que les concepts de transmission de documents par téléphone remontent à la fin du XIXe siècle, c'est Xerox qui crée le premier système de fax fiable et abordable. Le fax révolutionne la communication commerciale, permettant le partage de documents importants à travers les distances sans délai postal. Le fax devient ubiquitaire dans les bureaux aux années 1980 et 1990, essentiellement remplaçant le courrier express pour les documents importants. Cependant, la révolution Internet et le courrier électronique (email) remplacent largement le fax à partir des années 2000. Malgré le déclin du fax, certains secteurs (gouvernement, justice, médecine) continuent à utiliser le fax pour les raisons légales et de conformité.</t>
         </is>
       </c>
-      <c r="G265" s="19" t="n"/>
+      <c r="G265" s="19" t="inlineStr">
+        <is>
+          <t>Le principe du fax est en réalité antérieur au téléphone : l'inventeur écossais Alexander Bain avait déjà breveté un appareil de transmission d'images en 1843, plus de trente ans avant l'invention du téléphone par Alexander Graham Bell.</t>
+        </is>
+      </c>
       <c r="H265" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11807,7 +11879,11 @@
           <t>En 1938, l'inventeur américain Chester Carlson développe le procédé de xérographie (du grec "écriture sèche"), créant la photocopie moderne basée sur l'électrostatique plutôt que sur les processus chimiques humides. Carlson, électricien sans formation formelle en chimie, expérimente dans son petit atelier pour créer un processus de reproduction d'images secs et rapides. Son premier prototype fonctionne le 22 octobre 1938, créant la première xérocopy. Cependant, Carlson passe des années à chercher des investisseurs avant que Xerox Corporation (alors Haloid Company) ne brevète et commercialise sa technologie en 1959. La photocopieuse Xerox 914, lancée en 1959, révolutionne les bureaux en rendant la duplication de documents instantanée, bon marché et de haute qualité. Les photocopieuses deviennent indispensables aux bureaux modernes, facilitant la distribution d'information et la documentation administrative. Bien que les photocopieuses soient partiellement remplacées par l'impression numérique et le stockage électronique, elles restent présentes dans les bureaux modernes et les institutions gouvernementales.</t>
         </is>
       </c>
-      <c r="G266" s="19" t="n"/>
+      <c r="G266" s="19" t="inlineStr">
+        <is>
+          <t>Chester Carlson a mis au point la xérographie dans la cuisine de son appartement et a été refusé par plus de vingt entreprises (dont IBM et Kodak) avant que la société Haloid, rebaptisée plus tard Xerox, n'accepte de la commercialiser en 1944.</t>
+        </is>
+      </c>
       <c r="H266" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11842,7 +11918,11 @@
           <t>Le 30 avril 1956, Ampex, la compagnie américaine d'électronique, présente le VRX-1000, le premier magnétoscope professionnel utilisable pour enregistrer et rejouer des images de télévision. L'invention du magnétoscope révolutionne la télévision en permettant l'enregistrement de programmes pour une rediffusion ultérieure, au lieu de la diffusion en direct uniquement. Les magnétoscopes utilisant la technologie de la bande magnétique dominent la télévision professionnelle et domestique pendant 50 ans. L'invention du magnétoscope permet la création d'archives télévisées, la production d'émissions plus complexes, et la distribution de contenu à travers les fuseaux horaires. À la fin des années 1970, les magnétoscopes domestiques (Betamax, VHS) révolutionnent le divertissement domestique, permettant aux gens de regarder des films à domicile. La guerre de format entre Betamax et VHS résout en faveur du VHS, qui domine le marché domestique pendant 25 ans. Bien que les magnétoscopes soient remplacés par l'enregistrement numérique et le streaming, ils restent des appareils culturellement importants représentant l'ère pré-Internet du divertissement.</t>
         </is>
       </c>
-      <c r="G267" s="19" t="n"/>
+      <c r="G267" s="19" t="inlineStr">
+        <is>
+          <t>Le premier magnétoscope professionnel d'Ampex, le VRX-1000, coûtait environ 50 000 dollars en 1956 (bien plus de 500 000 dollars actuels) et n'était accessible qu'aux chaînes de télévision — il faudra attendre encore deux décennies pour un appareil abordable par le grand public.</t>
+        </is>
+      </c>
       <c r="H267" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11877,7 +11957,11 @@
           <t>En 1961, Bell Punch Company au Royaume-Uni crée la Sumlock Comptometer, le premier appareil de calcul entièrement électronique disposant d'une interface de touches de saisie. Cependant, c'est le Friden EC-130R de 1963 qui est généralement considéré comme la première calculatrice électronique vraiment commerciale pratique aux États-Unis. La calculatrice électronique révolutionne la comptabilité et l'ingénierie en remplaçant les logarithmes manuels et les règles à calcul par des calculs numériques rapides et précis. La miniaturisation des calculatrices s'accélère dans les années 1970, avec la création des premières calculatrices de poche portables par Texas Instruments et Hewlett-Packard. La calculatrice de poche révolutionne l'éducation, le commerce et la science en rendant les calculs complexes instantanément accessibles. Bien que les calculatrices modernes soient intégrées aux téléphones portables et aux ordinateurs, les calculatrices de poche spécialisées persistent pour les applications techniques et éducatives.</t>
         </is>
       </c>
-      <c r="G268" s="19" t="n"/>
+      <c r="G268" s="19" t="inlineStr">
+        <is>
+          <t>La calculatrice britannique ANITA (1961) ne comportait aucune pièce mécanique pour ses calculs, une première mondiale, mais pesait environ 13 kilos et utilisait des tubes d'affichage à cathode froide, les écrans à transistors n'existant pas encore.</t>
+        </is>
+      </c>
       <c r="H268" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11912,7 +11996,11 @@
           <t>En 1948, Philips, la compagnie électronique néerlandaise, développe et commercialise le disque longue durée (LP, 33 tours), une révolution dans la technologie d'enregistrement sonore. Le LP utilise un sillon microscopique plus étroit que sur les disques 78 tours précédents, permettant jusqu'à 23 minutes de musique par face. Quelques mois plus tard, Columbia Records introduit son propre format LP à 33⅓ tours, devenant le standard dominant. Indépendamment, RCA Victor développe le 45 tours (disque microsillon) pour les singles. Le LP révolutionne la musique en permettant l'enregistrement d'albums complets, favorisant la création de concept albums artistiquement cohérents. Le LP domine le marché de la musique pendant 40 ans, jusqu'à être remplacé par le CD à partir des années 1980. Paradoxalement, le vinyle revient en vogue au XXIe siècle auprès des audiophiles et des collectionneurs qui apprécient la qualité sonore supérieure et l'expérience tactile du vinyle. Aujourd'hui, les ventes de vinyle augmentent après des décennies de déclin, se redéfinissant comme un produit de luxe premium.</t>
         </is>
       </c>
-      <c r="G269" s="19" t="n"/>
+      <c r="G269" s="19" t="inlineStr">
+        <is>
+          <t>La vitesse de 33 tours et un tiers par minute a été choisie car c'était la plus lente permettant encore une reproduction sonore fiable avec les pointes de lecture de l'époque, offrant environ 22 minutes de musique par face contre 3 à 4 minutes pour un disque 78 tours.</t>
+        </is>
+      </c>
       <c r="H269" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11947,7 +12035,11 @@
           <t>En 1982, Philips et Sony, les géants de l'électronique, annoncent le Compact Disc (CD), une révolution dans le stockage et la lecture du son numérique. Le CD utilise un laser pour lire les données numériques gravées microscopiquement sur une surface réfléchissante, offrant une qualité sonore supérieure sans dégradation due à l'usure mécanique. Le premier CD commercialisé est "Philips' Laserdisc" de Philips en 1978 pour la vidéo, mais c'est le CD audio qui révolutionne la musique. Le CD se diffuse rapidement sur le marché grand public à partir de 1983, remplaçant progressivement le vinyle et les cassettes magnétiques. Le CD offre la durée, la durabilité, la qualité sonore et la commodité, établissant un nouveau standard pour la musique enregistrée. L'adoption du CD crée un marché de musique de plusieurs milliards de dollars, bien que ce marché soit ultérieurement menacé par la compression numériques des fichiers MP3 et le streaming. Bien que les CDs soient remplacés par le streaming numérique, ils restent populaires auprès de certains mélomanes appréciant la propriété physique du médium.</t>
         </is>
       </c>
-      <c r="G270" s="19" t="n"/>
+      <c r="G270" s="19" t="inlineStr">
+        <is>
+          <t>La durée de 74 minutes et le diamètre de 12 cm du CD auraient été fixés pour qu'un seul disque puisse contenir l'intégralité de la Neuvième Symphonie de Beethoven, à la demande du vice-président de Sony Norio Ohga, lui-même musicien de formation lyrique.</t>
+        </is>
+      </c>
       <c r="H270" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -11982,7 +12074,11 @@
           <t>Entre 1989 et 1993, une équipe d'ingénieurs allemands de la Fraunhofer Society, dirigée par le Dr. Karlheinz Brandenburg, développe le codec MP3 (MPEG-1 Audio Layer III), compressant les fichiers audio numériques de 90% tout en préservant une qualité sonore acceptable à l'oreille humaine. Le MP3 révolutionne la musique numérique en rendant possible le téléchargement et le partage de chansons sur Internet à des vitesses pratiques. Bien que le MP3 ne soit pas le premier format audio compressé, c'est lui qui atteint l'adoption de masse grâce à son équilibre entre compression et qualité. L'adoption du MP3 démocratise l'accès à la musique, permettant à chacun de créer des bibliothèques musicales numériques portables. Cependant, le MP3 facilite également le piratage de la musique, catalysant la crise de l'industrie discographique qui n'a pas su s'adapter au numérique. Ironiquement, c'est Steve Jobs et l'iTunes Store (2003) qui sauvent l'industrie musicale en proposant une alternative légale au piratage. Bien que le MP3 soit remplacé par des codecs plus efficaces (AAC, OPUS), son impact sur la révolution numérique de la musique reste incontournable.</t>
         </is>
       </c>
-      <c r="G271" s="19" t="n"/>
+      <c r="G271" s="19" t="inlineStr">
+        <is>
+          <t>Le format MP3 a failli disparaître dès 1991, un vote de l'industrie ayant presque retenu un format concurrent. L'équipe de Fraunhofer a affiné son algorithme de compression à l'oreille en utilisant en boucle un seul morceau enregistré à la maison : « Tom's Diner » de Suzanne Vega, choisi pour sa clarté quasi a cappella.</t>
+        </is>
+      </c>
       <c r="H271" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12017,7 +12113,11 @@
           <t>Le 16 avril 1997, Reed Hastings et Marc Randolph lancent Netflix, un service de location de films en DVD par courrier postal via Internet. Netflix révolutionne la location de films en éliminant les pénalités de retard (amende pour retard) qui caractérisaient Blockbuster et autres loueurs physiques de films. Les clients Netflix reçoivent les DVD dans leur boîte aux lettres, les regardent à leur rythme, et les retournent gratuitement via le courrier. Netflix fonctionne sur un modèle d'abonnement à forfait plutôt que par location unitaire, prédisant correctement que les consommateurs préfèrent la certitude d'un coût mensuel fixe. Netflix se divise en deux entités en 2011 : Netflix Streaming pour le contenu vidéo en ligne et Qwikster pour la location de DVD par courrier (Qwikster ferme en 2013). Netflix Streaming révolutionne le divertissement vidéo à partir de 2007, lorsque la société commence à offrir le streaming de contenu en direct. Netflix Streaming s'étend internationalement dans les années 2010, devenant un leader mondial du streaming vidéo. En 2024, Netflix compte plus de 260 millions d'abonnés et a redéfini le divertissement vidéo.</t>
         </is>
       </c>
-      <c r="G272" s="19" t="n"/>
+      <c r="G272" s="19" t="inlineStr">
+        <is>
+          <t>Reed Hastings a raconté avoir eu l'idée de Netflix après s'être vu facturer 40 dollars d'amende de retard par Blockbuster pour une cassette d'Apollo 13 — une anecdote qu'il a lui-même reconnu avoir sans doute simplifiée pour la presse.</t>
+        </is>
+      </c>
       <c r="H272" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12052,7 +12152,11 @@
           <t>En 1955, Eveready Battery Company commercialise la première batterie alcaline grand public, surpassant les batteries zinc-carbone en performance et en durée de vie. La batterie alcaline utilise un électrolyte alcalin (hydroxyde de potassium) au lieu d'un électrolyte acide, permettant une réaction chimique plus efficace. L'invention de la batterie alcaline révolutionne l'alimentation des appareils portables, permettant une autonomie 3 à 4 fois supérieure aux batteries zinc-carbone. Les piles alcalines deviennent rapidement le standard pour les appareils électroniques portables tels que les torches, les transistors-radio et les jouets. Les batteries alcalines dominent le marché des piles non-rechargeables pendant 60 ans, jusqu'à être partiellement remplacées par les batteries rechargeables lithium-ion. Aujourd'hui, les piles alcalines restent populaires pour les appareils occasionnels où la recharge est impratique. Les batteries alcalines jetables soulèvent également des enjeux environnementaux liés aux déchets électroniques et à la pollution des métaux lourds.</t>
         </is>
       </c>
-      <c r="G273" s="19" t="n"/>
+      <c r="G273" s="19" t="inlineStr">
+        <is>
+          <t>C'est l'ingénieur canadien Lewis Urry qui a mis au point la pile alcaline moderne chez Eveready dans les années 1950 ; elle stocke bien plus d'énergie que les anciennes piles zinc-carbone et reste aujourd'hui le format de pile domestique le plus répandu.</t>
+        </is>
+      </c>
       <c r="H273" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12087,7 +12191,11 @@
           <t>En 1962, Nick Holonyak Jr. chez General Electric crée la première diode électroluminescente (LED) visible à l'œil nu, une lumière rouge, révolutionnant le potentiel des semi-conducteurs pour produire de la lumière. Les LEDs émettent de la lumière par transition des électrons dans une jonction semi-conductrice, un processus beaucoup plus efficace que l'émission thermique des lampes incandescentes. Les premières LEDs rouges sont utilisées dans les indicateurs et les affichages numériques dans les années 1970, remplaçant les ampoules moins efficaces. L'invention de LEDs de différentes couleurs (orange, jaune, vert, bleu) s'étend au cours des décennies suivantes, culminant avec la création de la LED blanche en 1996 par Shuji Nakamura. Les LEDs blanches révolutionnent l'éclairage, offrant une efficacité énergétique jusqu'à 10 fois supérieure aux lampes incandescentes. L'adoption des LEDs pour l'éclairage général commence à la fin des années 2000, progressivement remplaçant les lampes incandescentes et fluorescentes. Nakamura reçoit le Prix Nobel en physique en 2014, reconnaissant l'importance de la LED bleue pour l'éclairage efficace. Aujourd'hui, les LEDs dominent le marché de l'éclairage et sont omniprésentes dans les appareils électroniques modernes.</t>
         </is>
       </c>
-      <c r="G274" s="19" t="n"/>
+      <c r="G274" s="19" t="inlineStr">
+        <is>
+          <t>La première LED rouge de Nick Holonyak était si faible qu'elle ne servait au départ que de voyant lumineux. Il avait pourtant prédit à l'époque qu'elle finirait par remplacer l'ampoule à incandescence — une prédiction qui a mis environ cinquante ans à se réaliser pleinement.</t>
+        </is>
+      </c>
       <c r="H274" s="19" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12122,7 +12230,11 @@
           <t>En 2050, selon les projections de l'étude majeure publiée dans "Science" (2018) par Jambeck et al., la masse totale de plastique accumulée dans les océans dépassera la biomasse totale des poissons. Cette projection repose sur les données montrant que 8 à 12 millions de tonnes de plastique entrent chaque année dans les océans. Le plastique se fragmente en microplastiques, pénétrant les chaînes alimentaires marines et terrestres, affectant les écosystèmes à tous les niveaux. Les poissons ingèrent les microplastiques, réduisant leur capacité à se nourrir et à se reproduire. Cette crise plastique menace la viabilité des pêcheries mondiales, source de protéines pour 3 milliards de personnes. Les projections supposent une continuation des tendances actuelles sans intervention majeure de réduction des plastiques. Cette date critique symbolise l'urgence de la transition vers une économie circulaire et sans plastique jetable.</t>
         </is>
       </c>
-      <c r="G275" s="20" t="inlineStr"/>
+      <c r="G275" s="20" t="inlineStr">
+        <is>
+          <t>La comparaison provient d'un rapport de 2016 de la Fondation Ellen MacArthur et du Forum économique mondial, dont la formule-choc originale — plus de plastique que de poissons dans l'océan d'ici 2050 — a depuis été reprise dans d'innombrables discours et médias.</t>
+        </is>
+      </c>
       <c r="H275" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12157,7 +12269,11 @@
           <t>Le rapport du Groupe d'Experts Intergouvernemental sur l'Évolution du Climat (GIEC) de 2021 projette une fonte quasi-totale de la calotte glaciaire du Groenland d'ici 2070 selon les scénarios d'émissions élevées (RCP 8.5/SSP5-8.5). Cette calotte contient environ 2,85 millions de kilomètres cubes de glace, représentant 7% du niveau des mers mondial. La fonte du Groenland s'accélère exponentiellement : elle a contribué à seulement 0,03 mm/an d'élévation du niveau des mers dans les années 1990, mais à 0,7 mm/an en 2010-2020. Les observations satellitaires montrent que la perte de masse annuelle a augmenté de 280% entre 2003 et 2019. Cette fonte aurait des conséquences catastrophiques : perturbation de la circulation thermohaline atlantique, élévation du niveau des mers menaçant les villes côtières, modification majeure des régimes climatiques mondiaux. Les écosystèmes arctiques, dépendants de la glace, disparaîtront, menaçant l'ours polaire, le phoque et d'autres espèces. Cette projection revient dans tous les rapports climatiques majeurs depuis 2013.</t>
         </is>
       </c>
-      <c r="G276" s="20" t="inlineStr"/>
+      <c r="G276" s="20" t="inlineStr">
+        <is>
+          <t>La calotte glaciaire du Groenland fait environ trois fois la superficie de la France et contient assez d'eau pour élever le niveau des mers de plus de 7 mètres si elle fondait intégralement — les projections à 2070-2100 n'envisagent qu'une fonte partielle.</t>
+        </is>
+      </c>
       <c r="H276" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12192,7 +12308,11 @@
           <t>Selon les projections démographiques des Nations Unies (2019, mise à jour 2022), la population mondiale atteindrait son pic vers 2070-2090, mais certaines projections plus pessimistes de l'Institut pour la Métrique de la Santé (IHME) de l'Université de Washington suggèrent un pic dès 2040 sous certains scénarios. Le pic démographique résulte de la convergence de plusieurs facteurs : baisse du taux de fertilité global (passé de 5,1 enfants/femme en 1960 à 2,3 en 2020), augmentation de l'éducation des femmes, accès à la contraception, urbanisation, et coûts économiques croissants d'élever les enfants. Après 2040, selon l'IHME, la population mondiale pourrait décliner de façon permanente, passant de 9,7 milliards à 8,8 milliards d'ici 2100. Cette décroissance sera inégale : l'Afrique subsaharienne continuera à croître, tandis que l'Europe, l'Asie de l'Est et l'Amérique Latine verront des déclins majeurs. Cette transition démographique aura des implications majeures pour l'économie, les systèmes de retraite, l'emploi, et l'utilisation des ressources.</t>
         </is>
       </c>
-      <c r="G277" s="20" t="inlineStr"/>
+      <c r="G277" s="20" t="inlineStr">
+        <is>
+          <t>Il s'agirait de l'un des retournements démographiques les plus rapides jamais projetés : il a fallu plus de 300 000 ans à l'humanité pour atteindre 1 milliard d'habitants (vers 1800), mais la population pourrait commencer à décliner en l'espace d'une seule vie humaine après son pic.</t>
+        </is>
+      </c>
       <c r="H277" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12227,7 +12347,11 @@
           <t>Les projections du Rapport Planète Vivante 2022 du Fonds mondial pour la nature (WWF) et les données du Centre de recherche sur la biodiversité (Zoological Society of London) indiquent un déclin de 50% à 75% des populations d'animaux vertébrés d'ici 2075 selon les scénarios pessimistes. Ce déclin résulte de la combinaison de la perte d'habitat (70% des forêts tropicales perdues), du changement climatique, de la pollution, de la surexploitation des ressources, et des maladies. Depuis 1970, les populations d'animaux sauvages ont chuté de 68% en moyenne. Le taux actuel d'extinction est 100 à 1000 fois plus élevé que le taux naturel d'extinction préalable. Les forêts tropicales, qui abritent 80% des espèces terrestres, disparaissent au taux de 10 millions d'hectares par an. Les écosystèmes aquatiques subissent un déclin encore plus rapide : 84% des populations de poissons d'eau douce ont disparu. Si ces tendances continuent, nous entrerions dans la sixième extinction de masse de l'histoire de la Terre, la première causée par une seule espèce : l'humanité.</t>
         </is>
       </c>
-      <c r="G278" s="20" t="inlineStr"/>
+      <c r="G278" s="20" t="inlineStr">
+        <is>
+          <t>L'indice Planète Vivante du WWF, source de cette projection, ne mesure pas le nombre d'espèces disparues mais le déclin moyen de la taille des populations animales suivies — une espèce peut donc toujours exister tout en étant beaucoup moins nombreuse qu'il y a 50 ans.</t>
+        </is>
+      </c>
       <c r="H278" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12262,7 +12386,11 @@
           <t>Le 6ème Rapport d'Évaluation du GIEC (2021) projette une élévation du niveau des mers global de 0,43 à 0,84 mètre d'ici 2100 selon le scénario modéré (SSP2-4.5), et jusqu'à 0,84 à 1,30 mètre selon le scénario pessimiste (SSP5-8.5). Cette élévation résulte de deux mécanismes principaux : la dilatation thermique de l'eau (contribution de 40%) et la fonte des glaciers terrestres et des calottes polaires (contribution de 60%). L'élévation du niveau des mers menace directement les populations côtières : 600 millions de personnes vivent dans des zones côtières moins de 10 mètres au-dessus du niveau de la mer. Les villes majeures comme Venise, la Nouvelle-Orléans, Bangkok, Le Caire, et Shanghai subissent déjà des inondations récurrentes d'eau de mer. Une élévation d'1 mètre inonderait 40% du delta du Nil, 17% du Bangladesh, et détruirait les atolls du Pacifique. Les impacts économiques sont estimés à des milliers de milliards de dollars en dégâts aux infrastructures, pertes agricoles, et déplacements de populations. C'est l'une des conséquences du changement climatique avec le plus haut degré de certitude scientifique.</t>
         </is>
       </c>
-      <c r="G279" s="20" t="inlineStr"/>
+      <c r="G279" s="20" t="inlineStr">
+        <is>
+          <t>Une élévation d'un mètre ne se contenterait pas d'inonder les côtes directement : elle repousserait aussi l'eau salée plus loin dans les fleuves et les nappes phréatiques, contaminant l'eau douce de villes comme La Nouvelle-Orléans bien avant que la mer ne les atteigne physiquement.</t>
+        </is>
+      </c>
       <c r="H279" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12297,7 +12425,11 @@
           <t>Des études publiées dans "Nature Climate Change" (2010, Sherwood et al., mise à jour 2020) et confirmées par le GIEC projettent que certaines régions tropicales humides pourraient atteindre des conditions où la thermorégulation humaine devient impossible d'ici 2100. Le thermomètre de boule humide (qui mesure la température perçue en tenant compte de l'humidité) dépasserait 35°C, la limite physiologique au-delà de laquelle le corps humain ne peut plus se refroidir par évaporation de la sueur. Cette projection concerne particulièrement les deltas fluviaux majeurs : le delta du Mékong (Cambodge, Vietnam), le delta du Gange-Brahmapoutre (Bangladesh, Inde), le Golfe Persique (Iran, Émirats arabes), et le nord de l'Inde. Ces régions regroupent plus d'1 milliard de personnes. L'inhabitabilité progressive forcerait des migrations massives sans précédent historique. Les activités de plein air deviendraient impossibles pendant plusieurs mois de l'année. L'agriculture tropicale, source de nourriture pour des milliards, serait gravement compromise. Cette limite est mathématiquement définie et s'appuie sur la thermodynamique biologique, pas sur des projections climatiques incertaines.</t>
         </is>
       </c>
-      <c r="G280" s="20" t="inlineStr"/>
+      <c r="G280" s="20" t="inlineStr">
+        <is>
+          <t>Une « température au thermomètre mouillé » de 35°C ne semble pas extrême sur un thermomètre classique, mais elle signifie que l'air est si chaud et humide que la sueur ne peut plus s'évaporer : une personne en bonne santé pourrait alors mourir d'un coup de chaleur en quelques heures, même à l'ombre et avec de l'eau à volonté.</t>
+        </is>
+      </c>
       <c r="H280" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12332,7 +12464,11 @@
           <t>Le rapport du GIEC et les études océanographiques du SCRIPPS Institution et de l'Institut océanographique de Monaco projettent une augmentation de 200% de l'acidité océanique (diminution du pH) d'ici 2200 par rapport aux niveaux pré-industriels. Cette acidification résulte de l'absorption de 25% à 30% des émissions de CO2 anthropogénique par les océans, transformant le CO2 en acide carbonique. Le pH océanique a déjà diminué de 0,1 unité depuis 1750, représentant une augmentation de 30% de l'acidité. Une augmentation de 200% supplémentaire (pH passant de 8,2 à ~7,7) détruirait les écosystèmes marins calcifiés : les mollusques, les crustacés, les coraux, et les ptéropodes (escargots marins de 500 micromètres) ne pourraient plus former leurs coquilles. Les larves de poisson perdraient leur capacité à localiser les récifs de reproduction. La chaîne alimentaire marine s'effondrerait. Les pêcheries commerciales, source de 1,5 milliard de dollars annuels, disparaîtraient. Les récifs coralliens, qui fournissent 25% des protéines marines à 500 millions de personnes, seraient complètement détruits. Cette acidification est équivalente au changement chimique survenu lors de la Grande Extinction du Permien (-252 millions d'années).</t>
         </is>
       </c>
-      <c r="G281" s="20" t="inlineStr"/>
+      <c r="G281" s="20" t="inlineStr">
+        <is>
+          <t>L'acidification des océans est parfois surnommée « l'autre problème du CO2 » : même si l'humanité arrêtait toute émission dès aujourd'hui, le pH des océans continuerait de baisser pendant des siècles, le temps que le carbone déjà absorbé soit neutralisé par les minéraux des fonds marins.</t>
+        </is>
+      </c>
       <c r="H281" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12367,7 +12503,11 @@
           <t>Selon les données de la NASA et du Centre des Objets Géocroiseurs (Planetary Defense Center), un impact d'astéroïde potentiellement catastrophique (&gt;1 km de diamètre) frappe statistiquement la Terre environ une fois tous les 500 000 à 1 million d'années. À l'échelle de 100 000 ans, la probabilité qu'un tel événement se produise est d'environ 10 à 20%. Les géocroiseurs de plus de 140 mètres, capables de détruire une région entière, frappent environ une fois tous les 10 000 ans. L'extinction des dinosaures (il y a 66 millions d'années) fut causée par un astéroïde de 10 kilomètres frappant le Yucatan. L'événement de Tunguska (1908) en Sibérie, causé par un astéroïde de 40 mètres, rasa 80 millions d'arbres. Actuellement, 90% des astéroïdes de plus de 1 km de diamètre proches de la Terre ont été catalogués, mais des milliers de plus petits astéroïdes restent indétectés. La NASA a lancé les missions DART (2022) et Hera pour développer des capacités de défense planétaire, testant la possibilité de dévier un astéroïde par impact cinétique. Le risque zéro n'existe pas : l'univers reste un environnement dangereux.</t>
         </is>
       </c>
-      <c r="G282" s="20" t="inlineStr"/>
+      <c r="G282" s="20" t="inlineStr">
+        <is>
+          <t>La mission DART de la NASA a testé avec succès la défense planétaire en 2022 en percutant délibérément l'astéroïde Dimorphos, raccourcissant son orbite de 32 minutes — la preuve qu'il serait possible de dévier un astéroïde menaçant, à condition d'avoir suffisamment de temps pour agir.</t>
+        </is>
+      </c>
       <c r="H282" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12402,7 +12542,11 @@
           <t>Le paléovolcanologue Christopher Harpel et l'United States Geological Survey (USGS) documentent que le supervolcan Yellowstone suit un cycle d'éruptions majeures (supereruptions) tous les 640 000 à 800 000 ans en moyenne. La dernière supereruption de Yellowstone remonte à 640 000 ans. Une nouvelle supereruption est donc statistiquement due. Une éruption de magnitude 8 (Volcanic Explosivity Index) injecterait 1000 kilomètres cubes de matériau dans l'atmosphère, créant une colonne de cendre s'élevant à 50 km d'altitude. Les conséquences seraient globales : la cendre recouvrirait les États-Unis d'une couche de 10 centimètres en quelques jours, rendant l'agriculture impossible. Les gaz volcaniques refroidiraient le climat de 10 à 20 degrés Celsius pendant 3 à 10 ans (hiver volcanique). Les récoltes échoueraient pendant 5 ans minimum. La famine et les guerres décimeraient les populations humaines. Cette éruption ferait pâlir la catastrophe du Toba (74 000 ans) qui a réduit la population humaine à quelques milliers d'individus. Les données sismiques montrent que Yellowstone se recharge lentement mais régulièrement.</t>
         </is>
       </c>
-      <c r="G283" s="20" t="inlineStr"/>
+      <c r="G283" s="20" t="inlineStr">
+        <is>
+          <t>La chambre magmatique de Yellowstone est surveillée par des centaines de sismomètres et de stations GPS ; les géologues rappellent que son activité actuelle (petits séismes, éruptions de geysers comme Old Faithful) est un comportement de fond parfaitement normal, et non le signe d'une supereruption imminente.</t>
+        </is>
+      </c>
       <c r="H283" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12437,7 +12581,11 @@
           <t>Sur le timescale d'un million d'années, la tectonique des plaques continue sa lente danse continentale. Selon les modèles de géodynamique de l'Institut de Physique du Globe (IPGP) et de l'Université de Cambridge, 1 million d'années correspond à environ 20 à 40 centimètres de mouvement des plaques continentales (selon les plaques). La Californie dérive vers le nord-ouest à 5 cm/an, ce qui représenterait 50 kilomètres de déplacement sur 1 million d'années. L'Afrique continue à se séparer de l'Eurasie, élargissant la mer Méditerranée. La côte Est de l'Amérique du Nord s'éloigne de l'Afrique de 2,5 cm/an. L'Australie dérive vers le nord. Bien que ces changements semblent imperceptibles à l'échelle humaine, ils reconfigurent complètement la géographie de la Terre à l'échelle géologique. De nouvelles chaînes de montagnes apparaissent par l'orogenèse. De vieux océans ferment. De nouveaux océans s'ouvrent. Les connexions biologiques entre continents changent, provoquant des isolations et des spéciations. C'est un processus continu depuis 2,5 milliards d'années qui explique la distribution actuelle des continents et des formes de vie.</t>
         </is>
       </c>
-      <c r="G284" s="20" t="inlineStr"/>
+      <c r="G284" s="20" t="inlineStr">
+        <is>
+          <t>Au rythme actuel de dérive des continents, Los Angeles et San Francisco, situées de part et d'autre de la faille de San Andreas, se rapprochent lentement l'une de l'autre et pourraient devenir des villes voisines dans environ 15 millions d'années.</t>
+        </is>
+      </c>
       <c r="H284" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12472,7 +12620,11 @@
           <t>Selon les modèles d'évolution stellaire confirmés par le physicien Carl Sagan et actualisés par l'astrophysique stellaire moderne, le Soleil augmente lentement sa luminosité tout au long de sa vie de séquence principale. Cette luminosité augmente en moyenne de 10% tous les 2 milliards d'années. Dans 2 milliards d'années, le Soleil sera 10% plus lumineux qu'aujourd'hui. Cela semble modeste, mais c'est catastrophique pour la Terre. Un Soleil 10% plus lumineux signifie que l'énergie reçue augmente de 21% (car l'énergie augmente avec le carré de la luminosité relative). Cette augmentation drastique du rayonnement solaire provoquera un emballement de l'effet de serre : l'eau s'évaporera des océans plus rapidement, créant plus de vapeur d'eau (un gaz à effet de serre puissant), ce qui augmentera la température, ce qui augmentera l'évaporation, dans une boucle de rétroaction positive. Les océans bouilliront en quelques millions d'années. L'atmosphère ressemblera à celle de Vénus : ultra-chaude, ultra-dense, écrasante. Toute vie complexe aura disparu bien avant (probablement dans 1-1,5 milliards d'années). C'est la limite thermique définitive de la vie terrestre.</t>
         </is>
       </c>
-      <c r="G285" s="20" t="inlineStr"/>
+      <c r="G285" s="20" t="inlineStr">
+        <is>
+          <t>Ce lent réchauffement du Soleil est le miroir inversé du « paradoxe du jeune Soleil faible » : au tout début de son histoire, il était environ 30 % moins lumineux qu'aujourd'hui, et pourtant la Terre est restée assez chaude pour conserver de l'eau liquide — un puzzle que les scientifiques affinent encore.</t>
+        </is>
+      </c>
       <c r="H285" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12507,7 +12659,11 @@
           <t>Dans environ 5 à 7 milliards d'années, le Soleil épuisera son carburant d'hydrogène dans son noyau et se transformera en géante rouge. C'est le destin inévitable de toutes les étoiles de la masse du Soleil, selon les modèles d'évolution stellaire de Hertzsprung-Russell (1911, actualisés). En phase de géante rouge, le Soleil augmentera son rayon de 250 fois, s'étendant potentiellement jusqu'à l'orbite actuelle de Vénus ou même de la Terre. Le Soleil engloutira définitivement Mercure et Vénus. La Terre sera soit engloutie, soit carbonisée et réduite à une roche stérile. Les océans s'évaporeront. L'atmosphère sera balayée. C'est la fin inévitable de la Terre. Pendant cette phase de géante rouge, le Soleil sera 1000 fois plus lumineux. Après quelques millions d'années en tant que géante rouge, le Soleil rejettera sa couche externe (nébuleuse planétaire) et s'effondrera en une naine blanche : une étoile morte de la taille de la Terre, d'une densité extrême (une cuillère à café pèserait des tonnes). La Terre, ou ce qu'il en restera, orbitera ce cadavre stellaire dans un univers en expansion infini. C'est le destin thermodynamique de tout système : vers l'entropie maximale.</t>
         </is>
       </c>
-      <c r="G286" s="20" t="inlineStr"/>
+      <c r="G286" s="20" t="inlineStr">
+        <is>
+          <t>En devenant une géante rouge, le Soleil perdra une telle quantité de masse par vent stellaire que l'orbite de la Terre devrait s'élargir : certains modèles suggèrent qu'elle pourrait de justesse échapper à l'engloutissement, pour ne devenir qu'un caillou calciné et sans atmosphère.</t>
+        </is>
+      </c>
       <c r="H286" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12542,7 +12698,11 @@
           <t>Selon les calculs d'astrophysiciens du Space Telescope Science Institute et de l'Université de Cambridge utilisant les données du satellite Gaia, la galaxie d'Andromède (distante de 2,5 millions d'années-lumière) se rapproche de la Voie lactée à une vitesse de 110 kilomètres par seconde. Dans environ 4,5 milliards d'années, Andromède et la Voie lactée collideront, fusionnant progressivement en une seule mégagalaxie (que certains ont surnommée "Milkomède" ou "Lactamedromeda"). Ce processus ne serait pas catastrophique aux échelles humaines locales : les distances interstellaires sont si vastes que les collisions réelles entre étoiles lors d'une fusion galactique sont statistiquement rares. Cependant, à l'échelle de 200 000 ans, Andromède aura sensiblement augmenté en taille apparente dans le ciel nocturne. Les perturbations gravitationnelles de la proximité d'Andromède pourraient déstabiliser les orbites de certains objets dans le nuage d'Oort, augmentant les risques d'impacts de comètes sur la Terre. La luminosité du ciel nocturne à l'approche de la fusion sera dramatiquement modifiée. Astronomiquement parlant, c'est une date clé où l'univers local change de structure.</t>
         </is>
       </c>
-      <c r="G287" s="20" t="inlineStr"/>
+      <c r="G287" s="20" t="inlineStr">
+        <is>
+          <t>Malgré leurs quelque mille milliards d'étoiles combinées, la collision entre la Voie lactée et Andromède devrait être presque sans conséquence pour chaque système stellaire pris individuellement : les distances entre étoiles sont si immenses que les collisions directes resteront extrêmement rares.</t>
+        </is>
+      </c>
       <c r="H287" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12577,7 +12737,11 @@
           <t>Sur une période d'1 million d'années, tous les cycles biologiques majeurs se manifestent. La durée moyenne de vie d'une espèce de mammifère est d'environ 1 à 2 millions d'années selon les données du Muséum américain d'histoire naturelle. L'Homo sapiens n'existe que depuis environ 300 000 ans. Statistiquement, l'humanité a peut-être 700 000 à 1 700 000 ans avant son extinction naturelle (par spéciation, divergence évolutive, ou remplacement par une espèce dérivée). L'évolution favorisera de nouvelles adaptations. Si le climat change, les humains évolueront ou divergeront en espèces distinctes. Les isolations géographiques créeront de nouveaux hominidés. Ou simplement, une compétition ou maladie émergente réduira l'humanité à l'extinction. Le taux d'extinction des espèces sur cette période historique n'est pas connaissable avec précision, mais peu d'espèces durent plus de 10 millions d'années sans transformation majeure. L'Homo sapiens, malgré sa technologie, reste sujet aux lois biologiques fondamentales. Toutefois, notre technologie future pourrait modifier ces règles : si l'humanité maîtrise l'édition génétique, elle pourrait prolonger (ou transformer) son existence. C'est une limite purement biologique, non une certitude.</t>
         </is>
       </c>
-      <c r="G288" s="20" t="inlineStr"/>
+      <c r="G288" s="20" t="inlineStr">
+        <is>
+          <t>Une espèce de mammifère survit en moyenne environ 1 million d'années avant de s'éteindre ou d'évoluer en autre chose — à cette aune, Homo sapiens, âgé d'environ 300 000 ans, est encore une espèce relativement jeune.</t>
+        </is>
+      </c>
       <c r="H288" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12612,7 +12776,11 @@
           <t>Les mammifères règnent depuis environ 225 millions d'années (depuis le Trias moyen), mais sur une période de 100 millions d'années supplémentaires, il est statistiquement probable qu'une nouvelle extinction de masse ou une transformation évolutive majeure éliminerait l'ordre des mammifères tel que nous le connaissons. L'histoire de la Terre montre 5 extinctions de masse majeures, chacune séparée de dizaines de millions d'années. Les conditions planétaires auront radicalement changé : le CO2, la température, les régimes de pluie, la topographie continentale seront méconnaissables. Les écosystèmes mondiaux se réorganiseront. Certaines niches écologiques seront occupées par de nouveaux groupes d'animaux issus de la radiation adaptative des survivants. Les arthropodes, extrêmement adaptatifs, pourraient dominer davantage. Ou une nouvelle classe de vertébrés (les descendants des oiseaux ou des reptiles marins) pourrait s'adapter aux niches actuellement occupées par les mammifères. L'extinction des dinosaures il y a 66 millions d'années a permis l'essor des mammifères. Le même processus peut se répéter. C'est le flux et reflux éternel de la vie terrestre, gouverné par la sélection naturelle et les catastrophes géologiques.</t>
         </is>
       </c>
-      <c r="G289" s="20" t="inlineStr"/>
+      <c r="G289" s="20" t="inlineStr">
+        <is>
+          <t>Les mammifères ne sont devenus les grands animaux dominants de la planète qu'après l'impact d'astéroïde qui a rayé les dinosaures non aviens de la carte il y a 66 millions d'années — avant cela, pendant plus de 150 millions d'années, ils sont restés de petites créatures nocturnes vivant dans l'ombre des reptiles.</t>
+        </is>
+      </c>
       <c r="H289" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12647,7 +12815,11 @@
           <t>Dans 3 milliards d'années, le Soleil sera environ 20 à 30% plus lumineux qu'aujourd'hui (suivant l'évolution linéaire d'augmentation de 10% tous les 2 milliards d'années). À ce stade, l'énergie reçue par la Terre aura augmenté d'environ 44 à 73%. Cette augmentation massive de l'énergie solaire causera un emballement de l'effet de serre. Mais bien avant l'ébullition complète des océans, la photosynthèse elle-même devient thermodynamiquement impossible. La photosynthèse est une réaction chimique basée sur l'absorption de photons de lumière visible (400-700 nm) par des molécules de chlorophylle. L'efficacité énergétique diminue si le spectre solaire change ou si la température de base augmente trop. À partir d'une augmentation de 15 à 20% du rayonnement solaire, les plantes expérimentent un stress thermique excessif : les enzymes de la photosynthèse se dénaturent, l'eau s'évapore des stomates avant d'être utilisée, et la productivité primaire s'effondre. Sans photosynthèse, l'oxygène atmosphérique (actuellement 21%) s'échappe lentement vers l'espace, et le CO2 s'accumule. Toute vie complexe dépendant de l'oxygène meurt. Seules les bactéries chimiotrophes survivent dans les profondeurs géothermales. C'est la fin du règne de la vie visible sur Terre.</t>
         </is>
       </c>
-      <c r="G290" s="20" t="inlineStr"/>
+      <c r="G290" s="20" t="inlineStr">
+        <is>
+          <t>La photosynthèse est déjà, aujourd'hui, la source d'énergie ultime de presque toutes les chaînes alimentaires de la planète, y compris des combustibles fossiles — sa disparition ne priverait donc pas seulement les plantes d'énergie, mais quasiment toute forme de vie à la fois.</t>
+        </is>
+      </c>
       <c r="H290" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12682,7 +12854,11 @@
           <t>Selon la théorie du rayonnement Hawking proposée par le physicien Stephen Hawking en 1974 et confirmée par la physique quantique moderne, tous les trous noirs s'évaporent lentement via l'émission de rayonnement Hawking. Plus un trou noir est petit, plus vite il s'évapore. Un trou noir de la masse du Soleil mettrait environ 10^67 années pour s'évaporer complètement (bien au-delà de l'âge actuel de l'univers de 13,8 milliards d'années). Cependant, les trous noirs stellaires de masse intermédiaire (100 à 10 000 masses solaires) s'évaporent plus rapidement : en environ 10^10 à 10^20 années. À l'échelle de 10^12 années, de nombreux petits trous noirs et trous noirs primordiaux auraient déjà disparu via l'évaporation Hawking. Les trous noirs supermassifs (millions de masses solaires) au cœur des galaxies persisteraient bien au-delà, mais les trous noirs stellaires intermédiaires auraient probablement évaporé. Cette évaporation libère l'énergie accumulée sous forme de rayonnement énergétique, se terminant progressivement en une explosion de rayons gamma. Les trous noirs, bien que parmi les objets les plus stables du cosmos, ne sont pas éternels. C'est une des rares preuves que l'univers tend vers l'équilibre (entropie maximale).</t>
         </is>
       </c>
-      <c r="G291" s="20" t="inlineStr"/>
+      <c r="G291" s="20" t="inlineStr">
+        <is>
+          <t>Stephen Hawking a proposé le rayonnement des trous noirs en 1974 précisément parce qu'il semblait violer une règle fondamentale de la physique (l'information ne peut pas être détruite) — le « paradoxe de l'information » qui en découle reste l'un des plus grands problèmes non résolus de la physique théorique.</t>
+        </is>
+      </c>
       <c r="H291" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12717,7 +12893,11 @@
           <t>À cette phase extrêmement lointaine, le cosmos aura radicalement changé. Toutes les étoiles auront brûlé leur carburant et explosé (dans les premières 10^14 années). Tous les trous noirs stellaires et trous noirs de masse intermédiaire auront évaporé via le rayonnement Hawking. Les trous noirs supermassifs au cœur des galaxies (de millions à milliards de masses solaires) seraient les derniers objets massifs de l'univers. À 10^30 années, seuls ces trous noirs géants subsisteraient, s'évaporant très lentement via le rayonnement Hawking (un trou noir d'1 milliard de masses solaires met environ 10^100 années à s'évaporer complètement). L'univers serait dominé par une soupe de photons primaires, neutrinos, et les radiations d'évaporation des trous noirs résiduels. La densité d'énergie serait incroyablement faible. Les températures seraient proches du zéro absolu. L'expansion de l'univers aurait dilué toute matière ordinaire à des distances incompréhensiblement grandes. C'est l'ère des trous noirs : l'avant-dernier acte de l'univers avant sa mort thermique complète.</t>
         </is>
       </c>
-      <c r="G292" s="20" t="inlineStr"/>
+      <c r="G292" s="20" t="inlineStr">
+        <is>
+          <t>À ce stade, un unique trou noir supermassif comme celui au centre de notre galaxie mettrait à lui seul environ 10^100 années à s'évaporer complètement — les trous noirs, même les plus « rapides », domineront donc l'univers pendant une durée presque incompréhensiblement plus longue que toute son histoire actuelle.</t>
+        </is>
+      </c>
       <c r="H292" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12752,7 +12932,11 @@
           <t>À cette échelle de temps incompréhensiblement lointaine (10^100 années, un nombre avec 100 zéros), le destin final de l'univers se réalise selon la deuxième loi de la thermodynamique : l'entropie augmente inexorablement vers un maximum. C'est la mort thermique ou "Big Freeze" de l'univers. À ce stade, tous les trous noirs auront évaporé. Toute énergie libre aura été convertie en rayonnement diffus. L'univers atteindrait un état d'équilibre thermique parfait : une température uniforme infinitésimale (proche du zéro absolu, ~10^-30 Kelvin). Aucun gradient d'énergie n'existerait. Aucun travail ne pourrait être fait. Aucune structure n'existerait. Pas de vie, pas de conscience, pas même de chimie. Juste des particules élémentaires infinitésimalement diluées, incapables d'interaction. Le temps lui-même deviendrait thermodynamiquement sans sens : sans processus, il n'existe pas de flèche du temps. C'est la fin absolue et définitive. Cet état est le dernier possible selon nos compréhensions actuelles de la physique. L'univers, issu du Big Bang il y a 13,8 milliards d'années, aura duré environ 10^120 fois plus longtemps qu'il n'a existé jusqu'à présent. C'est le destin entropique inévitable de toute réalité physique.</t>
         </is>
       </c>
-      <c r="G293" s="20" t="inlineStr"/>
+      <c r="G293" s="20" t="inlineStr">
+        <is>
+          <t>Le nombre 10^100 porte un nom : le « gogol », inventé en 1920 par Milton Sirotta, neveu âgé de 9 ans du mathématicien Edward Kasner, à qui ce dernier avait demandé de nommer un très grand nombre. Le mot a plus tard inspiré le nom de l'entreprise Google.</t>
+        </is>
+      </c>
       <c r="H293" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12787,7 +12971,11 @@
           <t>Il y a 3,8 milliards d'années, dans les océans primitifs de la Terre jeune, les premières formes de vie apparaissent : des bactéries simples, unicellulaires, sans noyau (procaryotes). Ces organismes sont tellement microscopiques qu'on ne peut les voir qu'au microscope. Elles vivent dans l'eau chaude des océans, se nourrissant de minéraux et d'énergie chimique provenant des cheminées hydrothermales sous-marines. Ces bactéries primitives créent progressivement des structures rocheuses en couches appelées "stromatolites" : ce sont les fossiles les plus anciens découverts sur Terre. Les stromatolites sont formés par l'accumulation de bactéries mortes et de sédiments, créant des dômes rocheux caractéristiques. Ces premières créatures n'ont pas besoin d'oxygène pour vivre (elles sont anaérobies). Elles se reproduisent en se divisant simplement en deux, transmettant leur matériel génétique (ADN) à leurs descendants. Cette apparition marque le début de la vie sur Terre et le début de l'évolution biologique : pendant les 3,8 milliards d'années suivantes, toutes les formes de vie complexes descendront de ces bactéries microscopiques. Sans cette étape, aucun animal, aucune plante, aucun humain n'existerait.</t>
         </is>
       </c>
-      <c r="G294" s="20" t="inlineStr"/>
+      <c r="G294" s="20" t="inlineStr">
+        <is>
+          <t>Des stromatolites vivants existent encore aujourd'hui dans quelques rares lieux extrêmement salés, notamment la baie Shark en Australie — il est donc possible d'observer en temps réel des structures bâties par des organismes proches des toutes premières formes de vie terrestres.</t>
+        </is>
+      </c>
       <c r="H294" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12822,7 +13010,11 @@
           <t>Il y a 2,7 milliards d'années, un événement gigantesque transforme la Terre : la "Grande Oxydation". Pendant 1,1 milliard d'années avant cela, les bactéries photosynthétiques (cyanobactéries) produisent lentement de l'oxygène en convertissant la lumière solaire en énergie chimique. Cet oxygène était d'abord consommé par des minéraux de fer dissous dans l'océan, créant les "formations de fer rubanées" (bandes alternées de fer et de roche). Mais à partir de 2,7 milliards d'années, l'oxygène s'accumule plus vite qu'il n'est consommé. Il s'échappe dans l'atmosphère, passant de presque 0% à environ 1% de l'atmosphère. Pour les bactéries anaérobies dominantes à cette époque, c'est une catastrophe : l'oxygène est un poison qui tue leurs cellules. Cet événement provoque la plus grande extinction de masse de l'histoire de la vie : 99% de la vie anaérobie disparaît. Seules survivent les bactéries capables d'utiliser l'oxygène pour respirer et produire plus d'énergie. Mais cette catastrophe crée aussi une opportunité : avec l'oxygène, les cellules peuvent respirer plus efficacement et accumuler plus d'énergie. Cela permettra l'apparition d'organismes plus grands et plus complexes. Sans la Grande Oxydation, les animaux et plantes complexes n'auraient jamais pu émerger.</t>
         </is>
       </c>
-      <c r="G295" s="20" t="inlineStr"/>
+      <c r="G295" s="20" t="inlineStr">
+        <is>
+          <t>Comme l'oxygène était toxique pour presque toute forme de vie de l'époque, certains scientifiques surnomment cet événement la « catastrophe de l'oxygène » : il pourrait s'agir, en proportion d'espèces disparues, de la plus grande extinction de masse de l'histoire de la Terre, bien qu'elle soit largement absente des récits populaires sur les extinctions.</t>
+        </is>
+      </c>
       <c r="H295" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12857,7 +13049,11 @@
           <t>Il y a 1,2 milliard d'années, une révolution silencieuse transforme la vie microscopique : l'apparition des cellules eucaryotes. Jusqu'à ce moment, toute la vie consiste en bactéries procaryotes : une simple goutte de cytoplasme avec de l'ADN flottant librement au centre. Soudain, certaines bactéries développent une membrane interne entourant leur ADN, créant une structure appelée "noyau". C'est comme si la cellule construisait une chambre de coffre-fort pour protéger ses gènes. Comment ? Les scientifiques pensent qu'une bactérie a avalé une autre bactérie, mais au lieu de la digérer, elles ont fusionné. C'est l'endosymbiose : une fusion bactérienne. Ces nouvelles cellules eucaryotes sont beaucoup plus grandes et plus complexes. Elles développent aussi des organelles : mitochondries (centrales électriques cellulaires), chloroplastes (panneaux solaires biologiques), réticulum endoplasmique (système de transport interne). Avec cette organisation interne, les cellules peuvent accumuler beaucoup plus d'énergie. Elles peuvent aussi se combiner pour former des organismes multicellulaires : les premiers protistes apparaissent (algues microscopiques). Ces cellules eucaryotes sont nos ancêtres directs. Sans cette évolution cellulaire, les plantes, les animaux, les champignons et les humains n'existeraient jamais.</t>
         </is>
       </c>
-      <c r="G296" s="20" t="inlineStr"/>
+      <c r="G296" s="20" t="inlineStr">
+        <is>
+          <t>Les mitochondries, les « centrales énergétiques » de nos cellules, possèdent encore aujourd'hui leur propre petit ADN séparé — une empreinte génétique héritée des bactéries libres dont elles seraient issues, avant d'être absorbées par une cellule plus grande.</t>
+        </is>
+      </c>
       <c r="H296" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12892,7 +13088,11 @@
           <t>Il y a 600 millions d'années, quelque chose d'extraordinaire se produit dans les océans : l'Explosion cambrienne. Pendant plus de 3 milliards d'années, la vie était dominée par des organismes microscopiques et quelques créatures molles et sans couleur. Puis, en quelques millions d'années seulement (un clin d'œil géologique), des centaines de nouvelles formes de vie complexes et bizarres émergent soudainement. Les fossiles montrent des trilobites (créatures blindées avec des yeux), des échinodermes (ancêtres des étoiles de mer), des mollusques (ancêtres des poulpes), des arthropodes (ancêtres des insectes et araignées). Pourquoi soudainement ? Les scientifiques pensent que plusieurs facteurs convergent : l'oxygène atmosphérique atteint finalement des niveaux suffisants pour supporter des animaux complexes. Les océans refroidissent légèrement après une ère glaciaire. Une mutation génétique majeure (gènes Hox) permet une plus grande variabilité corporelle. La compétition apparaît : les prédateurs apparaissent et forcent les proies à évoluer rapidement pour survivre. C'est une "course aux armements" biologique. Ces animaux cambriens sont nos ancêtres : leur diversité de corps et de stratégies de survie crée les plans de base de tous les animaux futurs. Les humains et tous les animaux terrestres descendent des survivants de cette explosion créative.</t>
         </is>
       </c>
-      <c r="G297" s="20" t="inlineStr"/>
+      <c r="G297" s="20" t="inlineStr">
+        <is>
+          <t>L'un des plus célèbres gisements fossiles de cette période, le Schiste de Burgess au Canada, conserve des détails de tissus mous si exceptionnels que certains animaux y étaient si étranges que les paléontologues les ont d'abord reconstitués à l'envers ou en marche arrière.</t>
+        </is>
+      </c>
       <c r="H297" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12927,7 +13127,11 @@
           <t>Il y a 500 millions d'années, dans les océans du Silurien, les premiers poissons apparaissent : les Ostracodermes. Ces créatures ressemblent à des petits têtards blindés, longues de quelques centimètres. Contrairement aux autres animaux marins, ils possèdent une innovation révolutionnaire : un squelette primitif fait de cartilage (comme celui des requins modernes) au lieu d'exosquelette externe. Mieux encore, ce squelette contient une moelle épinière et un cerveau primitif. C'est la naissance des vertébrés : le groupe auquel nous appartenons. Les Ostracodermes n'ont pas de mâchoires mobiles (ils aspirent leur nourriture), pas de nageoires paires, juste une bouche fixe. Mais ils sont efficaces : petit à petit, d'autres innovations apparaissent. Certains Ostracodermes développent des mâchoires flexibles, permettant une meilleure capture de nourriture. Certains développent des nageoires paires pour mieux contrôler leur mouvement dans l'eau. Sur des millions d'années, ces améliorations créent les poissons modernes : les placodermes (poissons à plaques osseuses), les chondrichthyens (requins et raies), puis les ostéichthyens (poissons osseux). Les humains sont des descendants très éloignés de ces premiers poissons : nos bras, nos jambes, notre crâne, notre colonne vertébrale viennent de cette lignée aquatique ancienne.</t>
         </is>
       </c>
-      <c r="G298" s="20" t="inlineStr"/>
+      <c r="G298" s="20" t="inlineStr">
+        <is>
+          <t>Ces poissons sans mâchoire n'avaient aucun moyen de mordre : ils se nourrissaient probablement en filtrant ou en aspirant leur nourriture sur le fond marin. Les mâchoires n'apparaîtront chez les vertébrés que des dizaines de millions d'années plus tard, formées à partir des mêmes os qui soutenaient autrefois les branchies.</t>
+        </is>
+      </c>
       <c r="H298" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12962,7 +13166,11 @@
           <t>Il y a 475 millions d'années, les continents sont totalement déserts : des roches nues sous un ciel sans couleur. Les plantes vivent uniquement dans l'océan. Puis, les premières plantes aquatiques découvrent comment survivre sur la terre sèche : les bryophytes primitives (ancêtres des mousses et hépatiques modernes). Comment ? Ces plantes développent plusieurs adaptations géniales. D'abord, un système de racines primitif qui s'enfonce dans le sol pour absorber l'eau et les nutriments minéraux. Ensuite, une cuticule cireuse sur la surface qui réduit l'évaporation : sans cette protection, la plante se dessécherait instantanément au contact de l'air. Troisièmement, un système de transport interne (vaisseaux) qui propage l'eau des racines aux feuilles. Enfin, des spores plutôt que des œufs pour se reproduire : les spores sont minuscules, légères, et peuvent voyager dans le vent sur de longues distances. Ces premières plantes sont minuscules, juste quelques centimètres, sans feuilles véritables, ressemblant à des mousses. Mais elles sont révolutionnaires. Elles transforment les roches nues en sol : leurs racines fracturent la roche, créant du terreau. Elles produisent de l'oxygène, modifiant l'atmosphère. Elles créent des habitats. Sur les millions d'années suivants, les plantes évoluent : des fougères plus grandes apparaissent (avec de vraies racines profondes), puis des plantes à graines, puis des fleurs. Sans cette colonisation terrestre, les animaux terrestres et les humains ne pourraient jamais exister.</t>
         </is>
       </c>
-      <c r="G299" s="20" t="inlineStr"/>
+      <c r="G299" s="20" t="inlineStr">
+        <is>
+          <t>Avant la colonisation végétale des terres, les continents ressemblaient sans doute davantage à Mars qu'à la Terre actuelle : de la roche et des sédiments nus, sans le moindre sol, celui-ci étant en grande partie le produit des racines des plantes qui fragmentent la pierre au fil des millions d'années.</t>
+        </is>
+      </c>
       <c r="H299" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -12997,7 +13205,11 @@
           <t>Il y a 360 millions d'années, quelque chose d'extraordinaire se produit dans les marécages et rivières du Carbonifère : les poissons développent des pattes et quittent l'eau. Ce sont les premiers amphibiens, comme le Tiktaalik et l'Ichthyostega. Comment des poissons deviennent-ils des créatures terrestres ? La clé est la nageoire : les nageoires paires des poissons (pectorales et pelviennes) évoluent progressivement en membres articulés (bras et jambes) avec os, articulations et muscles. Ces amphibiens primitifs gardent encore des caractéristiques de poisson : une queue aplatie pour nager, des branchies pour respirer sous l'eau. Mais ils développent aussi des poumons pour respirer l'air. Leurs nageoires deviennent de vraies pattes assez fortes pour supporter leur poids et les propulser sur la terre. Pourquoi quitter l'eau ? L'eau stagnante des marécages manque d'oxygène. Les amphibiens capables de ramper sur la terre et respirer l'air à la surface ont un avantage de survie énorme. Sur terre, ils découvrent un monde vierge rempli de nourriture (plantes, insectes) et sans prédateurs. Mais les premiers amphibiens restent dépendants de l'eau : ils doivent y retourner pour se reproduire, comme les grenouilles modernes. Sur les 100 millions d'années suivantes, certains amphibiens évoluent pour s'adapter à la vie terrestre complète. Ils développent une peau imperméable, des œufs avec coquille (pas besoin de l'eau pour la reproduction). Ce sont les reptiles. Et les humains, comme tous les mammifères terrestres, descendons de ces amphibiens intrépides qui ont osé explorer la terre.</t>
         </is>
       </c>
-      <c r="G300" s="20" t="inlineStr"/>
+      <c r="G300" s="20" t="inlineStr">
+        <is>
+          <t>Le célèbre fossile de transition Tiktaalik, découvert dans l'Arctique canadien en 2004, a été surnommé le « poisson-pattes » (fishapod) car il combine écailles et branchies de poisson avec un cou flexible et des ébauches de poignets utiles pour se déplacer sur la terre ferme.</t>
+        </is>
+      </c>
       <c r="H300" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13032,7 +13244,11 @@
           <t>Il y a 320 millions d'années, un événement biologique majeur transforme l'évolution terrestre : l'apparition des premiers vrais reptiles. Leur innovation clé ? L'œuf amniotique : un œuf avec une coquille imperméable contenant une poche d'eau (l'amnios) qui protège l'embryon. Pourquoi est-ce révolutionnaire ? Les amphibiens doivent retourner à l'eau pour pondre car leurs œufs sont mous et se déssèchent rapidement au soleil. Les reptiles, avec leur coquille dure, peuvent pondre loin de l'eau, sur la terre ferme. Cela signifie : indépendance totale de l'eau pour la reproduction. Plus besoin de revenir à l'eau chaque saison de reproduction. Les premiers reptiles amniotes ressemblent à des lézards, longs de quelques décimètres. Ils développent aussi une peau écailleuse imperméable qui retient l'eau, contrairement à la peau humide des amphibiens. Leurs pattes deviennent plus fortes, supportant leur corps de manière plus verticale. Ces adaptations les rendent extrêmement efficaces sur terre. Sur les 50 millions d'années suivantes, les reptiles se diversifient explosivement : certains deviennent énormes (les dinosaures), d'autres développent des ailes (les ptérosaures et oiseaux), d'autres une apparence mammalienne (les synapsides). Les reptiles dominent tous les écosystèmes terrestres pendant 250 millions d'années. Les humains descendons d'une lignée de petits reptiles synapsidés qui survivent à plusieurs extinctions de masse et finissent par devenir les mammifères.</t>
         </is>
       </c>
-      <c r="G301" s="20" t="inlineStr"/>
+      <c r="G301" s="20" t="inlineStr">
+        <is>
+          <t>L'œuf amniotique est parfois décrit comme l'une des grandes « inventions de survie » de l'évolution : ses membranes gèrent si bien les échanges gazeux, les déchets et l'humidité que ce même principe, à peine modifié, équipe encore tous les reptiles et tous les oiseaux actuels.</t>
+        </is>
+      </c>
       <c r="H301" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13067,7 +13283,11 @@
           <t>Il y a 300 millions d'années, dans les marécages du Carbonifère, apparaissent les synapsides : une lignée de reptiles qui semble ordinaire au premier abord. Les synapsides ressemblent à des reptiles normaux, ressemblant à des petits lézards ou à des pelycosaures (reptiles à voile de cheveux sur le dos). Mais ils possèdent une caractéristique unique : une fenêtre osseuse sur chaque côté du crâne (la fenêtre temporale), d'où s'attachent des muscles mâchoires puissants. Pourquoi est-ce important ? Ces muscles mâchoires permettent une morsure plus puissante et une meilleure mastication. Au cours des 100 millions d'années suivantes, les synapsides évoluent lentement mais sûrement vers quelque chose de plus étrange. Certains développent une posture de pattes plus verticale (sous le corps) plutôt qu'écartées sur les côtés comme les reptiles. Certains développent des dents différenciées : des incisives pour trancher, des canines pointues pour percer, des molaires pour broyer. C'est très différent des reptiles qui ont des dents uniformes. Certains développent une seule fenêtre osseuse supérieure au crâne plutôt que deux. Ces changements graduels transforment lentement les synapsides en quelque chose de nouveau : les cynodontes. Et les cynodontes, après 50 millions d'années d'évolution supplémentaire, deviendront les premiers mammifères vrais. Chaque humain vivant descend directement de ces synapsides apparemment ordinaires du Carbonifère.</t>
         </is>
       </c>
-      <c r="G302" s="20" t="inlineStr"/>
+      <c r="G302" s="20" t="inlineStr">
+        <is>
+          <t>La caractéristique qui définit les synapsides — un unique orifice derrière chaque orbite oculaire pour les muscles de la mâchoire — est précisément celle que les paléontologues utilisent pour retracer une lignée ininterrompue depuis ces animaux du Carbonifère jusqu'à l'humain actuel.</t>
+        </is>
+      </c>
       <c r="H302" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13102,7 +13322,11 @@
           <t>Il y a 250 millions d'années, c'est l'apocalypse biologique : l'Extinction du Permien, aussi appelée "la Grande Mort" (The Great Dying). C'est la pire extinction de masse dans toute l'histoire de la vie. Les chiffres sont terrifiants : 95% de toutes les espèces marines disparaissent. 70% de toutes les espèces de vertébrés terrestres disparaissent. Seules quelques espèces survivent et repeuplent le monde ensuite. Qu'est-ce qui cause ce cataclysme ? Les scientifiques déterminent plusieurs causes qui convergeaient à la même époque. D'abord, le "trappage sibérien" : dans la région de la Sibérie, d'énormes éruptions volcaniques massives se produisent pendant des milliers d'années. Ces volcans libèrent des millions de tonnes de cendres volcaniques, d'acide sulfurique, et surtout du dioxyde de carbone. Le CO2 crée un effet de serre massif : les températures mondiales augmentent de 5 à 10 degrés Celsius. Les océans se réchauffent dangereusement. Les zones côtières produisent moins d'oxygène. Les niveaux marins baissent. Les écosystèmes marins s'effondrent. De plus, les cendres volcaniques bloquent le soleil, tuant les plantes et créant une famine. Les animaux qui survivent sont ceux qui peuvent jeûner longtemps, tolérer les températures extrêmes, et s'adapter rapidement aux nouvelles conditions. Les synapsides survivent à cette extinction mieux que les autres reptiles. Après cet événement catastrophique, le monde est vide. Les synapsides survivants se diversifient rapidement pour remplir tous les rôles écologiques laissés vacants. Cet "reset" écologique crée les opportunités pour que les cynodontes (descendants synapsides) évoluent ensuite en mammifères. Sans cette extinction terrifiante, les dinosaures, pas les synapsides, auraient dominé le monde, et les mammifères n'auraient jamais existé.</t>
         </is>
       </c>
-      <c r="G303" s="20" t="inlineStr"/>
+      <c r="G303" s="20" t="inlineStr">
+        <is>
+          <t>L'extinction du Permien a été si sévère qu'elle est la seule des « cinq grandes » extinctions de masse à avoir sérieusement touché les insectes, un groupe pourtant réputé pour sa remarquable résistance à l'extinction tout au long de l'histoire de la Terre.</t>
+        </is>
+      </c>
       <c r="H303" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13137,7 +13361,11 @@
           <t>Il y a 220 millions d'années, au moment où les dinosaures commencent à dominer la Terre, un groupe de petits reptiles abandonne la compétition directe et se cache : les premiers mammifères. Ces créatures, comme le Morganucodon et l'Hadrocodium, sont minuscules : longues de seulement 10 à 30 centimètres, pesant quelques grammes, ressemblant à de petites musaraignes. Elles sont timides, nocturnes, se cachant sous terre et dans les arbres pendant le jour, sortant la nuit chercher nourriture. Pourquoi sont-elles "mammifères" ? Elles possèdent des caractéristiques que seuls les mammifères ont. D'abord, un crâne spécialisé avec une fenêtre osseuse pour les muscles mâchoires (héritage des synapsides). Deuxièmement, des dents différenciées : incisives, canines, molaires, permettant une mastication efficace. Troisièmement, trois os d'oreille interne (marteau, enclume, étrier) plutôt que les os de mâchoire de reptiles. Quatrièmement, un palais dur qui sépare la bouche de la respiration, permettant une respiration continue pendant la mastication. Ces adaptations rendent les premiers mammifères extrêmement efficaces pour chasser de petites proies (insectes, petits lézards) la nuit. Pendant 140 millions d'années, les mammifères restent petits et rares, toujours éclipsés par les dinosaures dominants. Mais quand les dinosaures s'éteignent soudainement (extinction K-T, il y a 66 millions d'années), les mammifères survivants évoluent rapidement pour remplir tous les rôles écologiques laissés vacants. Sans cette période d'évolution cachée, les mammifères ne seraient jamais devenus les créatures dominantes du monde actuel, et les humains n'existeraient pas.</t>
         </is>
       </c>
-      <c r="G304" s="20" t="inlineStr"/>
+      <c r="G304" s="20" t="inlineStr">
+        <is>
+          <t>Pendant environ 140 millions d'années — toute la durée du règne des dinosaures — les mammifères sont restés presque exclusivement petits et nocturnes, guère plus gros qu'une musaraigne actuelle, probablement pour éviter la concurrence et la prédation des reptiles qui dominaient le jour.</t>
+        </is>
+      </c>
       <c r="H304" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13172,7 +13400,11 @@
           <t>Il y a 1,5 million d'années, dans les vallées d'Afrique de l'Est (Éthiopie, Kenya), le Homo erectus franchit un cap extraordinaire : maîtriser le feu. Ce n'est pas qu'il découvre soudainement le feu. Les hominidés antérieurs (Homo habilis) ont probablement utilisé le feu naturel (provenant des éruptions volcaniques ou éclairs) occasionnellement. Mais Homo erectus fait quelque chose de révolutionnaire : il apprend à créer le feu intentionnellement et à le maintenir allumé. Comment ? En frappant des roches de silex contre du granit pour produire des étincelles, ou en frottant du bois pour créer de la chaleur. Pourquoi c'est révolutionnaire ? Le feu change absolument tout. D'abord, nutrition : la cuisson tue les bactéries dangereuses et les parasites dans la viande et les plantes. Elle rend aussi la nourriture plus facile à digérer, ce qui signifie que le corps absorbe plus de nutriments avec moins d'effort. Cela libère de l'énergie pour d'autres fonctions, notamment le cerveau. Deuxièmement, survie : le feu tient chaud, crucial pour les humains qui perdent rapidement la chaleur corporelle. Il repousse les prédateurs la nuit. Troisièmement, socialité : le feu rassemble les gens. Assis autour du feu, les humains commencent à socialiser, parler, raconter des histoires, enseigner aux enfants. C'est probablement quand le langage devient plus complexe. Quatrièmement, technologie : le feu peut être utilisé pour travailler le bois, la pierre, l'os. Il rend possible des outils plus sophistiqués. Avec le feu, Homo erectus peut migrer vers des régions froides (Europe du Nord, Asie). Pendant environ 1 million d'années, Homo erectus utilise le feu, se propageant à travers le monde. Ses descendants (Homo neanderthalensis, Homo sapiens) héritent de cette technologie révolutionnaire et la raffinent encore plus. Sans la maîtrise du feu, le cerveau humain ne se serait jamais aussi développé, et la civilisation n'existerait pas.</t>
         </is>
       </c>
-      <c r="G305" s="20" t="inlineStr"/>
+      <c r="G305" s="20" t="inlineStr">
+        <is>
+          <t>Selon « l'hypothèse de la cuisson » du primatologue Richard Wrangham, la digestion facilitée par les aliments cuits aurait libéré tellement d'énergie métabolique qu'elle aurait directement permis la croissance spectaculaire du cerveau humain — le feu pourrait donc être, en partie, la raison pour laquelle nous pensons comme nous le faisons.</t>
+        </is>
+      </c>
       <c r="H305" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13207,7 +13439,11 @@
           <t>Il y a 500 000 ans, une créature appelée Homo heidelbergensis vit en Afrique, en Europe et en Asie. C'est un individu fascinant qui représente une étape critique de l'évolution humaine. Homo heidelbergensis est plus grand et plus robuste que Homo erectus (taille humaine, poids 70-90 kg). Son crâne est plus grand avec un volume cérébral de 1200-1400 centimètres cubes (comparable aux humains modernes). Ses os sont plus épais, ses muscles plus puissants. Qu'est-ce qui le rend spécial ? Les données génétiques et fossiles suggèrent qu'Homo heidelbergensis est probablement l'ancêtre commun de deux espèces humaines différentes qui évoluent ensuite séparément. En Europe, où le climat devient très froid, Homo heidelbergensis évolue en Homo neanderthalensis (les Néandertaliens), avec des corps plus courts et trapus, adaptés au froid. En Afrique, où le climat reste chaud, Homo heidelbergensis évolue en Homo sapiens (nous), avec des corps plus longs et gracieux. Homo heidelbergensis lui-même est un chasseur efficace. Les preuves archéologiques montrent qu'il fabrique des bifaces (outils de pierre bifaciales) sophistiqués appelés "coups de poing" (hand axes). Il chasse probablement des animaux de grande taille en groupes coordonnés, nécessitant une communication complexe et une planification. Son cerveau suffisamment grand suggère qu'il possède un langage et une capacité à enseigner. C'est probablement la première espèce humaine avec une véritable culture transmissible. Homo heidelbergensis disparaît il y a environ 300 000 ans, remplacé par ses descendants plus spécialisés (Néandertal et Sapiens). Mais sans Homo heidelbergensis, ces deux branches distinctes d'humanité n'auraient jamais émergé.</t>
         </is>
       </c>
-      <c r="G306" s="20" t="inlineStr"/>
+      <c r="G306" s="20" t="inlineStr">
+        <is>
+          <t>Homo heidelbergensis doit son nom à une mâchoire découverte près de Heidelberg, en Allemagne, en 1907, par un ouvrier de carrière — un fossile toujours considéré comme l'une des pièces clés de l'arbre généalogique humain.</t>
+        </is>
+      </c>
       <c r="H306" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13242,7 +13478,11 @@
           <t>Il y a 430 000 ans, dans les grottes et vallées de l'Europe, une nouvelle espèce humaine émerge : Homo neanderthalensis, que nous appelons les Néandertaliens. Ils évoluent à partir d'Homo heidelbergensis pendant une période de glaciation intense. Le climat européen devient beaucoup plus froid et inhospitalier. Homo neanderthalensis développe une morphologie extrêmement bien adaptée au froid : corps trapus et robustes (plus courts mais plus lourds que Homo sapiens), crâne plus grand avec un cerveau légèrement plus gros que le nôtre (1450-1600 cm³ contre 1400 pour Sapiens). Leur corps trapu minimise la perte de chaleur (surface/volume réduit). Leurs extrémités (doigts, orteils, nez) sont plus courtes pour réduire la gelure. Leurs muscles sont massifs, leur densité osseuse très élevée, les rendant extrêmement forts (environ 20% plus forts qu'un humain moderne). Ils développent des outils de pierre raffinés appelés "industries moustériennes" : des racloirs, des lames, des pointes de lance pour chasser les mégafaunes (mammouths, bisons, rennes). Les preuves archéologiques suggèrent qu'ils vivent en petits groupes, chassent en coordonnés (nécessitant communication complexe), et ont peut-être un langage sophistiqué. Certaines preuves indiquent qu'ils prennent soin de leurs malades et blessés, et qu'ils enterrent leurs morts avec des rituels, suggérant une conscience de la mort et possiblement une spiritualité. Les Néandertaliens prospèrent en Europe et en Asie occidentale pendant environ 200 000 ans. Mais quand Homo sapiens arrive d'Afrique il y a 40 000 ans, mieux adapté aux changements climatiques rapides, les Néandertaliens entrent en déclin et disparaissent il y a environ 30 000 ans. Ironiquement, ils ne disparaissent pas complètement : environ 1-4% du génome de tous les humains non-africains contient de l'ADN néandertalien.</t>
         </is>
       </c>
-      <c r="G307" s="20" t="inlineStr"/>
+      <c r="G307" s="20" t="inlineStr">
+        <is>
+          <t>Les Néandertaliens avaient en moyenne un cerveau légèrement plus volumineux que celui des humains modernes, bien que de forme différente — plus allongé d'avant en arrière plutôt qu'arrondi — une différence dont la signification cognitive fait encore débat parmi les chercheurs.</t>
+        </is>
+      </c>
       <c r="H307" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13277,7 +13517,11 @@
           <t>Il y a 300 000 ans, quelque part en Afrique subsaharienne (probablement en Afrique du Sud et de l'Est), une nouvelle espèce humaine émerge : Homo sapiens archaïque. C'est nous, ou plutôt, ce sont nos ancêtres les plus directs. Les fossiles montrent une transition progressive depuis Homo heidelbergensis. Les changements majeurs : d'abord, le crâne s'aplatit. Chez Homo erectus et Homo heidelbergensis, le front fuit vers l'arrière et il y a un bourrelet proéminent au-dessus des yeux. Chez Homo sapiens, le front devient vertical, donnant du style à un menton (unique aux humains modernes). Deuxièmement, la face devient plus petite et gracile plutôt que robuste. Troisièmement, le cerveau se réorganise : la partie frontale s'agrandit (pensée abstraite, langage, planification), tandis que l'occipital s'arrondit. Homo sapiens archaïque (300 000 à 100 000 ans) n'est pas encore complètement "moderne" mais s'en rapproche. Ils fabriquent des outils de pierre sophistiqués, chassent efficacement et cuisent leur nourriture avec le feu depuis longtemps. Vers 200 000 ans, certains fossiles montrent les caractéristiques entièrement "modernes" : crâne arrondi, petite face, menton proéminent. C'est Homo sapiens moderne. Entre 100 000 et 70 000 ans, des groupes de Homo sapiens modernes commencent à quitter l'Afrique pour explorer le Moyen-Orient, puis l'Europe, l'Asie, l'Océanie : c'est la "Grande Migration" qui peuplera tous les continents. Sans cette émergence en Afrique, la branche Sapiens de l'humanité n'existerait pas.</t>
         </is>
       </c>
-      <c r="G308" s="20" t="inlineStr"/>
+      <c r="G308" s="20" t="inlineStr">
+        <is>
+          <t>Les plus anciens fossiles connus d'Homo sapiens, découverts à Jebel Irhoud au Maroc et datés d'environ 300 000 ans, ont repoussé de 100 000 ans l'origine admise de notre espèce par rapport à ce que l'on pensait encore une décennie plus tôt — un rappel que cette chronologie continue d'être révisée à chaque nouvelle découverte.</t>
+        </is>
+      </c>
       <c r="H308" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13312,7 +13556,11 @@
           <t>Il y a 280 000 ans, les Néandertaliens atteignent leur apogée en termes de population, de distribution géographique, et de sophistication technologique. À ce moment, environ 100 000 à 500 000 Néandertaliens vivent en Europe, Asie mineure, et Asie occidentale (du Portugal à la Sibérie). Ils maîtrisent une vaste gamme de technologies de chasse. L'industrie moustérienne (la technologie principale) produit des dizaines de types d'outils : des racloirs pour enlever la peau des animaux, des lames pointues pour découper la viande, des pointes de lance pour la chasse. La technique dite "Levallois" permet de préparer une pierre pour produire des lames pré-définies : un savoir-faire nécessitant apprentissage long et communication sophistiquée, probablement un véritable langage parlé. Les preuves archéologiques montrent qu'ils vivent en groupes d'environ 20-30 individus, chassant des mégafaunes (mammouths, rhinos laineux, bisons, chevaux) souvent en groupe coordonné. Les fossiles montrent des traumatismes similaires à ceux de cavaliers de rodéo, indiquant une chasse au corps à corps dangereuse mais productive. Certaines preuves fossiles suggèrent qu'ils s'occupent de membres blessés : un fossile montre un Néandertal ayant survécu des années avec un bras amputé, impossible sans l'aide du groupe, indiquant empathie et cohésion sociale. Des sites archéologiques montrent des restes de fleurs autour de squelettes, suggérant des sépultures rituelles. À cet apogée, les Néandertaliens semblent être une espèce entièrement intelligente et culturellement sophistiquée. Mais cette apogée est aussi le début du déclin : vers 50 000 ans, le climat change et Homo sapiens arrive d'Afrique, plus flexible et adaptatif. Les Néandertaliens déclinent lentement et le dernier disparaît il y a environ 30 000 ans.</t>
         </is>
       </c>
-      <c r="G309" s="20" t="inlineStr"/>
+      <c r="G309" s="20" t="inlineStr">
+        <is>
+          <t>Un squelette de Néandertalien découvert dans la grotte de Shanidar, en Irak, montre qu'il a survécu des années après avoir perdu un bras et être devenu sourd et en partie aveugle — des blessures qui auraient été fatales sans les soins prolongés de son groupe, l'un des plus anciens témoignages connus de compassion dans la lignée humaine.</t>
+        </is>
+      </c>
       <c r="H309" s="20" t="inlineStr">
         <is>
           <t>Avéré</t>
@@ -13321,494 +13569,550 @@
       <c r="I309" s="20" t="inlineStr"/>
     </row>
     <row r="310">
-      <c r="A310" t="n">
+      <c r="A310" s="20" t="n">
         <v>309</v>
       </c>
-      <c r="B310" t="inlineStr">
+      <c r="B310" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Anthropologie</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr">
+      <c r="C310" s="20" t="inlineStr">
         <is>
           <t>Première vague de migration de Sapiens hors d'Afrique</t>
         </is>
       </c>
-      <c r="D310" t="n">
+      <c r="D310" s="20" t="n">
         <v>-70000</v>
       </c>
-      <c r="E310" t="inlineStr">
+      <c r="E310" s="20" t="inlineStr">
         <is>
           <t>Les humains modernes commencent à quitter le continent africain</t>
         </is>
       </c>
-      <c r="F310" t="inlineStr">
+      <c r="F310" s="20" t="inlineStr">
         <is>
           <t>Il y a 70 000 ans, un groupe d'Homo sapiens quitte l'Afrique pour la première fois et se lance dans une aventure qui durera des millénaires : le peuplement du monde entier. Avant cette date, tous les humains modernes vivaient en Afrique, principalement en Afrique de l'Est et du Sud. Mais à cette époque, certains groupes décident de partir vers le nord, franchissant le Sinaï et se dirigeant vers le Moyen-Orient et l'Asie. Cette migration n'est pas une décision planifiée : c'est plutôt une lente expansion des territoires de chasse. Au fil des générations, les groupes s'éloignent progressivement de l'Afrique. Les raisons exactes de cette migration restent débattues : certains scientifiques pensent que des changements climatiques (assèchement du Sahara) les ont poussés à partir. D'autres pensent que c'est simplement le résultat naturel de la croissance démographique. Les premiers migrants franchissent le détroit de la mer Rouge, probablement par bateau ou radeau primitif, montrant une capacité à naviguer et à traverser l'eau. Ces premiers voyageurs sont extrêmement courageux : ils entrent dans des territoires inconnus, avec des climats différents, des animaux différents, une végétation différente. Beaucoup de groupes n'iront pas loin. Certains reviennent. Mais d'autres persévèrent et continuent vers l'est. Cette première vague de migration est cruciale : c'est le début du peuplement de l'Eurasie. Sans cette migration audacieuse, les humains seraient restés confinés à l'Afrique.</t>
         </is>
       </c>
-      <c r="G310" t="inlineStr"/>
-      <c r="H310" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I310" t="inlineStr"/>
+      <c r="G310" s="20" t="inlineStr">
+        <is>
+          <t>Les études génétiques suggèrent que tous les non-Africains actuels descendent d'une population fondatrice étonnamment restreinte — entre quelques centaines et quelques milliers d'individus seulement auraient quitté l'Afrique lors de cette vague migratoire.</t>
+        </is>
+      </c>
+      <c r="H310" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I310" s="20" t="inlineStr"/>
     </row>
     <row r="311">
-      <c r="A311" t="n">
+      <c r="A311" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="B311" t="inlineStr">
+      <c r="B311" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Anthropologie</t>
         </is>
       </c>
-      <c r="C311" t="inlineStr">
+      <c r="C311" s="20" t="inlineStr">
         <is>
           <t>Homo sapiens arrive en Asie du Sud-Est</t>
         </is>
       </c>
-      <c r="D311" t="n">
+      <c r="D311" s="20" t="n">
         <v>-65000</v>
       </c>
-      <c r="E311" t="inlineStr">
+      <c r="E311" s="20" t="inlineStr">
         <is>
           <t>Les premiers humains modernes atteignent l'Asie du Sud-Est</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr">
+      <c r="F311" s="20" t="inlineStr">
         <is>
           <t>Il y a 65 000 ans, des groupes d'Homo sapiens atteignent l'Asie du Sud-Est, une région qui comprend aujourd'hui la Thaïlande, la Malaisie, l'Indonésie et les Philippines. Ce voyage depuis l'Afrique a duré au moins 5 000 ans, les groupes se déplaçant lentement, génération après génération, à travers le Moyen-Orient, puis vers le sud et l'est. Les preuves archéologiques viennent de sites comme Ksar Akil (Liban), Qafzeh (Iran) et des grottes en Thaïlande datant de cette époque. Ces premiers Sapiens en Asie du Sud-Est rencontrent un environnement tropical dense, chaud et humide, très différent de l'Afrique. Ils doivent adapter leur technologie de chasse et leurs techniques de survie. Des fossiles et des artefacts montrent qu'ils fabriquent des outils en pierre sophistiqués, chassent des animaux variés, et collectent des plantes. Des coquillages avec des trous percés, trouvés dans les grottes thaïlandaises, suggèrent qu'ils fabriquent déjà des parures : des colliers ou des bracelets. Cela indique un sens esthétique, peut-être même un sens de l'identité personnelle ou de groupe. Ces humains vivent en petits groupes de 20-50 personnes, chassent et cueillent pour survivre. Ils développent progressivement une connaissance intime de leur environnement : quelles plantes sont comestibles, où trouver l'eau, quand et où migrer. Cette adaptation à l'environnement tropical est cruciale : elle prépare le terrain pour la future colonisation de l'Australie, qui aura lieu 15 000 ans plus tard. Sans cette arrivée en Asie du Sud-Est, les humains n'auraient jamais pu atteindre l'Australie.</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr"/>
-      <c r="H311" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I311" t="inlineStr"/>
+      <c r="G311" s="20" t="inlineStr">
+        <is>
+          <t>Des coquillages percés retrouvés dans des grottes thaïlandaises de cette période comptent parmi les plus anciens bijoux personnels jamais découverts, suggérant que ces premiers migrants avaient déjà un sens de l'identité individuelle ou collective exprimé par l'apparence.</t>
+        </is>
+      </c>
+      <c r="H311" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I311" s="20" t="inlineStr"/>
     </row>
     <row r="312">
-      <c r="A312" t="n">
+      <c r="A312" s="20" t="n">
         <v>311</v>
       </c>
-      <c r="B312" t="inlineStr">
+      <c r="B312" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Anthropologie</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr">
+      <c r="C312" s="20" t="inlineStr">
         <is>
           <t>Homo sapiens colonise l'Australie</t>
         </is>
       </c>
-      <c r="D312" t="n">
+      <c r="D312" s="20" t="n">
         <v>-50000</v>
       </c>
-      <c r="E312" t="inlineStr">
+      <c r="E312" s="20" t="inlineStr">
         <is>
           <t>Les humains atteignent l'Australie en traversant l'océan pour la première fois</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr">
+      <c r="F312" s="20" t="inlineStr">
         <is>
           <t>Il y a 50 000 ans, un événement extraordinaire se produit : des groupes d'Homo sapiens franchissent l'océan et arrivent en Australie. C'est la première fois que des humains quittent les continents connus (Afrique, Asie, Europe) pour coloniser une terre complètement isolée. Cette migration représente un exploit technologique et culturel majeur. Pour atteindre l'Australie, les humains doivent traverser des détroits maritimes. À cette époque, le niveau des mers est plus bas (la glace recouvre les pôles), mais le détroit de Timor, entre l'Asie du Sud-Est et l'Australie, reste impassable à pied. Les humains doivent donc utiliser des bateaux ou des radeaux. Les preuves archéologiques montrent que les premiers Australiens arrivent à Lake Mungo, dans le sud-est de l'Australie, et rapidement ils colonisent tout le continent. Des fossiles de 50 000 à 45 000 ans montrent que les humains s'implantent dans tous les environnements australiens : déserts, côtes, montagnes. Cette diversification rapide montre une grande adaptabilité. Les archéologues trouvent des sites de foyers (feux) montrant que ces premiers Australiens maîtrisent le feu. Ils fabriquent des outils en pierre, des harpons, des filets. Des squelettes montrent que la vie est dure : fractures, infections, malnutrition. Mais les groupes prospèrent. Une découverte fascinante : une peinture rupestre datée de plus de 51 000 ans montre un stencil de main (empreinte de main). C'est l'une des plus anciennes formes d'art connu, presque certainement créée par ces premiers Australiens. L'empreinte de main est un geste universel d'affirmation de présence : "J'étais là". Ces premiers Australiens développent une culture riche avec des peintures, des sculptures en bois (les boomerangs apparaissent vers 30 000 ans), et des traditions orales. Les Aborigènes australiens contemporains sont les descendants directs de ces premiers migrants, ce qui en fait l'une des cultures humaines les plus anciennes et les plus continues du monde.</t>
         </is>
       </c>
-      <c r="G312" t="inlineStr"/>
-      <c r="H312" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I312" t="inlineStr"/>
+      <c r="G312" s="20" t="inlineStr">
+        <is>
+          <t>Atteindre l'Australie nécessitait de traverser volontairement une étendue d'eau qui n'a jamais été totalement fermée, même au plus bas niveau des mers de l'ère glaciaire — il s'agit peut-être de la plus ancienne preuve d'utilisation d'embarcations connue dans le monde.</t>
+        </is>
+      </c>
+      <c r="H312" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I312" s="20" t="inlineStr"/>
     </row>
     <row r="313">
-      <c r="A313" t="n">
+      <c r="A313" s="20" t="n">
         <v>312</v>
       </c>
-      <c r="B313" t="inlineStr">
+      <c r="B313" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Anthropologie</t>
         </is>
       </c>
-      <c r="C313" t="inlineStr">
+      <c r="C313" s="20" t="inlineStr">
         <is>
           <t>Arrivée de Sapiens en Europe - Rencontre avec Néandertal</t>
         </is>
       </c>
-      <c r="D313" t="n">
+      <c r="D313" s="20" t="n">
         <v>-45000</v>
       </c>
-      <c r="E313" t="inlineStr">
+      <c r="E313" s="20" t="inlineStr">
         <is>
           <t>Les humains modernes arrivent en Europe et rencontrent pour la première fois les Néandertaliens</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr">
+      <c r="F313" s="20" t="inlineStr">
         <is>
           <t>Il y a 45 000 ans, un événement décisif se produit en Europe : les premiers Homo sapiens arrivent du Moyen-Orient et rencontrent les Néandertaliens qui vivent en Europe depuis 250 000 ans. C'est la première rencontre entre deux espèces humaines intelligentes. Cette arrivée est datée précisément grâce aux fossiles de Mladeč (Tchéquie) et des sites de culture Aurignacienne, qui montrent clairement des caractéristiques de Sapiens modernes. Pendant les 10 000 années suivantes, Sapiens et Néandertal coexistent en Europe, probablement dans des régions différentes, mais parfois en contact direct. Les preuves archéologiques et génétiques montrent que ces deux espèces interagissent. Des analyses ADN révèlent que tous les Sapiens non-africains modernes portent 1 à 4% d'ADN Néandertal, ce qui signifie qu'il y a eu métissage. Cela implique des rencontres pacifiques, au moins occasionnellement. Mais la coexistence n'est pas simplement pacifique : il y a probablement aussi compétition pour les ressources de chasse. Les deux espèces chassent les mêmes animaux (mammouths, rennes, bisons). Sapiens, avec sa technologie plus avancée (premiers outils en os, premiers vêtements cousus, premiers harpons), a un avantage. Progressivement, Néandertal décline. Les derniers Néandertaliens disparaissent vers 35 000-30 000 ans. Néanmoins, les preuves d'intermariage restent plus probantes que celles de conflits massifs. L'arrivée de Sapiens en Europe marque le début de la domination humaine moderne sur le continent et la fin de l'ère des Néandertaliens.</t>
         </is>
       </c>
-      <c r="G313" t="inlineStr"/>
-      <c r="H313" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I313" t="inlineStr"/>
+      <c r="G313" s="20" t="inlineStr">
+        <is>
+          <t>Presque toutes les personnes d'origine non africaine aujourd'hui portent une petite part d'ADN néandertalien (typiquement 1 à 4 %), héritée de rencontres comme celle-ci — les Néandertaliens n'ont donc jamais totalement disparu, ils ont en partie été absorbés dans le patrimoine génétique de Sapiens.</t>
+        </is>
+      </c>
+      <c r="H313" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I313" s="20" t="inlineStr"/>
     </row>
     <row r="314">
-      <c r="A314" t="n">
+      <c r="A314" s="20" t="n">
         <v>313</v>
       </c>
-      <c r="B314" t="inlineStr">
+      <c r="B314" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Culture</t>
         </is>
       </c>
-      <c r="C314" t="inlineStr">
+      <c r="C314" s="20" t="inlineStr">
         <is>
           <t>Explosion créative : art pariétal, sculpture et parures</t>
         </is>
       </c>
-      <c r="D314" t="n">
+      <c r="D314" s="20" t="n">
         <v>-40000</v>
       </c>
-      <c r="E314" t="inlineStr">
+      <c r="E314" s="20" t="inlineStr">
         <is>
           <t>Le comportement humain change radicalement avec l'apparition de l'art et de la symbolique</t>
         </is>
       </c>
-      <c r="F314" t="inlineStr">
+      <c r="F314" s="20" t="inlineStr">
         <is>
           <t>Il y a 40 000 ans, quelque chose de remarquable se produit chez les humains : une "explosion créative". Cette période marque le début d'une transformation culturelle majeure. Soudainement, les preuves archéologiques montrent des peintures rupestres, des sculptures, des bijoux, des outils élaborés. C'est comme si un interrupteur était actionné. Avant 40 000 ans, les preuves d'art symbolique sont rares et douteuses. Après 40 000 ans, l'art devient courant et sophistiqué. Les grottes d'Europe se remplissent de peintures magnifiques : mains stencilisées, animaux (chevaux, bisons, rhinocéros), signes abstraits. Ces peintures ne sont pas des gribouillages naïfs : elles montrent une compréhension de la perspective, de la proportion, du mouvement. Parallèlement, les sculptures apparaissent. La Vénus de Hohle Fels, en Allemagne, datée de 40 000 ans, est une petite figurine de femme nue, sculptée en ivoire, mesurant 6 centimètres. Les bijoux apparaissent aussi : colliers de dents d'animaux percées, bracelets de coquillages. Certains squelettes de 40 000 ans sont enterrés avec des parures, suggérant que la beauté personnelle et l'identité visuelle deviennent importantes. Pourquoi cette explosion créative survient-elle maintenant ? Les scientifiques débattent. Une théorie : le langage parlé devient plus sophistiqué, permettant une meilleure communication et une meilleure transmission des idées. Une autre : le cerveau humain atteint sa maturité cognitive complète, permettant l'abstraction et l'imaginaire. Une troisième : la population augmente, créant plus d'interaction entre les groupes et d'échange d'idées. Quelle qu'en soit la raison, cette explosion créative marque un tournant : les humains commencent à créer une culture, pas simplement à survivre.</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr"/>
-      <c r="H314" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I314" t="inlineStr"/>
+      <c r="G314" s="20" t="inlineStr">
+        <is>
+          <t>La Vénus de Hohle Fels, sculptée dans de l'ivoire de mammouth à cette époque, compte parmi les plus anciennes représentations non ambiguës d'un être humain connues dans le monde.</t>
+        </is>
+      </c>
+      <c r="H314" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I314" s="20" t="inlineStr"/>
     </row>
     <row r="315">
-      <c r="A315" t="n">
+      <c r="A315" s="20" t="n">
         <v>314</v>
       </c>
-      <c r="B315" t="inlineStr">
+      <c r="B315" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Anthropologie</t>
         </is>
       </c>
-      <c r="C315" t="inlineStr">
+      <c r="C315" s="20" t="inlineStr">
         <is>
           <t>Disparition du dernier Néandertal</t>
         </is>
       </c>
-      <c r="D315" t="n">
+      <c r="D315" s="20" t="n">
         <v>-35000</v>
       </c>
-      <c r="E315" t="inlineStr">
+      <c r="E315" s="20" t="inlineStr">
         <is>
           <t>Les Néandertaliens disparaissent, Homo sapiens devient la seule espèce humaine</t>
         </is>
       </c>
-      <c r="F315" t="inlineStr">
+      <c r="F315" s="20" t="inlineStr">
         <is>
           <t>Il y a 35 000 ans, le dernier Néandertal disparaît. C'est la fin d'une espèce qui a prospéré en Europe pendant 250 000 ans. Les derniers Néandertaliens vivent dans les régions isolées du sud de la Péninsule Ibérique (Espagne et Portugal), où le climat plus doux permet à quelques populations de survivre plus longtemps. Après 35 000 ans, aucune trace fossile de Néandertal n'existe. Homo sapiens est désormais seul. La disparition du Néandertal n'est pas instantanée : elle s'étale sur plusieurs milliers d'années, probablement de 45 000 à 35 000 ans. Pendant cette période, les deux espèces coexistent, mais Sapiens augmente progressivement ses populations tandis que Néandertal décline. Pourquoi Néandertal disparaît-il ? Les scientifiques proposent plusieurs théories : Sapiens le tue ou l'expulse de ses territoires ; Sapiens, plus adaptatif et plus créatif, a un avantage compétitif ; un changement climatique défavorable aux Néandertaliens pousse les populations vers l'extinction ; des maladies, probablement apportées par Sapiens, déciment les populations Néandertal. Probablement, c'est une combinaison de tous ces facteurs. Les preuves génétiques montrent que les deux espèces se sont métissées, laissant 1 à 4% d'ADN Néandertal chez tous les Sapiens non-africains. Ironiquement, Néandertal n'a pas entièrement disparu : son génome vit à travers nous. Certains gènes Néandertal spécifiquement liés à l'immunité ont probablement aidé Sapiens à s'adapter aux maladies eurasiatiques. La disparition de Néandertal est un moment charnière : pour la première fois en 5-6 millions d'années d'évolution humaine, il n'y a plus de compétition d'autres hominidés.</t>
         </is>
       </c>
-      <c r="G315" t="inlineStr"/>
-      <c r="H315" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I315" t="inlineStr"/>
+      <c r="G315" s="20" t="inlineStr">
+        <is>
+          <t>On sait aujourd'hui que Néandertaliens et Sapiens ont coexisté et se sont métissés pendant environ les 10 000 dernières années de l'existence des premiers en Europe — leur « disparition » ressemble donc moins à un effacement soudain qu'à une lente fusion démographique suivie d'un déclin.</t>
+        </is>
+      </c>
+      <c r="H315" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I315" s="20" t="inlineStr"/>
     </row>
     <row r="316">
-      <c r="A316" t="n">
+      <c r="A316" s="20" t="n">
         <v>315</v>
       </c>
-      <c r="B316" t="inlineStr">
+      <c r="B316" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Art</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr">
+      <c r="C316" s="20" t="inlineStr">
         <is>
           <t>Gravures et sculptures sophistiquées - Vénus de Willendorf</t>
         </is>
       </c>
-      <c r="D316" t="n">
+      <c r="D316" s="20" t="n">
         <v>-30000</v>
       </c>
-      <c r="E316" t="inlineStr">
+      <c r="E316" s="20" t="inlineStr">
         <is>
           <t>L'art figuratif devient courant et montre une compréhension profonde de la forme et de la beauté</t>
         </is>
       </c>
-      <c r="F316" t="inlineStr">
+      <c r="F316" s="20" t="inlineStr">
         <is>
           <t>Il y a 30 000 ans, les humains créent des sculptures de plus en plus sophistiquées. L'une des plus célèbres est la Vénus de Willendorf, découverte en Autriche, datée de 29 000 à 25 000 ans. C'est une petite figurine en calcaire de 11 centimètres de haut, qui représente une femme nue, avec des seins proéminents, un ventre rond, et les jambes atrophiées. Le visage n'a pas de traits distincts, mais la tête a un motif qui ressemble à des nattes ou des cheveux tressés. Pourquoi cette figurine ? Les archéologues ont proposé de nombreuses interprétations : une déesse de la fertilité (le corps gras et enceinte symbolise la fécondité), un autoportrait d'une femme enceinte, une poupée destinée à l'amusement des enfants, ou un objet magique supposé apporter la fertilité au groupe. Ce qui est clair : les humains, à cette époque, créent des objets sophistiqués avec intention symbolique, pas pratique. L'existence de la Vénus de Willendorf et d'autres figurines similaires (trouvées en Russie, en Europe centrale, en France) montre que la sculpture est une pratique courante. Les outils aussi deviennent plus sophistiqués : des aiguilles en os pour coudre les vêtements, des harpons barbelés pour la pêche, des bâtons de commandement. Les squelettes montrent que les humains vivent en meilleure santé : moins de fractures, moins d'infections. Les grottes contiennent des restes de foyers, de nourriture stockée, de matériaux bruts pour la fabrication d'outils, suggérant des habitats plus permanents et une meilleure organisation sociale. À 30 000 ans, les humains ne sont pas juste des survivants : ce sont des artistes, des artisans, des penseurs symboliques.</t>
         </is>
       </c>
-      <c r="G316" t="inlineStr"/>
-      <c r="H316" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I316" t="inlineStr"/>
+      <c r="G316" s="20" t="inlineStr">
+        <is>
+          <t>La Vénus de Willendorf a été sculptée dans un type de calcaire introuvable à proximité du site autrichien où elle a été découverte, ce qui laisse penser que la pierre — ou son sculpteur — a parcouru une distance non négligeable.</t>
+        </is>
+      </c>
+      <c r="H316" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I316" s="20" t="inlineStr"/>
     </row>
     <row r="317">
-      <c r="A317" t="n">
+      <c r="A317" s="20" t="n">
         <v>316</v>
       </c>
-      <c r="B317" t="inlineStr">
+      <c r="B317" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Art</t>
         </is>
       </c>
-      <c r="C317" t="inlineStr">
+      <c r="C317" s="20" t="inlineStr">
         <is>
           <t>Apogée de l'art pariétal - Grottes Chauvet et Lascaux</t>
         </is>
       </c>
-      <c r="D317" t="n">
+      <c r="D317" s="20" t="n">
         <v>-25000</v>
       </c>
-      <c r="E317" t="inlineStr">
+      <c r="E317" s="20" t="inlineStr">
         <is>
           <t>Les grottes remplies de peintures deviennent des galeries d'art majeures</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr">
+      <c r="F317" s="20" t="inlineStr">
         <is>
           <t>Il y a 25 000 ans, les grottes d'Europe contiennent des quantités massives de peintures et de gravures. Bien que la grotte Chauvet (en France) soit datée de 36 000 ans et la grotte Lascaux de 17 000 ans, la période de 25 000 ans représente l'apogée de l'art rupestre gravetien et pré-magdalénien. Ces grottes ne sont pas des habitats : ce sont des sanctuaires sacrés, des galeries d'art, des lieux de culte ou de rituel, souvent dans les parties les plus profondes et inaccessibles, dans l'obscurité totale. La grotte Chauvet, avec ses 400 peintures, contient des images magnifiques : chevaux, bisons, lions des cavernes, rhinocéros, disposées en suivant les contours naturels de la roche. Les pigments utilisés sont de l'ocre rouge et du charbon noir, appliqués avec les mains, des bâtons, peut-être des brosses primitives. Dans la grotte Chauvet, il y a environ 150 empreintes de mains, chacune unique, datées de 37 500 à 33 900 ans : parmi les plus anciennes preuves que les humains reconnaissent l'individualité et laissent une trace de leur passage. Pourquoi l'art ? Les théories incluent la magie de chasse, le chamanisme, la religion, le marquage identitaire de territoire, ou simplement l'esthétique. Probablement une combinaison de tout cela. En 1994, la grotte Chauvet est découverte par hasard par des spéléologues, les peintures pratiquement intactes, préservées par le calcaire et l'atmosphère stable de la grotte. Voir ces peintures est une connexion directe avec les humains d'il y a 36 000 ans, rappelant que le besoin de créer et d'exprimer la beauté est aussi vieux que l'humanité moderne.</t>
         </is>
       </c>
-      <c r="G317" t="inlineStr"/>
-      <c r="H317" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I317" t="inlineStr"/>
+      <c r="G317" s="20" t="inlineStr">
+        <is>
+          <t>Après l'ouverture au public de la grotte de Lascaux, découverte en 1940, la chaleur et le souffle des visiteurs ont provoqué l'apparition de moisissures et d'algues sur les peintures. La grotte a été fermée au public dès 1963, et une réplique complète, Lascaux II, a été construite à proximité pour permettre au public de continuer à admirer cet art sans l'abîmer.</t>
+        </is>
+      </c>
+      <c r="H317" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I317" s="20" t="inlineStr"/>
     </row>
     <row r="318">
-      <c r="A318" t="n">
+      <c r="A318" s="20" t="n">
         <v>317</v>
       </c>
-      <c r="B318" t="inlineStr">
+      <c r="B318" s="20" t="inlineStr">
         <is>
           <t>Technologie / Chasse</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr">
+      <c r="C318" s="20" t="inlineStr">
         <is>
           <t>Bow and arrow technology émerge</t>
         </is>
       </c>
-      <c r="D318" t="n">
+      <c r="D318" s="20" t="n">
         <v>-20000</v>
       </c>
-      <c r="E318" t="inlineStr">
+      <c r="E318" s="20" t="inlineStr">
         <is>
           <t>L'arc et la flèche révolutionnent la chasse et le combat</t>
         </is>
       </c>
-      <c r="F318" t="inlineStr">
+      <c r="F318" s="20" t="inlineStr">
         <is>
           <t>Il y a 20 000 ans, les preuves archéologiques montrent l'émergence d'une nouvelle technologie : l'arc et la flèche. Les plus anciennes preuves proviennent de sites en Afrique du Sud (Sibudu Cave) et en Europe (Stellmoor, Allemagne), datées entre 20 000 et 17 000 ans. Avant cela, les humains utilisent principalement des javelots lancés à la main ou des atlatls (bâtons de propulsion). Mais l'arc et la flèche offrent des avantages majeurs : plus de précision, plus de puissance, une portée plus grande (jusqu'à 50-100 mètres), et moins d'effort physique. Un chasseur peut rester à distance sécuritaire de sa proie, et les flèches sont beaucoup plus légères que les javelots, donc un chasseur peut en porter beaucoup plus. Les premières flèches sont faites de bois, de pierre (pointes) et de plumes (empennage), avec des pointes petites, finement taillées, triangulaires ou barbelées. Les squelettes de 20 000 ans montrent souvent des blessures compatibles avec des blessures de flèche. La maîtrise de l'arc et la flèche demande de la pratique, de la coordination, de la précision, renforçant la transmission culturelle entre générations. L'arc et la flèche ne sont pas juste une technologie de chasse : ils deviennent aussi une arme de guerre, augmentant l'efficacité mortelle des conflits mais aussi la capacité de défense d'un territoire par un petit groupe bien entraîné. Des millénaires plus tard, Gengis Khan utilisera des archers à cheval pour conquérir le monde.</t>
         </is>
       </c>
-      <c r="G318" t="inlineStr"/>
-      <c r="H318" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I318" t="inlineStr"/>
+      <c r="G318" s="20" t="inlineStr">
+        <is>
+          <t>Certaines des plus anciennes preuves supposées de l'usage de l'arc proviennent de minuscules pointes en pierre retrouvées dans la grotte de Sibudu, en Afrique du Sud — si petites qu'elles n'auraient pu fonctionner que comme pointes de flèches, ce qui repousserait l'origine de cette technologie de plusieurs dizaines de milliers d'années.</t>
+        </is>
+      </c>
+      <c r="H318" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I318" s="20" t="inlineStr"/>
     </row>
     <row r="319">
-      <c r="A319" t="n">
+      <c r="A319" s="20" t="n">
         <v>318</v>
       </c>
-      <c r="B319" t="inlineStr">
+      <c r="B319" s="20" t="inlineStr">
         <is>
           <t>Climatologie / Géologie</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr">
+      <c r="C319" s="20" t="inlineStr">
         <is>
           <t>Dernière période glaciaire - Last Glacial Maximum</t>
         </is>
       </c>
-      <c r="D319" t="n">
+      <c r="D319" s="20" t="n">
         <v>-18000</v>
       </c>
-      <c r="E319" t="inlineStr">
+      <c r="E319" s="20" t="inlineStr">
         <is>
           <t>Le froid atteint son maximum, les glaciers couvrent de vastes territoires</t>
         </is>
       </c>
-      <c r="F319" t="inlineStr">
+      <c r="F319" s="20" t="inlineStr">
         <is>
           <t>Il y a 18 000 ans, la Terre connaît le point culminant de la dernière période glaciaire : le "Last Glacial Maximum" (LGM). Les calottes glaciaires sont au maximum de leur extension : les glaciers d'Amérique du Nord couvrent tout le Canada et descendent jusqu'au Kentucky, l'Europe du Nord est couverte de glaciers épais, la Sibérie est un désert de glace. Le niveau des mers est 120-130 mètres plus bas qu'aujourd'hui. Des "terres de passage" apparaissent : le détroit de Béring devient la "Béringie", une vaste plaine terrestre que des humains traversent pour migrer de Sibérie vers l'Amérique du Nord. Le climat est extrêmement froid, les hivers catastrophiques, et la vie incroyablement difficile. Les humains fabriquent des vêtements épais en peau d'animal, construisent des abris semi-enterrés renforcés avec des os et des défenses de mammouths, et maîtrisent complètement le feu. Ils chassent les mégafaunes (mammouths, rhinocéros laineux, ours des cavernes) qui requièrent coordination de groupe, stratégie et courage. Le LGM dure environ 2 000-3 000 ans (de 23 000 à 19 000 ans, avec le maximum à 18 000 ans). La population humaine globale diminue, certains groupes se réfugiant dans des zones climatiques plus clémentes (Méditerranée, Afrique du Sud, Asie du Sud). Le LGM est considéré comme le "goulot d'étranglement démographique" de l'humanité : la population mondiale aurait été réduite à peut-être seulement 10 000-30 000 individus. Si l'espèce humaine avait échoué à survivre au LGM, l'humanité entière aurait disparu.</t>
         </is>
       </c>
-      <c r="G319" t="inlineStr"/>
-      <c r="H319" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I319" t="inlineStr"/>
+      <c r="G319" s="20" t="inlineStr">
+        <is>
+          <t>Une telle quantité de l'eau de la planète était alors enfermée dans les calottes glaciaires que le niveau des mers était environ 120 mètres plus bas qu'aujourd'hui : des terres aujourd'hui recouvertes par la Manche ou le détroit de Béring formaient alors un sol sec que l'on pouvait traverser à pied.</t>
+        </is>
+      </c>
+      <c r="H319" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I319" s="20" t="inlineStr"/>
     </row>
     <row r="320">
-      <c r="A320" t="n">
+      <c r="A320" s="20" t="n">
         <v>319</v>
       </c>
-      <c r="B320" t="inlineStr">
+      <c r="B320" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Domestication</t>
         </is>
       </c>
-      <c r="C320" t="inlineStr">
+      <c r="C320" s="20" t="inlineStr">
         <is>
           <t>Domestication du chien - premiers animaux domestiqués</t>
         </is>
       </c>
-      <c r="D320" t="n">
+      <c r="D320" s="20" t="n">
         <v>-15000</v>
       </c>
-      <c r="E320" t="inlineStr">
+      <c r="E320" s="20" t="inlineStr">
         <is>
           <t>Les loups commencent à être domestiqués et deviennent des chiens</t>
         </is>
       </c>
-      <c r="F320" t="inlineStr">
+      <c r="F320" s="20" t="inlineStr">
         <is>
           <t>Il y a 15 000 ans, un processus qui changera profondément la civilisation humaine commence : la domestication du chien, probablement le premier animal jamais domestiqué. Les preuves archéologiques proviennent de sites en Allemagne (Bonn-Oberkassel), en Israël (Eynan), et en Russie (Razboinichya Cave), où des restes de chiens datent de 15 000 à 14 000 ans. La théorie la plus acceptée : les loups, attirés par les déchets près des campements humains, commencent à scavenger. Les loups les moins agressifs s'approchent des humains, qui les tolèrent car ils aident à se débarrasser des déchets. Au fil des générations, une sélection naturelle et humaine se produit : les loups les plus calmes survivent mieux près des humains et se reproduisent. Graduellement, leur tempérament et leur apparence changent (oreilles qui tombent, queue qui s'enroule, pelage varié) : ce ne sont plus des loups, ce sont des chiens. Un fossile célèbre, le "Bonn-Oberkassel dog", est un chiot datant de 14 200 ans qui avait un problème dentaire congénital ; le fait qu'il ait survécu jusqu'à 6-7 mois suggère qu'il a été soigné et chéri par les humains, l'une des plus anciennes preuves d'une relation affective homme-animal. La domestication du chien a des impacts majeurs sur la chasse : les chiens aident à débusquer et rabattre le gibier, tracent les animaux blessés, et protègent les campements. Elle inspire aussi la domestication d'autres animaux : 10 000 ans plus tard, les humains domestiquent chèvres, moutons et vaches. Mais le chien arrive le premier, et la relation humain-chien dure jusqu'à aujourd'hui.</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr"/>
-      <c r="H320" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I320" t="inlineStr"/>
+      <c r="G320" s="20" t="inlineStr">
+        <is>
+          <t>Le « chien de Bonn-Oberkassel », un chiot enterré aux côtés de deux humains il y a environ 14 200 ans, souffrait d'une grave maladie et n'aurait pu survivre plusieurs semaines après l'infection que grâce à des soins et une alimentation intensifs — l'un des plus anciens signes connus d'attachement d'humains envers un animal malade.</t>
+        </is>
+      </c>
+      <c r="H320" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I320" s="20" t="inlineStr"/>
     </row>
     <row r="321">
-      <c r="A321" t="n">
+      <c r="A321" s="20" t="n">
         <v>320</v>
       </c>
-      <c r="B321" t="inlineStr">
+      <c r="B321" s="20" t="inlineStr">
         <is>
           <t>Climatologie</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr">
+      <c r="C321" s="20" t="inlineStr">
         <is>
           <t>Fin de l'Âge de Glace et début du réchauffement climatique</t>
         </is>
       </c>
-      <c r="D321" t="n">
+      <c r="D321" s="20" t="n">
         <v>-14000</v>
       </c>
-      <c r="E321" t="inlineStr">
+      <c r="E321" s="20" t="inlineStr">
         <is>
           <t>Les glaciers commencent à fondre massivement, le climat se réchauffe</t>
         </is>
       </c>
-      <c r="F321" t="inlineStr">
+      <c r="F321" s="20" t="inlineStr">
         <is>
           <t>Il y a 14 000 ans, le climat de la Terre commence une transformation majeure : la fin de la dernière période glaciaire. Après une période de refroidissement temporaire (le Dryas Inférieur, environ 12 800 ans, qui dure 1 200 ans), le Holocène débute à 11 700 ans, marquant vraiment le début d'une période interglaciaire chaude et stable. À 14 000 ans, les glaciers qui couvraient l'Amérique du Nord, l'Europe du Nord et la Sibérie commencent à fondre rapidement. Le niveau des mers remonte, la Béringie est submergée, les écosystèmes changent radicalement, et les mammouths et autres mégafaunes, adaptés au froid, déclinent et finissent par disparaître. Ce réchauffement climatique a des implications énormes pour la civilisation humaine. Dans le Croissant Fertile (région entre le Tigre et l'Euphrate en Mésopotamie), les conditions deviennent idéales pour certaines plantes sauvages, particulièrement les céréales comme le blé et l'orge. Les humains de cette région remarquent qu'une certaine plante produit des graines comestibles et commencent à les cueillir. Progressivement, sur les 2 000-3 000 ans suivants, ils passent de la cueillette simple à la "proto-agriculture", puis à l'agriculture complète, d'où émergera la révolution néolithique. Sans ce réchauffement climatique, l'agriculture n'aurait probablement jamais émergé, et sans agriculture, pas de civilisation : les empires, les villes, l'écriture, la complexité sociale découlent finalement de ce réchauffement climatique. Avec le temps plus doux et plus stable, les humains peuvent rester au même endroit (sédentarité), ce qui permet l'accumulation de biens, l'émergence de hiérarchie, et finalement la civilisation.</t>
         </is>
       </c>
-      <c r="G321" t="inlineStr"/>
-      <c r="H321" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I321" t="inlineStr"/>
+      <c r="G321" s="20" t="inlineStr">
+        <is>
+          <t>Ce réchauffement ne s'est pas fait sans à-coups : il a été interrompu par un coup de froid d'environ 1 200 ans appelé « Dryas récent », pendant lequel une partie de l'hémisphère nord est retombée dans des conditions quasi glaciaires avant que la tendance au réchauffement ne reprenne durablement.</t>
+        </is>
+      </c>
+      <c r="H321" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I321" s="20" t="inlineStr"/>
     </row>
     <row r="322">
-      <c r="A322" t="n">
+      <c r="A322" s="20" t="n">
         <v>321</v>
       </c>
-      <c r="B322" t="inlineStr">
+      <c r="B322" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Agriculture</t>
         </is>
       </c>
-      <c r="C322" t="inlineStr">
+      <c r="C322" s="20" t="inlineStr">
         <is>
           <t>Révolution néolithique : débuts de l'agriculture dans le Croissant Fertile</t>
         </is>
       </c>
-      <c r="D322" t="n">
+      <c r="D322" s="20" t="n">
         <v>-12000</v>
       </c>
-      <c r="E322" t="inlineStr">
+      <c r="E322" s="20" t="inlineStr">
         <is>
           <t>Les humains commencent à cultiver intentionnellement des plantes</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr">
+      <c r="F322" s="20" t="inlineStr">
         <is>
           <t>Il y a 12 000 ans, un changement révolutionnaire se produit : les humains commencent à cultiver délibérément des plantes. C'est le début de la révolution néolithique, qui débute dans le Croissant Fertile, une région qui s'étend du Nil en Égypte jusqu'au Tigre-Euphrate en Mésopotamie moderne. Les preuves archéologiques viennent de sites comme Jéricho, Çatalhöyük, Abu Hureyra, et Tell Aswad. Avant 12 000 ans, les humains sont tous des chasseurs-cueilleurs, se déplaçant saisonnièrement à la recherche de nourriture. Les scientifiques débattent des raisons du changement : réchauffement climatique rendant l'agriculture viable, pression démographique, ou abondance naturelle croissante de plantes sauvages nutritives. Les humains remarquent que planter les graines du blé récolté l'année précédente fait pousser de nouvelles plantes, et expérimentent la culture intentionnelle. Progressivement, au cours des siècles, ils sélectionnent les plantes avec les plus grosses graines et les meilleurs rendements : une sélection artificielle qui rend les plantes cultivées génétiquement distinctes des plantes sauvages. Parallèlement, la chasse devient plus difficile à mesure que les mégafaunes disparaissent, rendant l'agriculture plus attractive. À 10 000-9 000 ans, la transition est complète : les villages du Croissant Fertile cultivent blé, orge, pois et lentilles, et domestiquent chèvres, moutons et vaches. Ce passage a des impacts colossaux : rendement alimentaire plus élevé, sédentarité, accumulation de biens et de richesse, surplus permettant l'émergence de prêtres, guerriers et administrateurs, donc de hiérarchie sociale et finalement de l'État. Mais aussi des inconvénients : travail plus intensif, régime moins diversifié, vulnérabilité aux mauvaises récoltes, et augmentation des maladies infectieuses liées à la proximité du bétail et à la densité de population. La révolution agricole crée ainsi les conditions nécessaires à la civilisation.</t>
         </is>
       </c>
-      <c r="G322" t="inlineStr"/>
-      <c r="H322" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I322" t="inlineStr"/>
+      <c r="G322" s="20" t="inlineStr">
+        <is>
+          <t>Jéricho, l'un des sites clés de cette transition, est considérée par de nombreux archéologues comme la plus ancienne ville habitée sans interruption au monde : sa célèbre tour et ses murs de pierre datent d'environ 11 000 ans, bien avant l'invention de l'écriture, du métal ou de la roue.</t>
+        </is>
+      </c>
+      <c r="H322" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I322" s="20" t="inlineStr"/>
     </row>
     <row r="323">
-      <c r="A323" t="n">
+      <c r="A323" s="20" t="n">
         <v>322</v>
       </c>
-      <c r="B323" t="inlineStr">
+      <c r="B323" s="20" t="inlineStr">
         <is>
           <t>Archéologie / Agriculture</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr">
+      <c r="C323" s="20" t="inlineStr">
         <is>
           <t>Domestication du blé et de l'orge</t>
         </is>
       </c>
-      <c r="D323" t="n">
+      <c r="D323" s="20" t="n">
         <v>-11000</v>
       </c>
-      <c r="E323" t="inlineStr">
+      <c r="E323" s="20" t="inlineStr">
         <is>
           <t>Les céréales deviennent les cultures fondamentales</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr">
+      <c r="F323" s="20" t="inlineStr">
         <is>
           <t>Il y a 11 000 ans, la domestication du blé et de l'orge est bien établie dans le Croissant Fertile. Des sites archéologiques montrent que le blé "emmer" (Triticum turgidum dicoccoides) et l'orge (Hordeum vulgare) sont activement cultivés. Pourquoi ces deux plantes ? Elles offrent un rendement élevé en calories, une facilité de stockage (les grains secs se conservent longtemps), une facilité de culture, et contiennent protéines et vitamines. Les archéobotaniques distinguent le blé et l'orge sauvages des versions domestiquées par des caractéristiques morphologiques : le blé sauvage a un axe fragile qui se casse facilement et disperse les graines, tandis que le blé domestiqué a un axe dur qui ne se casse pas, permettant aux humains de récolter les épis entiers. Ce changement génétique, apparu progressivement sur plusieurs générations, rend la plante entièrement dépendante de l'homme pour sa reproduction. À 11 000 ans, le blé et l'orge domestiqués sont génétiquement distincts de leurs ancêtres sauvages, et les rendements s'améliorent chaque année : un agriculteur peut produire assez de céréales pour nourrir environ 2-3 fois plus de personnes qu'un chasseur-cueilleur sur la même surface. Cela permet à la population d'augmenter rapidement, et les villages qui cultivent le blé et l'orge grossissent, atteignant plusieurs centaines d'habitants dès 10 000 ans. Le stockage du blé dans des greniers crée une incitation à construire des bâtiments fortifiés et à organiser une défense collective. Plus tard, le surplus permet à certaines personnes de devenir guerriers à temps plein, et le blé et l'orge deviennent même des unités de monnaie avant l'apparition des pièces. Cette domestication crée une symbiose humains-plantes qui dure depuis plus de 10 000 ans.</t>
         </is>
       </c>
-      <c r="G323" t="inlineStr"/>
-      <c r="H323" t="inlineStr">
-        <is>
-          <t>Avéré</t>
-        </is>
-      </c>
-      <c r="I323" t="inlineStr"/>
+      <c r="G323" s="20" t="inlineStr">
+        <is>
+          <t>L'épi de blé sauvage se brise naturellement pour disperser ses graines, mais une mutation génétique rare produit un épi qui reste attaché à la tige : sans le savoir, les premiers agriculteurs ont sélectionné ce trait mutant à chaque récolte et replantation, modifiant durablement la génétique de la plante en quelques centaines de générations seulement.</t>
+        </is>
+      </c>
+      <c r="H323" s="20" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="I323" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -23365,840 +23669,840 @@
       </c>
     </row>
     <row r="477">
-      <c r="A477" t="n">
+      <c r="A477" s="20" t="n">
         <v>309</v>
       </c>
-      <c r="B477" t="inlineStr">
+      <c r="B477" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C477" t="inlineStr">
+      <c r="C477" s="20" t="inlineStr">
         <is>
           <t>Nature : Early dispersal of modern humans from Africa - Templeton (2002)</t>
         </is>
       </c>
-      <c r="D477" t="inlineStr">
+      <c r="D477" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/415546a</t>
         </is>
       </c>
     </row>
     <row r="478">
-      <c r="A478" t="n">
+      <c r="A478" s="20" t="n">
         <v>309</v>
       </c>
-      <c r="B478" t="inlineStr">
+      <c r="B478" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C478" t="inlineStr">
+      <c r="C478" s="20" t="inlineStr">
         <is>
           <t>PNAS : Genomic evidence for early human dispersal - Armitage et al. (2011)</t>
         </is>
       </c>
-      <c r="D478" t="inlineStr">
+      <c r="D478" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1100166108</t>
         </is>
       </c>
     </row>
     <row r="479">
-      <c r="A479" t="n">
+      <c r="A479" s="20" t="n">
         <v>309</v>
       </c>
-      <c r="B479" t="inlineStr">
+      <c r="B479" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C479" t="inlineStr">
+      <c r="C479" s="20" t="inlineStr">
         <is>
           <t>Science : Human genetic diversity and migration patterns - Li et al. (2008)</t>
         </is>
       </c>
-      <c r="D479" t="inlineStr">
+      <c r="D479" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1153717</t>
         </is>
       </c>
     </row>
     <row r="480">
-      <c r="A480" t="n">
+      <c r="A480" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="B480" t="inlineStr">
+      <c r="B480" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C480" t="inlineStr">
+      <c r="C480" s="20" t="inlineStr">
         <is>
           <t>PNAS : Early human dispersal to Southeast Asia - Demeter et al. (2012)</t>
         </is>
       </c>
-      <c r="D480" t="inlineStr">
+      <c r="D480" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1108887109</t>
         </is>
       </c>
     </row>
     <row r="481">
-      <c r="A481" t="n">
+      <c r="A481" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="B481" t="inlineStr">
+      <c r="B481" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C481" t="inlineStr">
+      <c r="C481" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Archaeological evidence of early Southeast Asian settlement - Higham &amp; Thosarat (2004)</t>
         </is>
       </c>
-      <c r="D481" t="inlineStr">
+      <c r="D481" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2003.12.003</t>
         </is>
       </c>
     </row>
     <row r="482">
-      <c r="A482" t="n">
+      <c r="A482" s="20" t="n">
         <v>310</v>
       </c>
-      <c r="B482" t="inlineStr">
+      <c r="B482" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C482" t="inlineStr">
+      <c r="C482" s="20" t="inlineStr">
         <is>
           <t>Quaternary Science Reviews : Human migration to Southeast Asia - Ono et al. (2018)</t>
         </is>
       </c>
-      <c r="D482" t="inlineStr">
+      <c r="D482" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.quascirev.2018.09.035</t>
         </is>
       </c>
     </row>
     <row r="483">
-      <c r="A483" t="n">
+      <c r="A483" s="20" t="n">
         <v>311</v>
       </c>
-      <c r="B483" t="inlineStr">
+      <c r="B483" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C483" t="inlineStr">
+      <c r="C483" s="20" t="inlineStr">
         <is>
           <t>Nature : Dating of Australian rock art and early human dispersal - Clarkson et al. (2017)</t>
         </is>
       </c>
-      <c r="D483" t="inlineStr">
+      <c r="D483" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/s41586-017-0008-8</t>
         </is>
       </c>
     </row>
     <row r="484">
-      <c r="A484" t="n">
+      <c r="A484" s="20" t="n">
         <v>311</v>
       </c>
-      <c r="B484" t="inlineStr">
+      <c r="B484" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C484" t="inlineStr">
+      <c r="C484" s="20" t="inlineStr">
         <is>
           <t>PNAS : Earliest known art in Australia - Aubert et al. (2014)</t>
         </is>
       </c>
-      <c r="D484" t="inlineStr">
+      <c r="D484" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1408356111</t>
         </is>
       </c>
     </row>
     <row r="485">
-      <c r="A485" t="n">
+      <c r="A485" s="20" t="n">
         <v>311</v>
       </c>
-      <c r="B485" t="inlineStr">
+      <c r="B485" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C485" t="inlineStr">
+      <c r="C485" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Settlement patterns in early Australia - O'Connell &amp; Allen (2012)</t>
         </is>
       </c>
-      <c r="D485" t="inlineStr">
+      <c r="D485" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2012.05.010</t>
         </is>
       </c>
     </row>
     <row r="486">
-      <c r="A486" t="n">
+      <c r="A486" s="20" t="n">
         <v>312</v>
       </c>
-      <c r="B486" t="inlineStr">
+      <c r="B486" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C486" t="inlineStr">
+      <c r="C486" s="20" t="inlineStr">
         <is>
           <t>Nature : Fossil evidence of Sapiens arrival in Europe - Higham et al. (2014)</t>
         </is>
       </c>
-      <c r="D486" t="inlineStr">
+      <c r="D486" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature13621</t>
         </is>
       </c>
     </row>
     <row r="487">
-      <c r="A487" t="n">
+      <c r="A487" s="20" t="n">
         <v>312</v>
       </c>
-      <c r="B487" t="inlineStr">
+      <c r="B487" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C487" t="inlineStr">
+      <c r="C487" s="20" t="inlineStr">
         <is>
           <t>Science : Ancient DNA of Neanderthals and Sapiens - Green et al. (2010)</t>
         </is>
       </c>
-      <c r="D487" t="inlineStr">
+      <c r="D487" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1188021</t>
         </is>
       </c>
     </row>
     <row r="488">
-      <c r="A488" t="n">
+      <c r="A488" s="20" t="n">
         <v>312</v>
       </c>
-      <c r="B488" t="inlineStr">
+      <c r="B488" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C488" t="inlineStr">
+      <c r="C488" s="20" t="inlineStr">
         <is>
           <t>PNAS : Neandertal-Sapiens introgression - Castellano et al. (2014)</t>
         </is>
       </c>
-      <c r="D488" t="inlineStr">
+      <c r="D488" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1320099111</t>
         </is>
       </c>
     </row>
     <row r="489">
-      <c r="A489" t="n">
+      <c r="A489" s="20" t="n">
         <v>313</v>
       </c>
-      <c r="B489" t="inlineStr">
+      <c r="B489" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C489" t="inlineStr">
+      <c r="C489" s="20" t="inlineStr">
         <is>
           <t>Nature : Aurignacian symbolic behavior in Europe - Mellars (2005)</t>
         </is>
       </c>
-      <c r="D489" t="inlineStr">
+      <c r="D489" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature03674</t>
         </is>
       </c>
     </row>
     <row r="490">
-      <c r="A490" t="n">
+      <c r="A490" s="20" t="n">
         <v>313</v>
       </c>
-      <c r="B490" t="inlineStr">
+      <c r="B490" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C490" t="inlineStr">
+      <c r="C490" s="20" t="inlineStr">
         <is>
           <t>PNAS : Early artistic expression in Africa and Europe - Conard et al. (2009)</t>
         </is>
       </c>
-      <c r="D490" t="inlineStr">
+      <c r="D490" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0900157106</t>
         </is>
       </c>
     </row>
     <row r="491">
-      <c r="A491" t="n">
+      <c r="A491" s="20" t="n">
         <v>313</v>
       </c>
-      <c r="B491" t="inlineStr">
+      <c r="B491" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C491" t="inlineStr">
+      <c r="C491" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : The evolution of symbolic behavior - Mithen (2007)</t>
         </is>
       </c>
-      <c r="D491" t="inlineStr">
+      <c r="D491" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2006.07.001</t>
         </is>
       </c>
     </row>
     <row r="492">
-      <c r="A492" t="n">
+      <c r="A492" s="20" t="n">
         <v>314</v>
       </c>
-      <c r="B492" t="inlineStr">
+      <c r="B492" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C492" t="inlineStr">
+      <c r="C492" s="20" t="inlineStr">
         <is>
           <t>PNAS : Timing of Neanderthal extinction - Higham et al. (2014)</t>
         </is>
       </c>
-      <c r="D492" t="inlineStr">
+      <c r="D492" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1405035111</t>
         </is>
       </c>
     </row>
     <row r="493">
-      <c r="A493" t="n">
+      <c r="A493" s="20" t="n">
         <v>314</v>
       </c>
-      <c r="B493" t="inlineStr">
+      <c r="B493" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C493" t="inlineStr">
+      <c r="C493" s="20" t="inlineStr">
         <is>
           <t>Nature : Neanderthal extinction and climate - Finlayson et al. (2006)</t>
         </is>
       </c>
-      <c r="D493" t="inlineStr">
+      <c r="D493" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature04585</t>
         </is>
       </c>
     </row>
     <row r="494">
-      <c r="A494" t="n">
+      <c r="A494" s="20" t="n">
         <v>314</v>
       </c>
-      <c r="B494" t="inlineStr">
+      <c r="B494" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C494" t="inlineStr">
+      <c r="C494" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Reasons for Neanderthal extinction - Shea (2006)</t>
         </is>
       </c>
-      <c r="D494" t="inlineStr">
+      <c r="D494" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhevol.2006.04.001</t>
         </is>
       </c>
     </row>
     <row r="495">
-      <c r="A495" t="n">
+      <c r="A495" s="20" t="n">
         <v>315</v>
       </c>
-      <c r="B495" t="inlineStr">
+      <c r="B495" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C495" t="inlineStr">
+      <c r="C495" s="20" t="inlineStr">
         <is>
           <t>Journal of Archaeological Research : Paleolithic figurines and their meaning - Conard (2009)</t>
         </is>
       </c>
-      <c r="D495" t="inlineStr">
+      <c r="D495" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s10814-009-9030-1</t>
         </is>
       </c>
     </row>
     <row r="496">
-      <c r="A496" t="n">
+      <c r="A496" s="20" t="n">
         <v>315</v>
       </c>
-      <c r="B496" t="inlineStr">
+      <c r="B496" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C496" t="inlineStr">
+      <c r="C496" s="20" t="inlineStr">
         <is>
           <t>PNAS : Venus figurines - Conard &amp; Malina (2008)</t>
         </is>
       </c>
-      <c r="D496" t="inlineStr">
+      <c r="D496" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0710975105</t>
         </is>
       </c>
     </row>
     <row r="497">
-      <c r="A497" t="n">
+      <c r="A497" s="20" t="n">
         <v>315</v>
       </c>
-      <c r="B497" t="inlineStr">
+      <c r="B497" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C497" t="inlineStr">
+      <c r="C497" s="20" t="inlineStr">
         <is>
           <t>Current Biology : Dating of Venus figurines - Higham et al. (2012)</t>
         </is>
       </c>
-      <c r="D497" t="inlineStr">
+      <c r="D497" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cub.2012.07.021</t>
         </is>
       </c>
     </row>
     <row r="498">
-      <c r="A498" t="n">
+      <c r="A498" s="20" t="n">
         <v>316</v>
       </c>
-      <c r="B498" t="inlineStr">
+      <c r="B498" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C498" t="inlineStr">
+      <c r="C498" s="20" t="inlineStr">
         <is>
           <t>Nature : Dating and study of Chauvet Cave - Clottes et al. (1995)</t>
         </is>
       </c>
-      <c r="D498" t="inlineStr">
+      <c r="D498" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/375231a0</t>
         </is>
       </c>
     </row>
     <row r="499">
-      <c r="A499" t="n">
+      <c r="A499" s="20" t="n">
         <v>316</v>
       </c>
-      <c r="B499" t="inlineStr">
+      <c r="B499" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C499" t="inlineStr">
+      <c r="C499" s="20" t="inlineStr">
         <is>
           <t>PNAS : Chauvet Cave radiocarbon dating - Quiles et al. (2016)</t>
         </is>
       </c>
-      <c r="D499" t="inlineStr">
+      <c r="D499" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1502651112</t>
         </is>
       </c>
     </row>
     <row r="500">
-      <c r="A500" t="n">
+      <c r="A500" s="20" t="n">
         <v>316</v>
       </c>
-      <c r="B500" t="inlineStr">
+      <c r="B500" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C500" t="inlineStr">
+      <c r="C500" s="20" t="inlineStr">
         <is>
           <t>Journal of Human Evolution : Interpretation of Paleolithic art - Lewis-Williams (2002)</t>
         </is>
       </c>
-      <c r="D500" t="inlineStr">
+      <c r="D500" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S0047-2484(02)00024-4</t>
         </is>
       </c>
     </row>
     <row r="501">
-      <c r="A501" t="n">
+      <c r="A501" s="20" t="n">
         <v>317</v>
       </c>
-      <c r="B501" t="inlineStr">
+      <c r="B501" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C501" t="inlineStr">
+      <c r="C501" s="20" t="inlineStr">
         <is>
           <t>Journal of Archaeological Science : Early bow and arrow technology - Shea &amp; Sisk (2010)</t>
         </is>
       </c>
-      <c r="D501" t="inlineStr">
+      <c r="D501" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jas.2009.11.013</t>
         </is>
       </c>
     </row>
     <row r="502">
-      <c r="A502" t="n">
+      <c r="A502" s="20" t="n">
         <v>317</v>
       </c>
-      <c r="B502" t="inlineStr">
+      <c r="B502" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C502" t="inlineStr">
+      <c r="C502" s="20" t="inlineStr">
         <is>
           <t>PNAS : Origin of projectile weaponry - Lombard &amp; Phillipson (2010)</t>
         </is>
       </c>
-      <c r="D502" t="inlineStr">
+      <c r="D502" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1001885107</t>
         </is>
       </c>
     </row>
     <row r="503">
-      <c r="A503" t="n">
+      <c r="A503" s="20" t="n">
         <v>317</v>
       </c>
-      <c r="B503" t="inlineStr">
+      <c r="B503" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C503" t="inlineStr">
+      <c r="C503" s="20" t="inlineStr">
         <is>
           <t>American Antiquity : African origins of archery - Lombard (2005)</t>
         </is>
       </c>
-      <c r="D503" t="inlineStr">
+      <c r="D503" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.2307/40035648</t>
         </is>
       </c>
     </row>
     <row r="504">
-      <c r="A504" t="n">
+      <c r="A504" s="20" t="n">
         <v>318</v>
       </c>
-      <c r="B504" t="inlineStr">
+      <c r="B504" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C504" t="inlineStr">
+      <c r="C504" s="20" t="inlineStr">
         <is>
           <t>Science : Last Glacial Maximum reconstruction - Mix et al. (2001)</t>
         </is>
       </c>
-      <c r="D504" t="inlineStr">
+      <c r="D504" s="20" t="inlineStr">
         <is>
           <t>https://www.science.org/doi/10.1126/science.1059133</t>
         </is>
       </c>
     </row>
     <row r="505">
-      <c r="A505" t="n">
+      <c r="A505" s="20" t="n">
         <v>318</v>
       </c>
-      <c r="B505" t="inlineStr">
+      <c r="B505" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C505" t="inlineStr">
+      <c r="C505" s="20" t="inlineStr">
         <is>
           <t>Quaternary Research : Human adaptation to LGM - Gamble (1999)</t>
         </is>
       </c>
-      <c r="D505" t="inlineStr">
+      <c r="D505" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1006/qres.1999.2080</t>
         </is>
       </c>
     </row>
     <row r="506">
-      <c r="A506" t="n">
+      <c r="A506" s="20" t="n">
         <v>318</v>
       </c>
-      <c r="B506" t="inlineStr">
+      <c r="B506" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C506" t="inlineStr">
+      <c r="C506" s="20" t="inlineStr">
         <is>
           <t>PNAS : Population genetics of Last Glacial Maximum - Excoffier et al. (2005)</t>
         </is>
       </c>
-      <c r="D506" t="inlineStr">
+      <c r="D506" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0500448102</t>
         </is>
       </c>
     </row>
     <row r="507">
-      <c r="A507" t="n">
+      <c r="A507" s="20" t="n">
         <v>319</v>
       </c>
-      <c r="B507" t="inlineStr">
+      <c r="B507" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C507" t="inlineStr">
+      <c r="C507" s="20" t="inlineStr">
         <is>
           <t>PNAS : Ancient dog genomics - Parker et al. (2004)</t>
         </is>
       </c>
-      <c r="D507" t="inlineStr">
+      <c r="D507" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0401913101</t>
         </is>
       </c>
     </row>
     <row r="508">
-      <c r="A508" t="n">
+      <c r="A508" s="20" t="n">
         <v>319</v>
       </c>
-      <c r="B508" t="inlineStr">
+      <c r="B508" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C508" t="inlineStr">
+      <c r="C508" s="20" t="inlineStr">
         <is>
           <t>Nature Ecology &amp; Evolution : Early dog domestication - Larson et al. (2012)</t>
         </is>
       </c>
-      <c r="D508" t="inlineStr">
+      <c r="D508" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature11159</t>
         </is>
       </c>
     </row>
     <row r="509">
-      <c r="A509" t="n">
+      <c r="A509" s="20" t="n">
         <v>319</v>
       </c>
-      <c r="B509" t="inlineStr">
+      <c r="B509" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C509" t="inlineStr">
+      <c r="C509" s="20" t="inlineStr">
         <is>
           <t>Current Biology : Dog domestication genetics - Freedman et al. (2014)</t>
         </is>
       </c>
-      <c r="D509" t="inlineStr">
+      <c r="D509" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cub.2014.03.024</t>
         </is>
       </c>
     </row>
     <row r="510">
-      <c r="A510" t="n">
+      <c r="A510" s="20" t="n">
         <v>320</v>
       </c>
-      <c r="B510" t="inlineStr">
+      <c r="B510" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C510" t="inlineStr">
+      <c r="C510" s="20" t="inlineStr">
         <is>
           <t>Nature : Holocene climate change and human settlement - Mayewski et al. (2004)</t>
         </is>
       </c>
-      <c r="D510" t="inlineStr">
+      <c r="D510" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature02805</t>
         </is>
       </c>
     </row>
     <row r="511">
-      <c r="A511" t="n">
+      <c r="A511" s="20" t="n">
         <v>320</v>
       </c>
-      <c r="B511" t="inlineStr">
+      <c r="B511" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C511" t="inlineStr">
+      <c r="C511" s="20" t="inlineStr">
         <is>
           <t>PNAS : Younger Dryas climate event - Firestone et al. (2007)</t>
         </is>
       </c>
-      <c r="D511" t="inlineStr">
+      <c r="D511" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0707213104</t>
         </is>
       </c>
     </row>
     <row r="512">
-      <c r="A512" t="n">
+      <c r="A512" s="20" t="n">
         <v>320</v>
       </c>
-      <c r="B512" t="inlineStr">
+      <c r="B512" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C512" t="inlineStr">
+      <c r="C512" s="20" t="inlineStr">
         <is>
           <t>Quaternary Science Reviews : Climate transitions and cultural change - Roberts &amp; Brayshaw (2002)</t>
         </is>
       </c>
-      <c r="D512" t="inlineStr">
+      <c r="D512" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S0277-3791(01)00083-3</t>
         </is>
       </c>
     </row>
     <row r="513">
-      <c r="A513" t="n">
+      <c r="A513" s="20" t="n">
         <v>321</v>
       </c>
-      <c r="B513" t="inlineStr">
+      <c r="B513" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C513" t="inlineStr">
+      <c r="C513" s="20" t="inlineStr">
         <is>
           <t>PNAS : Origins of agriculture in the Fertile Crescent - Zeder (2011)</t>
         </is>
       </c>
-      <c r="D513" t="inlineStr">
+      <c r="D513" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.1100999108</t>
         </is>
       </c>
     </row>
     <row r="514">
-      <c r="A514" t="n">
+      <c r="A514" s="20" t="n">
         <v>321</v>
       </c>
-      <c r="B514" t="inlineStr">
+      <c r="B514" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C514" t="inlineStr">
+      <c r="C514" s="20" t="inlineStr">
         <is>
           <t>Journal of Archaeological Research : Neolithic transition - Bellwood (2005)</t>
         </is>
       </c>
-      <c r="D514" t="inlineStr">
+      <c r="D514" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s10814-005-6142-0</t>
         </is>
       </c>
     </row>
     <row r="515">
-      <c r="A515" t="n">
+      <c r="A515" s="20" t="n">
         <v>321</v>
       </c>
-      <c r="B515" t="inlineStr">
+      <c r="B515" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C515" t="inlineStr">
+      <c r="C515" s="20" t="inlineStr">
         <is>
           <t>Nature : Early crop development - Purugganan &amp; Fuller (2009)</t>
         </is>
       </c>
-      <c r="D515" t="inlineStr">
+      <c r="D515" s="20" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/nature08808</t>
         </is>
       </c>
     </row>
     <row r="516">
-      <c r="A516" t="n">
+      <c r="A516" s="20" t="n">
         <v>322</v>
       </c>
-      <c r="B516" t="inlineStr">
+      <c r="B516" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C516" t="inlineStr">
+      <c r="C516" s="20" t="inlineStr">
         <is>
           <t>PNAS : Wheat domestication - Tanno &amp; Willcox (2006)</t>
         </is>
       </c>
-      <c r="D516" t="inlineStr">
+      <c r="D516" s="20" t="inlineStr">
         <is>
           <t>https://www.pnas.org/doi/10.1073/pnas.0510618103</t>
         </is>
       </c>
     </row>
     <row r="517">
-      <c r="A517" t="n">
+      <c r="A517" s="20" t="n">
         <v>322</v>
       </c>
-      <c r="B517" t="inlineStr">
+      <c r="B517" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C517" t="inlineStr">
+      <c r="C517" s="20" t="inlineStr">
         <is>
           <t>Journal of Archaeological Science : Barley domestication in the Near East - Badr et al. (2000)</t>
         </is>
       </c>
-      <c r="D517" t="inlineStr">
+      <c r="D517" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1006/jasc.2000.0520</t>
         </is>
       </c>
     </row>
     <row r="518">
-      <c r="A518" t="n">
+      <c r="A518" s="20" t="n">
         <v>322</v>
       </c>
-      <c r="B518" t="inlineStr">
+      <c r="B518" s="20" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
       </c>
-      <c r="C518" t="inlineStr">
+      <c r="C518" s="20" t="inlineStr">
         <is>
           <t>Current Biology : Early wheat and barley cultivation - Fuller et al. (2011)</t>
         </is>
       </c>
-      <c r="D518" t="inlineStr">
+      <c r="D518" s="20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cub.2011.06.045</t>
         </is>

</xml_diff>

<commit_message>
Categories bonus (Cinema/TV/Jeux video/Manga) + fantome de drag corrige
- Cinema, Television et Jeux video passent en categories "bonus" :
  decochees par defaut, regroupees a la fin de la liste des filtres,
  avec un style dore pour bien les distinguer des categories normales.
- Nouvelle categorie Manga (bonus egalement) avec 15 cartes sur les
  mangas les plus connus (One Piece, Dragon Ball, Naruto, Death Note,
  Attaque des Titans, Demon Slayer, etc.), date = premiere parution du
  tome 1.
- Le fantome affiche pendant un glisser-deposer montre desormais toute
  la carte (bordure, titre, date) et non plus seulement l'image brute :
  les <img> de carte etaient nativement "draggable" par le navigateur,
  ce qui court-circuitait le drag-and-drop personnalise du parent.
</commit_message>
<xml_diff>
--- a/data/cartes_maitre.xlsx
+++ b/data/cartes_maitre.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L460"/>
+  <dimension ref="A1:L475"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="44.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7.04" customWidth="1" style="10" min="1" max="1"/>
@@ -23335,6 +23335,651 @@
         </is>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" s="16" t="n">
+        <v>460</v>
+      </c>
+      <c r="B461" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C461" s="16" t="inlineStr">
+        <is>
+          <t>One Piece - Tome 1</t>
+        </is>
+      </c>
+      <c r="D461" s="16" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E461" s="16" t="inlineStr">
+        <is>
+          <t>Eiichirō Oda publie le premier tome de One Piece, qui deviendra le manga le plus vendu de l'histoire.</t>
+        </is>
+      </c>
+      <c r="F461" s="16" t="inlineStr">
+        <is>
+          <t>Après un peu plus de cinq mois de prépublication hebdomadaire dans le Weekly Shōnen Jump, Eiichirō Oda voit son manga de pirates compilé pour la première fois en un tome relié le 24 décembre 1997. L'histoire suit Monkey D. Luffy, un jeune pirate au corps élastique après avoir mangé un fruit du démon, parti à la recherche du trésor légendaire « One Piece » pour devenir le roi des pirates. Le succès, modeste au départ, grandit progressivement jusqu'à faire de la série le manga le plus vendu de tous les temps, avec plus de 500 millions d'exemplaires écoulés dans le monde et une adaptation animée diffusée sans interruption depuis 1999.</t>
+        </is>
+      </c>
+      <c r="G461" s="16" t="inlineStr">
+        <is>
+          <t>Eiichirō Oda affirme avoir déjà écrit la scène finale de la série dans un cahier tenu secret dès les débuts de la prépublication - un scénario complet qu'il suivrait depuis l'origine, malgré des dizaines de milliers de pages publiées entretemps.</t>
+        </is>
+      </c>
+      <c r="H461" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J461" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="16" t="n">
+        <v>461</v>
+      </c>
+      <c r="B462" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C462" s="16" t="inlineStr">
+        <is>
+          <t>Dragon Ball - Tome 1</t>
+        </is>
+      </c>
+      <c r="D462" s="16" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E462" s="16" t="inlineStr">
+        <is>
+          <t>Akira Toriyama publie le premier tome de Dragon Ball, qui va populariser le manga et l'anime en Occident.</t>
+        </is>
+      </c>
+      <c r="F462" s="16" t="inlineStr">
+        <is>
+          <t>Sérialisé depuis novembre 1984 dans le Weekly Shōnen Jump, Dragon Ball d'Akira Toriyama est compilé en un premier tome relié le 10 septembre 1985. Inspiré du roman classique chinois La Pérégrination vers l'Ouest, le manga suit Son Goku, jeune garçon à la force surhumaine et à la queue de singe, parti à la recherche des sept Dragon Balls capables d'exaucer un vœu. Vendue à plus de 260 millions d'exemplaires dans le monde, la série et son adaptation animée jouent un rôle déterminant dans la popularisation du manga et de l'anime hors du Japon, en particulier en France dans les années 1990.</t>
+        </is>
+      </c>
+      <c r="G462" s="16" t="inlineStr">
+        <is>
+          <t>Le nom « Dragon Ball » ferait en partie référence à un jeu de mots avec le sport du baseball, dont Toriyama était très amateur, bien que l'inspiration principale du récit reste le roman chinois La Pérégrination vers l'Ouest.</t>
+        </is>
+      </c>
+      <c r="H462" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J462" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="16" t="n">
+        <v>462</v>
+      </c>
+      <c r="B463" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C463" s="16" t="inlineStr">
+        <is>
+          <t>Naruto - Tome 1</t>
+        </is>
+      </c>
+      <c r="D463" s="16" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E463" s="16" t="inlineStr">
+        <is>
+          <t>Masashi Kishimoto publie le premier tome de Naruto, pilier du Weekly Shōnen Jump des années 2000.</t>
+        </is>
+      </c>
+      <c r="F463" s="16" t="inlineStr">
+        <is>
+          <t>Après ses débuts en septembre 1999 dans le Weekly Shōnen Jump, Naruto est compilé en un premier tome relié le 3 mars 2000. Le manga de Masashi Kishimoto suit Naruto Uzumaki, jeune ninja rejeté par les habitants de son village parce qu'il abrite en lui un démon-renard scellé à sa naissance, et dont le rêve est de devenir le chef (Hokage) de son village pour être enfin reconnu. Vendue à plus de 250 millions d'exemplaires dans le monde, la série contribue fortement, aux côtés de One Piece et Bleach, à ce que la presse spécialisée surnomme le « Big Three » du Weekly Shōnen Jump des années 2000.</t>
+        </is>
+      </c>
+      <c r="G463" s="16" t="inlineStr">
+        <is>
+          <t>Masashi Kishimoto avait initialement conçu Naruto comme un ninja capable de se transformer littéralement en renard et obsédé par la nourriture plutôt que par les ramens - des idées abandonnées avant la publication du tout premier chapitre.</t>
+        </is>
+      </c>
+      <c r="H463" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J463" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="16" t="n">
+        <v>463</v>
+      </c>
+      <c r="B464" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C464" s="16" t="inlineStr">
+        <is>
+          <t>Détective Conan - Tome 1</t>
+        </is>
+      </c>
+      <c r="D464" s="16" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E464" s="16" t="inlineStr">
+        <is>
+          <t>Gōshō Aoyama publie le premier tome de Détective Conan, devenu un phénomène culturel au Japon.</t>
+        </is>
+      </c>
+      <c r="F464" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis janvier 1994 dans le Weekly Shōnen Sunday, Détective Conan (Meitantei Conan) de Gōshō Aoyama est compilé en un premier tome le 18 juin 1994. L'histoire suit Shin'ichi Kudō, lycéen surdoué en résolution d'enquêtes, transformé malgré lui en enfant de six ans après avoir été empoisonné par une organisation criminelle, et contraint de vivre caché sous l'identité de « Conan Edogawa » tout en continuant secrètement à résoudre des affaires criminelles. Avec plus de 250 millions d'exemplaires vendus, la série est devenue l'un des piliers du manga policier et un phénomène culturel durable au Japon, où son adaptation animée et ses films sortent en salle chaque année depuis 1997.</t>
+        </is>
+      </c>
+      <c r="G464" s="16" t="inlineStr">
+        <is>
+          <t>Le nom d'emprunt « Conan Edogawa » choisi par le héros est un double hommage voulu par Gōshō Aoyama : à l'écrivain britannique Arthur Conan Doyle, créateur de Sherlock Holmes, et au romancier japonais Edogawa Ranpo, pionnier du roman policier nippon.</t>
+        </is>
+      </c>
+      <c r="H464" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J464" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="16" t="n">
+        <v>464</v>
+      </c>
+      <c r="B465" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C465" s="16" t="inlineStr">
+        <is>
+          <t>Slam Dunk - Tome 1</t>
+        </is>
+      </c>
+      <c r="D465" s="16" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E465" s="16" t="inlineStr">
+        <is>
+          <t>Takehiko Inoue publie le premier tome de Slam Dunk, manga de basket-ball culte au Japon.</t>
+        </is>
+      </c>
+      <c r="F465" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis octobre 1990 dans le Weekly Shōnen Jump, Slam Dunk de Takehiko Inoue est compilé en un premier tome le 18 septembre 1990. Le manga suit Hanamichi Sakuragi, lycéen bagarreur au tempérament explosif, qui rejoint le club de basket-ball de son lycée dans l'espoir de séduire une camarade et découvre peu à peu une véritable passion pour ce sport. Vendue à plus de 170 millions d'exemplaires, la série est créditée d'avoir considérablement popularisé la pratique du basket-ball auprès des jeunes Japonais dans les années 1990.</t>
+        </is>
+      </c>
+      <c r="G465" s="16" t="inlineStr">
+        <is>
+          <t>Takehiko Inoue a mis fin à la série à l'apogée de sa popularité commerciale, contre l'avis de son éditeur, afin de préserver la cohérence de son histoire plutôt que de la prolonger artificiellement - un choix rare dans l'industrie du manga.</t>
+        </is>
+      </c>
+      <c r="H465" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J465" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="16" t="n">
+        <v>465</v>
+      </c>
+      <c r="B466" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C466" s="16" t="inlineStr">
+        <is>
+          <t>Demon Slayer - Tome 1</t>
+        </is>
+      </c>
+      <c r="D466" s="16" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E466" s="16" t="inlineStr">
+        <is>
+          <t>Koyoharu Gotōge publie le premier tome de Demon Slayer, futur phénomène mondial de la fin des années 2010.</t>
+        </is>
+      </c>
+      <c r="F466" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis février 2016 dans le Weekly Shōnen Jump, Kimetsu no Yaiba (Demon Slayer) de Koyoharu Gotōge est compilé en un premier tome le 3 juin 2016. Le manga suit Tanjirō Kamado, jeune garçon devenu pourfendeur de démons après le massacre de sa famille et la transformation de sa sœur cadette Nezuko en démone, qu'il cherche à guérir tout en la protégeant. D'abord modestement accueillie, la série connaît un succès fulgurant à partir de 2019 grâce à son adaptation animée par le studio ufotable, dépassant les 150 millions d'exemplaires vendus et devenant un phénomène culturel mondial, porté notamment par le succès record du film Le Train de l'infini au box-office japonais.</t>
+        </is>
+      </c>
+      <c r="G466" s="16" t="inlineStr">
+        <is>
+          <t>Koyoharu Gotōge, dont le visage et le genre n'ont jamais été officiellement dévoilés au public, se représente exclusivement sous la forme d'un dessin d'alligator portant des lunettes dans ses apparitions et remerciements publiés en fin de tome.</t>
+        </is>
+      </c>
+      <c r="H466" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J466" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="16" t="n">
+        <v>466</v>
+      </c>
+      <c r="B467" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C467" s="16" t="inlineStr">
+        <is>
+          <t>L'Attaque des Titans - Tome 1</t>
+        </is>
+      </c>
+      <c r="D467" s="16" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E467" s="16" t="inlineStr">
+        <is>
+          <t>Hajime Isayama publie le premier tome de L'Attaque des Titans, dont l'intrigue bouleverse les codes du manga d'action.</t>
+        </is>
+      </c>
+      <c r="F467" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis septembre 2009 dans le Bessatsu Shōnen Magazine, Shingeki no Kyojin (L'Attaque des Titans) de Hajime Isayama est compilé en un premier tome le 17 mars 2010. L'histoire se déroule dans un monde où l'humanité survit retranchée derrière d'immenses murailles, seule protection contre des géants humanoïdes dévoreurs d'hommes appelés Titans, et suit Eren Jäger après la destruction de son village natal. Reconnue pour la noirceur de son intrigue et ses multiples retournements narratifs, la série se vend à plus de 140 millions d'exemplaires et son adaptation animée, débutée en 2013, est saluée comme l'une des plus marquantes de la décennie 2010.</t>
+        </is>
+      </c>
+      <c r="G467" s="16" t="inlineStr">
+        <is>
+          <t>Hajime Isayama a expliqué avoir eu l'idée des Titans après une rencontre déroutante avec un client ivre au comportement agressif et disproportionné dans un bar - une image d'irrationalité écrasante face à laquelle l'humanité serait totalement démunie.</t>
+        </is>
+      </c>
+      <c r="H467" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J467" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="16" t="n">
+        <v>467</v>
+      </c>
+      <c r="B468" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C468" s="16" t="inlineStr">
+        <is>
+          <t>Death Note - Tome 1</t>
+        </is>
+      </c>
+      <c r="D468" s="16" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E468" s="16" t="inlineStr">
+        <is>
+          <t>Tsugumi Ōba et Takeshi Obata publient le premier tome de Death Note, thriller psychologique devenu culte.</t>
+        </is>
+      </c>
+      <c r="F468" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis décembre 2003 dans le Weekly Shōnen Jump, Death Note, scénarisé par Tsugumi Ōba et dessiné par Takeshi Obata, est compilé en un premier tome le 2 avril 2004. Le manga suit Light Yagami, lycéen brillant qui trouve un cahier surnaturel permettant de tuer quiconque dont le nom y est inscrit, et qui entreprend d'éliminer les criminels du monde entier pour devenir le dieu d'un nouvel ordre moral, avant d'être traqué par un détective énigmatique surnommé L. Salué pour la sophistication de son intrigue en forme de duel intellectuel, le manga se vend à plus de 30 millions d'exemplaires et connaît plusieurs adaptations, en anime comme au cinéma.</t>
+        </is>
+      </c>
+      <c r="G468" s="16" t="inlineStr">
+        <is>
+          <t>L'identité réelle de Tsugumi Ōba, scénariste de la série, n'a jamais été révélée publiquement : le nom est un pseudonyme, et même le genre de l'auteur n'a jamais été confirmé officiellement par l'éditeur Shūeisha.</t>
+        </is>
+      </c>
+      <c r="H468" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J468" s="16" t="inlineStr">
+        <is>
+          <t>facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="16" t="n">
+        <v>468</v>
+      </c>
+      <c r="B469" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C469" s="16" t="inlineStr">
+        <is>
+          <t>Fullmetal Alchemist - Tome 1</t>
+        </is>
+      </c>
+      <c r="D469" s="16" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E469" s="16" t="inlineStr">
+        <is>
+          <t>Hiromu Arakawa publie le premier tome de Fullmetal Alchemist, saga d'alchimie saluée pour la rigueur de son scénario.</t>
+        </is>
+      </c>
+      <c r="F469" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis juillet 2001 dans le magazine Monthly Shōnen Gangan, Hagane no Renkinjutsushi (Fullmetal Alchemist) d'Hiromu Arakawa est compilé en un premier tome le 22 janvier 2002. L'histoire suit les frères Edward et Alphonse Elric, jeunes alchimistes ayant perdu respectivement un bras et une jambe, et un corps entier, lors d'une tentative interdite de ressusciter leur mère, et partis à la recherche de la légendaire pierre philosophale pour retrouver ce qu'ils ont perdu. Saluée pour la cohérence de son univers fondé sur la loi de l'échange équivalent, la série se vend à plus de 80 millions d'exemplaires et est réputée, fait rare, pour avoir mené à terme dans le manga sa propre histoire complète après qu'une première adaptation animée s'en fut écartée.</t>
+        </is>
+      </c>
+      <c r="G469" s="16" t="inlineStr">
+        <is>
+          <t>Hiromu Arakawa, ancienne fille d'éleveurs de vaches laitières à Hokkaidō avant de devenir mangaka, se représente traditionnellement sous les traits d'une vache dans ses apparitions et notes d'auteur, plutôt que sous son apparence réelle.</t>
+        </is>
+      </c>
+      <c r="H469" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J469" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="16" t="n">
+        <v>469</v>
+      </c>
+      <c r="B470" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C470" s="16" t="inlineStr">
+        <is>
+          <t>My Hero Academia - Tome 1</t>
+        </is>
+      </c>
+      <c r="D470" s="16" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E470" s="16" t="inlineStr">
+        <is>
+          <t>Kōhei Horikoshi publie le premier tome de My Hero Academia, qui relance le genre du super-héros dans le manga.</t>
+        </is>
+      </c>
+      <c r="F470" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis juillet 2014 dans le Weekly Shōnen Jump, Boku no Hero Academia (My Hero Academia) de Kōhei Horikoshi est compilé en un premier tome le 4 novembre 2014. Dans un monde où 80% de la population possède un pouvoir surnaturel appelé « Alter », le manga suit Izuku Midoriya, l'un des rares nés sans pouvoir, qui rêve malgré tout de devenir un héros professionnel et se voit transmettre exceptionnellement le pouvoir du plus grand héros en exercice, All Might. Portée par un mélange d'action, d'humour et de formation initiatique façon lycée de super-héros, la série dépasse les 90 millions d'exemplaires vendus et contribue au renouveau du genre super-héroïque dans le manga des années 2010.</t>
+        </is>
+      </c>
+      <c r="G470" s="16" t="inlineStr">
+        <is>
+          <t>Kōhei Horikoshi avait conçu plusieurs projets préliminaires également centrés sur les super-pouvoirs avant My Hero Academia, refusés par son éditeur car jugés trop proches des comics américains plutôt que d'un manga shōnen classique.</t>
+        </is>
+      </c>
+      <c r="H470" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J470" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="16" t="n">
+        <v>470</v>
+      </c>
+      <c r="B471" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C471" s="16" t="inlineStr">
+        <is>
+          <t>Bleach - Tome 1</t>
+        </is>
+      </c>
+      <c r="D471" s="16" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E471" s="16" t="inlineStr">
+        <is>
+          <t>Tite Kubo publie le premier tome de Bleach, qui rejoindra Naruto et One Piece au sommet du Shōnen Jump.</t>
+        </is>
+      </c>
+      <c r="F471" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis août 2001 dans le Weekly Shōnen Jump, Bleach de Tite Kubo est compilé en un premier tome le 5 janvier 2002. Le manga suit Ichigo Kurosaki, lycéen capable de voir les fantômes, qui hérite malgré lui des pouvoirs d'un shinigami (dieu de la mort) chargé de guider les âmes des défunts vers l'au-delà et de combattre les esprits maléfiques appelés Hollows. Portée par un univers visuel très marqué et des combats chorégraphiés, la série se vend à plus de 130 millions d'exemplaires et fait, aux côtés de One Piece et Naruto, partie du « Big Three » ayant dominé le Weekly Shōnen Jump durant les années 2000.</t>
+        </is>
+      </c>
+      <c r="G471" s="16" t="inlineStr">
+        <is>
+          <t>Le titre « Bleach » (eau de Javel) n'a aucun rapport direct avec l'intrigue : Tite Kubo l'aurait choisi pour l'association visuelle entre le blanc de l'eau de Javel et la robe des shinigamis, qu'il imaginait à l'origine presque blanche avant d'opter finalement pour le noir.</t>
+        </is>
+      </c>
+      <c r="H471" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J471" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="16" t="n">
+        <v>471</v>
+      </c>
+      <c r="B472" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C472" s="16" t="inlineStr">
+        <is>
+          <t>JoJo's Bizarre Adventure - Tome 1</t>
+        </is>
+      </c>
+      <c r="D472" s="16" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E472" s="16" t="inlineStr">
+        <is>
+          <t>Hirohiko Araki publie le premier tome de JoJo's Bizarre Adventure, saga culte à l'esthétique unique.</t>
+        </is>
+      </c>
+      <c r="F472" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis janvier 1987 dans le Weekly Shōnen Jump, JoJo no Kimyō na Bōken (JoJo's Bizarre Adventure) d'Hirohiko Araki est compilé en un premier tome le 10 août 1987. La série, organisée en plusieurs parties indépendantes centrées chacune sur un descendant différent de la famille Joestar, débute avec l'affrontement entre Jonathan Joestar et son frère adoptif Dio Brando devenu vampire. Reconnaissable entre tous les mangas pour son style graphique très maniériste inspiré de la mode et de la sculpture occidentales, ainsi que pour l'introduction du concept des « Stands » à partir de sa troisième partie, la série s'est vendue à plus de 120 millions d'exemplaires et exerce une influence marquée sur l'esthétique manga et la pop culture japonaise.</t>
+        </is>
+      </c>
+      <c r="G472" s="16" t="inlineStr">
+        <is>
+          <t>Hirohiko Araki, passionné de peinture de la Renaissance italienne, aurait puisé une grande partie de ses poses de personnages emblématiques - souvent qualifiées de « poses JoJo » par les fans - directement dans des tableaux classiques et des publicités de mode occidentales des années 1980.</t>
+        </is>
+      </c>
+      <c r="H472" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J472" s="16" t="inlineStr">
+        <is>
+          <t>difficile</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="16" t="n">
+        <v>472</v>
+      </c>
+      <c r="B473" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C473" s="16" t="inlineStr">
+        <is>
+          <t>Sailor Moon - Tome 1</t>
+        </is>
+      </c>
+      <c r="D473" s="16" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E473" s="16" t="inlineStr">
+        <is>
+          <t>Naoko Takeuchi publie le premier tome de Sailor Moon, série fondatrice du genre magical girl moderne.</t>
+        </is>
+      </c>
+      <c r="F473" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis février 1992 dans le magazine mensuel Nakayoshi, Bishōjo Senshi Sailor Moon de Naoko Takeuchi est compilé en un premier tome le 6 juillet 1992. Le manga suit Usagi Tsukino, collégienne maladroite qui découvre pouvoir se transformer en guerrière légendaire, Sailor Moon, aux côtés d'autres héroïnes incarnant chacune une planète du système solaire, pour combattre les forces du mal et protéger la Terre. Best-seller mondial du genre « magical girl » avec plus de 46 millions d'exemplaires vendus, la série a durablement marqué la culture populaire des années 1990 et a largement contribué, via son adaptation animée diffusée dans de nombreux pays dont la France, à l'essor international du manga auprès d'un jeune public féminin.</t>
+        </is>
+      </c>
+      <c r="G473" s="16" t="inlineStr">
+        <is>
+          <t>Naoko Takeuchi avait initialement imaginé le personnage principal comme un garçon avant de le transformer en héroïne féminine, une décision qui donnera naissance à l'un des archétypes les plus copiés de l'histoire du manga.</t>
+        </is>
+      </c>
+      <c r="H473" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J473" s="16" t="inlineStr">
+        <is>
+          <t>moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="16" t="n">
+        <v>473</v>
+      </c>
+      <c r="B474" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C474" s="16" t="inlineStr">
+        <is>
+          <t>Akira - Tome 1</t>
+        </is>
+      </c>
+      <c r="D474" s="16" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E474" s="16" t="inlineStr">
+        <is>
+          <t>Katsuhiro Ōtomo publie le premier tome d'Akira, chef-d'œuvre de science-fiction qui va révolutionner le manga et l'animation.</t>
+        </is>
+      </c>
+      <c r="F474" s="16" t="inlineStr">
+        <is>
+          <t>Prépublié depuis décembre 1982 dans le magazine Young Magazine, Akira de Katsuhiro Ōtomo est compilé en un premier tome le 14 septembre 1984. L'histoire se déroule dans le Néo-Tokyo dystopique de 2019, reconstruit après la destruction de la capitale japonaise par une explosion mystérieuse, et suit un jeune motard, Tetsuo Shima, dont les pouvoirs psychiques incontrôlables menacent de déclencher une nouvelle catastrophe. Salué pour la précision quasi architecturale de son dessin et la noirceur de son propos, le manga inspire directement le film d'animation homonyme réalisé par Ōtomo lui-même en 1988, considéré comme l'un des jalons majeurs ayant fait connaître l'animation japonaise en Occident.</t>
+        </is>
+      </c>
+      <c r="G474" s="16" t="inlineStr">
+        <is>
+          <t>Katsuhiro Ōtomo aurait dessiné certaines planches d'Akira représentant la destruction de Tokyo avec un tel luxe de détails architecturaux qu'elles ont, par la suite, été citées en exemple par des urbanistes japonais pour illustrer des scénarios de reconstruction urbaine post-catastrophe.</t>
+        </is>
+      </c>
+      <c r="H474" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J474" s="16" t="inlineStr">
+        <is>
+          <t>difficile</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="16" t="n">
+        <v>474</v>
+      </c>
+      <c r="B475" s="16" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="C475" s="16" t="inlineStr">
+        <is>
+          <t>Astro Boy</t>
+        </is>
+      </c>
+      <c r="D475" s="16" t="n">
+        <v>1952</v>
+      </c>
+      <c r="E475" s="16" t="inlineStr">
+        <is>
+          <t>Osamu Tezuka lance la prépublication d'Astro Boy, œuvre fondatrice qui façonne les codes du manga moderne.</t>
+        </is>
+      </c>
+      <c r="F475" s="16" t="inlineStr">
+        <is>
+          <t>Le 3 avril 1952, Osamu Tezuka entame dans le magazine Shōnen la prépublication de Tetsuwan Atom (Astro Boy), l'histoire d'un robot à l'apparence d'enfant, doté de sentiments et de super-pouvoirs, créé par un savant en deuil de son fils puis adopté par un second scientifique qui en fait un défenseur de la justice. Surnommé le « dieu du manga », Tezuka y invente ou popularise nombre de codes graphiques et narratifs devenus des standards du médium (grands yeux expressifs, découpage cinématographique des cases, thématiques de science-fiction morale). La série, prépubliée jusqu'en 1968, donne naissance en 1963 à la première série d'animation télévisée japonaise hebdomadaire, posant les fondations industrielles et esthétiques de l'anime moderne.</t>
+        </is>
+      </c>
+      <c r="G475" s="16" t="inlineStr">
+        <is>
+          <t>Osamu Tezuka, également docteur en médecine, a doté Astro Boy d'une date de naissance officielle fixée au 7 avril 2003 par la fiction elle-même - une date qui a donné lieu, au Japon, à de véritables commémorations médiatiques et scientifiques lorsqu'elle a été atteinte dans la réalité.</t>
+        </is>
+      </c>
+      <c r="H475" s="16" t="inlineStr">
+        <is>
+          <t>Avéré</t>
+        </is>
+      </c>
+      <c r="J475" s="16" t="inlineStr">
+        <is>
+          <t>difficile</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -23348,7 +23993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F912"/>
+  <dimension ref="A1:F938"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="16" min="1" max="1"/>
@@ -41609,6 +42254,526 @@
         </is>
       </c>
     </row>
+    <row r="913">
+      <c r="A913" s="16" t="n">
+        <v>460</v>
+      </c>
+      <c r="B913" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C913" s="16" t="inlineStr">
+        <is>
+          <t>One Piece (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D913" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/One_Piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="16" t="n">
+        <v>460</v>
+      </c>
+      <c r="B914" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C914" s="16" t="inlineStr">
+        <is>
+          <t>Eiichirō Oda (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D914" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Eiichir%C5%8D_Oda</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="16" t="n">
+        <v>461</v>
+      </c>
+      <c r="B915" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C915" s="16" t="inlineStr">
+        <is>
+          <t>Dragon Ball (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D915" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Dragon_Ball</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="16" t="n">
+        <v>461</v>
+      </c>
+      <c r="B916" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C916" s="16" t="inlineStr">
+        <is>
+          <t>Akira Toriyama (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D916" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Akira_Toriyama</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="16" t="n">
+        <v>462</v>
+      </c>
+      <c r="B917" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C917" s="16" t="inlineStr">
+        <is>
+          <t>Naruto (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D917" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Naruto</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="16" t="n">
+        <v>462</v>
+      </c>
+      <c r="B918" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C918" s="16" t="inlineStr">
+        <is>
+          <t>Masashi Kishimoto (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D918" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Masashi_Kishimoto</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="16" t="n">
+        <v>463</v>
+      </c>
+      <c r="B919" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C919" s="16" t="inlineStr">
+        <is>
+          <t>Détective Conan (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D919" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/D%C3%A9tective_Conan</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="16" t="n">
+        <v>463</v>
+      </c>
+      <c r="B920" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C920" s="16" t="inlineStr">
+        <is>
+          <t>Gōshō Aoyama (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D920" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/G%C5%8Dsh%C5%8D_Aoyama</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="16" t="n">
+        <v>464</v>
+      </c>
+      <c r="B921" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C921" s="16" t="inlineStr">
+        <is>
+          <t>Slam Dunk (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D921" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/From_TV_Animation_Slam_Dunk</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="16" t="n">
+        <v>464</v>
+      </c>
+      <c r="B922" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C922" s="16" t="inlineStr">
+        <is>
+          <t>Takehiko Inoue (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D922" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Takehiko_Inoue</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="16" t="n">
+        <v>465</v>
+      </c>
+      <c r="B923" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C923" s="16" t="inlineStr">
+        <is>
+          <t>Demon Slayer / Kimetsu no Yaiba (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D923" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Demon_Slayer:_Kimetsu_no_Yaiba</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="16" t="n">
+        <v>466</v>
+      </c>
+      <c r="B924" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C924" s="16" t="inlineStr">
+        <is>
+          <t>L'Attaque des Titans (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D924" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/L%27Attaque_des_Titans</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="16" t="n">
+        <v>466</v>
+      </c>
+      <c r="B925" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C925" s="16" t="inlineStr">
+        <is>
+          <t>Hajime Isayama (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D925" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Hajime_Isayama</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="16" t="n">
+        <v>467</v>
+      </c>
+      <c r="B926" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C926" s="16" t="inlineStr">
+        <is>
+          <t>Death Note (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D926" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Death_Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="16" t="n">
+        <v>468</v>
+      </c>
+      <c r="B927" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C927" s="16" t="inlineStr">
+        <is>
+          <t>Fullmetal Alchemist (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D927" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Fullmetal_Alchemist</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="16" t="n">
+        <v>468</v>
+      </c>
+      <c r="B928" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C928" s="16" t="inlineStr">
+        <is>
+          <t>Hiromu Arakawa (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D928" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Hiromu_Arakawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="16" t="n">
+        <v>469</v>
+      </c>
+      <c r="B929" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C929" s="16" t="inlineStr">
+        <is>
+          <t>My Hero Academia (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D929" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Boku_no_Hero_Academia</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="16" t="n">
+        <v>470</v>
+      </c>
+      <c r="B930" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C930" s="16" t="inlineStr">
+        <is>
+          <t>Bleach (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D930" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Bleach</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="16" t="n">
+        <v>471</v>
+      </c>
+      <c r="B931" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C931" s="16" t="inlineStr">
+        <is>
+          <t>JoJo's Bizarre Adventure (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D931" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/JoJo's_Bizarre_Adventure</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="16" t="n">
+        <v>471</v>
+      </c>
+      <c r="B932" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C932" s="16" t="inlineStr">
+        <is>
+          <t>Hirohiko Araki (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D932" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Hirohiko_Araki</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="16" t="n">
+        <v>472</v>
+      </c>
+      <c r="B933" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C933" s="16" t="inlineStr">
+        <is>
+          <t>Sailor Moon (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D933" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Sailor_Moon</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="16" t="n">
+        <v>472</v>
+      </c>
+      <c r="B934" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C934" s="16" t="inlineStr">
+        <is>
+          <t>Naoko Takeuchi (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D934" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Naoko_Takeuchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="16" t="n">
+        <v>473</v>
+      </c>
+      <c r="B935" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C935" s="16" t="inlineStr">
+        <is>
+          <t>Akira (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D935" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Akira_(manga)</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="16" t="n">
+        <v>473</v>
+      </c>
+      <c r="B936" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C936" s="16" t="inlineStr">
+        <is>
+          <t>Katsuhiro Ōtomo (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D936" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Katsuhiro_%C5%8Ctomo</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="16" t="n">
+        <v>474</v>
+      </c>
+      <c r="B937" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C937" s="16" t="inlineStr">
+        <is>
+          <t>Astro Boy / Astro, le petit robot (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D937" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Astro,_le_petit_robot</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="16" t="n">
+        <v>474</v>
+      </c>
+      <c r="B938" s="16" t="inlineStr">
+        <is>
+          <t>wikipedia</t>
+        </is>
+      </c>
+      <c r="C938" s="16" t="inlineStr">
+        <is>
+          <t>Osamu Tezuka (Wikipédia)</t>
+        </is>
+      </c>
+      <c r="D938" s="16" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Osamushi_Tezuka</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>